<commit_message>
plan_compras: Stein viernes y Franco domingo confirmados por Gonzalo (20/09)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -120,7 +120,7 @@
     <t>2026-09-20</t>
   </si>
   <si>
-    <t>domingo (supuesto 20/09)</t>
+    <t>confirmado por Gonzalo 20/09: cargo domingo</t>
   </si>
   <si>
     <t>Gilson</t>
@@ -138,7 +138,7 @@
     <t>Stein</t>
   </si>
   <si>
-    <t>dia supuesto (no lo dijo)</t>
+    <t>confirmado por Gonzalo 20/09: viernes</t>
   </si>
   <si>
     <t>Agrocurupa</t>

</xml_diff>

<commit_message>
plan_compras: Milciades lunes y martes (2 mas), Gilson pasa al viernes (Gonzalo 20/09)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
   <si>
     <t>fecha</t>
   </si>
@@ -126,6 +126,9 @@
     <t>Gilson</t>
   </si>
   <si>
+    <t>Gonzalo 20/09: al final carga viernes (era martes)</t>
+  </si>
+  <si>
     <t>Chabat</t>
   </si>
   <si>
@@ -142,6 +145,12 @@
   </si>
   <si>
     <t>Agrocurupa</t>
+  </si>
+  <si>
+    <t>Gonzalo 20/09</t>
+  </si>
+  <si>
+    <t>Milciades, agregado el 20/09</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -229,7 +238,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/MM/yyyy"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -261,7 +272,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -271,6 +282,7 @@
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -281,7 +293,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -778,10 +790,10 @@
     </row>
     <row r="16">
       <c r="A16" s="1">
-        <v>46287</v>
+        <v>46290</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C16" s="0" t="s">
         <v>33</v>
@@ -805,7 +817,7 @@
         <v>15</v>
       </c>
       <c r="J16" s="0" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17">
@@ -889,7 +901,7 @@
         <v>24</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G19" s="0" t="s">
         <v>14</v>
@@ -918,10 +930,10 @@
         <v>23</v>
       </c>
       <c r="E20" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="F20" s="0" t="s">
         <v>37</v>
-      </c>
-      <c r="F20" s="0" t="s">
-        <v>36</v>
       </c>
       <c r="G20" s="0" t="s">
         <v>14</v>
@@ -950,10 +962,10 @@
         <v>23</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G21" s="0" t="s">
         <v>14</v>
@@ -982,7 +994,7 @@
         <v>23</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F22" s="0" t="s">
         <v>31</v>
@@ -997,7 +1009,7 @@
         <v>15</v>
       </c>
       <c r="J22" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="23">
@@ -1046,7 +1058,7 @@
         <v>23</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F24" s="0" t="s">
         <v>31</v>
@@ -1094,6 +1106,70 @@
       </c>
       <c r="J25" s="0" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9">
+        <v>46286</v>
+      </c>
+      <c r="B26" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="D26" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H26" s="0">
+        <v>980</v>
+      </c>
+      <c r="I26" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="J26" s="0" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9">
+        <v>46287</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H27" s="0">
+        <v>980</v>
+      </c>
+      <c r="I27" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="J27" s="0" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1116,7 +1192,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>23</v>
@@ -1125,7 +1201,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>8</v>
@@ -1148,10 +1224,10 @@
         <v>1230</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3">
@@ -1168,10 +1244,10 @@
         <v>1230</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4">
@@ -1188,10 +1264,10 @@
         <v>1230</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5">
@@ -1208,10 +1284,10 @@
         <v>1230</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6">
@@ -1228,10 +1304,10 @@
         <v>1230</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7">
@@ -1248,10 +1324,10 @@
         <v>1230</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1269,57 +1345,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1367,10 +1443,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3">
@@ -1384,10 +1460,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4">
@@ -1395,16 +1471,16 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5">
@@ -1412,16 +1488,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1457,10 +1533,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="G1" s="8" t="s">
         <v>8</v>
@@ -1486,7 +1562,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3">
@@ -1509,7 +1585,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4">
@@ -1520,7 +1596,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -1532,7 +1608,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5">
@@ -1543,7 +1619,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -1555,7 +1631,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6">
@@ -1563,7 +1639,7 @@
         <v>46281</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C6" s="0" t="s">
         <v>23</v>
@@ -1578,7 +1654,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7">
@@ -1586,7 +1662,7 @@
         <v>46281</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C7" s="0" t="s">
         <v>12</v>
@@ -1601,7 +1677,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8">
@@ -1609,10 +1685,10 @@
         <v>46281</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -1624,7 +1700,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9">
@@ -1632,10 +1708,10 @@
         <v>46281</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -1647,7 +1723,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10">
@@ -1670,7 +1746,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11">
@@ -1693,7 +1769,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12">
@@ -1704,7 +1780,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -1716,7 +1792,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13">
@@ -1727,7 +1803,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -1739,7 +1815,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan_compras: venta por semana (15.000 sem 21/09, 17.000 sem 28/09 en adelante) en simulador y ventas_plan
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t>fecha</t>
   </si>
@@ -159,10 +159,25 @@
     <t>BO</t>
   </si>
   <si>
-    <t>promedio 4 reportes ERP (sem 38) x 6 dias</t>
-  </si>
-  <si>
-    <t>reemplazar por el plan de ventas</t>
+    <t>promedio ERP sem 38 (ya paso)</t>
+  </si>
+  <si>
+    <t>total 13700 · mix BR 52,6 % / PY 38,4 % / BO 9,0 % (reportes ERP sem 38)</t>
+  </si>
+  <si>
+    <t>Gonzalo 20/09: estimado 15.000</t>
+  </si>
+  <si>
+    <t>total 15000 · mix BR 52,6 % / PY 38,4 % / BO 9,0 % (reportes ERP sem 38)</t>
+  </si>
+  <si>
+    <t>Gonzalo 20/09: estimado 17.000</t>
+  </si>
+  <si>
+    <t>total 17000 · mix BR 52,6 % / PY 38,4 % / BO 9,0 % (reportes ERP sem 38)</t>
+  </si>
+  <si>
+    <t>SUPUESTO = semana anterior (confirmar)</t>
   </si>
   <si>
     <t>notas</t>
@@ -276,12 +291,12 @@
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1109,7 +1124,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="9">
+      <c r="A26" s="8">
         <v>46286</v>
       </c>
       <c r="B26" s="0" t="s">
@@ -1141,7 +1156,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="9">
+      <c r="A27" s="8">
         <v>46287</v>
       </c>
       <c r="B27" s="0" t="s">
@@ -1191,34 +1206,34 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="9">
         <v>46279</v>
       </c>
       <c r="B2" s="0">
-        <v>7200</v>
+        <v>7210</v>
       </c>
       <c r="C2" s="0">
-        <v>5250</v>
+        <v>5260</v>
       </c>
       <c r="D2" s="0">
         <v>1230</v>
@@ -1231,103 +1246,103 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3">
+      <c r="A3" s="9">
         <v>46286</v>
       </c>
       <c r="B3" s="0">
-        <v>7200</v>
+        <v>7890</v>
       </c>
       <c r="C3" s="0">
-        <v>5250</v>
+        <v>5760</v>
       </c>
       <c r="D3" s="0">
-        <v>1230</v>
+        <v>1350</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3">
+      <c r="A4" s="9">
         <v>46293</v>
       </c>
       <c r="B4" s="0">
-        <v>7200</v>
+        <v>8940</v>
       </c>
       <c r="C4" s="0">
-        <v>5250</v>
+        <v>6530</v>
       </c>
       <c r="D4" s="0">
-        <v>1230</v>
+        <v>1530</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3">
+      <c r="A5" s="9">
         <v>46300</v>
       </c>
       <c r="B5" s="0">
-        <v>7200</v>
+        <v>8940</v>
       </c>
       <c r="C5" s="0">
-        <v>5250</v>
+        <v>6530</v>
       </c>
       <c r="D5" s="0">
-        <v>1230</v>
+        <v>1530</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3">
+      <c r="A6" s="9">
         <v>46307</v>
       </c>
       <c r="B6" s="0">
-        <v>7200</v>
+        <v>8940</v>
       </c>
       <c r="C6" s="0">
-        <v>5250</v>
+        <v>6530</v>
       </c>
       <c r="D6" s="0">
-        <v>1230</v>
+        <v>1530</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3">
+      <c r="A7" s="9">
         <v>46314</v>
       </c>
       <c r="B7" s="0">
-        <v>7200</v>
+        <v>8940</v>
       </c>
       <c r="C7" s="0">
-        <v>5250</v>
+        <v>6530</v>
       </c>
       <c r="D7" s="0">
-        <v>1230</v>
+        <v>1530</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1345,57 +1360,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1416,24 +1431,24 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5">
+      <c r="A2" s="4">
         <v>46282</v>
       </c>
       <c r="B2" s="0" t="s">
@@ -1443,14 +1458,14 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5">
+      <c r="A3" s="4">
         <v>46282</v>
       </c>
       <c r="B3" s="0" t="s">
@@ -1460,14 +1475,14 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="4">
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
@@ -1477,27 +1492,27 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5">
+      <c r="A5" s="4">
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1520,30 +1535,30 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="8" t="s">
+      <c r="E1" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" s="7" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7">
+      <c r="A2" s="6">
         <v>46280</v>
       </c>
       <c r="B2" s="0" t="s">
@@ -1562,11 +1577,11 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7">
+      <c r="A3" s="6">
         <v>46280</v>
       </c>
       <c r="B3" s="0" t="s">
@@ -1585,11 +1600,11 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7">
+      <c r="A4" s="6">
         <v>46280</v>
       </c>
       <c r="B4" s="0" t="s">
@@ -1608,18 +1623,18 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7">
+      <c r="A5" s="6">
         <v>46280</v>
       </c>
       <c r="B5" s="0" t="s">
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -1631,15 +1646,15 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7">
+      <c r="A6" s="6">
         <v>46281</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C6" s="0" t="s">
         <v>23</v>
@@ -1654,15 +1669,15 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7">
+      <c r="A7" s="6">
         <v>46281</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C7" s="0" t="s">
         <v>12</v>
@@ -1677,15 +1692,15 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7">
+      <c r="A8" s="6">
         <v>46281</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C8" s="0" t="s">
         <v>46</v>
@@ -1700,18 +1715,18 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7">
+      <c r="A9" s="6">
         <v>46281</v>
       </c>
       <c r="B9" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" s="0" t="s">
         <v>69</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>64</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -1723,11 +1738,11 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7">
+      <c r="A10" s="6">
         <v>46284</v>
       </c>
       <c r="B10" s="0" t="s">
@@ -1746,11 +1761,11 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7">
+      <c r="A11" s="6">
         <v>46284</v>
       </c>
       <c r="B11" s="0" t="s">
@@ -1769,11 +1784,11 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7">
+      <c r="A12" s="6">
         <v>46284</v>
       </c>
       <c r="B12" s="0" t="s">
@@ -1792,18 +1807,18 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7">
+      <c r="A13" s="6">
         <v>46284</v>
       </c>
       <c r="B13" s="0" t="s">
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -1815,7 +1830,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cargas 2026 + plan_compras: semanas 38-40 segun las notas de Gonzalo del 25/09 (sem 21-26 con precios; sem 28/09-03/10 planificada)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
   <si>
     <t>fecha</t>
   </si>
@@ -120,37 +120,94 @@
     <t>2026-09-20</t>
   </si>
   <si>
-    <t>confirmado por Gonzalo 20/09: cargo domingo</t>
+    <t>Etimex</t>
+  </si>
+  <si>
+    <t>Gonzalo 25/09 (nota)</t>
+  </si>
+  <si>
+    <t>nota 25/09: martes, R$ 38</t>
+  </si>
+  <si>
+    <t>Axt</t>
+  </si>
+  <si>
+    <t>nota 25/09: viernes, R$ 36</t>
+  </si>
+  <si>
+    <t>Agrocurupa</t>
+  </si>
+  <si>
+    <t>Nilton</t>
+  </si>
+  <si>
+    <t>nota 25/09: viernes, precio ilegible (3?)</t>
   </si>
   <si>
     <t>Gilson</t>
   </si>
   <si>
-    <t>Gonzalo 20/09: al final carga viernes (era martes)</t>
+    <t>nota 25/09: viernes, R$ 42</t>
+  </si>
+  <si>
+    <t>nota 25/09: Franco 3, domingo</t>
+  </si>
+  <si>
+    <t>nota 25/09: Franco 3, lunes</t>
+  </si>
+  <si>
+    <t>nota 25/09: Franco 3, martes</t>
+  </si>
+  <si>
+    <t>nota 25/09: Alvarito 2, lunes</t>
+  </si>
+  <si>
+    <t>nota 25/09: Alvarito 2, martes</t>
+  </si>
+  <si>
+    <t>nota 25/09: Milciades 2, lunes</t>
+  </si>
+  <si>
+    <t>nota 25/09: Milciades 2, martes</t>
+  </si>
+  <si>
+    <t>mie</t>
+  </si>
+  <si>
+    <t>2026-09-27</t>
+  </si>
+  <si>
+    <t>nota 25/09: cuarta</t>
+  </si>
+  <si>
+    <t>nota 25/09: sexta</t>
   </si>
   <si>
     <t>Chabat</t>
   </si>
   <si>
+    <t>nota 25/09: tersa</t>
+  </si>
+  <si>
     <t>Josemar</t>
   </si>
   <si>
+    <t>Stein</t>
+  </si>
+  <si>
     <t>Marconi</t>
   </si>
   <si>
-    <t>Stein</t>
-  </si>
-  <si>
-    <t>confirmado por Gonzalo 20/09: viernes</t>
-  </si>
-  <si>
-    <t>Agrocurupa</t>
-  </si>
-  <si>
-    <t>Gonzalo 20/09</t>
-  </si>
-  <si>
-    <t>Milciades, agregado el 20/09</t>
+    <t>nota 25/09: Milciades 1, dia no indicado (supuesto lunes)</t>
+  </si>
+  <si>
+    <t>nota 25/09: Diego 2, dia no indicado (supuesto lunes)</t>
+  </si>
+  <si>
+    <t>nota 25/09: Diego 2, dia no indicado (supuesto martes)</t>
+  </si>
+  <si>
+    <t>nota 25/09: Alvarito 1, dia no indicado (supuesto lunes)</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -238,9 +295,6 @@
   </si>
   <si>
     <t>reporte ERP 15/09</t>
-  </si>
-  <si>
-    <t>mie</t>
   </si>
   <si>
     <t>reporte ERP 16/09</t>
@@ -308,7 +362,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -708,103 +762,103 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1">
-        <v>46285</v>
+      <c r="A13" s="9">
+        <v>46287</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C13" s="0" t="s">
         <v>33</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H13" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J13" s="0" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1">
-        <v>46286</v>
+      <c r="A14" s="9">
+        <v>46290</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C14" s="0" t="s">
         <v>33</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="H14" s="0">
-        <v>980</v>
+        <v>936</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1">
-        <v>46286</v>
+      <c r="A15" s="9">
+        <v>46290</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C15" s="0" t="s">
         <v>33</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H15" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J15" s="0" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1">
+      <c r="A16" s="9">
         <v>46290</v>
       </c>
       <c r="B16" s="0" t="s">
@@ -817,62 +871,62 @@
         <v>23</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H16" s="0">
         <v>1008</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J16" s="0" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1">
-        <v>46287</v>
+      <c r="A17" s="9">
+        <v>46285</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C17" s="0" t="s">
         <v>33</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G17" s="0" t="s">
         <v>14</v>
       </c>
       <c r="H17" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J17" s="0" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1">
-        <v>46287</v>
+      <c r="A18" s="9">
+        <v>46286</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C18" s="0" t="s">
         <v>33</v>
@@ -893,213 +947,213 @@
         <v>980</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J18" s="0" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1">
-        <v>46290</v>
+      <c r="A19" s="9">
+        <v>46287</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C19" s="0" t="s">
         <v>33</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G19" s="0" t="s">
         <v>14</v>
       </c>
       <c r="H19" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I19" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J19" s="0" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1">
-        <v>46290</v>
+      <c r="A20" s="9">
+        <v>46286</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C20" s="0" t="s">
         <v>33</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G20" s="0" t="s">
         <v>14</v>
       </c>
       <c r="H20" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I20" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J20" s="0" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1">
-        <v>46290</v>
+      <c r="A21" s="9">
+        <v>46287</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C21" s="0" t="s">
         <v>33</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G21" s="0" t="s">
         <v>14</v>
       </c>
       <c r="H21" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I21" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J21" s="0" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1">
-        <v>46290</v>
+      <c r="A22" s="9">
+        <v>46286</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C22" s="0" t="s">
         <v>33</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="G22" s="0" t="s">
         <v>14</v>
       </c>
       <c r="H22" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I22" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J22" s="0" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1">
-        <v>46290</v>
+      <c r="A23" s="9">
+        <v>46287</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C23" s="0" t="s">
         <v>33</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="H23" s="0">
-        <v>936</v>
+        <v>980</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J23" s="0" t="s">
-        <v>14</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1">
-        <v>46290</v>
+      <c r="A24" s="9">
+        <v>46295</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="D24" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H24" s="0">
         <v>1008</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J24" s="0" t="s">
-        <v>14</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1">
-        <v>46291</v>
+      <c r="A25" s="9">
+        <v>46297</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="D25" s="0" t="s">
         <v>23</v>
@@ -1111,80 +1165,432 @@
         <v>25</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H25" s="0">
         <v>1008</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J25" s="0" t="s">
-        <v>14</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8">
-        <v>46286</v>
+      <c r="A26" s="9">
+        <v>46295</v>
       </c>
       <c r="B26" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D26" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E26" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="F26" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G26" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H26" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I26" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J26" s="0" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9">
+        <v>46297</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C27" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D27" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E27" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="F27" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G27" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H27" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I27" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J27" s="0" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9">
+        <v>46294</v>
+      </c>
+      <c r="B28" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D28" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E28" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F28" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="G28" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H28" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I28" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J28" s="0" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9">
+        <v>46297</v>
+      </c>
+      <c r="B29" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C29" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D29" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E29" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F29" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="G29" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H29" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I29" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J29" s="0" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9">
+        <v>46297</v>
+      </c>
+      <c r="B30" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D30" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E30" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="F30" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G30" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="H30" s="0">
+        <v>936</v>
+      </c>
+      <c r="I30" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J30" s="0" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9">
+        <v>46297</v>
+      </c>
+      <c r="B31" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C31" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D31" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E31" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="F31" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G31" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H31" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I31" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J31" s="0" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9">
+        <v>46297</v>
+      </c>
+      <c r="B32" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C32" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D32" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E32" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="F32" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G32" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H32" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I32" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J32" s="0" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9">
+        <v>46297</v>
+      </c>
+      <c r="B33" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C33" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D33" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E33" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="F33" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G33" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H33" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I33" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J33" s="0" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9">
+        <v>46297</v>
+      </c>
+      <c r="B34" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C34" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D34" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E34" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F34" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="G34" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H34" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I34" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J34" s="0" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9">
+        <v>46293</v>
+      </c>
+      <c r="B35" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="C26" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="D26" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E26" s="0" t="s">
+      <c r="C35" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D35" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="F26" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G26" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H26" s="0">
+      <c r="F35" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G35" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H35" s="0">
         <v>980</v>
       </c>
-      <c r="I26" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="J26" s="0" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="8">
-        <v>46287</v>
-      </c>
-      <c r="B27" s="0" t="s">
+      <c r="I35" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J35" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9">
+        <v>46293</v>
+      </c>
+      <c r="B36" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D36" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="F36" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G36" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H36" s="0">
+        <v>980</v>
+      </c>
+      <c r="I36" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J36" s="0" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9">
+        <v>46294</v>
+      </c>
+      <c r="B37" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="C27" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="D27" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E27" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="F27" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G27" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H27" s="0">
+      <c r="C37" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D37" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="F37" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G37" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H37" s="0">
         <v>980</v>
       </c>
-      <c r="I27" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="J27" s="0" t="s">
-        <v>44</v>
+      <c r="I37" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J37" s="0" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9">
+        <v>46293</v>
+      </c>
+      <c r="B38" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C38" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D38" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="F38" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G38" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H38" s="0">
+        <v>980</v>
+      </c>
+      <c r="I38" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J38" s="0" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1207,7 +1613,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -1216,7 +1622,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>8</v>
@@ -1226,7 +1632,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9">
+      <c r="A2" s="8">
         <v>46279</v>
       </c>
       <c r="B2" s="0">
@@ -1239,14 +1645,14 @@
         <v>1230</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>48</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9">
+      <c r="A3" s="8">
         <v>46286</v>
       </c>
       <c r="B3" s="0">
@@ -1259,14 +1665,14 @@
         <v>1350</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9">
+      <c r="A4" s="8">
         <v>46293</v>
       </c>
       <c r="B4" s="0">
@@ -1279,14 +1685,14 @@
         <v>1530</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9">
+      <c r="A5" s="8">
         <v>46300</v>
       </c>
       <c r="B5" s="0">
@@ -1299,14 +1705,14 @@
         <v>1530</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9">
+      <c r="A6" s="8">
         <v>46307</v>
       </c>
       <c r="B6" s="0">
@@ -1319,14 +1725,14 @@
         <v>1530</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9">
+      <c r="A7" s="8">
         <v>46314</v>
       </c>
       <c r="B7" s="0">
@@ -1339,10 +1745,10 @@
         <v>1530</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1360,57 +1766,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1458,10 +1864,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3">
@@ -1475,10 +1881,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4">
@@ -1486,16 +1892,16 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5">
@@ -1503,16 +1909,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1548,10 +1954,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -1577,7 +1983,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3">
@@ -1600,7 +2006,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4">
@@ -1611,7 +2017,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -1623,7 +2029,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5">
@@ -1634,7 +2040,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -1646,7 +2052,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6">
@@ -1654,7 +2060,7 @@
         <v>46281</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="C6" s="0" t="s">
         <v>23</v>
@@ -1669,7 +2075,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7">
@@ -1677,7 +2083,7 @@
         <v>46281</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="C7" s="0" t="s">
         <v>12</v>
@@ -1692,7 +2098,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8">
@@ -1700,10 +2106,10 @@
         <v>46281</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -1715,7 +2121,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
     </row>
     <row r="9">
@@ -1723,10 +2129,10 @@
         <v>46281</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -1738,7 +2144,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10">
@@ -1761,7 +2167,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11">
@@ -1784,7 +2190,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12">
@@ -1795,7 +2201,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -1807,7 +2213,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13">
@@ -1818,7 +2224,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -1830,7 +2236,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
conteo de camaras 26/09 (fotos + listado ERP por camara): BR 9709, PY 15617, BO 1646; simulador arranca del 26/09
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
   <si>
     <t>fecha</t>
   </si>
@@ -286,6 +286,21 @@
   </si>
   <si>
     <t>referencia; Ecuador no entra en el plan</t>
+  </si>
+  <si>
+    <t>fuentes\stock\2026-09-26_conteo_camaras.xlsx</t>
+  </si>
+  <si>
+    <t>ZAC 8701 (listado ERP por camara) + Coronel Raiz cam 5 1.008 (supuesto Brasil: 1.008 = un camion BR)</t>
+  </si>
+  <si>
+    <t>ZAC 13673 (listado ERP por camara) + Coronel Raiz cam 2 1.944 (supuesto Paraguay, como el 17/09)</t>
+  </si>
+  <si>
+    <t>ZAC camaras 2, 25 y 30 (Porvenir). OJO: la foto de Bolivia dice CAM 2 = 423 y el ERP 23 (camara 2 total 111): se tomo el ERP</t>
+  </si>
+  <si>
+    <t>solo ZAC (Coronel Raiz no vino); referencia, Ecuador no entra en el plan</t>
   </si>
   <si>
     <t>kg</t>
@@ -344,7 +359,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -355,6 +370,7 @@
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1830,7 +1846,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -1923,6 +1939,74 @@
       </c>
       <c r="E5" s="0" t="s">
         <v>89</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11">
+        <v>46291</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="0">
+        <v>9709</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11">
+        <v>46291</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="0">
+        <v>15617</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11">
+        <v>46291</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="0">
+        <v>1646</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11">
+        <v>46291</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="C9" s="0">
+        <v>6833</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1958,10 +2042,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -1987,7 +2071,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3">
@@ -2010,7 +2094,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4">
@@ -2033,7 +2117,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5">
@@ -2056,7 +2140,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6">
@@ -2079,7 +2163,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7">
@@ -2102,7 +2186,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8">
@@ -2125,7 +2209,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9">
@@ -2148,7 +2232,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10">
@@ -2171,7 +2255,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11">
@@ -2194,7 +2278,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12">
@@ -2217,7 +2301,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="13">
@@ -2240,7 +2324,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14">
@@ -2263,7 +2347,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
@@ -2286,7 +2370,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16">
@@ -2309,7 +2393,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17">
@@ -2332,7 +2416,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan_compras: venta sem 28/09 = 16.000 (BO 1 carga, resto BR/PY); simulador regenerado
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
   <si>
     <t>fecha</t>
   </si>
@@ -228,13 +228,16 @@
     <t>total 15000 · mix BR 52,6 % / PY 38,4 % / BO 9,0 % (reportes ERP sem 38)</t>
   </si>
   <si>
-    <t>Gonzalo 20/09: estimado 17.000</t>
+    <t>Gonzalo 27/09: se pide vender 16.000; Bolivia 1 carga, el resto PY y BR</t>
+  </si>
+  <si>
+    <t>total 16.000 = BO 1.050 (1 carga) + BR 8640 + PY 6310 (resto repartido con el mix BR/PY del ERP sem 38, 'no importa el orden')</t>
+  </si>
+  <si>
+    <t>SUPUESTO = semana anterior (confirmar)</t>
   </si>
   <si>
     <t>total 17000 · mix BR 52,6 % / PY 38,4 % / BO 9,0 % (reportes ERP sem 38)</t>
-  </si>
-  <si>
-    <t>SUPUESTO = semana anterior (confirmar)</t>
   </si>
   <si>
     <t>notas</t>
@@ -1696,13 +1699,13 @@
         <v>46293</v>
       </c>
       <c r="B4" s="0">
-        <v>8940</v>
+        <v>8640</v>
       </c>
       <c r="C4" s="0">
-        <v>6530</v>
+        <v>6310</v>
       </c>
       <c r="D4" s="0">
-        <v>1530</v>
+        <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
         <v>70</v>
@@ -1728,7 +1731,7 @@
         <v>72</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6">
@@ -1748,7 +1751,7 @@
         <v>72</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7">
@@ -1768,7 +1771,7 @@
         <v>72</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1786,57 +1789,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1884,10 +1887,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3">
@@ -1901,10 +1904,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4">
@@ -1918,10 +1921,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5">
@@ -1929,16 +1932,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6">
@@ -1952,10 +1955,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7">
@@ -1969,10 +1972,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8">
@@ -1986,10 +1989,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9">
@@ -1997,16 +2000,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -2042,10 +2045,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -2071,7 +2074,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3">
@@ -2094,7 +2097,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4">
@@ -2117,7 +2120,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5">
@@ -2128,7 +2131,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -2140,7 +2143,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6">
@@ -2163,7 +2166,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7">
@@ -2186,7 +2189,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8">
@@ -2209,7 +2212,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9">
@@ -2220,7 +2223,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -2232,7 +2235,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10">
@@ -2255,7 +2258,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
@@ -2278,7 +2281,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
@@ -2301,7 +2304,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
@@ -2312,7 +2315,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -2324,7 +2327,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
@@ -2347,7 +2350,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15">
@@ -2358,7 +2361,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -2370,7 +2373,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16">
@@ -2393,7 +2396,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17">
@@ -2416,7 +2419,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan_compras: un solo stock de banana (BR + PY + BO) con minimo 22.500 al sabado, Bolivia incluida; lag por origen; supuesto 5 camiones PY por semana (dom-mar)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -10,13 +10,14 @@
     <sheet name="notas" sheetId="3" r:id="rId4"/>
     <sheet name="conteo" sheetId="4" r:id="rId5"/>
     <sheet name="ventas_erp" sheetId="5" r:id="rId6"/>
+    <sheet name="supuestos" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="106">
   <si>
     <t>fecha</t>
   </si>
@@ -322,6 +323,18 @@
   </si>
   <si>
     <t>reporte ERP 26/09 10:16</t>
+  </si>
+  <si>
+    <t>clave</t>
+  </si>
+  <si>
+    <t>valor</t>
+  </si>
+  <si>
+    <t>py_camiones_semana</t>
+  </si>
+  <si>
+    <t>Gonzalo 27/09/2026: Paraguay carga domingo, lunes y martes (entra siempre en la semana); por lo general 5/6 camiones. Se usa en las semanas sin cargas PY dictadas ni en el Plan.</t>
   </si>
 </sst>
 </file>
@@ -2425,4 +2438,41 @@
   </sheetData>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="20.870376586914062" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="159.2061767578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="0">
+        <v>5</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>105</v>
+      </c>
+    </row>
+  </sheetData>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
plan de compras: carga extra Stein mie 30/09 (Nilton); resumen: 'falta 1 camion' en singular y texto en log en modo prueba
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
   <si>
     <t>fecha</t>
   </si>
@@ -209,6 +209,12 @@
   </si>
   <si>
     <t>nota 25/09: Alvarito 1, nota completa 25/09: lunes confirmado</t>
+  </si>
+  <si>
+    <t>Gonzalo 27/09 (chat)</t>
+  </si>
+  <si>
+    <t>carga extra: "asi cierro mejor pensando en futuro" (ademas de la sexta ya dictada)</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -398,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -1627,6 +1633,38 @@
       </c>
       <c r="J38" s="0" t="s">
         <v>63</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9">
+        <v>46295</v>
+      </c>
+      <c r="B39" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C39" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D39" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E39" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="F39" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G39" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H39" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I39" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="J39" s="0" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1649,7 +1687,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -1658,7 +1696,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>8</v>
@@ -1681,10 +1719,10 @@
         <v>1230</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3">
@@ -1701,10 +1739,10 @@
         <v>1350</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4">
@@ -1721,10 +1759,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5">
@@ -1741,10 +1779,10 @@
         <v>1530</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6">
@@ -1761,10 +1799,10 @@
         <v>1530</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7">
@@ -1781,10 +1819,10 @@
         <v>1530</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1802,57 +1840,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1900,10 +1938,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3">
@@ -1917,10 +1955,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4">
@@ -1928,16 +1966,16 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5">
@@ -1945,16 +1983,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6">
@@ -1968,10 +2006,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7">
@@ -1985,10 +2023,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8">
@@ -1996,16 +2034,16 @@
         <v>46291</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C8" s="0">
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9">
@@ -2013,16 +2051,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -2058,10 +2096,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -2087,7 +2125,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
@@ -2110,7 +2148,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4">
@@ -2121,7 +2159,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -2133,7 +2171,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -2144,7 +2182,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -2156,7 +2194,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6">
@@ -2179,7 +2217,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7">
@@ -2202,7 +2240,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8">
@@ -2213,7 +2251,7 @@
         <v>51</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -2225,7 +2263,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9">
@@ -2236,7 +2274,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -2248,7 +2286,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10">
@@ -2271,7 +2309,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11">
@@ -2294,7 +2332,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12">
@@ -2305,7 +2343,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -2317,7 +2355,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13">
@@ -2328,7 +2366,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -2340,7 +2378,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14">
@@ -2363,7 +2401,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="15">
@@ -2374,7 +2412,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -2386,7 +2424,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16">
@@ -2409,7 +2447,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17">
@@ -2420,7 +2458,7 @@
         <v>29</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D17" s="0">
         <v>134</v>
@@ -2432,7 +2470,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2452,10 +2490,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -2463,13 +2501,13 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: venta semanal real por origen (ERP jul-sep) en xlsx/JSON/Excel; sigma real, mix real en supuestos; Excel con grupos PY, Diego Fernandez y notas legibles
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -11,13 +11,14 @@
     <sheet name="conteo" sheetId="4" r:id="rId5"/>
     <sheet name="ventas_erp" sheetId="5" r:id="rId6"/>
     <sheet name="supuestos" sheetId="6" r:id="rId7"/>
+    <sheet name="ventas_semanales" sheetId="7" r:id="rId8"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
   <si>
     <t>fecha</t>
   </si>
@@ -223,16 +224,13 @@
     <t>BO</t>
   </si>
   <si>
-    <t>promedio ERP sem 38 (ya paso)</t>
-  </si>
-  <si>
-    <t>total 13700 · mix BR 52,6 % / PY 38,4 % / BO 9,0 % (reportes ERP sem 38)</t>
-  </si>
-  <si>
-    <t>Gonzalo 20/09: estimado 15.000</t>
-  </si>
-  <si>
-    <t>total 15000 · mix BR 52,6 % / PY 38,4 % / BO 9,0 % (reportes ERP sem 38)</t>
+    <t>REAL ERP (captura 29/09/2026)</t>
+  </si>
+  <si>
+    <t>total 15851 real (antes: total 13700 · mix BR 52,6 % / PY 38,4 % / BO 9,0 % (reportes ERP sem 38))</t>
+  </si>
+  <si>
+    <t>total 14845 real (antes: total 15000 · mix BR 52,6 % / PY 38,4 % / BO 9,0 % (reportes ERP sem 38))</t>
   </si>
   <si>
     <t>Gonzalo 27/09: se pide vender 16.000; Bolivia 1 carga, el resto PY y BR</t>
@@ -244,7 +242,7 @@
     <t>SUPUESTO = semana anterior (confirmar)</t>
   </si>
   <si>
-    <t>total 17000 · mix BR 52,6 % / PY 38,4 % / BO 9,0 % (reportes ERP sem 38)</t>
+    <t>total 17000 · mix real ERP ult. 4 sem (31/08-21/09): BR 61.7 % / PY 31.2 % / BO 7.1 %</t>
   </si>
   <si>
     <t>notas</t>
@@ -341,6 +339,18 @@
   </si>
   <si>
     <t>Gonzalo 27/09/2026: Paraguay carga domingo, lunes y martes (entra siempre en la semana); por lo general 5/6 camiones. Se usa en las semanas sin cargas PY dictadas ni en el Plan.</t>
+  </si>
+  <si>
+    <t>sabado</t>
+  </si>
+  <si>
+    <t>total_banana</t>
+  </si>
+  <si>
+    <t>ERP, venta semanal por agrupacion (captura 29/09/2026, fuentes\ventas)</t>
+  </si>
+  <si>
+    <t>Venta real en cajas por semana (lunes a sabado) y origen, del reporte semanal del ERP. total_banana = BR + PY + BO (Ecuador va por otro canal). Agregar una fila por semana cerrada; el paso 5j la lleva al JSON (ventas_reales) y la planilla Excel la usa para el desvio y el desvio estandar.</t>
   </si>
 </sst>
 </file>
@@ -381,7 +391,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -394,6 +404,8 @@
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1710,13 +1722,13 @@
         <v>46279</v>
       </c>
       <c r="B2" s="0">
-        <v>7210</v>
+        <v>8590</v>
       </c>
       <c r="C2" s="0">
-        <v>5260</v>
+        <v>5769</v>
       </c>
       <c r="D2" s="0">
-        <v>1230</v>
+        <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
         <v>68</v>
@@ -1730,19 +1742,19 @@
         <v>46286</v>
       </c>
       <c r="B3" s="0">
-        <v>7890</v>
+        <v>7919</v>
       </c>
       <c r="C3" s="0">
-        <v>5760</v>
+        <v>6221</v>
       </c>
       <c r="D3" s="0">
-        <v>1350</v>
+        <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" s="0" t="s">
         <v>70</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="4">
@@ -1759,10 +1771,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" s="0" t="s">
         <v>72</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="5">
@@ -1770,19 +1782,19 @@
         <v>46300</v>
       </c>
       <c r="B5" s="0">
-        <v>8940</v>
+        <v>10496</v>
       </c>
       <c r="C5" s="0">
-        <v>6530</v>
+        <v>5304</v>
       </c>
       <c r="D5" s="0">
-        <v>1530</v>
+        <v>1200</v>
       </c>
       <c r="E5" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" s="0" t="s">
         <v>74</v>
-      </c>
-      <c r="F5" s="0" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="6">
@@ -1790,19 +1802,19 @@
         <v>46307</v>
       </c>
       <c r="B6" s="0">
-        <v>8940</v>
+        <v>10496</v>
       </c>
       <c r="C6" s="0">
-        <v>6530</v>
+        <v>5304</v>
       </c>
       <c r="D6" s="0">
-        <v>1530</v>
+        <v>1200</v>
       </c>
       <c r="E6" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="F6" s="0" t="s">
         <v>74</v>
-      </c>
-      <c r="F6" s="0" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="7">
@@ -1810,19 +1822,19 @@
         <v>46314</v>
       </c>
       <c r="B7" s="0">
-        <v>8940</v>
+        <v>10496</v>
       </c>
       <c r="C7" s="0">
-        <v>6530</v>
+        <v>5304</v>
       </c>
       <c r="D7" s="0">
-        <v>1530</v>
+        <v>1200</v>
       </c>
       <c r="E7" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="F7" s="0" t="s">
         <v>74</v>
-      </c>
-      <c r="F7" s="0" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1840,57 +1852,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1938,10 +1950,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="E2" s="0" t="s">
         <v>87</v>
-      </c>
-      <c r="E2" s="0" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="3">
@@ -1955,10 +1967,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4">
@@ -1972,10 +1984,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5">
@@ -1983,16 +1995,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6">
@@ -2006,10 +2018,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="E6" s="0" t="s">
         <v>93</v>
-      </c>
-      <c r="E6" s="0" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="7">
@@ -2023,10 +2035,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8">
@@ -2040,10 +2052,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9">
@@ -2051,16 +2063,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2096,10 +2108,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>98</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>99</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -2125,7 +2137,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3">
@@ -2148,7 +2160,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4">
@@ -2171,7 +2183,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5">
@@ -2182,7 +2194,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -2194,7 +2206,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6">
@@ -2217,7 +2229,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -2240,7 +2252,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">
@@ -2263,7 +2275,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -2274,7 +2286,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -2286,7 +2298,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10">
@@ -2309,7 +2321,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11">
@@ -2332,7 +2344,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12">
@@ -2355,7 +2367,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13">
@@ -2366,7 +2378,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -2378,7 +2390,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14">
@@ -2401,7 +2413,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15">
@@ -2412,7 +2424,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -2424,7 +2436,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16">
@@ -2447,7 +2459,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="17">
@@ -2470,7 +2482,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -2490,10 +2502,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="0" t="s">
         <v>104</v>
-      </c>
-      <c r="B1" s="0" t="s">
-        <v>105</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -2501,13 +2513,371 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
+        <v>106</v>
+      </c>
+    </row>
+  </sheetData>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="8" max="8" width="70" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="12" t="s">
         <v>107</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13">
+        <v>46209</v>
+      </c>
+      <c r="B2" s="13">
+        <v>46214</v>
+      </c>
+      <c r="C2" s="0">
+        <v>8884</v>
+      </c>
+      <c r="D2" s="0">
+        <v>4896</v>
+      </c>
+      <c r="E2" s="0">
+        <v>713</v>
+      </c>
+      <c r="F2" s="0">
+        <v>7277</v>
+      </c>
+      <c r="G2" s="0">
+        <f>C2+D2+E2</f>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13">
+        <v>46216</v>
+      </c>
+      <c r="B3" s="13">
+        <v>46221</v>
+      </c>
+      <c r="C3" s="0">
+        <v>8547</v>
+      </c>
+      <c r="D3" s="0">
+        <v>3607</v>
+      </c>
+      <c r="E3" s="0">
+        <v>344</v>
+      </c>
+      <c r="F3" s="0">
+        <v>6900</v>
+      </c>
+      <c r="G3" s="0">
+        <f>C3+D3+E3</f>
+      </c>
+      <c r="H3" s="0" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13">
+        <v>46223</v>
+      </c>
+      <c r="B4" s="13">
+        <v>46228</v>
+      </c>
+      <c r="C4" s="0">
+        <v>11589</v>
+      </c>
+      <c r="D4" s="0">
+        <v>2140</v>
+      </c>
+      <c r="E4" s="0">
+        <v>1025</v>
+      </c>
+      <c r="F4" s="0">
+        <v>7601</v>
+      </c>
+      <c r="G4" s="0">
+        <f>C4+D4+E4</f>
+      </c>
+      <c r="H4" s="0" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13">
+        <v>46230</v>
+      </c>
+      <c r="B5" s="13">
+        <v>46235</v>
+      </c>
+      <c r="C5" s="0">
+        <v>9196</v>
+      </c>
+      <c r="D5" s="0">
+        <v>4748</v>
+      </c>
+      <c r="E5" s="0">
+        <v>0</v>
+      </c>
+      <c r="F5" s="0">
+        <v>7884</v>
+      </c>
+      <c r="G5" s="0">
+        <f>C5+D5+E5</f>
+      </c>
+      <c r="H5" s="0" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13">
+        <v>46237</v>
+      </c>
+      <c r="B6" s="13">
+        <v>46242</v>
+      </c>
+      <c r="C6" s="0">
+        <v>9880</v>
+      </c>
+      <c r="D6" s="0">
+        <v>5192</v>
+      </c>
+      <c r="E6" s="0">
+        <v>866</v>
+      </c>
+      <c r="F6" s="0">
+        <v>7601</v>
+      </c>
+      <c r="G6" s="0">
+        <f>C6+D6+E6</f>
+      </c>
+      <c r="H6" s="0" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13">
+        <v>46244</v>
+      </c>
+      <c r="B7" s="13">
+        <v>46249</v>
+      </c>
+      <c r="C7" s="0">
+        <v>6972</v>
+      </c>
+      <c r="D7" s="0">
+        <v>6201</v>
+      </c>
+      <c r="E7" s="0">
+        <v>1816</v>
+      </c>
+      <c r="F7" s="0">
+        <v>6647</v>
+      </c>
+      <c r="G7" s="0">
+        <f>C7+D7+E7</f>
+      </c>
+      <c r="H7" s="0" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13">
+        <v>46251</v>
+      </c>
+      <c r="B8" s="13">
+        <v>46256</v>
+      </c>
+      <c r="C8" s="0">
+        <v>8041</v>
+      </c>
+      <c r="D8" s="0">
+        <v>5861</v>
+      </c>
+      <c r="E8" s="0">
+        <v>34</v>
+      </c>
+      <c r="F8" s="0">
+        <v>6290</v>
+      </c>
+      <c r="G8" s="0">
+        <f>C8+D8+E8</f>
+      </c>
+      <c r="H8" s="0" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13">
+        <v>46258</v>
+      </c>
+      <c r="B9" s="13">
+        <v>46263</v>
+      </c>
+      <c r="C9" s="0">
+        <v>6633</v>
+      </c>
+      <c r="D9" s="0">
+        <v>7058</v>
+      </c>
+      <c r="E9" s="0">
+        <v>1051</v>
+      </c>
+      <c r="F9" s="0">
+        <v>4669</v>
+      </c>
+      <c r="G9" s="0">
+        <f>C9+D9+E9</f>
+      </c>
+      <c r="H9" s="0" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13">
+        <v>46265</v>
+      </c>
+      <c r="B10" s="13">
+        <v>46270</v>
+      </c>
+      <c r="C10" s="0">
+        <v>11032</v>
+      </c>
+      <c r="D10" s="0">
+        <v>5369</v>
+      </c>
+      <c r="E10" s="0">
+        <v>873</v>
+      </c>
+      <c r="F10" s="0">
+        <v>7102</v>
+      </c>
+      <c r="G10" s="0">
+        <f>C10+D10+E10</f>
+      </c>
+      <c r="H10" s="0" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13">
+        <v>46272</v>
+      </c>
+      <c r="B11" s="13">
+        <v>46277</v>
+      </c>
+      <c r="C11" s="0">
+        <v>12293</v>
+      </c>
+      <c r="D11" s="0">
+        <v>2770</v>
+      </c>
+      <c r="E11" s="0">
+        <v>1486</v>
+      </c>
+      <c r="F11" s="0">
+        <v>6924</v>
+      </c>
+      <c r="G11" s="0">
+        <f>C11+D11+E11</f>
+      </c>
+      <c r="H11" s="0" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13">
+        <v>46279</v>
+      </c>
+      <c r="B12" s="13">
+        <v>46284</v>
+      </c>
+      <c r="C12" s="0">
+        <v>8590</v>
+      </c>
+      <c r="D12" s="0">
+        <v>5769</v>
+      </c>
+      <c r="E12" s="0">
+        <v>1492</v>
+      </c>
+      <c r="F12" s="0">
+        <v>6673</v>
+      </c>
+      <c r="G12" s="0">
+        <f>C12+D12+E12</f>
+      </c>
+      <c r="H12" s="0" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13">
+        <v>46286</v>
+      </c>
+      <c r="B13" s="13">
+        <v>46291</v>
+      </c>
+      <c r="C13" s="0">
+        <v>7919</v>
+      </c>
+      <c r="D13" s="0">
+        <v>6221</v>
+      </c>
+      <c r="E13" s="0">
+        <v>705</v>
+      </c>
+      <c r="F13" s="0">
+        <v>6718</v>
+      </c>
+      <c r="G13" s="0">
+        <f>C13+D13+E13</f>
+      </c>
+      <c r="H13" s="0" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: cargas dictadas semana 05-10/10 (BR 11, PY 6)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
   <si>
     <t>fecha</t>
   </si>
@@ -216,6 +216,45 @@
   </si>
   <si>
     <t>carga extra: "asi cierro mejor pensando en futuro" (ademas de la sexta ya dictada)</t>
+  </si>
+  <si>
+    <t>2026-10-04</t>
+  </si>
+  <si>
+    <t>Gonzalo 30/09 (chat)</t>
+  </si>
+  <si>
+    <t>nota 30/09: tersa; transportista supuesto = semana anterior</t>
+  </si>
+  <si>
+    <t>nota 30/09: sexta; transportista supuesto = semana anterior</t>
+  </si>
+  <si>
+    <t>nota 30/09: cuarta; transportista supuesto = semana anterior</t>
+  </si>
+  <si>
+    <t>nota 30/09: sabado (descarga martes 13, suma a la semana siguiente); transportista supuesto = semana anterior</t>
+  </si>
+  <si>
+    <t>nota 30/09: Milciades 2, lunes</t>
+  </si>
+  <si>
+    <t>nota 30/09: Milciades 2, martes</t>
+  </si>
+  <si>
+    <t>nota 30/09: Diego 2, lunes</t>
+  </si>
+  <si>
+    <t>nota 30/09: Diego 2, martes</t>
+  </si>
+  <si>
+    <t>Paraguay GM</t>
+  </si>
+  <si>
+    <t>nota 30/09: Guido 1, miercoles (con 4 dias descarga domingo 11: suma a la semana siguiente)</t>
+  </si>
+  <si>
+    <t>nota 30/09: Alvarito 1, lunes</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -416,7 +455,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -1677,6 +1716,550 @@
       </c>
       <c r="J39" s="0" t="s">
         <v>65</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9">
+        <v>46301</v>
+      </c>
+      <c r="B40" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C40" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D40" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E40" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="F40" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="G40" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H40" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I40" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J40" s="0" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9">
+        <v>46304</v>
+      </c>
+      <c r="B41" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C41" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D41" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E41" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="F41" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="G41" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H41" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I41" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J41" s="0" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="9">
+        <v>46302</v>
+      </c>
+      <c r="B42" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C42" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E42" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="F42" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G42" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H42" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I42" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J42" s="0" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9">
+        <v>46304</v>
+      </c>
+      <c r="B43" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C43" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D43" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E43" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="F43" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G43" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H43" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I43" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J43" s="0" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9">
+        <v>46301</v>
+      </c>
+      <c r="B44" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C44" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D44" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E44" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="F44" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G44" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="H44" s="0">
+        <v>936</v>
+      </c>
+      <c r="I44" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J44" s="0" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9">
+        <v>46305</v>
+      </c>
+      <c r="B45" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C45" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D45" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E45" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="F45" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G45" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="H45" s="0">
+        <v>936</v>
+      </c>
+      <c r="I45" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J45" s="0" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9">
+        <v>46302</v>
+      </c>
+      <c r="B46" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C46" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D46" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E46" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F46" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="G46" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H46" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I46" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J46" s="0" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9">
+        <v>46304</v>
+      </c>
+      <c r="B47" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C47" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D47" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E47" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F47" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="G47" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H47" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I47" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J47" s="0" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9">
+        <v>46304</v>
+      </c>
+      <c r="B48" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C48" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D48" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E48" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="F48" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G48" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H48" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I48" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J48" s="0" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="9">
+        <v>46301</v>
+      </c>
+      <c r="B49" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C49" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D49" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E49" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="F49" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G49" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H49" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I49" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J49" s="0" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9">
+        <v>46304</v>
+      </c>
+      <c r="B50" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C50" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D50" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E50" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F50" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="G50" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H50" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I50" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J50" s="0" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9">
+        <v>46300</v>
+      </c>
+      <c r="B51" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C51" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D51" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="F51" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G51" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H51" s="0">
+        <v>980</v>
+      </c>
+      <c r="I51" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J51" s="0" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="9">
+        <v>46301</v>
+      </c>
+      <c r="B52" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C52" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D52" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E52" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="F52" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G52" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H52" s="0">
+        <v>980</v>
+      </c>
+      <c r="I52" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J52" s="0" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="9">
+        <v>46300</v>
+      </c>
+      <c r="B53" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C53" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D53" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E53" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="F53" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G53" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H53" s="0">
+        <v>980</v>
+      </c>
+      <c r="I53" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J53" s="0" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="9">
+        <v>46301</v>
+      </c>
+      <c r="B54" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C54" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D54" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E54" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="F54" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G54" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H54" s="0">
+        <v>980</v>
+      </c>
+      <c r="I54" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J54" s="0" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="9">
+        <v>46302</v>
+      </c>
+      <c r="B55" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C55" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D55" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="F55" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G55" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H55" s="0">
+        <v>980</v>
+      </c>
+      <c r="I55" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J55" s="0" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9">
+        <v>46300</v>
+      </c>
+      <c r="B56" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C56" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D56" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E56" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="F56" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G56" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H56" s="0">
+        <v>980</v>
+      </c>
+      <c r="I56" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J56" s="0" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1699,7 +2282,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -1708,7 +2291,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>8</v>
@@ -1731,10 +2314,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3">
@@ -1751,10 +2334,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4">
@@ -1771,10 +2354,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5">
@@ -1791,10 +2374,10 @@
         <v>1200</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6">
@@ -1811,10 +2394,10 @@
         <v>1200</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7">
@@ -1831,10 +2414,10 @@
         <v>1200</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -1852,57 +2435,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -1950,10 +2533,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
@@ -1967,10 +2550,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4">
@@ -1978,16 +2561,16 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5">
@@ -1995,16 +2578,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6">
@@ -2018,10 +2601,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7">
@@ -2035,10 +2618,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8">
@@ -2046,16 +2629,16 @@
         <v>46291</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C8" s="0">
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9">
@@ -2063,16 +2646,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2108,10 +2691,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -2137,7 +2720,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3">
@@ -2160,7 +2743,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4">
@@ -2171,7 +2754,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -2183,7 +2766,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5">
@@ -2194,7 +2777,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -2206,7 +2789,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6">
@@ -2229,7 +2812,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7">
@@ -2252,7 +2835,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8">
@@ -2263,7 +2846,7 @@
         <v>51</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -2275,7 +2858,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9">
@@ -2286,7 +2869,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -2298,7 +2881,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10">
@@ -2321,7 +2904,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
     </row>
     <row r="11">
@@ -2344,7 +2927,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12">
@@ -2355,7 +2938,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -2367,7 +2950,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
     </row>
     <row r="13">
@@ -2378,7 +2961,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -2390,7 +2973,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14">
@@ -2413,7 +2996,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15">
@@ -2424,7 +3007,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -2436,7 +3019,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16">
@@ -2459,7 +3042,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
     </row>
     <row r="17">
@@ -2470,7 +3053,7 @@
         <v>29</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="D17" s="0">
         <v>134</v>
@@ -2482,7 +3065,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -2502,10 +3085,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -2513,13 +3096,13 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -2539,10 +3122,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -2551,13 +3134,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -2586,7 +3169,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3">
@@ -2612,7 +3195,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4">
@@ -2638,7 +3221,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5">
@@ -2664,7 +3247,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6">
@@ -2690,7 +3273,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7">
@@ -2716,7 +3299,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8">
@@ -2742,7 +3325,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9">
@@ -2768,7 +3351,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10">
@@ -2794,7 +3377,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11">
@@ -2820,7 +3403,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12">
@@ -2846,7 +3429,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13">
@@ -2872,12 +3455,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: semana 05-10/10 version final (BR 11 con Josemar mar y Cassio mie+sab; PY 5, sin Guido)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
   <si>
     <t>fecha</t>
   </si>
@@ -248,13 +248,16 @@
     <t>nota 30/09: Diego 2, martes</t>
   </si>
   <si>
-    <t>Paraguay GM</t>
-  </si>
-  <si>
-    <t>nota 30/09: Guido 1, miercoles (con 4 dias descarga domingo 11: suma a la semana siguiente)</t>
-  </si>
-  <si>
     <t>nota 30/09: Alvarito 1, lunes</t>
+  </si>
+  <si>
+    <t>Gonzalo 01/10 (chat)</t>
+  </si>
+  <si>
+    <t>nota 01/10: tersa; transportista supuesto = semana anterior</t>
+  </si>
+  <si>
+    <t>nota 01/10: cuarta (antes martes, sacada el 30/09); transportista supuesto</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -1816,10 +1819,10 @@
     </row>
     <row r="43">
       <c r="A43" s="9">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C43" s="0" t="s">
         <v>66</v>
@@ -1828,30 +1831,30 @@
         <v>23</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="H43" s="0">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I43" s="0" t="s">
         <v>67</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9">
-        <v>46305</v>
+        <v>46302</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="C44" s="0" t="s">
         <v>66</v>
@@ -1860,30 +1863,30 @@
         <v>23</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="H44" s="0">
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="I44" s="0" t="s">
         <v>67</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C45" s="0" t="s">
         <v>66</v>
@@ -1907,7 +1910,7 @@
         <v>67</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="46">
@@ -1924,13 +1927,13 @@
         <v>23</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="G46" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H46" s="0">
         <v>1008</v>
@@ -1944,10 +1947,10 @@
     </row>
     <row r="47">
       <c r="A47" s="9">
-        <v>46304</v>
+        <v>46301</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C47" s="0" t="s">
         <v>66</v>
@@ -1956,7 +1959,7 @@
         <v>23</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="F47" s="0" t="s">
         <v>40</v>
@@ -1971,15 +1974,15 @@
         <v>67</v>
       </c>
       <c r="J47" s="0" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9">
-        <v>46301</v>
+        <v>46304</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C48" s="0" t="s">
         <v>66</v>
@@ -1988,13 +1991,13 @@
         <v>23</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H48" s="0">
         <v>1008</v>
@@ -2003,47 +2006,47 @@
         <v>67</v>
       </c>
       <c r="J48" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="9">
-        <v>46304</v>
+        <v>46300</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C49" s="0" t="s">
         <v>66</v>
       </c>
       <c r="D49" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="F49" s="0" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="G49" s="0" t="s">
         <v>14</v>
       </c>
       <c r="H49" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I49" s="0" t="s">
         <v>67</v>
       </c>
       <c r="J49" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="9">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C50" s="0" t="s">
         <v>66</v>
@@ -2067,15 +2070,15 @@
         <v>67</v>
       </c>
       <c r="J50" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="9">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C51" s="0" t="s">
         <v>66</v>
@@ -2084,7 +2087,7 @@
         <v>12</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F51" s="0" t="s">
         <v>14</v>
@@ -2099,15 +2102,15 @@
         <v>67</v>
       </c>
       <c r="J51" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="9">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C52" s="0" t="s">
         <v>66</v>
@@ -2131,15 +2134,15 @@
         <v>67</v>
       </c>
       <c r="J52" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="9">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C53" s="0" t="s">
         <v>66</v>
@@ -2148,7 +2151,7 @@
         <v>12</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F53" s="0" t="s">
         <v>14</v>
@@ -2163,71 +2166,71 @@
         <v>67</v>
       </c>
       <c r="J53" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="9">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C54" s="0" t="s">
         <v>66</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H54" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="J54" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="9">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="C55" s="0" t="s">
         <v>66</v>
       </c>
       <c r="D55" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="H55" s="0">
-        <v>980</v>
+        <v>936</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="J55" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -2250,7 +2253,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -2259,7 +2262,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>8</v>
@@ -2282,10 +2285,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3">
@@ -2302,10 +2305,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4">
@@ -2322,10 +2325,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5">
@@ -2342,10 +2345,10 @@
         <v>1200</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6">
@@ -2362,10 +2365,10 @@
         <v>1200</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7">
@@ -2382,10 +2385,10 @@
         <v>1200</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -2403,57 +2406,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -2501,10 +2504,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3">
@@ -2518,10 +2521,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4">
@@ -2529,16 +2532,16 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5">
@@ -2546,16 +2549,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6">
@@ -2569,10 +2572,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7">
@@ -2586,10 +2589,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8">
@@ -2597,16 +2600,16 @@
         <v>46291</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C8" s="0">
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9">
@@ -2614,16 +2617,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -2659,10 +2662,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -2688,7 +2691,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3">
@@ -2711,7 +2714,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4">
@@ -2722,7 +2725,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -2734,7 +2737,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5">
@@ -2745,7 +2748,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -2757,7 +2760,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6">
@@ -2780,7 +2783,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7">
@@ -2803,7 +2806,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8">
@@ -2814,7 +2817,7 @@
         <v>51</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -2826,7 +2829,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9">
@@ -2837,7 +2840,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -2849,7 +2852,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10">
@@ -2872,7 +2875,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11">
@@ -2895,7 +2898,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12">
@@ -2906,7 +2909,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -2918,7 +2921,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13">
@@ -2929,7 +2932,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -2941,7 +2944,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14">
@@ -2964,7 +2967,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15">
@@ -2975,7 +2978,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -2987,7 +2990,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16">
@@ -3010,7 +3013,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17">
@@ -3021,7 +3024,7 @@
         <v>29</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D17" s="0">
         <v>134</v>
@@ -3033,7 +3036,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -3053,10 +3056,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3064,13 +3067,13 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -3090,10 +3093,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3102,13 +3105,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3137,7 +3140,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3">
@@ -3163,7 +3166,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4">
@@ -3189,7 +3192,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5">
@@ -3215,7 +3218,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6">
@@ -3241,7 +3244,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7">
@@ -3267,7 +3270,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8">
@@ -3293,7 +3296,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9">
@@ -3319,7 +3322,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10">
@@ -3345,7 +3348,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11">
@@ -3371,7 +3374,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12">
@@ -3397,7 +3400,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13">
@@ -3423,12 +3426,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: minimo 25.000 al sabado (verano) y 1 camion de Bolivia por semana como supuesto, en WhatsApp/simulador/Excel
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="129">
   <si>
     <t>fecha</t>
   </si>
@@ -381,6 +381,18 @@
   </si>
   <si>
     <t>Gonzalo 27/09/2026: Paraguay carga domingo, lunes y martes (entra siempre en la semana); por lo general 5/6 camiones. Se usa en las semanas sin cargas PY dictadas ni en el Plan.</t>
+  </si>
+  <si>
+    <t>bo_camiones_semana</t>
+  </si>
+  <si>
+    <t>Gonzalo 01/10/2026: "de Bolivia vamos a descargar uno por semana siempre". Se agrega un camion BO supuesto en cada semana de venta sin descarga BO, cargado 6 dias antes del lunes (si esa fecha no paso).</t>
+  </si>
+  <si>
+    <t>minimo_cajas_sabado</t>
+  </si>
+  <si>
+    <t>Gonzalo 01/10/2026: "comienza el calor en Uruguay, levanta las ventas, quieren mantener 25 mil cajas al cierre del sabado contando todo, PY BOL y BR". Antes 22.500 (27/09).</t>
   </si>
   <si>
     <t>sabado</t>
@@ -3046,7 +3058,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.870376586914062" customWidth="1"/>
@@ -3074,6 +3086,28 @@
       </c>
       <c r="C2" s="0" t="s">
         <v>120</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="B3" s="0">
+        <v>1</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="B4" s="0">
+        <v>25000</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -3096,7 +3130,7 @@
         <v>80</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3111,7 +3145,7 @@
         <v>104</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3140,7 +3174,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3">
@@ -3166,7 +3200,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4">
@@ -3192,7 +3226,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5">
@@ -3218,7 +3252,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6">
@@ -3244,7 +3278,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7">
@@ -3270,7 +3304,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8">
@@ -3296,7 +3330,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9">
@@ -3322,7 +3356,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10">
@@ -3348,7 +3382,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11">
@@ -3374,7 +3408,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12">
@@ -3400,7 +3434,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13">
@@ -3426,12 +3460,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Guido martes 13/10; supuestos PY completan hasta 5 cuando hay dictadas parciales
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="133">
   <si>
     <t>fecha</t>
   </si>
@@ -261,6 +261,15 @@
   </si>
   <si>
     <t>nota 01/10 (v4): sexta (Gonzalo: "prefiero cerrar en casi 25 mil que casi 26 mil"); transportista supuesto = semana anterior</t>
+  </si>
+  <si>
+    <t>2026-10-11</t>
+  </si>
+  <si>
+    <t>Paraguay GM</t>
+  </si>
+  <si>
+    <t>nota 01/10: Guido 1, martes 13 (reactivacion; sin cargar desde julio). Con 4 dias descarga el sabado 17.</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -473,7 +482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -2214,6 +2223,32 @@
       </c>
       <c r="J54" s="0" t="s">
         <v>80</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="9">
+        <v>46308</v>
+      </c>
+      <c r="B55" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C55" s="0" t="s">
+        <v>81</v>
+      </c>
+      <c r="D55" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="H55" s="0">
+        <v>980</v>
+      </c>
+      <c r="I55" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="J55" s="0" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -2236,7 +2271,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -2245,7 +2280,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>8</v>
@@ -2268,10 +2303,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3">
@@ -2288,10 +2323,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4">
@@ -2308,10 +2343,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5">
@@ -2328,10 +2363,10 @@
         <v>1278</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6">
@@ -2348,10 +2383,10 @@
         <v>1278</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7">
@@ -2368,10 +2403,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -2389,57 +2424,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2487,10 +2522,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3">
@@ -2504,10 +2539,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4">
@@ -2515,16 +2550,16 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5">
@@ -2532,16 +2567,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6">
@@ -2555,10 +2590,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7">
@@ -2572,10 +2607,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8">
@@ -2583,16 +2618,16 @@
         <v>46291</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C8" s="0">
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9">
@@ -2600,16 +2635,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -2645,10 +2680,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -2674,7 +2709,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3">
@@ -2697,7 +2732,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4">
@@ -2708,7 +2743,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -2720,7 +2755,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5">
@@ -2731,7 +2766,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -2743,7 +2778,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6">
@@ -2766,7 +2801,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7">
@@ -2789,7 +2824,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8">
@@ -2800,7 +2835,7 @@
         <v>51</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -2812,7 +2847,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9">
@@ -2823,7 +2858,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -2835,7 +2870,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10">
@@ -2858,7 +2893,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11">
@@ -2881,7 +2916,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12">
@@ -2892,7 +2927,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -2904,7 +2939,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13">
@@ -2915,7 +2950,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -2927,7 +2962,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14">
@@ -2950,7 +2985,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15">
@@ -2961,7 +2996,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -2973,7 +3008,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16">
@@ -2996,7 +3031,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17">
@@ -3007,7 +3042,7 @@
         <v>29</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D17" s="0">
         <v>134</v>
@@ -3019,7 +3054,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -3039,10 +3074,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3050,35 +3085,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B3" s="0">
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -3098,10 +3133,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3110,13 +3145,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3145,7 +3180,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3">
@@ -3171,7 +3206,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4">
@@ -3197,7 +3232,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5">
@@ -3223,7 +3258,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6">
@@ -3249,7 +3284,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7">
@@ -3275,7 +3310,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8">
@@ -3301,7 +3336,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9">
@@ -3327,7 +3362,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10">
@@ -3353,7 +3388,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11">
@@ -3379,7 +3414,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12">
@@ -3405,7 +3440,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13">
@@ -3431,12 +3466,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: semanas 05-10/10 (final) y 12-17/10 dictadas por Gonzalo
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -221,55 +221,55 @@
     <t>2026-10-04</t>
   </si>
   <si>
-    <t>Gonzalo 30/09 (chat)</t>
-  </si>
-  <si>
-    <t>nota 30/09: tersa; transportista supuesto = semana anterior</t>
-  </si>
-  <si>
-    <t>nota 30/09: sexta; transportista supuesto = semana anterior</t>
-  </si>
-  <si>
-    <t>nota 30/09: cuarta; transportista supuesto = semana anterior</t>
-  </si>
-  <si>
-    <t>nota 30/09: Milciades 2, lunes</t>
-  </si>
-  <si>
-    <t>nota 30/09: Milciades 2, martes</t>
-  </si>
-  <si>
-    <t>nota 30/09: Diego 2, lunes</t>
-  </si>
-  <si>
-    <t>nota 30/09: Diego 2, martes</t>
-  </si>
-  <si>
-    <t>nota 30/09: Alvarito 1, lunes</t>
-  </si>
-  <si>
-    <t>Gonzalo 01/10 (chat)</t>
-  </si>
-  <si>
-    <t>nota 01/10: tersa; transportista supuesto = semana anterior</t>
-  </si>
-  <si>
-    <t>nota 01/10: cuarta (antes martes, sacada el 30/09); transportista supuesto</t>
-  </si>
-  <si>
-    <t>Gonzalo 01/10 (chat, v3)</t>
-  </si>
-  <si>
-    <t>nota 01/10 (v4): sexta (Gonzalo: "prefiero cerrar en casi 25 mil que casi 26 mil"); transportista supuesto = semana anterior</t>
+    <t>Gonzalo 02/10 (chat)</t>
+  </si>
+  <si>
+    <t>nota 02/10: tersa; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>nota 02/10: sexta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>nota 02/10: cuarta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>nota 02/10: segunda; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>Celso</t>
+  </si>
+  <si>
+    <t>nota 02/10: cuarta. PRODUCTOR NUEVO: no esta en productores.xlsx ni en Aloha; falta nombre completo y transporte</t>
+  </si>
+  <si>
+    <t>nota 02/10: Milciades 2, lunes</t>
+  </si>
+  <si>
+    <t>nota 02/10: Milciades 2, martes</t>
+  </si>
+  <si>
+    <t>nota 02/10: Diego 2, lunes</t>
+  </si>
+  <si>
+    <t>nota 02/10: Diego 2, martes</t>
+  </si>
+  <si>
+    <t>nota 02/10: Alvarito 1, lunes</t>
   </si>
   <si>
     <t>2026-10-11</t>
   </si>
   <si>
+    <t>nota 02/10: sabado (descarga martes 20, semana siguiente); transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>nota 02/10: cuarta. PRODUCTOR NUEVO (ver semana anterior)</t>
+  </si>
+  <si>
     <t>Paraguay GM</t>
   </si>
   <si>
-    <t>nota 01/10: Guido 1, martes 13 (reactivacion; sin cargar desde julio). Con 4 dias descarga el sabado 17.</t>
+    <t>nota 02/10: Guido 1, martes (reactivacion; descarga sabado 17)</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -482,7 +482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -1855,16 +1855,16 @@
         <v>23</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="H43" s="0">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I43" s="0" t="s">
         <v>67</v>
@@ -1875,10 +1875,10 @@
     </row>
     <row r="44">
       <c r="A44" s="9">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C44" s="0" t="s">
         <v>66</v>
@@ -1902,15 +1902,15 @@
         <v>67</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C45" s="0" t="s">
         <v>66</v>
@@ -1919,13 +1919,13 @@
         <v>23</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>58</v>
+        <v>24</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H45" s="0">
         <v>1008</v>
@@ -1934,15 +1934,15 @@
         <v>67</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="9">
-        <v>46304</v>
+        <v>46301</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C46" s="0" t="s">
         <v>66</v>
@@ -1951,13 +1951,13 @@
         <v>23</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="G46" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H46" s="0">
         <v>1008</v>
@@ -1966,24 +1966,24 @@
         <v>67</v>
       </c>
       <c r="J46" s="0" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="9">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="C47" s="0" t="s">
         <v>66</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="F47" s="0" t="s">
         <v>14</v>
@@ -1992,21 +1992,21 @@
         <v>14</v>
       </c>
       <c r="H47" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I47" s="0" t="s">
         <v>67</v>
       </c>
       <c r="J47" s="0" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C48" s="0" t="s">
         <v>66</v>
@@ -2030,15 +2030,15 @@
         <v>67</v>
       </c>
       <c r="J48" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="9">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C49" s="0" t="s">
         <v>66</v>
@@ -2047,7 +2047,7 @@
         <v>12</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F49" s="0" t="s">
         <v>14</v>
@@ -2062,15 +2062,15 @@
         <v>67</v>
       </c>
       <c r="J49" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="9">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C50" s="0" t="s">
         <v>66</v>
@@ -2094,15 +2094,15 @@
         <v>67</v>
       </c>
       <c r="J50" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="9">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C51" s="0" t="s">
         <v>66</v>
@@ -2111,7 +2111,7 @@
         <v>12</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F51" s="0" t="s">
         <v>14</v>
@@ -2126,91 +2126,91 @@
         <v>67</v>
       </c>
       <c r="J51" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="9">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C52" s="0" t="s">
         <v>66</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G52" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H52" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I52" s="0" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="J52" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="9">
-        <v>46302</v>
+        <v>46308</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="D53" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H53" s="0">
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="J53" s="0" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="9">
-        <v>46304</v>
+        <v>46312</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="D54" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="G54" s="0" t="s">
         <v>34</v>
@@ -2219,7 +2219,7 @@
         <v>1008</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="J54" s="0" t="s">
         <v>80</v>
@@ -2227,27 +2227,481 @@
     </row>
     <row r="55">
       <c r="A55" s="9">
+        <v>46309</v>
+      </c>
+      <c r="B55" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C55" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D55" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E55" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="F55" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G55" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H55" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I55" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J55" s="0" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9">
+        <v>46311</v>
+      </c>
+      <c r="B56" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C56" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D56" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E56" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="F56" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G56" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H56" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I56" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J56" s="0" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="9">
         <v>46308</v>
       </c>
-      <c r="B55" s="0" t="s">
+      <c r="B57" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="C55" s="0" t="s">
+      <c r="C57" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D57" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E57" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="F57" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G57" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="H57" s="0">
+        <v>936</v>
+      </c>
+      <c r="I57" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J57" s="0" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="9">
+        <v>46311</v>
+      </c>
+      <c r="B58" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C58" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D58" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E58" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="F58" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G58" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="H58" s="0">
+        <v>936</v>
+      </c>
+      <c r="I58" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J58" s="0" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="9">
+        <v>46309</v>
+      </c>
+      <c r="B59" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C59" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D59" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E59" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F59" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="G59" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H59" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I59" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J59" s="0" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="9">
+        <v>46311</v>
+      </c>
+      <c r="B60" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C60" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D60" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E60" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F60" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="G60" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H60" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I60" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J60" s="0" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="9">
+        <v>46309</v>
+      </c>
+      <c r="B61" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C61" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D61" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E61" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="F61" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G61" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H61" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I61" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J61" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="D55" s="0" t="s">
+    </row>
+    <row r="62">
+      <c r="A62" s="9">
+        <v>46309</v>
+      </c>
+      <c r="B62" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C62" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D62" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E62" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F62" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="G62" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H62" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I62" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J62" s="0" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="9">
+        <v>46311</v>
+      </c>
+      <c r="B63" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C63" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D63" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E63" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="F63" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G63" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H63" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I63" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J63" s="0" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="9">
+        <v>46307</v>
+      </c>
+      <c r="B64" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C64" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D64" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="E55" s="0" t="s">
+      <c r="E64" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="F64" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G64" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H64" s="0">
+        <v>980</v>
+      </c>
+      <c r="I64" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J64" s="0" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="9">
+        <v>46307</v>
+      </c>
+      <c r="B65" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C65" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D65" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E65" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="F65" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G65" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H65" s="0">
+        <v>980</v>
+      </c>
+      <c r="I65" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J65" s="0" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="9">
+        <v>46308</v>
+      </c>
+      <c r="B66" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C66" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D66" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E66" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="F66" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G66" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H66" s="0">
+        <v>980</v>
+      </c>
+      <c r="I66" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J66" s="0" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="9">
+        <v>46307</v>
+      </c>
+      <c r="B67" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C67" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D67" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E67" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="F67" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G67" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H67" s="0">
+        <v>980</v>
+      </c>
+      <c r="I67" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J67" s="0" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="9">
+        <v>46308</v>
+      </c>
+      <c r="B68" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C68" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D68" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E68" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="F68" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G68" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H68" s="0">
+        <v>980</v>
+      </c>
+      <c r="I68" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J68" s="0" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="9">
+        <v>46308</v>
+      </c>
+      <c r="B69" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C69" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D69" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E69" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="H55" s="0">
+      <c r="F69" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G69" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H69" s="0">
         <v>980</v>
       </c>
-      <c r="I55" s="0" t="s">
-        <v>76</v>
-      </c>
-      <c r="J55" s="0" t="s">
+      <c r="I69" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="J69" s="0" t="s">
         <v>83</v>
       </c>
     </row>

</xml_diff>

<commit_message>
conteo de camaras 03/10 (BR 12.269, PY 9.676, BO 1.500): cierre 23.445, plan regenerado; WhatsApp muestra el sabado contado como cierre real
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
   <si>
     <t>fecha</t>
   </si>
@@ -369,6 +369,21 @@
   </si>
   <si>
     <t>ZAC 6833 + Coronel Raiz 14904; referencia, Ecuador no entra en el plan</t>
+  </si>
+  <si>
+    <t>fuentes\stock\2026-10-03_conteo_camaras.xlsx</t>
+  </si>
+  <si>
+    <t>planilla de camaras de Gonzalo (CAM naranja = Brasil): ZAC 10253 en 10 camaras + Coronel Raiz cam 4 2016</t>
+  </si>
+  <si>
+    <t>planilla de camaras (CAM gris = Paraguay): ZAC 9676 en 8 camaras</t>
+  </si>
+  <si>
+    <t>planilla Bolivia: ZAC cam 30 (750, gas 29-sep) y cam 25 (750)</t>
+  </si>
+  <si>
+    <t>planilla Carton: solo ZAC, 7 camaras; Coronel Raiz no vino; referencia, Ecuador no entra en el plan</t>
   </si>
   <si>
     <t>kg</t>
@@ -463,7 +478,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -478,6 +493,7 @@
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2944,7 +2960,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -3105,6 +3121,74 @@
       </c>
       <c r="E9" s="0" t="s">
         <v>116</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14">
+        <v>46298</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="0">
+        <v>12269</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14">
+        <v>46298</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="0">
+        <v>9676</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14">
+        <v>46298</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="C12" s="0">
+        <v>1500</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="E12" s="0" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14">
+        <v>46298</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="C13" s="0">
+        <v>7993</v>
+      </c>
+      <c r="D13" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="E13" s="0" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -3140,10 +3224,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3169,7 +3253,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3">
@@ -3192,7 +3276,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4">
@@ -3215,7 +3299,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5">
@@ -3238,7 +3322,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6">
@@ -3261,7 +3345,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7">
@@ -3284,7 +3368,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8">
@@ -3307,7 +3391,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9">
@@ -3330,7 +3414,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10">
@@ -3353,7 +3437,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11">
@@ -3376,7 +3460,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12">
@@ -3399,7 +3483,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13">
@@ -3422,7 +3506,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="14">
@@ -3445,7 +3529,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15">
@@ -3468,7 +3552,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="16">
@@ -3491,7 +3575,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17">
@@ -3514,7 +3598,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -3534,10 +3618,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3545,35 +3629,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B3" s="0">
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -3596,7 +3680,7 @@
         <v>86</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3611,7 +3695,7 @@
         <v>110</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3640,7 +3724,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3">
@@ -3666,7 +3750,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4">
@@ -3692,7 +3776,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5">
@@ -3718,7 +3802,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6">
@@ -3744,7 +3828,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7">
@@ -3770,7 +3854,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8">
@@ -3796,7 +3880,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9">
@@ -3822,7 +3906,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10">
@@ -3848,7 +3932,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11">
@@ -3874,7 +3958,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12">
@@ -3900,7 +3984,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13">
@@ -3926,12 +4010,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: venta de la semana del 05/10 planificada en 17.000 (Gonzalo)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="142">
   <si>
     <t>fecha</t>
   </si>
@@ -297,6 +297,12 @@
   </si>
   <si>
     <t>total 16.000 = BO 1.050 (1 carga) + BR 8640 + PY 6310 (resto repartido con el mix BR/PY del ERP sem 38, 'no importa el orden')</t>
+  </si>
+  <si>
+    <t>Gonzalo 03/10: "la venta semana que viene esta planificada en 17 mil cajas"</t>
+  </si>
+  <si>
+    <t>total 17.000 = BO 1.050 (1 carga) + BR 10593 + PY 5357 (resto repartido con el mix BR/PY del ERP ult. 4 sem, 61,7/31,2)</t>
   </si>
   <si>
     <t>SUPUESTO 18.000 (Gonzalo 01/10: "si sube es a 18 mil la venta, no mas"; verano)</t>
@@ -2830,13 +2836,13 @@
         <v>46300</v>
       </c>
       <c r="B5" s="0">
-        <v>11106</v>
+        <v>10593</v>
       </c>
       <c r="C5" s="0">
-        <v>5616</v>
+        <v>5357</v>
       </c>
       <c r="D5" s="0">
-        <v>1278</v>
+        <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
         <v>93</v>
@@ -2859,10 +2865,10 @@
         <v>1278</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7">
@@ -2879,10 +2885,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2900,57 +2906,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -2998,10 +3004,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3">
@@ -3015,10 +3021,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4">
@@ -3032,10 +3038,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5">
@@ -3043,16 +3049,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6">
@@ -3066,10 +3072,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7">
@@ -3083,10 +3089,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8">
@@ -3100,10 +3106,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9">
@@ -3111,16 +3117,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10">
@@ -3134,10 +3140,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11">
@@ -3151,10 +3157,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12">
@@ -3168,10 +3174,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13">
@@ -3179,16 +3185,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -3224,10 +3230,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3253,7 +3259,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3">
@@ -3276,7 +3282,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4">
@@ -3299,7 +3305,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5">
@@ -3310,7 +3316,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -3322,7 +3328,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6">
@@ -3345,7 +3351,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7">
@@ -3368,7 +3374,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8">
@@ -3391,7 +3397,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9">
@@ -3402,7 +3408,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -3414,7 +3420,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10">
@@ -3437,7 +3443,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11">
@@ -3460,7 +3466,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12">
@@ -3483,7 +3489,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13">
@@ -3494,7 +3500,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -3506,7 +3512,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14">
@@ -3529,7 +3535,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15">
@@ -3540,7 +3546,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -3552,7 +3558,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16">
@@ -3575,7 +3581,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="17">
@@ -3598,7 +3604,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -3618,10 +3624,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3629,35 +3635,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B3" s="0">
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -3680,7 +3686,7 @@
         <v>86</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3692,10 +3698,10 @@
         <v>87</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3724,7 +3730,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3">
@@ -3750,7 +3756,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4">
@@ -3776,7 +3782,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5">
@@ -3802,7 +3808,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6">
@@ -3828,7 +3834,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7">
@@ -3854,7 +3860,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="8">
@@ -3880,7 +3886,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="9">
@@ -3906,7 +3912,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10">
@@ -3932,7 +3938,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11">
@@ -3958,7 +3964,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12">
@@ -3984,7 +3990,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13">
@@ -4010,12 +4016,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Cassio del viernes 02/10 contado una sola vez (Aloha ya lo tiene); sab 10/10 27.371, sab 17/10 faltan 2
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -510,7 +510,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -1435,16 +1435,16 @@
         <v>23</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G29" s="0" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H29" s="0">
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="I29" s="0" t="s">
         <v>35</v>
@@ -1467,7 +1467,7 @@
         <v>23</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="F30" s="0" t="s">
         <v>40</v>
@@ -1499,7 +1499,7 @@
         <v>23</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F31" s="0" t="s">
         <v>40</v>
@@ -1531,13 +1531,13 @@
         <v>23</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F32" s="0" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="G32" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H32" s="0">
         <v>1008</v>
@@ -1551,34 +1551,34 @@
     </row>
     <row r="33">
       <c r="A33" s="9">
-        <v>46297</v>
+        <v>46293</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C33" s="0" t="s">
         <v>52</v>
       </c>
       <c r="D33" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="G33" s="0" t="s">
         <v>14</v>
       </c>
       <c r="H33" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I33" s="0" t="s">
         <v>35</v>
       </c>
       <c r="J33" s="0" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34">
@@ -1595,7 +1595,7 @@
         <v>12</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F34" s="0" t="s">
         <v>14</v>
@@ -1610,15 +1610,15 @@
         <v>35</v>
       </c>
       <c r="J34" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C35" s="0" t="s">
         <v>52</v>
@@ -1642,15 +1642,15 @@
         <v>35</v>
       </c>
       <c r="J35" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C36" s="0" t="s">
         <v>52</v>
@@ -1659,7 +1659,7 @@
         <v>12</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F36" s="0" t="s">
         <v>14</v>
@@ -1674,59 +1674,59 @@
         <v>35</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="C37" s="0" t="s">
         <v>52</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H37" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="J37" s="0" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9">
-        <v>46295</v>
+        <v>46301</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="D38" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="G38" s="0" t="s">
         <v>34</v>
@@ -1735,18 +1735,18 @@
         <v>1008</v>
       </c>
       <c r="I38" s="0" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J38" s="0" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9">
-        <v>46301</v>
+        <v>46304</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C39" s="0" t="s">
         <v>66</v>
@@ -1770,15 +1770,15 @@
         <v>67</v>
       </c>
       <c r="J39" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="9">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C40" s="0" t="s">
         <v>66</v>
@@ -1787,10 +1787,10 @@
         <v>23</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="G40" s="0" t="s">
         <v>34</v>
@@ -1802,7 +1802,7 @@
         <v>67</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="41">
@@ -1819,16 +1819,16 @@
         <v>23</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="H41" s="0">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I41" s="0" t="s">
         <v>67</v>
@@ -1851,16 +1851,16 @@
         <v>23</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="G42" s="0" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="H42" s="0">
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="I42" s="0" t="s">
         <v>67</v>
@@ -1871,10 +1871,10 @@
     </row>
     <row r="43">
       <c r="A43" s="9">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="C43" s="0" t="s">
         <v>66</v>
@@ -1898,15 +1898,15 @@
         <v>67</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C44" s="0" t="s">
         <v>66</v>
@@ -1915,13 +1915,13 @@
         <v>23</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H44" s="0">
         <v>1008</v>
@@ -1930,15 +1930,15 @@
         <v>67</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C45" s="0" t="s">
         <v>66</v>
@@ -1947,13 +1947,13 @@
         <v>23</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H45" s="0">
         <v>1008</v>
@@ -1962,24 +1962,24 @@
         <v>67</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="9">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="C46" s="0" t="s">
         <v>66</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>72</v>
+        <v>19</v>
       </c>
       <c r="F46" s="0" t="s">
         <v>14</v>
@@ -1988,21 +1988,21 @@
         <v>14</v>
       </c>
       <c r="H46" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I46" s="0" t="s">
         <v>67</v>
       </c>
       <c r="J46" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="9">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C47" s="0" t="s">
         <v>66</v>
@@ -2026,15 +2026,15 @@
         <v>67</v>
       </c>
       <c r="J47" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C48" s="0" t="s">
         <v>66</v>
@@ -2043,7 +2043,7 @@
         <v>12</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F48" s="0" t="s">
         <v>14</v>
@@ -2058,15 +2058,15 @@
         <v>67</v>
       </c>
       <c r="J48" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="9">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C49" s="0" t="s">
         <v>66</v>
@@ -2090,15 +2090,15 @@
         <v>67</v>
       </c>
       <c r="J49" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="9">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C50" s="0" t="s">
         <v>66</v>
@@ -2107,7 +2107,7 @@
         <v>12</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F50" s="0" t="s">
         <v>14</v>
@@ -2122,47 +2122,47 @@
         <v>67</v>
       </c>
       <c r="J50" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="9">
-        <v>46300</v>
+        <v>46308</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="D51" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G51" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H51" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I51" s="0" t="s">
         <v>67</v>
       </c>
       <c r="J51" s="0" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="9">
-        <v>46308</v>
+        <v>46312</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C52" s="0" t="s">
         <v>79</v>
@@ -2186,15 +2186,15 @@
         <v>67</v>
       </c>
       <c r="J52" s="0" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="9">
-        <v>46312</v>
+        <v>46309</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="C53" s="0" t="s">
         <v>79</v>
@@ -2203,10 +2203,10 @@
         <v>23</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="G53" s="0" t="s">
         <v>34</v>
@@ -2218,15 +2218,15 @@
         <v>67</v>
       </c>
       <c r="J53" s="0" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="9">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C54" s="0" t="s">
         <v>79</v>
@@ -2250,15 +2250,15 @@
         <v>67</v>
       </c>
       <c r="J54" s="0" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="9">
-        <v>46311</v>
+        <v>46308</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C55" s="0" t="s">
         <v>79</v>
@@ -2267,30 +2267,30 @@
         <v>23</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="H55" s="0">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I55" s="0" t="s">
         <v>67</v>
       </c>
       <c r="J55" s="0" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="9">
-        <v>46308</v>
+        <v>46311</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C56" s="0" t="s">
         <v>79</v>
@@ -2314,15 +2314,15 @@
         <v>67</v>
       </c>
       <c r="J56" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="9">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C57" s="0" t="s">
         <v>79</v>
@@ -2331,30 +2331,30 @@
         <v>23</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="H57" s="0">
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="I57" s="0" t="s">
         <v>67</v>
       </c>
       <c r="J57" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="9">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C58" s="0" t="s">
         <v>79</v>
@@ -2378,15 +2378,15 @@
         <v>67</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="9">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="B59" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C59" s="0" t="s">
         <v>79</v>
@@ -2395,10 +2395,10 @@
         <v>23</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="G59" s="0" t="s">
         <v>14</v>
@@ -2410,7 +2410,7 @@
         <v>67</v>
       </c>
       <c r="J59" s="0" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
     </row>
     <row r="60">
@@ -2427,10 +2427,10 @@
         <v>23</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="G60" s="0" t="s">
         <v>14</v>
@@ -2442,15 +2442,15 @@
         <v>67</v>
       </c>
       <c r="J60" s="0" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="9">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C61" s="0" t="s">
         <v>79</v>
@@ -2459,13 +2459,13 @@
         <v>23</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H61" s="0">
         <v>1008</v>
@@ -2474,39 +2474,39 @@
         <v>67</v>
       </c>
       <c r="J61" s="0" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="9">
-        <v>46311</v>
+        <v>46307</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C62" s="0" t="s">
         <v>79</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G62" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H62" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I62" s="0" t="s">
         <v>67</v>
       </c>
       <c r="J62" s="0" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
     </row>
     <row r="63">
@@ -2523,7 +2523,7 @@
         <v>12</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F63" s="0" t="s">
         <v>14</v>
@@ -2538,15 +2538,15 @@
         <v>67</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="9">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B64" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C64" s="0" t="s">
         <v>79</v>
@@ -2570,15 +2570,15 @@
         <v>67</v>
       </c>
       <c r="J64" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="9">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="B65" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C65" s="0" t="s">
         <v>79</v>
@@ -2587,7 +2587,7 @@
         <v>12</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F65" s="0" t="s">
         <v>14</v>
@@ -2602,15 +2602,15 @@
         <v>67</v>
       </c>
       <c r="J65" s="0" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="9">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C66" s="0" t="s">
         <v>79</v>
@@ -2634,7 +2634,7 @@
         <v>67</v>
       </c>
       <c r="J66" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="67">
@@ -2651,7 +2651,7 @@
         <v>12</v>
       </c>
       <c r="E67" s="0" t="s">
-        <v>19</v>
+        <v>82</v>
       </c>
       <c r="F67" s="0" t="s">
         <v>14</v>
@@ -2666,70 +2666,38 @@
         <v>67</v>
       </c>
       <c r="J67" s="0" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="9">
-        <v>46308</v>
+        <v>46295</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C68" s="0" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="D68" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E68" s="0" t="s">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="F68" s="0" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G68" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H68" s="0">
-        <v>980</v>
+        <v>936</v>
       </c>
       <c r="I68" s="0" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="J68" s="0" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="9">
-        <v>46295</v>
-      </c>
-      <c r="B69" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="C69" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="D69" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E69" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="F69" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G69" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H69" s="0">
-        <v>936</v>
-      </c>
-      <c r="I69" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="J69" s="0" t="s">
         <v>85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
plan de compras: manda el dictado sobre las solicitadas de Aloha (regla nueva), dictado del 06/10 de las semanas 05-10 y 12-17, venta 16.000
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="154">
   <si>
     <t>fecha</t>
   </si>
@@ -218,64 +218,100 @@
     <t>carga extra: "asi cierro mejor pensando en futuro" (ademas de la sexta ya dictada)</t>
   </si>
   <si>
+    <t>Gonzalo 02/10 (precios de la semana)</t>
+  </si>
+  <si>
+    <t>carga real: cuarta Nilton, R$ 35 (no estaba dictada)</t>
+  </si>
+  <si>
     <t>2026-10-04</t>
   </si>
   <si>
-    <t>Gonzalo 02/10 (chat)</t>
-  </si>
-  <si>
-    <t>nota 02/10: tersa; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>nota 02/10: sexta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>nota 02/10: cuarta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>nota 02/10: segunda; transportista supuesto = habitual</t>
+    <t>Gonzalo 06/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Fisher 2: tersa; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Fisher 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Agro 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Cassio 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Ivo 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Ivo 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Gilson 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Josemar 1: tersa</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Stein 1: tersa</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Marconi 1: sexta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Milciades 2: lunes</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Milciades 2: martes</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Diego 2: lunes</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Diego 2: martes</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Alvarito 1: lunes</t>
+  </si>
+  <si>
+    <t>2026-10-11</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Fisher 1: sabado (descarga martes 20, semana siguiente)</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Agro 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Agro 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Cassio 2: tersa</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Cassio 2: sexta</t>
   </si>
   <si>
     <t>Celso</t>
   </si>
   <si>
-    <t>nota 02/10: cuarta. PRODUCTOR NUEVO: no esta en productores.xlsx ni en Aloha; falta nombre completo y transporte</t>
-  </si>
-  <si>
-    <t>nota 02/10: Milciades 2, lunes</t>
-  </si>
-  <si>
-    <t>nota 02/10: Milciades 2, martes</t>
-  </si>
-  <si>
-    <t>nota 02/10: Diego 2, lunes</t>
-  </si>
-  <si>
-    <t>nota 02/10: Diego 2, martes</t>
-  </si>
-  <si>
-    <t>nota 02/10: Alvarito 1, lunes</t>
-  </si>
-  <si>
-    <t>2026-10-11</t>
-  </si>
-  <si>
-    <t>nota 02/10: sabado (descarga martes 20, semana siguiente); transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>nota 02/10: cuarta. PRODUCTOR NUEVO (ver semana anterior)</t>
+    <t>dictado 06/10: Celso 1: cuarta. PRODUCTOR NUEVO: falta nombre completo y transporte</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Marconi 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Josemar 1: sexta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Stein 1: sexta</t>
   </si>
   <si>
     <t>Paraguay GM</t>
   </si>
   <si>
-    <t>nota 02/10: Guido 1, martes (reactivacion; descarga sabado 17)</t>
-  </si>
-  <si>
-    <t>Gonzalo 02/10 (precios de la semana)</t>
-  </si>
-  <si>
-    <t>carga real: cuarta Nilton, R$ 35 (no estaba dictada)</t>
+    <t>dictado 06/10: Guido 1: martes</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -299,10 +335,10 @@
     <t>total 16.000 = BO 1.050 (1 carga) + BR 8640 + PY 6310 (resto repartido con el mix BR/PY del ERP sem 38, 'no importa el orden')</t>
   </si>
   <si>
-    <t>Gonzalo 03/10: "la venta semana que viene esta planificada en 17 mil cajas"</t>
-  </si>
-  <si>
-    <t>total 17.000 = BO 1.050 (1 carga) + BR 10593 + PY 5357 (resto repartido con el mix BR/PY del ERP ult. 4 sem, 61,7/31,2)</t>
+    <t>Gonzalo 06/10: "venta esta semana va a ser de 16 mil, la venta fallo ayer lunes" (el 03/10 habia dicho 17.000)</t>
+  </si>
+  <si>
+    <t>total 16.000 = BO 1.050 (1 carga) + BR 9929 + PY 5021 (resto con el mix BR/PY del ERP ult. 4 sem)</t>
   </si>
   <si>
     <t>SUPUESTO 18.000 (Gonzalo 01/10: "si sube es a 18 mil la venta, no mas"; verano)</t>
@@ -484,7 +520,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -500,6 +536,7 @@
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -510,7 +547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -1711,45 +1748,45 @@
     </row>
     <row r="38">
       <c r="A38" s="9">
-        <v>46301</v>
+        <v>46295</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="D38" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="G38" s="0" t="s">
         <v>34</v>
       </c>
       <c r="H38" s="0">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I38" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="J38" s="0" t="s">
         <v>67</v>
       </c>
-      <c r="J38" s="0" t="s">
+    </row>
+    <row r="39">
+      <c r="A39" s="15">
+        <v>46301</v>
+      </c>
+      <c r="B39" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C39" s="0" t="s">
         <v>68</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="9">
-        <v>46304</v>
-      </c>
-      <c r="B39" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="C39" s="0" t="s">
-        <v>66</v>
       </c>
       <c r="D39" s="0" t="s">
         <v>23</v>
@@ -1767,117 +1804,117 @@
         <v>1008</v>
       </c>
       <c r="I39" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J39" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="9">
-        <v>46302</v>
+      <c r="A40" s="15">
+        <v>46304</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D40" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H40" s="0">
         <v>1008</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="9">
+      <c r="A41" s="15">
         <v>46302</v>
       </c>
       <c r="B41" s="0" t="s">
         <v>51</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D41" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="H41" s="0">
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J41" s="0" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="9">
+      <c r="A42" s="15">
         <v>46302</v>
       </c>
       <c r="B42" s="0" t="s">
         <v>51</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D42" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="G42" s="0" t="s">
         <v>14</v>
       </c>
       <c r="H42" s="0">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I42" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J42" s="0" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="9">
-        <v>46300</v>
+      <c r="A43" s="15">
+        <v>46302</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D43" s="0" t="s">
         <v>23</v>
@@ -1886,7 +1923,7 @@
         <v>24</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="G43" s="0" t="s">
         <v>14</v>
@@ -1895,59 +1932,59 @@
         <v>1008</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="9">
-        <v>46301</v>
+      <c r="A44" s="15">
+        <v>46304</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D44" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>58</v>
+        <v>24</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H44" s="0">
         <v>1008</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="9">
+      <c r="A45" s="15">
         <v>46302</v>
       </c>
       <c r="B45" s="0" t="s">
         <v>51</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D45" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>72</v>
+        <v>42</v>
       </c>
       <c r="F45" s="0" t="s">
         <v>14</v>
@@ -1959,27 +1996,27 @@
         <v>1008</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="9">
-        <v>46300</v>
+      <c r="A46" s="15">
+        <v>46301</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>19</v>
+        <v>57</v>
       </c>
       <c r="F46" s="0" t="s">
         <v>14</v>
@@ -1988,30 +2025,30 @@
         <v>14</v>
       </c>
       <c r="H46" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I46" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J46" s="0" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="9">
+      <c r="A47" s="15">
         <v>46301</v>
       </c>
       <c r="B47" s="0" t="s">
         <v>20</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>19</v>
+        <v>58</v>
       </c>
       <c r="F47" s="0" t="s">
         <v>14</v>
@@ -2020,62 +2057,62 @@
         <v>14</v>
       </c>
       <c r="H47" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I47" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J47" s="0" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="9">
+      <c r="A48" s="15">
+        <v>46304</v>
+      </c>
+      <c r="B48" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C48" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="D48" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E48" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F48" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G48" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H48" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I48" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="J48" s="0" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="15">
         <v>46300</v>
       </c>
-      <c r="B48" s="0" t="s">
+      <c r="B49" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="C48" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="D48" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E48" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F48" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G48" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H48" s="0">
-        <v>980</v>
-      </c>
-      <c r="I48" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="J48" s="0" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="9">
-        <v>46301</v>
-      </c>
-      <c r="B49" s="0" t="s">
-        <v>20</v>
-      </c>
       <c r="C49" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D49" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F49" s="0" t="s">
         <v>14</v>
@@ -2087,27 +2124,27 @@
         <v>980</v>
       </c>
       <c r="I49" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J49" s="0" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="9">
-        <v>46300</v>
+      <c r="A50" s="15">
+        <v>46301</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C50" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D50" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F50" s="0" t="s">
         <v>14</v>
@@ -2119,283 +2156,283 @@
         <v>980</v>
       </c>
       <c r="I50" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J50" s="0" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="9">
-        <v>46308</v>
+      <c r="A51" s="15">
+        <v>46300</v>
       </c>
       <c r="B51" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C51" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="D51" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="F51" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G51" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H51" s="0">
+        <v>980</v>
+      </c>
+      <c r="I51" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="J51" s="0" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="15">
+        <v>46301</v>
+      </c>
+      <c r="B52" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="C51" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="D51" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E51" s="0" t="s">
+      <c r="C52" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="D52" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E52" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="F52" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G52" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H52" s="0">
+        <v>980</v>
+      </c>
+      <c r="I52" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="J52" s="0" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="15">
+        <v>46300</v>
+      </c>
+      <c r="B53" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C53" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="D53" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E53" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="F53" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G53" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H53" s="0">
+        <v>980</v>
+      </c>
+      <c r="I53" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="J53" s="0" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="15">
+        <v>46312</v>
+      </c>
+      <c r="B54" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C54" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="D54" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E54" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="F51" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="G51" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H51" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I51" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="J51" s="0" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="9">
-        <v>46312</v>
-      </c>
-      <c r="B52" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="C52" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="D52" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E52" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="F52" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="G52" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H52" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I52" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="J52" s="0" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="9">
-        <v>46309</v>
-      </c>
-      <c r="B53" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="C53" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="D53" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E53" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="F53" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G53" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H53" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I53" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="J53" s="0" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="9">
-        <v>46311</v>
-      </c>
-      <c r="B54" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="C54" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="D54" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E54" s="0" t="s">
-        <v>39</v>
-      </c>
       <c r="F54" s="0" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H54" s="0">
         <v>1008</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J54" s="0" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="15">
+        <v>46309</v>
+      </c>
+      <c r="B55" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C55" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="D55" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E55" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="F55" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G55" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H55" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I55" s="0" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="9">
-        <v>46308</v>
-      </c>
-      <c r="B55" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="C55" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="D55" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E55" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="F55" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="G55" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="H55" s="0">
-        <v>936</v>
-      </c>
-      <c r="I55" s="0" t="s">
-        <v>67</v>
-      </c>
       <c r="J55" s="0" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="9">
+      <c r="A56" s="15">
         <v>46311</v>
       </c>
       <c r="B56" s="0" t="s">
         <v>22</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D56" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E56" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="F56" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G56" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H56" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I56" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="J56" s="0" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="15">
+        <v>46308</v>
+      </c>
+      <c r="B57" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C57" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="D57" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E57" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="F56" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="G56" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="H56" s="0">
+      <c r="F57" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G57" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H57" s="0">
         <v>936</v>
       </c>
-      <c r="I56" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="J56" s="0" t="s">
+      <c r="I57" s="0" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="9">
-        <v>46309</v>
-      </c>
-      <c r="B57" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="C57" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="D57" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E57" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="F57" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="G57" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H57" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I57" s="0" t="s">
-        <v>67</v>
-      </c>
       <c r="J57" s="0" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="9">
+      <c r="A58" s="15">
         <v>46311</v>
       </c>
       <c r="B58" s="0" t="s">
         <v>22</v>
       </c>
       <c r="C58" s="0" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D58" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="G58" s="0" t="s">
         <v>14</v>
       </c>
       <c r="H58" s="0">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="9">
+      <c r="A59" s="15">
         <v>46309</v>
       </c>
       <c r="B59" s="0" t="s">
         <v>51</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D59" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="F59" s="0" t="s">
         <v>14</v>
@@ -2407,30 +2444,30 @@
         <v>1008</v>
       </c>
       <c r="I59" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J59" s="0" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="9">
-        <v>46309</v>
+      <c r="A60" s="15">
+        <v>46311</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D60" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="G60" s="0" t="s">
         <v>14</v>
@@ -2439,91 +2476,91 @@
         <v>1008</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J60" s="0" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="9">
-        <v>46311</v>
+      <c r="A61" s="15">
+        <v>46309</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D61" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>57</v>
+        <v>91</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H61" s="0">
         <v>1008</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J61" s="0" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="15">
+        <v>46309</v>
+      </c>
+      <c r="B62" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C62" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="D62" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E62" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F62" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G62" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H62" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I62" s="0" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="9">
-        <v>46307</v>
-      </c>
-      <c r="B62" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="C62" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="D62" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E62" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="F62" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G62" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H62" s="0">
-        <v>980</v>
-      </c>
-      <c r="I62" s="0" t="s">
-        <v>67</v>
-      </c>
       <c r="J62" s="0" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="9">
-        <v>46307</v>
+      <c r="A63" s="15">
+        <v>46311</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D63" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="F63" s="0" t="s">
         <v>14</v>
@@ -2532,30 +2569,30 @@
         <v>14</v>
       </c>
       <c r="H63" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="9">
-        <v>46308</v>
+      <c r="A64" s="15">
+        <v>46311</v>
       </c>
       <c r="B64" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>13</v>
+        <v>58</v>
       </c>
       <c r="F64" s="0" t="s">
         <v>14</v>
@@ -2564,30 +2601,30 @@
         <v>14</v>
       </c>
       <c r="H64" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J64" s="0" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="9">
+      <c r="A65" s="15">
         <v>46307</v>
       </c>
       <c r="B65" s="0" t="s">
         <v>18</v>
       </c>
       <c r="C65" s="0" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D65" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F65" s="0" t="s">
         <v>14</v>
@@ -2599,27 +2636,27 @@
         <v>980</v>
       </c>
       <c r="I65" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J65" s="0" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="9">
-        <v>46308</v>
+      <c r="A66" s="15">
+        <v>46307</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C66" s="0" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D66" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F66" s="0" t="s">
         <v>14</v>
@@ -2631,27 +2668,27 @@
         <v>980</v>
       </c>
       <c r="I66" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J66" s="0" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="9">
+      <c r="A67" s="15">
         <v>46308</v>
       </c>
       <c r="B67" s="0" t="s">
         <v>20</v>
       </c>
       <c r="C67" s="0" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D67" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E67" s="0" t="s">
-        <v>82</v>
+        <v>13</v>
       </c>
       <c r="F67" s="0" t="s">
         <v>14</v>
@@ -2663,42 +2700,106 @@
         <v>980</v>
       </c>
       <c r="I67" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J67" s="0" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="9">
-        <v>46295</v>
+      <c r="A68" s="15">
+        <v>46307</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="C68" s="0" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="D68" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E68" s="0" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F68" s="0" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G68" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H68" s="0">
-        <v>936</v>
+        <v>980</v>
       </c>
       <c r="I68" s="0" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="J68" s="0" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="15">
+        <v>46308</v>
+      </c>
+      <c r="B69" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C69" s="0" t="s">
         <v>85</v>
+      </c>
+      <c r="D69" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E69" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="F69" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G69" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H69" s="0">
+        <v>980</v>
+      </c>
+      <c r="I69" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="J69" s="0" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="15">
+        <v>46308</v>
+      </c>
+      <c r="B70" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C70" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="D70" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E70" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F70" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G70" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H70" s="0">
+        <v>980</v>
+      </c>
+      <c r="I70" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="J70" s="0" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -2721,7 +2822,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -2730,7 +2831,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>8</v>
@@ -2753,10 +2854,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3">
@@ -2773,10 +2874,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4">
@@ -2793,10 +2894,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5">
@@ -2804,19 +2905,19 @@
         <v>46300</v>
       </c>
       <c r="B5" s="0">
-        <v>10593</v>
+        <v>9929</v>
       </c>
       <c r="C5" s="0">
-        <v>5357</v>
+        <v>5021</v>
       </c>
       <c r="D5" s="0">
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6">
@@ -2833,10 +2934,10 @@
         <v>1278</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7">
@@ -2853,10 +2954,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -2874,57 +2975,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -2972,10 +3073,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3">
@@ -2989,10 +3090,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4">
@@ -3000,16 +3101,16 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5">
@@ -3017,16 +3118,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6">
@@ -3040,10 +3141,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7">
@@ -3057,10 +3158,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8">
@@ -3068,16 +3169,16 @@
         <v>46291</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C8" s="0">
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9">
@@ -3085,16 +3186,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10">
@@ -3108,10 +3209,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
     </row>
     <row r="11">
@@ -3125,10 +3226,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12">
@@ -3136,16 +3237,16 @@
         <v>46298</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C12" s="0">
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="13">
@@ -3153,16 +3254,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -3198,10 +3299,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3227,7 +3328,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3">
@@ -3250,7 +3351,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4">
@@ -3261,7 +3362,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -3273,7 +3374,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5">
@@ -3284,7 +3385,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -3296,7 +3397,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6">
@@ -3319,7 +3420,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7">
@@ -3342,7 +3443,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8">
@@ -3353,7 +3454,7 @@
         <v>51</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -3365,7 +3466,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9">
@@ -3376,7 +3477,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -3388,7 +3489,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10">
@@ -3411,7 +3512,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11">
@@ -3434,7 +3535,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12">
@@ -3445,7 +3546,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -3457,7 +3558,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13">
@@ -3468,7 +3569,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -3480,7 +3581,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14">
@@ -3503,7 +3604,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15">
@@ -3514,7 +3615,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -3526,7 +3627,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16">
@@ -3549,7 +3650,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17">
@@ -3560,7 +3661,7 @@
         <v>29</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="D17" s="0">
         <v>134</v>
@@ -3572,7 +3673,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -3592,10 +3693,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3603,35 +3704,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="B3" s="0">
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -3651,10 +3752,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3663,13 +3764,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3698,7 +3799,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3">
@@ -3724,7 +3825,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4">
@@ -3750,7 +3851,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5">
@@ -3776,7 +3877,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6">
@@ -3802,7 +3903,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7">
@@ -3828,7 +3929,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8">
@@ -3854,7 +3955,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9">
@@ -3880,7 +3981,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10">
@@ -3906,7 +4007,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11">
@@ -3932,7 +4033,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="12">
@@ -3958,7 +4059,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13">
@@ -3984,12 +4085,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: dictado corregido de la semana 05-10/10 (BR 8: sin Gilson/Josemar/Marconi, con Celso); sab 10 28.371, sab 17 faltan 2
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="160">
   <si>
     <t>fecha</t>
   </si>
@@ -224,94 +224,112 @@
     <t>carga real: cuarta Nilton, R$ 35 (no estaba dictada)</t>
   </si>
   <si>
+    <t>2026-10-11</t>
+  </si>
+  <si>
+    <t>Gonzalo 06/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Fisher 1: sabado (descarga martes 20, semana siguiente)</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Agro 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Agro 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Cassio 2: tersa</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Cassio 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Ivo 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Ivo 2: sexta</t>
+  </si>
+  <si>
+    <t>Celso</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Celso 1: cuarta. PRODUCTOR NUEVO: falta nombre completo y transporte</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Marconi 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Josemar 1: sexta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Stein 1: sexta</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Alvarito 1: lunes</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Diego 2: lunes</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Diego 2: martes</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Milciades 2: lunes</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Milciades 2: martes</t>
+  </si>
+  <si>
+    <t>Paraguay GM</t>
+  </si>
+  <si>
+    <t>dictado 06/10: Guido 1: martes</t>
+  </si>
+  <si>
     <t>2026-10-04</t>
   </si>
   <si>
-    <t>Gonzalo 06/10 (chat)</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Fisher 2: tersa; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Fisher 2: sexta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Agro 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Cassio 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Ivo 2: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Ivo 2: sexta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Gilson 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Josemar 1: tersa</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Stein 1: tersa</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Marconi 1: sexta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Milciades 2: lunes</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Milciades 2: martes</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Diego 2: lunes</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Diego 2: martes</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Alvarito 1: lunes</t>
-  </si>
-  <si>
-    <t>2026-10-11</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Fisher 1: sabado (descarga martes 20, semana siguiente)</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Agro 2: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Agro 2: sexta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Cassio 2: tersa</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Cassio 2: sexta</t>
-  </si>
-  <si>
-    <t>Celso</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Celso 1: cuarta. PRODUCTOR NUEVO: falta nombre completo y transporte</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Marconi 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Josemar 1: sexta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Stein 1: sexta</t>
-  </si>
-  <si>
-    <t>Paraguay GM</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Guido 1: martes</t>
+    <t>Gonzalo 06/10 (chat, 2da version)</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Fisher 2: tersa; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Fisher 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Agro 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Cassio 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Celso 1: cuarta. PRODUCTOR NUEVO: falta nombre completo y transporte</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Ivo 2: tersa</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Ivo 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Stein 1: tersa</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Milciades 2: lunes</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Milciades 2: martes</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Diego 2: lunes</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Diego 2: martes</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Alvarito 1: lunes</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -520,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -537,6 +555,7 @@
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -547,7 +566,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -1780,10 +1799,10 @@
     </row>
     <row r="39">
       <c r="A39" s="15">
-        <v>46301</v>
+        <v>46312</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C39" s="0" t="s">
         <v>68</v>
@@ -1795,10 +1814,10 @@
         <v>30</v>
       </c>
       <c r="F39" s="0" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G39" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H39" s="0">
         <v>1008</v>
@@ -1812,10 +1831,10 @@
     </row>
     <row r="40">
       <c r="A40" s="15">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C40" s="0" t="s">
         <v>68</v>
@@ -1824,7 +1843,7 @@
         <v>23</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="F40" s="0" t="s">
         <v>14</v>
@@ -1844,10 +1863,10 @@
     </row>
     <row r="41">
       <c r="A41" s="15">
-        <v>46302</v>
+        <v>46311</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C41" s="0" t="s">
         <v>68</v>
@@ -1876,10 +1895,10 @@
     </row>
     <row r="42">
       <c r="A42" s="15">
-        <v>46302</v>
+        <v>46308</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C42" s="0" t="s">
         <v>68</v>
@@ -1908,10 +1927,10 @@
     </row>
     <row r="43">
       <c r="A43" s="15">
-        <v>46302</v>
+        <v>46311</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C43" s="0" t="s">
         <v>68</v>
@@ -1920,7 +1939,7 @@
         <v>23</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F43" s="0" t="s">
         <v>14</v>
@@ -1929,7 +1948,7 @@
         <v>14</v>
       </c>
       <c r="H43" s="0">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I43" s="0" t="s">
         <v>69</v>
@@ -1940,10 +1959,10 @@
     </row>
     <row r="44">
       <c r="A44" s="15">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C44" s="0" t="s">
         <v>68</v>
@@ -1972,10 +1991,10 @@
     </row>
     <row r="45">
       <c r="A45" s="15">
-        <v>46302</v>
+        <v>46311</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C45" s="0" t="s">
         <v>68</v>
@@ -1984,7 +2003,7 @@
         <v>23</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="F45" s="0" t="s">
         <v>14</v>
@@ -2004,10 +2023,10 @@
     </row>
     <row r="46">
       <c r="A46" s="15">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C46" s="0" t="s">
         <v>68</v>
@@ -2016,7 +2035,7 @@
         <v>23</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="F46" s="0" t="s">
         <v>14</v>
@@ -2031,15 +2050,15 @@
         <v>69</v>
       </c>
       <c r="J46" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="15">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C47" s="0" t="s">
         <v>68</v>
@@ -2048,7 +2067,7 @@
         <v>23</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F47" s="0" t="s">
         <v>14</v>
@@ -2063,12 +2082,12 @@
         <v>69</v>
       </c>
       <c r="J47" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="15">
-        <v>46304</v>
+        <v>46311</v>
       </c>
       <c r="B48" s="0" t="s">
         <v>22</v>
@@ -2080,7 +2099,7 @@
         <v>23</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F48" s="0" t="s">
         <v>14</v>
@@ -2095,24 +2114,24 @@
         <v>69</v>
       </c>
       <c r="J48" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="15">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C49" s="0" t="s">
         <v>68</v>
       </c>
       <c r="D49" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>19</v>
+        <v>58</v>
       </c>
       <c r="F49" s="0" t="s">
         <v>14</v>
@@ -2121,21 +2140,21 @@
         <v>14</v>
       </c>
       <c r="H49" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I49" s="0" t="s">
         <v>69</v>
       </c>
       <c r="J49" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="15">
-        <v>46301</v>
+        <v>46307</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C50" s="0" t="s">
         <v>68</v>
@@ -2144,7 +2163,7 @@
         <v>12</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F50" s="0" t="s">
         <v>14</v>
@@ -2159,12 +2178,12 @@
         <v>69</v>
       </c>
       <c r="J50" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="15">
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="B51" s="0" t="s">
         <v>18</v>
@@ -2191,12 +2210,12 @@
         <v>69</v>
       </c>
       <c r="J51" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="15">
-        <v>46301</v>
+        <v>46308</v>
       </c>
       <c r="B52" s="0" t="s">
         <v>20</v>
@@ -2223,12 +2242,12 @@
         <v>69</v>
       </c>
       <c r="J52" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="15">
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="B53" s="0" t="s">
         <v>18</v>
@@ -2240,7 +2259,7 @@
         <v>12</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F53" s="0" t="s">
         <v>14</v>
@@ -2255,24 +2274,24 @@
         <v>69</v>
       </c>
       <c r="J53" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="15">
-        <v>46312</v>
+        <v>46308</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F54" s="0" t="s">
         <v>14</v>
@@ -2281,7 +2300,7 @@
         <v>14</v>
       </c>
       <c r="H54" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I54" s="0" t="s">
         <v>69</v>
@@ -2292,19 +2311,19 @@
     </row>
     <row r="55">
       <c r="A55" s="15">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C55" s="0" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="D55" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>39</v>
+        <v>87</v>
       </c>
       <c r="F55" s="0" t="s">
         <v>14</v>
@@ -2313,62 +2332,62 @@
         <v>14</v>
       </c>
       <c r="H55" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I55" s="0" t="s">
         <v>69</v>
       </c>
       <c r="J55" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="15">
-        <v>46311</v>
+      <c r="A56" s="16">
+        <v>46301</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D56" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H56" s="0">
         <v>1008</v>
       </c>
       <c r="I56" s="0" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="J56" s="0" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="15">
-        <v>46308</v>
+      <c r="A57" s="16">
+        <v>46304</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C57" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D57" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F57" s="0" t="s">
         <v>14</v>
@@ -2377,30 +2396,30 @@
         <v>14</v>
       </c>
       <c r="H57" s="0">
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="J57" s="0" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="16">
+        <v>46302</v>
+      </c>
+      <c r="B58" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C58" s="0" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="15">
-        <v>46311</v>
-      </c>
-      <c r="B58" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="C58" s="0" t="s">
-        <v>85</v>
-      </c>
       <c r="D58" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="F58" s="0" t="s">
         <v>14</v>
@@ -2409,30 +2428,30 @@
         <v>14</v>
       </c>
       <c r="H58" s="0">
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="15">
-        <v>46309</v>
+      <c r="A59" s="16">
+        <v>46302</v>
       </c>
       <c r="B59" s="0" t="s">
         <v>51</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D59" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F59" s="0" t="s">
         <v>14</v>
@@ -2441,30 +2460,30 @@
         <v>14</v>
       </c>
       <c r="H59" s="0">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I59" s="0" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="J59" s="0" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="15">
-        <v>46311</v>
+      <c r="A60" s="16">
+        <v>46302</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D60" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>24</v>
+        <v>77</v>
       </c>
       <c r="F60" s="0" t="s">
         <v>14</v>
@@ -2476,27 +2495,27 @@
         <v>1008</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="J60" s="0" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="15">
-        <v>46309</v>
+      <c r="A61" s="16">
+        <v>46301</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D61" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>91</v>
+        <v>24</v>
       </c>
       <c r="F61" s="0" t="s">
         <v>14</v>
@@ -2508,27 +2527,27 @@
         <v>1008</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="J61" s="0" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="15">
-        <v>46309</v>
+      <c r="A62" s="16">
+        <v>46302</v>
       </c>
       <c r="B62" s="0" t="s">
         <v>51</v>
       </c>
       <c r="C62" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D62" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="F62" s="0" t="s">
         <v>14</v>
@@ -2540,27 +2559,27 @@
         <v>1008</v>
       </c>
       <c r="I62" s="0" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="J62" s="0" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="15">
-        <v>46311</v>
+      <c r="A63" s="16">
+        <v>46301</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D63" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F63" s="0" t="s">
         <v>14</v>
@@ -2572,27 +2591,27 @@
         <v>1008</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="15">
-        <v>46311</v>
+      <c r="A64" s="16">
+        <v>46300</v>
       </c>
       <c r="B64" s="0" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>58</v>
+        <v>19</v>
       </c>
       <c r="F64" s="0" t="s">
         <v>14</v>
@@ -2601,30 +2620,30 @@
         <v>14</v>
       </c>
       <c r="H64" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="J64" s="0" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="15">
-        <v>46307</v>
+      <c r="A65" s="16">
+        <v>46301</v>
       </c>
       <c r="B65" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C65" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D65" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F65" s="0" t="s">
         <v>14</v>
@@ -2636,21 +2655,21 @@
         <v>980</v>
       </c>
       <c r="I65" s="0" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="J65" s="0" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="15">
-        <v>46307</v>
+      <c r="A66" s="16">
+        <v>46300</v>
       </c>
       <c r="B66" s="0" t="s">
         <v>18</v>
       </c>
       <c r="C66" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D66" s="0" t="s">
         <v>12</v>
@@ -2668,21 +2687,21 @@
         <v>980</v>
       </c>
       <c r="I66" s="0" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="J66" s="0" t="s">
-        <v>82</v>
+        <v>101</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="15">
-        <v>46308</v>
+      <c r="A67" s="16">
+        <v>46301</v>
       </c>
       <c r="B67" s="0" t="s">
         <v>20</v>
       </c>
       <c r="C67" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D67" s="0" t="s">
         <v>12</v>
@@ -2700,27 +2719,27 @@
         <v>980</v>
       </c>
       <c r="I67" s="0" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="J67" s="0" t="s">
-        <v>83</v>
+        <v>102</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="15">
-        <v>46307</v>
+      <c r="A68" s="16">
+        <v>46300</v>
       </c>
       <c r="B68" s="0" t="s">
         <v>18</v>
       </c>
       <c r="C68" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D68" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E68" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F68" s="0" t="s">
         <v>14</v>
@@ -2732,74 +2751,10 @@
         <v>980</v>
       </c>
       <c r="I68" s="0" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="J68" s="0" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="15">
-        <v>46308</v>
-      </c>
-      <c r="B69" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="C69" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="D69" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E69" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="F69" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G69" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H69" s="0">
-        <v>980</v>
-      </c>
-      <c r="I69" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="J69" s="0" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="15">
-        <v>46308</v>
-      </c>
-      <c r="B70" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="C70" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="D70" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E70" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="F70" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G70" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H70" s="0">
-        <v>980</v>
-      </c>
-      <c r="I70" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="J70" s="0" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2822,7 +2777,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -2831,7 +2786,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>8</v>
@@ -2854,10 +2809,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3">
@@ -2874,10 +2829,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4">
@@ -2894,10 +2849,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5">
@@ -2914,10 +2869,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6">
@@ -2934,10 +2889,10 @@
         <v>1278</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7">
@@ -2954,10 +2909,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -2975,57 +2930,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -3073,10 +3028,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3">
@@ -3090,10 +3045,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4">
@@ -3101,16 +3056,16 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5">
@@ -3118,16 +3073,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6">
@@ -3141,10 +3096,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7">
@@ -3158,10 +3113,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8">
@@ -3169,16 +3124,16 @@
         <v>46291</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C8" s="0">
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9">
@@ -3186,16 +3141,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10">
@@ -3209,10 +3164,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11">
@@ -3226,10 +3181,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12">
@@ -3237,16 +3192,16 @@
         <v>46298</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C12" s="0">
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13">
@@ -3254,16 +3209,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -3299,10 +3254,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3328,7 +3283,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3">
@@ -3351,7 +3306,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4">
@@ -3362,7 +3317,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -3374,7 +3329,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5">
@@ -3385,7 +3340,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -3397,7 +3352,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6">
@@ -3420,7 +3375,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7">
@@ -3443,7 +3398,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8">
@@ -3454,7 +3409,7 @@
         <v>51</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -3466,7 +3421,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="9">
@@ -3477,7 +3432,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -3489,7 +3444,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10">
@@ -3512,7 +3467,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11">
@@ -3535,7 +3490,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12">
@@ -3546,7 +3501,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -3558,7 +3513,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13">
@@ -3569,7 +3524,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -3581,7 +3536,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14">
@@ -3604,7 +3559,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15">
@@ -3615,7 +3570,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -3627,7 +3582,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
     </row>
     <row r="16">
@@ -3650,7 +3605,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
     </row>
     <row r="17">
@@ -3661,7 +3616,7 @@
         <v>29</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D17" s="0">
         <v>134</v>
@@ -3673,7 +3628,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -3693,10 +3648,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3704,35 +3659,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B3" s="0">
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -3752,10 +3707,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3764,13 +3719,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3799,7 +3754,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3">
@@ -3825,7 +3780,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4">
@@ -3851,7 +3806,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5">
@@ -3877,7 +3832,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6">
@@ -3903,7 +3858,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7">
@@ -3929,7 +3884,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8">
@@ -3955,7 +3910,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9">
@@ -3981,7 +3936,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10">
@@ -4007,7 +3962,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11">
@@ -4033,7 +3988,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="12">
@@ -4059,7 +4014,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13">
@@ -4085,12 +4040,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: venta de la semana del 12/10 en 17.000 (Gonzalo); sab 17/10 24.277, falta 1
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="162">
   <si>
     <t>fecha</t>
   </si>
@@ -357,6 +357,12 @@
   </si>
   <si>
     <t>total 16.000 = BO 1.050 (1 carga) + BR 9929 + PY 5021 (resto con el mix BR/PY del ERP ult. 4 sem)</t>
+  </si>
+  <si>
+    <t>Gonzalo 06/10: "la segunda semana la venta es de 17 no 18"</t>
+  </si>
+  <si>
+    <t>total 17.000 = BO 1.050 (1 carga) + BR 10593 + PY 5357 (resto con el mix BR/PY del ERP ult. 4 sem)</t>
   </si>
   <si>
     <t>SUPUESTO 18.000 (Gonzalo 01/10: "si sube es a 18 mil la venta, no mas"; verano)</t>
@@ -2880,13 +2886,13 @@
         <v>46307</v>
       </c>
       <c r="B6" s="0">
-        <v>11106</v>
+        <v>10593</v>
       </c>
       <c r="C6" s="0">
-        <v>5616</v>
+        <v>5357</v>
       </c>
       <c r="D6" s="0">
-        <v>1278</v>
+        <v>1050</v>
       </c>
       <c r="E6" s="0" t="s">
         <v>113</v>
@@ -2909,10 +2915,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -2930,57 +2936,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -3028,10 +3034,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3">
@@ -3045,10 +3051,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4">
@@ -3062,10 +3068,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5">
@@ -3073,16 +3079,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6">
@@ -3096,10 +3102,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7">
@@ -3113,10 +3119,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8">
@@ -3130,10 +3136,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9">
@@ -3141,16 +3147,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10">
@@ -3164,10 +3170,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11">
@@ -3181,10 +3187,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12">
@@ -3198,10 +3204,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13">
@@ -3209,16 +3215,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -3254,10 +3260,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3283,7 +3289,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3">
@@ -3306,7 +3312,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4">
@@ -3329,7 +3335,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5">
@@ -3340,7 +3346,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -3352,7 +3358,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6">
@@ -3375,7 +3381,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7">
@@ -3398,7 +3404,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8">
@@ -3421,7 +3427,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9">
@@ -3432,7 +3438,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -3444,7 +3450,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10">
@@ -3467,7 +3473,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11">
@@ -3490,7 +3496,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="12">
@@ -3513,7 +3519,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13">
@@ -3524,7 +3530,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -3536,7 +3542,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14">
@@ -3559,7 +3565,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15">
@@ -3570,7 +3576,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -3582,7 +3588,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="16">
@@ -3605,7 +3611,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="17">
@@ -3628,7 +3634,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -3648,10 +3654,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3659,35 +3665,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B3" s="0">
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -3710,7 +3716,7 @@
         <v>104</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3722,10 +3728,10 @@
         <v>105</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3754,7 +3760,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3">
@@ -3780,7 +3786,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4">
@@ -3806,7 +3812,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5">
@@ -3832,7 +3838,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6">
@@ -3858,7 +3864,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7">
@@ -3884,7 +3890,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8">
@@ -3910,7 +3916,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9">
@@ -3936,7 +3942,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10">
@@ -3962,7 +3968,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11">
@@ -3988,7 +3994,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12">
@@ -4014,7 +4020,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13">
@@ -4040,12 +4046,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: dictado del 07/10 para la semana 12-17/10 (BR 10, PY 5 incl. HF domingo); sab 17/10 23.297, faltan 2
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="160">
   <si>
     <t>fecha</t>
   </si>
@@ -224,112 +224,106 @@
     <t>carga real: cuarta Nilton, R$ 35 (no estaba dictada)</t>
   </si>
   <si>
+    <t>2026-10-04</t>
+  </si>
+  <si>
+    <t>Gonzalo 06/10 (chat, 2da version)</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Fisher 2: tersa; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Fisher 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Agro 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Cassio 1: cuarta</t>
+  </si>
+  <si>
+    <t>Celso</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Celso 1: cuarta. PRODUCTOR NUEVO: falta nombre completo y transporte</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Ivo 2: tersa</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Ivo 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Stein 1: tersa</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Milciades 2: lunes</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Milciades 2: martes</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Diego 2: lunes</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Diego 2: martes</t>
+  </si>
+  <si>
+    <t>dictado 06/10 (corregido): Alvarito 1: lunes</t>
+  </si>
+  <si>
     <t>2026-10-11</t>
   </si>
   <si>
-    <t>Gonzalo 06/10 (chat)</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Fisher 1: sabado (descarga martes 20, semana siguiente)</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Agro 2: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Agro 2: sexta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Cassio 2: tersa</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Cassio 2: sexta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Ivo 2: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Ivo 2: sexta</t>
-  </si>
-  <si>
-    <t>Celso</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Celso 1: cuarta. PRODUCTOR NUEVO: falta nombre completo y transporte</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Marconi 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Josemar 1: sexta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Stein 1: sexta</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Alvarito 1: lunes</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Diego 2: lunes</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Diego 2: martes</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Milciades 2: lunes</t>
-  </si>
-  <si>
-    <t>dictado 06/10: Milciades 2: martes</t>
+    <t>Gonzalo 07/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Fisher 2: tersa; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Fisher 2: sabado (descarga martes 20, semana siguiente)</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Stein 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Stein 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Agro 1: sexta</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Cassio 2: tersa</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Cassio 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Ivo 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Marconi 1: sexta</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Josemar 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Alvarito 1: lunes</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Diego 1: lunes</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Milciades 1: lunes</t>
   </si>
   <si>
     <t>Paraguay GM</t>
   </si>
   <si>
-    <t>dictado 06/10: Guido 1: martes</t>
-  </si>
-  <si>
-    <t>2026-10-04</t>
-  </si>
-  <si>
-    <t>Gonzalo 06/10 (chat, 2da version)</t>
-  </si>
-  <si>
-    <t>dictado 06/10 (corregido): Fisher 2: tersa; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 06/10 (corregido): Fisher 2: sexta</t>
-  </si>
-  <si>
-    <t>dictado 06/10 (corregido): Agro 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 06/10 (corregido): Cassio 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 06/10 (corregido): Celso 1: cuarta. PRODUCTOR NUEVO: falta nombre completo y transporte</t>
-  </si>
-  <si>
-    <t>dictado 06/10 (corregido): Ivo 2: tersa</t>
-  </si>
-  <si>
-    <t>dictado 06/10 (corregido): Ivo 2: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 06/10 (corregido): Stein 1: tersa</t>
-  </si>
-  <si>
-    <t>dictado 06/10 (corregido): Milciades 2: lunes</t>
-  </si>
-  <si>
-    <t>dictado 06/10 (corregido): Milciades 2: martes</t>
-  </si>
-  <si>
-    <t>dictado 06/10 (corregido): Diego 2: lunes</t>
-  </si>
-  <si>
-    <t>dictado 06/10 (corregido): Diego 2: martes</t>
-  </si>
-  <si>
-    <t>dictado 06/10 (corregido): Alvarito 1: lunes</t>
+    <t>dictado 07/10: Guido 1: martes</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Hugo 1: domingo (Hugo = HF)</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -572,7 +566,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -1805,10 +1799,10 @@
     </row>
     <row r="39">
       <c r="A39" s="15">
-        <v>46312</v>
+        <v>46301</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C39" s="0" t="s">
         <v>68</v>
@@ -1820,10 +1814,10 @@
         <v>30</v>
       </c>
       <c r="F39" s="0" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G39" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H39" s="0">
         <v>1008</v>
@@ -1837,10 +1831,10 @@
     </row>
     <row r="40">
       <c r="A40" s="15">
-        <v>46309</v>
+        <v>46304</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C40" s="0" t="s">
         <v>68</v>
@@ -1849,7 +1843,7 @@
         <v>23</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="F40" s="0" t="s">
         <v>14</v>
@@ -1869,10 +1863,10 @@
     </row>
     <row r="41">
       <c r="A41" s="15">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C41" s="0" t="s">
         <v>68</v>
@@ -1901,10 +1895,10 @@
     </row>
     <row r="42">
       <c r="A42" s="15">
-        <v>46308</v>
+        <v>46302</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C42" s="0" t="s">
         <v>68</v>
@@ -1933,10 +1927,10 @@
     </row>
     <row r="43">
       <c r="A43" s="15">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C43" s="0" t="s">
         <v>68</v>
@@ -1945,7 +1939,7 @@
         <v>23</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="F43" s="0" t="s">
         <v>14</v>
@@ -1954,21 +1948,21 @@
         <v>14</v>
       </c>
       <c r="H43" s="0">
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="I43" s="0" t="s">
         <v>69</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="15">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C44" s="0" t="s">
         <v>68</v>
@@ -1992,15 +1986,15 @@
         <v>69</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="15">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C45" s="0" t="s">
         <v>68</v>
@@ -2024,15 +2018,15 @@
         <v>69</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="15">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C46" s="0" t="s">
         <v>68</v>
@@ -2041,7 +2035,7 @@
         <v>23</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F46" s="0" t="s">
         <v>14</v>
@@ -2061,19 +2055,19 @@
     </row>
     <row r="47">
       <c r="A47" s="15">
-        <v>46309</v>
+        <v>46300</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="C47" s="0" t="s">
         <v>68</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="F47" s="0" t="s">
         <v>14</v>
@@ -2082,7 +2076,7 @@
         <v>14</v>
       </c>
       <c r="H47" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I47" s="0" t="s">
         <v>69</v>
@@ -2093,19 +2087,19 @@
     </row>
     <row r="48">
       <c r="A48" s="15">
-        <v>46311</v>
+        <v>46301</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C48" s="0" t="s">
         <v>68</v>
       </c>
       <c r="D48" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="F48" s="0" t="s">
         <v>14</v>
@@ -2114,7 +2108,7 @@
         <v>14</v>
       </c>
       <c r="H48" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I48" s="0" t="s">
         <v>69</v>
@@ -2125,19 +2119,19 @@
     </row>
     <row r="49">
       <c r="A49" s="15">
-        <v>46311</v>
+        <v>46300</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C49" s="0" t="s">
         <v>68</v>
       </c>
       <c r="D49" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="F49" s="0" t="s">
         <v>14</v>
@@ -2146,7 +2140,7 @@
         <v>14</v>
       </c>
       <c r="H49" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I49" s="0" t="s">
         <v>69</v>
@@ -2157,10 +2151,10 @@
     </row>
     <row r="50">
       <c r="A50" s="15">
-        <v>46307</v>
+        <v>46301</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C50" s="0" t="s">
         <v>68</v>
@@ -2169,7 +2163,7 @@
         <v>12</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F50" s="0" t="s">
         <v>14</v>
@@ -2189,7 +2183,7 @@
     </row>
     <row r="51">
       <c r="A51" s="15">
-        <v>46307</v>
+        <v>46300</v>
       </c>
       <c r="B51" s="0" t="s">
         <v>18</v>
@@ -2201,7 +2195,7 @@
         <v>12</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F51" s="0" t="s">
         <v>14</v>
@@ -2220,52 +2214,52 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="15">
+      <c r="A52" s="16">
         <v>46308</v>
       </c>
       <c r="B52" s="0" t="s">
         <v>20</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G52" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H52" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I52" s="0" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="J52" s="0" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="16">
+        <v>46312</v>
+      </c>
+      <c r="B53" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C53" s="0" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="15">
-        <v>46307</v>
-      </c>
-      <c r="B53" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="C53" s="0" t="s">
-        <v>68</v>
-      </c>
       <c r="D53" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F53" s="0" t="s">
         <v>14</v>
@@ -2274,62 +2268,62 @@
         <v>14</v>
       </c>
       <c r="H53" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="J53" s="0" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B54" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C54" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="D54" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E54" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="F54" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G54" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H54" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I54" s="0" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="15">
-        <v>46308</v>
-      </c>
-      <c r="B54" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="C54" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="D54" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E54" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="F54" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G54" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H54" s="0">
-        <v>980</v>
-      </c>
-      <c r="I54" s="0" t="s">
-        <v>69</v>
-      </c>
       <c r="J54" s="0" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="15">
-        <v>46308</v>
+      <c r="A55" s="16">
+        <v>46311</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C55" s="0" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="D55" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="F55" s="0" t="s">
         <v>14</v>
@@ -2338,62 +2332,62 @@
         <v>14</v>
       </c>
       <c r="H55" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="J55" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="16">
-        <v>46301</v>
+        <v>46311</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D56" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H56" s="0">
         <v>1008</v>
       </c>
       <c r="I56" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="J56" s="0" t="s">
         <v>90</v>
-      </c>
-      <c r="J56" s="0" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="16">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C57" s="0" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D57" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F57" s="0" t="s">
         <v>14</v>
@@ -2402,30 +2396,30 @@
         <v>14</v>
       </c>
       <c r="H57" s="0">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J57" s="0" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="16">
-        <v>46302</v>
+        <v>46311</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C58" s="0" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D58" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="F58" s="0" t="s">
         <v>14</v>
@@ -2434,30 +2428,30 @@
         <v>14</v>
       </c>
       <c r="H58" s="0">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="16">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="B59" s="0" t="s">
         <v>51</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D59" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F59" s="0" t="s">
         <v>14</v>
@@ -2466,30 +2460,30 @@
         <v>14</v>
       </c>
       <c r="H59" s="0">
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="I59" s="0" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J59" s="0" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="16">
-        <v>46302</v>
+        <v>46311</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D60" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="F60" s="0" t="s">
         <v>14</v>
@@ -2501,27 +2495,27 @@
         <v>1008</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J60" s="0" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="16">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D61" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="F61" s="0" t="s">
         <v>14</v>
@@ -2533,27 +2527,27 @@
         <v>1008</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J61" s="0" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="16">
-        <v>46302</v>
+        <v>46307</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="C62" s="0" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F62" s="0" t="s">
         <v>14</v>
@@ -2562,30 +2556,30 @@
         <v>14</v>
       </c>
       <c r="H62" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I62" s="0" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J62" s="0" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="16">
-        <v>46301</v>
+        <v>46307</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D63" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="F63" s="0" t="s">
         <v>14</v>
@@ -2594,24 +2588,24 @@
         <v>14</v>
       </c>
       <c r="H63" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="16">
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="B64" s="0" t="s">
         <v>18</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D64" s="0" t="s">
         <v>12</v>
@@ -2629,27 +2623,27 @@
         <v>980</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J64" s="0" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="16">
-        <v>46301</v>
+        <v>46308</v>
       </c>
       <c r="B65" s="0" t="s">
         <v>20</v>
       </c>
       <c r="C65" s="0" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D65" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>19</v>
+        <v>99</v>
       </c>
       <c r="F65" s="0" t="s">
         <v>14</v>
@@ -2661,7 +2655,7 @@
         <v>980</v>
       </c>
       <c r="I65" s="0" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J65" s="0" t="s">
         <v>100</v>
@@ -2669,19 +2663,19 @@
     </row>
     <row r="66">
       <c r="A66" s="16">
-        <v>46300</v>
+        <v>46306</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C66" s="0" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D66" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F66" s="0" t="s">
         <v>14</v>
@@ -2693,74 +2687,10 @@
         <v>980</v>
       </c>
       <c r="I66" s="0" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J66" s="0" t="s">
         <v>101</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="16">
-        <v>46301</v>
-      </c>
-      <c r="B67" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="C67" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="D67" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E67" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F67" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G67" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H67" s="0">
-        <v>980</v>
-      </c>
-      <c r="I67" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="J67" s="0" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="16">
-        <v>46300</v>
-      </c>
-      <c r="B68" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="C68" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="D68" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E68" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="F68" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G68" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H68" s="0">
-        <v>980</v>
-      </c>
-      <c r="I68" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="J68" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2783,7 +2713,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -2792,7 +2722,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>8</v>
@@ -2815,10 +2745,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3">
@@ -2835,10 +2765,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="F3" s="0" t="s">
         <v>106</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="4">
@@ -2855,10 +2785,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5">
@@ -2875,10 +2805,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6">
@@ -2895,10 +2825,10 @@
         <v>1050</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7">
@@ -2915,10 +2845,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -2936,57 +2866,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -3034,10 +2964,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3">
@@ -3051,10 +2981,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="E3" s="0" t="s">
         <v>128</v>
-      </c>
-      <c r="E3" s="0" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="4">
@@ -3062,16 +2992,16 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5">
@@ -3079,16 +3009,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6">
@@ -3102,10 +3032,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7">
@@ -3119,10 +3049,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="E7" s="0" t="s">
         <v>134</v>
-      </c>
-      <c r="E7" s="0" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="8">
@@ -3130,16 +3060,16 @@
         <v>46291</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C8" s="0">
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9">
@@ -3147,16 +3077,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10">
@@ -3170,10 +3100,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11">
@@ -3187,10 +3117,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="E11" s="0" t="s">
         <v>139</v>
-      </c>
-      <c r="E11" s="0" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="12">
@@ -3198,16 +3128,16 @@
         <v>46298</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C12" s="0">
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13">
@@ -3215,16 +3145,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -3260,10 +3190,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3289,7 +3219,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3">
@@ -3312,7 +3242,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4">
@@ -3323,7 +3253,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -3335,7 +3265,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5">
@@ -3346,7 +3276,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -3358,7 +3288,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6">
@@ -3381,7 +3311,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7">
@@ -3404,7 +3334,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8">
@@ -3415,7 +3345,7 @@
         <v>51</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -3427,7 +3357,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="9">
@@ -3438,7 +3368,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -3450,7 +3380,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10">
@@ -3473,7 +3403,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11">
@@ -3496,7 +3426,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12">
@@ -3507,7 +3437,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -3519,7 +3449,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13">
@@ -3530,7 +3460,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -3542,7 +3472,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14">
@@ -3565,7 +3495,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15">
@@ -3576,7 +3506,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -3588,7 +3518,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="16">
@@ -3611,7 +3541,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="17">
@@ -3622,7 +3552,7 @@
         <v>29</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D17" s="0">
         <v>134</v>
@@ -3634,7 +3564,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -3654,10 +3584,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3665,35 +3595,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B3" s="0">
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -3713,10 +3643,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3725,13 +3655,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3760,7 +3690,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3">
@@ -3786,7 +3716,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4">
@@ -3812,7 +3742,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5">
@@ -3838,7 +3768,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6">
@@ -3864,7 +3794,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7">
@@ -3890,7 +3820,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8">
@@ -3916,7 +3846,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9">
@@ -3942,7 +3872,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10">
@@ -3968,7 +3898,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11">
@@ -3994,7 +3924,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="12">
@@ -4020,7 +3950,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13">
@@ -4046,12 +3976,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Gilson miercoles 14/10 agregado a la semana 12-17/10; sab 17/10 24.305, falta 1
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="162">
   <si>
     <t>fecha</t>
   </si>
@@ -324,6 +324,12 @@
   </si>
   <si>
     <t>dictado 07/10: Hugo 1: domingo (Hugo = HF)</t>
+  </si>
+  <si>
+    <t>Gonzalo 07/10 (chat, 2da version)</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Gilson 1: cuarta (agregado en la segunda version); transportista supuesto = habitual</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -538,7 +544,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -556,6 +562,7 @@
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -566,7 +573,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:J67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -2691,6 +2698,38 @@
       </c>
       <c r="J66" s="0" t="s">
         <v>101</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="17">
+        <v>46309</v>
+      </c>
+      <c r="B67" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C67" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="D67" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E67" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="F67" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G67" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H67" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I67" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J67" s="0" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2713,7 +2752,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -2722,7 +2761,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>8</v>
@@ -2745,10 +2784,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3">
@@ -2765,10 +2804,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4">
@@ -2785,10 +2824,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5">
@@ -2805,10 +2844,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6">
@@ -2825,10 +2864,10 @@
         <v>1050</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7">
@@ -2845,10 +2884,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -2866,57 +2905,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -2964,10 +3003,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3">
@@ -2981,10 +3020,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4">
@@ -2992,16 +3031,16 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5">
@@ -3009,16 +3048,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6">
@@ -3032,10 +3071,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7">
@@ -3049,10 +3088,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8">
@@ -3060,16 +3099,16 @@
         <v>46291</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C8" s="0">
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9">
@@ -3077,16 +3116,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10">
@@ -3100,10 +3139,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11">
@@ -3117,10 +3156,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12">
@@ -3128,16 +3167,16 @@
         <v>46298</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C12" s="0">
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13">
@@ -3145,16 +3184,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -3190,10 +3229,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3219,7 +3258,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3">
@@ -3242,7 +3281,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4">
@@ -3253,7 +3292,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -3265,7 +3304,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5">
@@ -3276,7 +3315,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -3288,7 +3327,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6">
@@ -3311,7 +3350,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7">
@@ -3334,7 +3373,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8">
@@ -3345,7 +3384,7 @@
         <v>51</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -3357,7 +3396,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9">
@@ -3368,7 +3407,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -3380,7 +3419,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10">
@@ -3403,7 +3442,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11">
@@ -3426,7 +3465,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="12">
@@ -3437,7 +3476,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -3449,7 +3488,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13">
@@ -3460,7 +3499,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -3472,7 +3511,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14">
@@ -3495,7 +3534,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15">
@@ -3506,7 +3545,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -3518,7 +3557,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="16">
@@ -3541,7 +3580,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="17">
@@ -3552,7 +3591,7 @@
         <v>29</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D17" s="0">
         <v>134</v>
@@ -3564,7 +3603,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -3584,10 +3623,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3595,35 +3634,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B3" s="0">
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -3643,10 +3682,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3655,13 +3694,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3690,7 +3729,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3">
@@ -3716,7 +3755,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4">
@@ -3742,7 +3781,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5">
@@ -3768,7 +3807,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6">
@@ -3794,7 +3833,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7">
@@ -3820,7 +3859,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8">
@@ -3846,7 +3885,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9">
@@ -3872,7 +3911,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10">
@@ -3898,7 +3937,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11">
@@ -3924,7 +3963,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12">
@@ -3950,7 +3989,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13">
@@ -3976,12 +4015,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Agro pasa del viernes 16 al miercoles 14; sab 17/10 cierra en 25.313
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -290,7 +290,7 @@
     <t>dictado 07/10: Stein 2: sexta</t>
   </si>
   <si>
-    <t>dictado 07/10: Agro 1: sexta</t>
+    <t>dictado 07/10: Agro 1: era sexta, Gonzalo 07/10 "agro pasa para cuarta entonces" (para cerrar el sab 17); transportista supuesto = habitual</t>
   </si>
   <si>
     <t>dictado 07/10: Cassio 2: tersa</t>
@@ -2350,10 +2350,10 @@
     </row>
     <row r="56">
       <c r="A56" s="16">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C56" s="0" t="s">
         <v>84</v>

</xml_diff>

<commit_message>
plan de compras: 12 pallets de banana de Furlani en camion mixto el martes 13 (432 cajas); sab 17/10 25.745
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="164">
   <si>
     <t>fecha</t>
   </si>
@@ -330,6 +330,12 @@
   </si>
   <si>
     <t>dictado 07/10: Gilson 1: cuarta (agregado en la segunda version); transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>Furlani</t>
+  </si>
+  <si>
+    <t>dictado 07/10: "martes 13 tenemos 12 palet de banana que va a cargar con exoticos", "de Furlani"; 12 pallets x 36 cajas = 432 (carga parcial, camion mixto con exoticos). Si Aloha lo registra como Varios/Exoticos el plan no lo cuenta y esta fila queda</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -544,7 +550,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -563,6 +569,7 @@
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -573,7 +580,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J67"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -2730,6 +2737,38 @@
       </c>
       <c r="J67" s="0" t="s">
         <v>103</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="18">
+        <v>46308</v>
+      </c>
+      <c r="B68" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C68" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="D68" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E68" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="F68" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G68" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H68" s="0">
+        <v>432</v>
+      </c>
+      <c r="I68" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="J68" s="0" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -2752,7 +2791,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -2761,7 +2800,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>8</v>
@@ -2784,10 +2823,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3">
@@ -2804,10 +2843,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4">
@@ -2824,10 +2863,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5">
@@ -2844,10 +2883,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6">
@@ -2864,10 +2903,10 @@
         <v>1050</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7">
@@ -2884,10 +2923,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -2905,57 +2944,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -3003,10 +3042,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3">
@@ -3020,10 +3059,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4">
@@ -3031,16 +3070,16 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5">
@@ -3048,16 +3087,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6">
@@ -3071,10 +3110,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7">
@@ -3088,10 +3127,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8">
@@ -3099,16 +3138,16 @@
         <v>46291</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C8" s="0">
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9">
@@ -3116,16 +3155,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10">
@@ -3139,10 +3178,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11">
@@ -3156,10 +3195,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="12">
@@ -3167,16 +3206,16 @@
         <v>46298</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C12" s="0">
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13">
@@ -3184,16 +3223,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -3229,10 +3268,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3258,7 +3297,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3">
@@ -3281,7 +3320,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4">
@@ -3292,7 +3331,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -3304,7 +3343,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5">
@@ -3315,7 +3354,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -3327,7 +3366,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6">
@@ -3350,7 +3389,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7">
@@ -3373,7 +3412,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8">
@@ -3384,7 +3423,7 @@
         <v>51</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -3396,7 +3435,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9">
@@ -3407,7 +3446,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -3419,7 +3458,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10">
@@ -3442,7 +3481,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11">
@@ -3465,7 +3504,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12">
@@ -3476,7 +3515,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -3488,7 +3527,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="13">
@@ -3499,7 +3538,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -3511,7 +3550,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14">
@@ -3534,7 +3573,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="15">
@@ -3545,7 +3584,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -3557,7 +3596,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="16">
@@ -3580,7 +3619,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="17">
@@ -3591,7 +3630,7 @@
         <v>29</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D17" s="0">
         <v>134</v>
@@ -3603,7 +3642,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -3623,10 +3662,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3634,35 +3673,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B3" s="0">
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -3682,10 +3721,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3694,13 +3733,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3729,7 +3768,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3">
@@ -3755,7 +3794,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4">
@@ -3781,7 +3820,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5">
@@ -3807,7 +3846,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6">
@@ -3833,7 +3872,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7">
@@ -3859,7 +3898,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8">
@@ -3885,7 +3924,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9">
@@ -3911,7 +3950,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10">
@@ -3937,7 +3976,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11">
@@ -3963,7 +4002,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12">
@@ -3989,7 +4028,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13">
@@ -4015,12 +4054,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Shapo viernes 16/10 agregado a la semana 12-17; sab 24/10 18.663
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="166">
   <si>
     <t>fecha</t>
   </si>
@@ -336,6 +336,12 @@
   </si>
   <si>
     <t>dictado 07/10: "martes 13 tenemos 12 palet de banana que va a cargar con exoticos", "de Furlani"; 12 pallets x 36 cajas = 432 (carga parcial, camion mixto con exoticos). Si Aloha lo registra como Varios/Exoticos el plan no lo cuenta y esta fila queda</t>
+  </si>
+  <si>
+    <t>Shapo</t>
+  </si>
+  <si>
+    <t>dictado 07/10: Shapo 1: sexta (agregado en la tercera version del dictado de la semana 12-17)</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -550,7 +556,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -570,6 +576,7 @@
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -580,7 +587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -2769,6 +2776,38 @@
       </c>
       <c r="J68" s="0" t="s">
         <v>105</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="19">
+        <v>46311</v>
+      </c>
+      <c r="B69" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C69" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="D69" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E69" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="F69" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G69" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H69" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I69" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="J69" s="0" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -2791,7 +2830,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -2800,7 +2839,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>8</v>
@@ -2823,10 +2862,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3">
@@ -2843,10 +2882,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4">
@@ -2863,10 +2902,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5">
@@ -2883,10 +2922,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6">
@@ -2903,10 +2942,10 @@
         <v>1050</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7">
@@ -2923,10 +2962,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -2944,57 +2983,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -3042,10 +3081,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3">
@@ -3059,10 +3098,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4">
@@ -3070,16 +3109,16 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5">
@@ -3087,16 +3126,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6">
@@ -3110,10 +3149,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7">
@@ -3127,10 +3166,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="8">
@@ -3138,16 +3177,16 @@
         <v>46291</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C8" s="0">
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="9">
@@ -3155,16 +3194,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10">
@@ -3178,10 +3217,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11">
@@ -3195,10 +3234,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12">
@@ -3206,16 +3245,16 @@
         <v>46298</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C12" s="0">
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13">
@@ -3223,16 +3262,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -3268,10 +3307,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3297,7 +3336,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3">
@@ -3320,7 +3359,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4">
@@ -3331,7 +3370,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -3343,7 +3382,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5">
@@ -3354,7 +3393,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -3366,7 +3405,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6">
@@ -3389,7 +3428,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7">
@@ -3412,7 +3451,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8">
@@ -3423,7 +3462,7 @@
         <v>51</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -3435,7 +3474,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9">
@@ -3446,7 +3485,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -3458,7 +3497,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10">
@@ -3481,7 +3520,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11">
@@ -3504,7 +3543,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="12">
@@ -3515,7 +3554,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -3527,7 +3566,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13">
@@ -3538,7 +3577,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -3550,7 +3589,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14">
@@ -3573,7 +3612,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15">
@@ -3584,7 +3623,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -3596,7 +3635,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="16">
@@ -3619,7 +3658,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="17">
@@ -3630,7 +3669,7 @@
         <v>29</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D17" s="0">
         <v>134</v>
@@ -3642,7 +3681,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -3662,10 +3701,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3673,35 +3712,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B3" s="0">
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -3721,10 +3760,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3733,13 +3772,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3768,7 +3807,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3">
@@ -3794,7 +3833,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4">
@@ -3820,7 +3859,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="5">
@@ -3846,7 +3885,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6">
@@ -3872,7 +3911,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7">
@@ -3898,7 +3937,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="8">
@@ -3924,7 +3963,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9">
@@ -3950,7 +3989,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10">
@@ -3976,7 +4015,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="11">
@@ -4002,7 +4041,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12">
@@ -4028,7 +4067,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13">
@@ -4054,12 +4093,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Paraguay a 3 por el precio de USD 8 (redictado 12-17), supuestos PY solo en semanas sin dictar; sab 17/10 24.793
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
   <si>
     <t>fecha</t>
   </si>
@@ -275,73 +275,64 @@
     <t>2026-10-11</t>
   </si>
   <si>
-    <t>Gonzalo 07/10 (chat)</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Fisher 2: tersa; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Fisher 2: sabado (descarga martes 20, semana siguiente)</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Stein 2: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Stein 2: sexta</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Agro 1: era sexta, Gonzalo 07/10 "agro pasa para cuarta entonces" (para cerrar el sab 17); transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Cassio 2: tersa</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Cassio 2: sexta</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Ivo 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Marconi 1: sexta</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Josemar 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Alvarito 1: lunes</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Diego 1: lunes</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Milciades 1: lunes</t>
+    <t>Gonzalo 08/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Fisher 2: cuarta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Fisher 2: sabado (descarga martes 20, semana siguiente)</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Stein 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Stein 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Agro 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Cassio 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Cassio 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Ivo 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Marconi 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Josemar 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Gilson 1: cuarta</t>
+  </si>
+  <si>
+    <t>Shapo</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Shapo 1: sexta</t>
+  </si>
+  <si>
+    <t>Furlani</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): 12 pallets de banana en camion mixto con exoticos (dictado 07/10, se mantiene)</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Alvarito 1: lunes</t>
+  </si>
+  <si>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Milciades 1: lunes</t>
   </si>
   <si>
     <t>Paraguay GM</t>
   </si>
   <si>
-    <t>dictado 07/10: Guido 1: martes</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Hugo 1: domingo (Hugo = HF)</t>
-  </si>
-  <si>
-    <t>Gonzalo 07/10 (chat, 2da version)</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Gilson 1: cuarta (agregado en la segunda version); transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>Furlani</t>
-  </si>
-  <si>
-    <t>dictado 07/10: "martes 13 tenemos 12 palet de banana que va a cargar con exoticos", "de Furlani"; 12 pallets x 36 cajas = 432 (carga parcial, camion mixto con exoticos). Si Aloha lo registra como Varios/Exoticos el plan no lo cuenta y esta fila queda</t>
-  </si>
-  <si>
-    <t>Shapo</t>
-  </si>
-  <si>
-    <t>dictado 07/10: Shapo 1: sexta (agregado en la tercera version del dictado de la semana 12-17)</t>
+    <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Guido 1: martes</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -556,7 +547,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -574,9 +565,6 @@
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -587,7 +575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -2236,10 +2224,10 @@
     </row>
     <row r="52">
       <c r="A52" s="16">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C52" s="0" t="s">
         <v>84</v>
@@ -2396,10 +2384,10 @@
     </row>
     <row r="57">
       <c r="A57" s="16">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C57" s="0" t="s">
         <v>84</v>
@@ -2492,10 +2480,10 @@
     </row>
     <row r="60">
       <c r="A60" s="16">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C60" s="0" t="s">
         <v>84</v>
@@ -2556,19 +2544,19 @@
     </row>
     <row r="62">
       <c r="A62" s="16">
-        <v>46307</v>
+        <v>46309</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="C62" s="0" t="s">
         <v>84</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="F62" s="0" t="s">
         <v>14</v>
@@ -2577,7 +2565,7 @@
         <v>14</v>
       </c>
       <c r="H62" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I62" s="0" t="s">
         <v>85</v>
@@ -2588,19 +2576,19 @@
     </row>
     <row r="63">
       <c r="A63" s="16">
-        <v>46307</v>
+        <v>46311</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C63" s="0" t="s">
         <v>84</v>
       </c>
       <c r="D63" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>13</v>
+        <v>97</v>
       </c>
       <c r="F63" s="0" t="s">
         <v>14</v>
@@ -2609,30 +2597,30 @@
         <v>14</v>
       </c>
       <c r="H63" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I63" s="0" t="s">
         <v>85</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="16">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B64" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C64" s="0" t="s">
         <v>84</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>19</v>
+        <v>99</v>
       </c>
       <c r="F64" s="0" t="s">
         <v>14</v>
@@ -2641,21 +2629,21 @@
         <v>14</v>
       </c>
       <c r="H64" s="0">
-        <v>980</v>
+        <v>432</v>
       </c>
       <c r="I64" s="0" t="s">
         <v>85</v>
       </c>
       <c r="J64" s="0" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="16">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="B65" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C65" s="0" t="s">
         <v>84</v>
@@ -2664,7 +2652,7 @@
         <v>12</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>99</v>
+        <v>21</v>
       </c>
       <c r="F65" s="0" t="s">
         <v>14</v>
@@ -2679,15 +2667,15 @@
         <v>85</v>
       </c>
       <c r="J65" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="16">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C66" s="0" t="s">
         <v>84</v>
@@ -2696,7 +2684,7 @@
         <v>12</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F66" s="0" t="s">
         <v>14</v>
@@ -2711,103 +2699,39 @@
         <v>85</v>
       </c>
       <c r="J66" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="17">
-        <v>46309</v>
+      <c r="A67" s="16">
+        <v>46308</v>
       </c>
       <c r="B67" s="0" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C67" s="0" t="s">
         <v>84</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E67" s="0" t="s">
-        <v>42</v>
+        <v>103</v>
       </c>
       <c r="F67" s="0" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G67" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H67" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I67" s="0" t="s">
-        <v>102</v>
+        <v>85</v>
       </c>
       <c r="J67" s="0" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="18">
-        <v>46308</v>
-      </c>
-      <c r="B68" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="C68" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="D68" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E68" s="0" t="s">
         <v>104</v>
-      </c>
-      <c r="F68" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G68" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H68" s="0">
-        <v>432</v>
-      </c>
-      <c r="I68" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="J68" s="0" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="19">
-        <v>46311</v>
-      </c>
-      <c r="B69" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="C69" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="D69" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E69" s="0" t="s">
-        <v>106</v>
-      </c>
-      <c r="F69" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G69" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H69" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I69" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="J69" s="0" t="s">
-        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -2830,7 +2754,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -2839,7 +2763,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>8</v>
@@ -2862,10 +2786,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3">
@@ -2882,10 +2806,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4">
@@ -2902,10 +2826,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5">
@@ -2922,10 +2846,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6">
@@ -2942,10 +2866,10 @@
         <v>1050</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7">
@@ -2962,10 +2886,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -2983,57 +2907,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -3081,10 +3005,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3">
@@ -3098,10 +3022,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4">
@@ -3109,16 +3033,16 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="E4" s="0" t="s">
         <v>132</v>
-      </c>
-      <c r="E4" s="0" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="5">
@@ -3126,16 +3050,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6">
@@ -3149,10 +3073,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7">
@@ -3166,10 +3090,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8">
@@ -3177,16 +3101,16 @@
         <v>46291</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C8" s="0">
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="E8" s="0" t="s">
         <v>138</v>
-      </c>
-      <c r="E8" s="0" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="9">
@@ -3194,16 +3118,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10">
@@ -3217,10 +3141,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11">
@@ -3234,10 +3158,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12">
@@ -3245,16 +3169,16 @@
         <v>46298</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C12" s="0">
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
+        <v>140</v>
+      </c>
+      <c r="E12" s="0" t="s">
         <v>143</v>
-      </c>
-      <c r="E12" s="0" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="13">
@@ -3262,16 +3186,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -3307,10 +3231,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3336,7 +3260,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3">
@@ -3359,7 +3283,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4">
@@ -3370,7 +3294,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -3382,7 +3306,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5">
@@ -3393,7 +3317,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -3405,7 +3329,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6">
@@ -3428,7 +3352,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7">
@@ -3451,7 +3375,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8">
@@ -3462,7 +3386,7 @@
         <v>51</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -3474,7 +3398,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9">
@@ -3485,7 +3409,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -3497,7 +3421,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10">
@@ -3520,7 +3444,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="11">
@@ -3543,7 +3467,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="12">
@@ -3554,7 +3478,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -3566,7 +3490,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="13">
@@ -3577,7 +3501,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -3589,7 +3513,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14">
@@ -3612,7 +3536,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="15">
@@ -3623,7 +3547,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -3635,7 +3559,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16">
@@ -3658,7 +3582,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="17">
@@ -3669,7 +3593,7 @@
         <v>29</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D17" s="0">
         <v>134</v>
@@ -3681,7 +3605,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -3701,10 +3625,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3712,35 +3636,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B2" s="0">
         <v>5</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B3" s="0">
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -3760,10 +3684,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3772,13 +3696,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3807,7 +3731,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3">
@@ -3833,7 +3757,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4">
@@ -3859,7 +3783,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5">
@@ -3885,7 +3809,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6">
@@ -3911,7 +3835,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7">
@@ -3937,7 +3861,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8">
@@ -3963,7 +3887,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9">
@@ -3989,7 +3913,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10">
@@ -4015,7 +3939,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11">
@@ -4041,7 +3965,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12">
@@ -4067,7 +3991,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13">
@@ -4093,12 +4017,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: sin supuestos de Paraguay ni Bolivia (solo cuentan Aloha y lo dictado); sab 17/10 23.743
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -482,13 +482,13 @@
     <t>py_camiones_semana</t>
   </si>
   <si>
-    <t>Gonzalo 27/09/2026: Paraguay carga domingo, lunes y martes (entra siempre en la semana); por lo general 5/6 camiones. Se usa en las semanas sin cargas PY dictadas ni en el Plan.</t>
+    <t>Gonzalo 08/10/2026: "no hables de supuestos, si no te pase cargas no cuenta". Era 5 (27/09). Con 0 el generador no agrega camiones PY supuestos en ninguna semana.</t>
   </si>
   <si>
     <t>bo_camiones_semana</t>
   </si>
   <si>
-    <t>Gonzalo 01/10/2026: "de Bolivia vamos a descargar uno por semana siempre". Se agrega un camion BO supuesto en cada semana de venta sin descarga BO, cargado 6 dias antes del lunes (si esa fecha no paso).</t>
+    <t>Gonzalo 08/10/2026: "no hables de supuestos, si no te pase cargas no cuenta". Era 1 (01/10: "de Bolivia uno por semana siempre"). Con 0 solo cuentan las cargas BO reales de Aloha o dictadas.</t>
   </si>
   <si>
     <t>minimo_cajas_sabado</t>
@@ -3639,7 +3639,7 @@
         <v>153</v>
       </c>
       <c r="B2" s="0">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>154</v>
@@ -3650,7 +3650,7 @@
         <v>155</v>
       </c>
       <c r="B3" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>156</v>

</xml_diff>

<commit_message>
plan de compras: venta prevista automatica = promedio real de 10 semanas (Aloha) salvo dictado; sab 17/10 24.260
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="161">
   <si>
     <t>fecha</t>
   </si>
@@ -362,16 +362,10 @@
     <t>total 16.000 = BO 1.050 (1 carga) + BR 9929 + PY 5021 (resto con el mix BR/PY del ERP ult. 4 sem)</t>
   </si>
   <si>
-    <t>Gonzalo 06/10: "la segunda semana la venta es de 17 no 18"</t>
-  </si>
-  <si>
-    <t>total 17.000 = BO 1.050 (1 carga) + BR 10593 + PY 5357 (resto con el mix BR/PY del ERP ult. 4 sem)</t>
-  </si>
-  <si>
-    <t>SUPUESTO 18.000 (Gonzalo 01/10: "si sube es a 18 mil la venta, no mas"; verano)</t>
-  </si>
-  <si>
-    <t>total 18000 · mix real ERP ult. 4 sem (31/08-21/09): BR 61,7 % / PY 31,2 % / BO 7,1 %</t>
+    <t>AUTO</t>
+  </si>
+  <si>
+    <t>Gonzalo 11/10/2026 "vamos por el 1": venta prevista = promedio real de las ultimas 10 semanas (Aloha); el generador pisa BR/PY/BO en cada corrida. Si Gonzalo dicta una semana, poner fuente "Gonzalo dd/MM..." y sus numeros.</t>
   </si>
   <si>
     <t>notas</t>
@@ -2886,10 +2880,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -2907,57 +2901,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -3005,10 +2999,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3">
@@ -3022,10 +3016,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" s="0" t="s">
         <v>129</v>
-      </c>
-      <c r="E3" s="0" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="4">
@@ -3039,10 +3033,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5">
@@ -3050,16 +3044,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6">
@@ -3073,10 +3067,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7">
@@ -3090,10 +3084,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
+        <v>133</v>
+      </c>
+      <c r="E7" s="0" t="s">
         <v>135</v>
-      </c>
-      <c r="E7" s="0" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="8">
@@ -3107,10 +3101,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9">
@@ -3118,16 +3112,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10">
@@ -3141,10 +3135,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11">
@@ -3158,10 +3152,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="E11" s="0" t="s">
         <v>140</v>
-      </c>
-      <c r="E11" s="0" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="12">
@@ -3175,10 +3169,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="13">
@@ -3186,16 +3180,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -3231,10 +3225,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3260,7 +3254,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3">
@@ -3283,7 +3277,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4">
@@ -3306,7 +3300,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5">
@@ -3317,7 +3311,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -3329,7 +3323,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6">
@@ -3352,7 +3346,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7">
@@ -3375,7 +3369,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8">
@@ -3398,7 +3392,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9">
@@ -3409,7 +3403,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -3421,7 +3415,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10">
@@ -3444,7 +3438,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="11">
@@ -3467,7 +3461,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="12">
@@ -3490,7 +3484,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="13">
@@ -3501,7 +3495,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -3513,7 +3507,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14">
@@ -3536,7 +3530,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15">
@@ -3547,7 +3541,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -3559,7 +3553,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="16">
@@ -3582,7 +3576,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="17">
@@ -3605,7 +3599,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -3625,10 +3619,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3636,35 +3630,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -3687,7 +3681,7 @@
         <v>105</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3699,10 +3693,10 @@
         <v>106</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3731,7 +3725,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3">
@@ -3757,7 +3751,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4">
@@ -3783,7 +3777,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5">
@@ -3809,7 +3803,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6">
@@ -3835,7 +3829,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7">
@@ -3861,7 +3855,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8">
@@ -3887,7 +3881,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9">
@@ -3913,7 +3907,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10">
@@ -3939,7 +3933,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="11">
@@ -3965,7 +3959,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12">
@@ -3991,7 +3985,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="13">
@@ -4017,12 +4011,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: camion de Bolivia (Banexfrut) dictado para la semana 12-17/10; sab 17 cierra 25.310
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="164">
   <si>
     <t>fecha</t>
   </si>
@@ -335,10 +335,19 @@
     <t>dictado 08/10 (PY pide USD 8, Paraguay baja a 3): Guido 1: martes</t>
   </si>
   <si>
+    <t>BO</t>
+  </si>
+  <si>
+    <t>Banexfrut</t>
+  </si>
+  <si>
+    <t>Gonzalo 11/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 11/10: Gonzalo 11/10: "semana que viene descargamos 1 camion de Bol como siempre"; carga viernes como las anteriores de Banexfrut (descarga jue 15)</t>
+  </si>
+  <si>
     <t>semana_lunes</t>
-  </si>
-  <si>
-    <t>BO</t>
   </si>
   <si>
     <t>REAL ERP (captura 29/09/2026)</t>
@@ -541,7 +550,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -559,6 +568,7 @@
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -569,7 +579,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J67"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -2726,6 +2736,38 @@
       </c>
       <c r="J67" s="0" t="s">
         <v>104</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="17">
+        <v>46304</v>
+      </c>
+      <c r="B68" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C68" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="D68" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="E68" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="F68" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G68" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H68" s="0">
+        <v>1050</v>
+      </c>
+      <c r="I68" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="J68" s="0" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -2748,7 +2790,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -2757,7 +2799,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>8</v>
@@ -2780,10 +2822,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3">
@@ -2800,10 +2842,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4">
@@ -2820,10 +2862,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5">
@@ -2840,10 +2882,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6">
@@ -2860,10 +2902,10 @@
         <v>1050</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7">
@@ -2880,10 +2922,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -2901,57 +2943,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -2999,10 +3041,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3">
@@ -3016,10 +3058,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4">
@@ -3027,16 +3069,16 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5">
@@ -3044,16 +3086,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6">
@@ -3067,10 +3109,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7">
@@ -3084,10 +3126,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8">
@@ -3095,16 +3137,16 @@
         <v>46291</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C8" s="0">
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9">
@@ -3112,16 +3154,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10">
@@ -3135,10 +3177,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11">
@@ -3152,10 +3194,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="12">
@@ -3163,16 +3205,16 @@
         <v>46298</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C12" s="0">
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13">
@@ -3180,16 +3222,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -3225,10 +3267,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3254,7 +3296,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3">
@@ -3277,7 +3319,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4">
@@ -3288,7 +3330,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -3300,7 +3342,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5">
@@ -3311,7 +3353,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -3323,7 +3365,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6">
@@ -3346,7 +3388,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7">
@@ -3369,7 +3411,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8">
@@ -3380,7 +3422,7 @@
         <v>51</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -3392,7 +3434,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9">
@@ -3403,7 +3445,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -3415,7 +3457,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10">
@@ -3438,7 +3480,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11">
@@ -3461,7 +3503,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12">
@@ -3472,7 +3514,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -3484,7 +3526,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="13">
@@ -3495,7 +3537,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -3507,7 +3549,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14">
@@ -3530,7 +3572,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="15">
@@ -3541,7 +3583,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -3553,7 +3595,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="16">
@@ -3576,7 +3618,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="17">
@@ -3587,7 +3629,7 @@
         <v>29</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D17" s="0">
         <v>134</v>
@@ -3599,7 +3641,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -3619,10 +3661,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3630,35 +3672,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -3678,10 +3720,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3690,13 +3732,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3725,7 +3767,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3">
@@ -3751,7 +3793,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4">
@@ -3777,7 +3819,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5">
@@ -3803,7 +3845,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6">
@@ -3829,7 +3871,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7">
@@ -3855,7 +3897,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8">
@@ -3881,7 +3923,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9">
@@ -3907,7 +3949,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10">
@@ -3933,7 +3975,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11">
@@ -3959,7 +4001,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12">
@@ -3985,7 +4027,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13">
@@ -4011,12 +4053,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: camion de Bolivia dictado para la semana 19-24/10 (descarga jue 22); faltan 11
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
   <si>
     <t>fecha</t>
   </si>
@@ -345,6 +345,9 @@
   </si>
   <si>
     <t>dictado 11/10: Gonzalo 11/10: "semana que viene descargamos 1 camion de Bol como siempre"; carga viernes como las anteriores de Banexfrut (descarga jue 15)</t>
+  </si>
+  <si>
+    <t>dictado 11/10: Gonzalo 11/10: "semana 19 se descarga jueves el Bol" (descarga jue 22, carga vie 16 como las anteriores)</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -550,7 +553,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -569,6 +572,7 @@
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -579,7 +583,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -2768,6 +2772,38 @@
       </c>
       <c r="J68" s="0" t="s">
         <v>108</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="18">
+        <v>46311</v>
+      </c>
+      <c r="B69" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C69" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="D69" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="E69" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="F69" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G69" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H69" s="0">
+        <v>1050</v>
+      </c>
+      <c r="I69" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="J69" s="0" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2790,7 +2826,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -2822,10 +2858,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3">
@@ -2842,10 +2878,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4">
@@ -2862,10 +2898,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5">
@@ -2882,10 +2918,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6">
@@ -2902,10 +2938,10 @@
         <v>1050</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7">
@@ -2922,10 +2958,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -2943,57 +2979,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -3041,10 +3077,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3">
@@ -3058,10 +3094,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4">
@@ -3075,10 +3111,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5">
@@ -3086,16 +3122,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6">
@@ -3109,10 +3145,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7">
@@ -3126,10 +3162,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8">
@@ -3143,10 +3179,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="9">
@@ -3154,16 +3190,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10">
@@ -3177,10 +3213,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="11">
@@ -3194,10 +3230,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12">
@@ -3211,10 +3247,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="13">
@@ -3222,16 +3258,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -3267,10 +3303,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3296,7 +3332,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3">
@@ -3319,7 +3355,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4">
@@ -3342,7 +3378,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5">
@@ -3353,7 +3389,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -3365,7 +3401,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6">
@@ -3388,7 +3424,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7">
@@ -3411,7 +3447,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8">
@@ -3434,7 +3470,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9">
@@ -3445,7 +3481,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -3457,7 +3493,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10">
@@ -3480,7 +3516,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11">
@@ -3503,7 +3539,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="12">
@@ -3526,7 +3562,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="13">
@@ -3537,7 +3573,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -3549,7 +3585,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="14">
@@ -3572,7 +3608,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="15">
@@ -3583,7 +3619,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -3595,7 +3631,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16">
@@ -3618,7 +3654,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="17">
@@ -3641,7 +3677,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -3661,10 +3697,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3672,35 +3708,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -3720,10 +3756,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3735,10 +3771,10 @@
         <v>105</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3767,7 +3803,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3">
@@ -3793,7 +3829,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4">
@@ -3819,7 +3855,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5">
@@ -3845,7 +3881,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6">
@@ -3871,7 +3907,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7">
@@ -3897,7 +3933,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8">
@@ -3923,7 +3959,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9">
@@ -3949,7 +3985,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10">
@@ -3975,7 +4011,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11">
@@ -4001,7 +4037,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12">
@@ -4027,7 +4063,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13">
@@ -4053,12 +4089,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: dictado de la semana 19-25/10 (12 BR + 5 PY con dias); sab 24 cierra 22.750, faltan 3
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
   <si>
     <t>fecha</t>
   </si>
@@ -348,6 +348,63 @@
   </si>
   <si>
     <t>dictado 11/10: Gonzalo 11/10: "semana 19 se descarga jueves el Bol" (descarga jue 22, carga vie 16 como las anteriores)</t>
+  </si>
+  <si>
+    <t>2026-10-18</t>
+  </si>
+  <si>
+    <t>Gonzalo 13/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Fisher 2: cuarta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Fisher 2: sexta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Cassio 2: tersa; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Cassio 2: sexta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Ivo 1: cuarta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Agro 1: cuarta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Stein 1: cuarta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Gilson 1: cuarta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Josemar 1: cuarta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Marconi 1: sexta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Furlani 1: sexta (camion entero)</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Shapo 1: sexta</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Milciades 1: lunes</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Alvarito 1: martes</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Diego 1: martes</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Guido 1: lunes</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Hugo 1: domingo (arranca la semana)</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -553,7 +610,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -573,6 +630,7 @@
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -583,7 +641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -2804,6 +2862,550 @@
       </c>
       <c r="J69" s="0" t="s">
         <v>109</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="19">
+        <v>46316</v>
+      </c>
+      <c r="B70" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C70" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D70" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E70" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="F70" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="G70" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H70" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I70" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J70" s="0" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="19">
+        <v>46318</v>
+      </c>
+      <c r="B71" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C71" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D71" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E71" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="F71" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="G71" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H71" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I71" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J71" s="0" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="19">
+        <v>46315</v>
+      </c>
+      <c r="B72" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C72" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D72" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E72" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="F72" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G72" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="H72" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I72" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J72" s="0" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="19">
+        <v>46318</v>
+      </c>
+      <c r="B73" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C73" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D73" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E73" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="F73" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G73" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="H73" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I73" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J73" s="0" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="19">
+        <v>46316</v>
+      </c>
+      <c r="B74" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C74" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D74" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E74" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F74" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="G74" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H74" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I74" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J74" s="0" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="19">
+        <v>46316</v>
+      </c>
+      <c r="B75" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C75" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D75" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E75" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="F75" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G75" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H75" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I75" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J75" s="0" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="19">
+        <v>46316</v>
+      </c>
+      <c r="B76" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C76" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D76" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E76" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="F76" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G76" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H76" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I76" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J76" s="0" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="19">
+        <v>46316</v>
+      </c>
+      <c r="B77" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C77" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D77" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E77" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="F77" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G77" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H77" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I77" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J77" s="0" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="19">
+        <v>46316</v>
+      </c>
+      <c r="B78" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C78" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D78" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E78" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="F78" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G78" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H78" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I78" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J78" s="0" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="19">
+        <v>46318</v>
+      </c>
+      <c r="B79" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C79" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D79" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E79" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F79" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="G79" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H79" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I79" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J79" s="0" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="19">
+        <v>46318</v>
+      </c>
+      <c r="B80" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C80" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D80" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E80" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="F80" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G80" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H80" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I80" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J80" s="0" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="19">
+        <v>46318</v>
+      </c>
+      <c r="B81" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C81" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D81" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E81" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="F81" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G81" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H81" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I81" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J81" s="0" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="19">
+        <v>46314</v>
+      </c>
+      <c r="B82" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C82" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D82" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E82" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="F82" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G82" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H82" s="0">
+        <v>980</v>
+      </c>
+      <c r="I82" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J82" s="0" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="19">
+        <v>46315</v>
+      </c>
+      <c r="B83" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C83" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D83" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E83" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="F83" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G83" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H83" s="0">
+        <v>980</v>
+      </c>
+      <c r="I83" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J83" s="0" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="19">
+        <v>46315</v>
+      </c>
+      <c r="B84" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C84" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D84" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E84" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="F84" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G84" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H84" s="0">
+        <v>980</v>
+      </c>
+      <c r="I84" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J84" s="0" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="19">
+        <v>46314</v>
+      </c>
+      <c r="B85" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C85" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D85" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E85" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="F85" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G85" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H85" s="0">
+        <v>980</v>
+      </c>
+      <c r="I85" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J85" s="0" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="19">
+        <v>46313</v>
+      </c>
+      <c r="B86" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="C86" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D86" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E86" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="F86" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G86" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H86" s="0">
+        <v>980</v>
+      </c>
+      <c r="I86" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J86" s="0" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -2826,7 +3428,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -2858,10 +3460,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>112</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3">
@@ -2878,10 +3480,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4">
@@ -2898,10 +3500,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5">
@@ -2918,10 +3520,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6">
@@ -2938,10 +3540,10 @@
         <v>1050</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7">
@@ -2958,10 +3560,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -2979,57 +3581,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>120</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -3077,10 +3679,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3">
@@ -3094,10 +3696,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>133</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4">
@@ -3111,10 +3713,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>134</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5">
@@ -3122,16 +3724,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
     </row>
     <row r="6">
@@ -3145,10 +3747,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>138</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7">
@@ -3162,10 +3764,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8">
@@ -3179,10 +3781,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>140</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9">
@@ -3190,16 +3792,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>141</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10">
@@ -3213,10 +3815,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>143</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11">
@@ -3230,10 +3832,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>144</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12">
@@ -3247,10 +3849,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>145</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13">
@@ -3258,16 +3860,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>146</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -3303,10 +3905,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>147</v>
+        <v>166</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>148</v>
+        <v>167</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3332,7 +3934,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3">
@@ -3355,7 +3957,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4">
@@ -3378,7 +3980,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5">
@@ -3389,7 +3991,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -3401,7 +4003,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
     </row>
     <row r="6">
@@ -3424,7 +4026,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>150</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7">
@@ -3447,7 +4049,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>150</v>
+        <v>169</v>
       </c>
     </row>
     <row r="8">
@@ -3470,7 +4072,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>150</v>
+        <v>169</v>
       </c>
     </row>
     <row r="9">
@@ -3481,7 +4083,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -3493,7 +4095,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>150</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10">
@@ -3516,7 +4118,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>151</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11">
@@ -3539,7 +4141,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>151</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12">
@@ -3562,7 +4164,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>151</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13">
@@ -3573,7 +4175,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -3585,7 +4187,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>151</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14">
@@ -3608,7 +4210,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15">
@@ -3619,7 +4221,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -3631,7 +4233,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
     </row>
     <row r="16">
@@ -3654,7 +4256,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
     </row>
     <row r="17">
@@ -3677,7 +4279,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -3697,10 +4299,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>154</v>
+        <v>173</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -3708,35 +4310,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>158</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>159</v>
+        <v>178</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>160</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -3756,10 +4358,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>161</v>
+        <v>180</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -3771,10 +4373,10 @@
         <v>105</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>162</v>
+        <v>181</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -3803,7 +4405,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3">
@@ -3829,7 +4431,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4">
@@ -3855,7 +4457,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5">
@@ -3881,7 +4483,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6">
@@ -3907,7 +4509,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7">
@@ -3933,7 +4535,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
     </row>
     <row r="8">
@@ -3959,7 +4561,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
     </row>
     <row r="9">
@@ -3985,7 +4587,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
     </row>
     <row r="10">
@@ -4011,7 +4613,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
     </row>
     <row r="11">
@@ -4037,7 +4639,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12">
@@ -4063,7 +4665,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13">
@@ -4089,12 +4691,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Cassio y Fisher a 3 cargas en la semana 19-25/10; sab 24 cierra 22.729, faltan 3
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="186">
   <si>
     <t>fecha</t>
   </si>
@@ -405,6 +405,12 @@
   </si>
   <si>
     <t>dictado 13/10: Hugo 1: domingo (arranca la semana)</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Cassio 3: tersa, cuarta y sexta (Gonzalo 13/10: "casio carga 3 martes miercoles y viernes"; se suma la cuarta); transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 13/10: Fisher 3: tersa, cuarta y sexta (Gonzalo 13/10: "fisher tambien, 3 martes miercoles y viernes"; se suma la tersa); transportista supuesto = habitual</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -610,7 +616,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -631,6 +637,8 @@
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -641,7 +649,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J86"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -3406,6 +3414,70 @@
       </c>
       <c r="J86" s="0" t="s">
         <v>128</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="20">
+        <v>46316</v>
+      </c>
+      <c r="B87" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C87" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D87" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E87" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="F87" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="G87" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="H87" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I87" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J87" s="0" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="21">
+        <v>46315</v>
+      </c>
+      <c r="B88" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C88" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D88" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E88" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="F88" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="G88" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H88" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I88" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J88" s="0" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -3428,7 +3500,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -3460,10 +3532,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3">
@@ -3480,10 +3552,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4">
@@ -3500,10 +3572,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5">
@@ -3520,10 +3592,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6">
@@ -3540,10 +3612,10 @@
         <v>1050</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7">
@@ -3560,10 +3632,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -3581,57 +3653,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -3679,10 +3751,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3">
@@ -3696,10 +3768,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4">
@@ -3713,10 +3785,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5">
@@ -3724,16 +3796,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6">
@@ -3747,10 +3819,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7">
@@ -3764,10 +3836,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8">
@@ -3781,10 +3853,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9">
@@ -3792,16 +3864,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10">
@@ -3815,10 +3887,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="11">
@@ -3832,10 +3904,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="12">
@@ -3849,10 +3921,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13">
@@ -3860,16 +3932,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -3905,10 +3977,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -3934,7 +4006,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3">
@@ -3957,7 +4029,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4">
@@ -3980,7 +4052,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5">
@@ -3991,7 +4063,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -4003,7 +4075,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6">
@@ -4026,7 +4098,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7">
@@ -4049,7 +4121,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8">
@@ -4072,7 +4144,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="9">
@@ -4083,7 +4155,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -4095,7 +4167,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="10">
@@ -4118,7 +4190,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="11">
@@ -4141,7 +4213,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12">
@@ -4164,7 +4236,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13">
@@ -4175,7 +4247,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -4187,7 +4259,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="14">
@@ -4210,7 +4282,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="15">
@@ -4221,7 +4293,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -4233,7 +4305,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="16">
@@ -4256,7 +4328,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="17">
@@ -4279,7 +4351,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -4299,10 +4371,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -4310,35 +4382,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -4358,10 +4430,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -4373,10 +4445,10 @@
         <v>105</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -4405,7 +4477,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3">
@@ -4431,7 +4503,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4">
@@ -4457,7 +4529,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5">
@@ -4483,7 +4555,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="6">
@@ -4509,7 +4581,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7">
@@ -4535,7 +4607,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8">
@@ -4561,7 +4633,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9">
@@ -4587,7 +4659,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="10">
@@ -4613,7 +4685,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11">
@@ -4639,7 +4711,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="12">
@@ -4665,7 +4737,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="13">
@@ -4691,12 +4763,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: dictado definitivo de la semana 19-25/10 (17 BR + 5 PY); sab 24 cierra 26.784
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="191">
   <si>
     <t>fecha</t>
   </si>
@@ -353,64 +353,79 @@
     <t>2026-10-18</t>
   </si>
   <si>
-    <t>Gonzalo 13/10 (chat)</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Fisher 2: cuarta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Fisher 2: sexta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Cassio 2: tersa; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Cassio 2: sexta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Ivo 1: cuarta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Agro 1: cuarta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Stein 1: cuarta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Gilson 1: cuarta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Josemar 1: cuarta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Marconi 1: sexta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Furlani 1: sexta (camion entero)</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Shapo 1: sexta</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Milciades 1: lunes</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Alvarito 1: martes</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Diego 1: martes</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Guido 1: lunes</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Hugo 1: domingo (arranca la semana)</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Cassio 3: tersa, cuarta y sexta (Gonzalo 13/10: "casio carga 3 martes miercoles y viernes"; se suma la cuarta); transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 13/10: Fisher 3: tersa, cuarta y sexta (Gonzalo 13/10: "fisher tambien, 3 martes miercoles y viernes"; se suma la tersa); transportista supuesto = habitual</t>
+    <t>Gonzalo 14/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Fisher 2: tersa; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Fisher 2: sexta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Cassio 3: tersa; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Cassio 3: cuarta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Cassio 3: sexta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Celso 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Ivo 1: cuarta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Agro 2: cuarta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Agro 2: sexta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>Muller Fabricio</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Miuller Fabricio 2: tersa</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Miuller Fabricio 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Stein 2: cuarta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Stein 2: sexta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Gilson 1: cuarta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Marconi 1: cuarta; transportista supuesto = habitual</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Shapo 1: sexta</t>
+  </si>
+  <si>
+    <t>Wagner</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Wagner 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Milciades 1: lunes</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Alvarito 1: martes</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Diego 2: lunes</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Diego 2: martes</t>
+  </si>
+  <si>
+    <t>dictado 14/10: Guido 1: lunes</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -616,7 +631,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
@@ -637,8 +652,6 @@
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -649,7 +662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
@@ -2874,10 +2887,10 @@
     </row>
     <row r="70">
       <c r="A70" s="19">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="B70" s="0" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C70" s="0" t="s">
         <v>110</v>
@@ -2970,10 +2983,10 @@
     </row>
     <row r="73">
       <c r="A73" s="19">
-        <v>46318</v>
+        <v>46316</v>
       </c>
       <c r="B73" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C73" s="0" t="s">
         <v>110</v>
@@ -3002,10 +3015,10 @@
     </row>
     <row r="74">
       <c r="A74" s="19">
-        <v>46316</v>
+        <v>46318</v>
       </c>
       <c r="B74" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C74" s="0" t="s">
         <v>110</v>
@@ -3014,13 +3027,13 @@
         <v>23</v>
       </c>
       <c r="E74" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F74" s="0" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="G74" s="0" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="H74" s="0">
         <v>1008</v>
@@ -3046,13 +3059,13 @@
         <v>23</v>
       </c>
       <c r="E75" s="0" t="s">
-        <v>39</v>
+        <v>74</v>
       </c>
       <c r="F75" s="0" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G75" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H75" s="0">
         <v>1008</v>
@@ -3078,13 +3091,13 @@
         <v>23</v>
       </c>
       <c r="E76" s="0" t="s">
-        <v>58</v>
+        <v>24</v>
       </c>
       <c r="F76" s="0" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="G76" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H76" s="0">
         <v>1008</v>
@@ -3110,7 +3123,7 @@
         <v>23</v>
       </c>
       <c r="E77" s="0" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F77" s="0" t="s">
         <v>40</v>
@@ -3130,10 +3143,10 @@
     </row>
     <row r="78">
       <c r="A78" s="19">
-        <v>46316</v>
+        <v>46318</v>
       </c>
       <c r="B78" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C78" s="0" t="s">
         <v>110</v>
@@ -3142,7 +3155,7 @@
         <v>23</v>
       </c>
       <c r="E78" s="0" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="F78" s="0" t="s">
         <v>40</v>
@@ -3162,10 +3175,10 @@
     </row>
     <row r="79">
       <c r="A79" s="19">
-        <v>46318</v>
+        <v>46315</v>
       </c>
       <c r="B79" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C79" s="0" t="s">
         <v>110</v>
@@ -3174,10 +3187,10 @@
         <v>23</v>
       </c>
       <c r="E79" s="0" t="s">
-        <v>59</v>
+        <v>121</v>
       </c>
       <c r="F79" s="0" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="G79" s="0" t="s">
         <v>14</v>
@@ -3189,7 +3202,7 @@
         <v>111</v>
       </c>
       <c r="J79" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="80">
@@ -3206,7 +3219,7 @@
         <v>23</v>
       </c>
       <c r="E80" s="0" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="F80" s="0" t="s">
         <v>14</v>
@@ -3221,15 +3234,15 @@
         <v>111</v>
       </c>
       <c r="J80" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="19">
-        <v>46318</v>
+        <v>46316</v>
       </c>
       <c r="B81" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C81" s="0" t="s">
         <v>110</v>
@@ -3238,13 +3251,13 @@
         <v>23</v>
       </c>
       <c r="E81" s="0" t="s">
-        <v>97</v>
+        <v>58</v>
       </c>
       <c r="F81" s="0" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G81" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H81" s="0">
         <v>1008</v>
@@ -3253,120 +3266,120 @@
         <v>111</v>
       </c>
       <c r="J81" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="19">
-        <v>46314</v>
+        <v>46318</v>
       </c>
       <c r="B82" s="0" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C82" s="0" t="s">
         <v>110</v>
       </c>
       <c r="D82" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E82" s="0" t="s">
-        <v>19</v>
+        <v>58</v>
       </c>
       <c r="F82" s="0" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G82" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H82" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I82" s="0" t="s">
         <v>111</v>
       </c>
       <c r="J82" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="19">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B83" s="0" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C83" s="0" t="s">
         <v>110</v>
       </c>
       <c r="D83" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E83" s="0" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="F83" s="0" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G83" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H83" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I83" s="0" t="s">
         <v>111</v>
       </c>
       <c r="J83" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="19">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B84" s="0" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C84" s="0" t="s">
         <v>110</v>
       </c>
       <c r="D84" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E84" s="0" t="s">
-        <v>13</v>
+        <v>59</v>
       </c>
       <c r="F84" s="0" t="s">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="G84" s="0" t="s">
         <v>14</v>
       </c>
       <c r="H84" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I84" s="0" t="s">
         <v>111</v>
       </c>
       <c r="J84" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="19">
-        <v>46314</v>
+        <v>46318</v>
       </c>
       <c r="B85" s="0" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C85" s="0" t="s">
         <v>110</v>
       </c>
       <c r="D85" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E85" s="0" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="F85" s="0" t="s">
         <v>14</v>
@@ -3375,30 +3388,30 @@
         <v>14</v>
       </c>
       <c r="H85" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I85" s="0" t="s">
         <v>111</v>
       </c>
       <c r="J85" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="19">
-        <v>46313</v>
+        <v>46316</v>
       </c>
       <c r="B86" s="0" t="s">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="C86" s="0" t="s">
         <v>110</v>
       </c>
       <c r="D86" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E86" s="0" t="s">
-        <v>17</v>
+        <v>129</v>
       </c>
       <c r="F86" s="0" t="s">
         <v>14</v>
@@ -3407,49 +3420,49 @@
         <v>14</v>
       </c>
       <c r="H86" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I86" s="0" t="s">
         <v>111</v>
       </c>
       <c r="J86" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="20">
-        <v>46316</v>
+      <c r="A87" s="19">
+        <v>46314</v>
       </c>
       <c r="B87" s="0" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="C87" s="0" t="s">
         <v>110</v>
       </c>
       <c r="D87" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E87" s="0" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F87" s="0" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G87" s="0" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="H87" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I87" s="0" t="s">
         <v>111</v>
       </c>
       <c r="J87" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="21">
+      <c r="A88" s="19">
         <v>46315</v>
       </c>
       <c r="B88" s="0" t="s">
@@ -3459,25 +3472,121 @@
         <v>110</v>
       </c>
       <c r="D88" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F88" s="0" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G88" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H88" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I88" s="0" t="s">
         <v>111</v>
       </c>
       <c r="J88" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="19">
+        <v>46314</v>
+      </c>
+      <c r="B89" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C89" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D89" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E89" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="F89" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G89" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H89" s="0">
+        <v>980</v>
+      </c>
+      <c r="I89" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J89" s="0" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="19">
+        <v>46315</v>
+      </c>
+      <c r="B90" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C90" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D90" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E90" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="F90" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G90" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H90" s="0">
+        <v>980</v>
+      </c>
+      <c r="I90" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J90" s="0" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="19">
+        <v>46314</v>
+      </c>
+      <c r="B91" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C91" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D91" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E91" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="F91" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G91" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H91" s="0">
+        <v>980</v>
+      </c>
+      <c r="I91" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="J91" s="0" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -3500,7 +3609,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -3532,10 +3641,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3">
@@ -3552,10 +3661,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4">
@@ -3572,10 +3681,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5">
@@ -3592,10 +3701,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6">
@@ -3612,10 +3721,10 @@
         <v>1050</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7">
@@ -3632,10 +3741,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -3653,57 +3762,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -3751,10 +3860,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3">
@@ -3768,10 +3877,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4">
@@ -3785,10 +3894,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5">
@@ -3796,16 +3905,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6">
@@ -3819,10 +3928,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7">
@@ -3836,10 +3945,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8">
@@ -3853,10 +3962,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9">
@@ -3864,16 +3973,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10">
@@ -3887,10 +3996,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="11">
@@ -3904,10 +4013,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12">
@@ -3921,10 +4030,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="13">
@@ -3932,16 +4041,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -3977,10 +4086,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -4006,7 +4115,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3">
@@ -4029,7 +4138,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4">
@@ -4052,7 +4161,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5">
@@ -4063,7 +4172,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -4075,7 +4184,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6">
@@ -4098,7 +4207,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7">
@@ -4121,7 +4230,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="8">
@@ -4144,7 +4253,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="9">
@@ -4155,7 +4264,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -4167,7 +4276,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="10">
@@ -4190,7 +4299,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="11">
@@ -4213,7 +4322,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="12">
@@ -4236,7 +4345,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="13">
@@ -4247,7 +4356,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -4259,7 +4368,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="14">
@@ -4282,7 +4391,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15">
@@ -4293,7 +4402,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -4305,7 +4414,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="16">
@@ -4328,7 +4437,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="17">
@@ -4351,7 +4460,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -4371,10 +4480,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -4382,35 +4491,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="B4" s="0">
         <v>25000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -4430,10 +4539,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -4445,10 +4554,10 @@
         <v>105</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -4477,7 +4586,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3">
@@ -4503,7 +4612,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4">
@@ -4529,7 +4638,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5">
@@ -4555,7 +4664,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6">
@@ -4581,7 +4690,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="7">
@@ -4607,7 +4716,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="8">
@@ -4633,7 +4742,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9">
@@ -4659,7 +4768,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10">
@@ -4685,7 +4794,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11">
@@ -4711,7 +4820,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12">
@@ -4737,7 +4846,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="13">
@@ -4763,12 +4872,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: objetivo del sabado 27.000 (pedido de Uruguay); sab 24 26.784, falta 1
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -578,7 +578,7 @@
     <t>minimo_cajas_sabado</t>
   </si>
   <si>
-    <t>Gonzalo 01/10/2026: "comienza el calor en Uruguay, levanta las ventas, quieren mantener 25 mil cajas al cierre del sabado contando todo, PY BOL y BR". Antes 22.500 (27/09).</t>
+    <t>Gonzalo 14/10/2026: "Uruguay quiere cierre de los sabados a 27 mil" (antes 25.000 desde el 01/10; 22.500 antes)</t>
   </si>
   <si>
     <t>sabado</t>
@@ -4516,7 +4516,7 @@
         <v>185</v>
       </c>
       <c r="B4" s="0">
-        <v>25000</v>
+        <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
         <v>186</v>

</xml_diff>

<commit_message>
plan de compras: dictado de la tarde de la semana 19-25/10 (19 BR + 3 PY, con transportistas); sab 24 26.840, falta 1
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="192">
   <si>
     <t>fecha</t>
   </si>
@@ -353,79 +353,82 @@
     <t>2026-10-18</t>
   </si>
   <si>
-    <t>Gonzalo 14/10 (chat)</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Fisher 2: tersa; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Fisher 2: sexta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Cassio 3: tersa; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Cassio 3: cuarta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Cassio 3: sexta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Celso 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Ivo 1: cuarta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Agro 2: cuarta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Agro 2: sexta; transportista supuesto = habitual</t>
+    <t>Gonzalo 14/10 tarde (chat)</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Fisher 2: tersa</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Fisher 2: sexta</t>
   </si>
   <si>
     <t>Muller Fabricio</t>
   </si>
   <si>
-    <t>dictado 14/10: Miuller Fabricio 2: tersa</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Miuller Fabricio 2: sexta</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Stein 2: cuarta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Stein 2: sexta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Gilson 1: cuarta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Marconi 1: cuarta; transportista supuesto = habitual</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Shapo 1: sexta</t>
+    <t>dictado 14/10 tarde: Miuller Fabricio 2 (via Curuca): tersa</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Miuller Fabricio 2 (via Curuca): sexta</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Stein 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Stein 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Cassio 3: tersa</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Cassio 3: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Cassio 3: sexta</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Celso 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Ivo 1: cuarta</t>
+  </si>
+  <si>
+    <t>Jaime Zimerman</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Jaime Zimerman 1: cuarta (nuevo; no es el Jaime viejo)</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Agro 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Agro 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Gilson 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Gilson 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Marconi 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Shapo 1: cuarta</t>
   </si>
   <si>
     <t>Wagner</t>
   </si>
   <si>
-    <t>dictado 14/10: Wagner 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Milciades 1: lunes</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Alvarito 1: martes</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Diego 2: lunes</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Diego 2: martes</t>
-  </si>
-  <si>
-    <t>dictado 14/10: Guido 1: lunes</t>
+    <t>dictado 14/10 tarde: Wagner 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Milciades 1: lunes</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Alvarito 1: martes</t>
+  </si>
+  <si>
+    <t>dictado 14/10 tarde: Guido 1: lunes</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -2963,13 +2966,13 @@
         <v>23</v>
       </c>
       <c r="E72" s="0" t="s">
-        <v>26</v>
+        <v>114</v>
       </c>
       <c r="F72" s="0" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="G72" s="0" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="H72" s="0">
         <v>1008</v>
@@ -2978,15 +2981,15 @@
         <v>111</v>
       </c>
       <c r="J72" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="19">
-        <v>46316</v>
+        <v>46318</v>
       </c>
       <c r="B73" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C73" s="0" t="s">
         <v>110</v>
@@ -2995,13 +2998,13 @@
         <v>23</v>
       </c>
       <c r="E73" s="0" t="s">
-        <v>26</v>
+        <v>114</v>
       </c>
       <c r="F73" s="0" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="G73" s="0" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="H73" s="0">
         <v>1008</v>
@@ -3010,15 +3013,15 @@
         <v>111</v>
       </c>
       <c r="J73" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="19">
-        <v>46318</v>
+        <v>46316</v>
       </c>
       <c r="B74" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C74" s="0" t="s">
         <v>110</v>
@@ -3027,13 +3030,13 @@
         <v>23</v>
       </c>
       <c r="E74" s="0" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="F74" s="0" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="G74" s="0" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="H74" s="0">
         <v>1008</v>
@@ -3042,15 +3045,15 @@
         <v>111</v>
       </c>
       <c r="J74" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="19">
-        <v>46316</v>
+        <v>46318</v>
       </c>
       <c r="B75" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C75" s="0" t="s">
         <v>110</v>
@@ -3059,10 +3062,10 @@
         <v>23</v>
       </c>
       <c r="E75" s="0" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="F75" s="0" t="s">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="G75" s="0" t="s">
         <v>14</v>
@@ -3074,15 +3077,15 @@
         <v>111</v>
       </c>
       <c r="J75" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="19">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="B76" s="0" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C76" s="0" t="s">
         <v>110</v>
@@ -3091,13 +3094,13 @@
         <v>23</v>
       </c>
       <c r="E76" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F76" s="0" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="G76" s="0" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="H76" s="0">
         <v>1008</v>
@@ -3106,7 +3109,7 @@
         <v>111</v>
       </c>
       <c r="J76" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="77">
@@ -3123,7 +3126,7 @@
         <v>23</v>
       </c>
       <c r="E77" s="0" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="F77" s="0" t="s">
         <v>40</v>
@@ -3138,7 +3141,7 @@
         <v>111</v>
       </c>
       <c r="J77" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="78">
@@ -3155,7 +3158,7 @@
         <v>23</v>
       </c>
       <c r="E78" s="0" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="F78" s="0" t="s">
         <v>40</v>
@@ -3170,15 +3173,15 @@
         <v>111</v>
       </c>
       <c r="J78" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="19">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B79" s="0" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C79" s="0" t="s">
         <v>110</v>
@@ -3187,13 +3190,13 @@
         <v>23</v>
       </c>
       <c r="E79" s="0" t="s">
-        <v>121</v>
+        <v>74</v>
       </c>
       <c r="F79" s="0" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G79" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H79" s="0">
         <v>1008</v>
@@ -3207,10 +3210,10 @@
     </row>
     <row r="80">
       <c r="A80" s="19">
-        <v>46318</v>
+        <v>46316</v>
       </c>
       <c r="B80" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C80" s="0" t="s">
         <v>110</v>
@@ -3219,13 +3222,13 @@
         <v>23</v>
       </c>
       <c r="E80" s="0" t="s">
-        <v>121</v>
+        <v>24</v>
       </c>
       <c r="F80" s="0" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G80" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H80" s="0">
         <v>1008</v>
@@ -3251,13 +3254,13 @@
         <v>23</v>
       </c>
       <c r="E81" s="0" t="s">
-        <v>58</v>
+        <v>124</v>
       </c>
       <c r="F81" s="0" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G81" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H81" s="0">
         <v>1008</v>
@@ -3266,15 +3269,15 @@
         <v>111</v>
       </c>
       <c r="J81" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="19">
-        <v>46318</v>
+        <v>46316</v>
       </c>
       <c r="B82" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C82" s="0" t="s">
         <v>110</v>
@@ -3283,7 +3286,7 @@
         <v>23</v>
       </c>
       <c r="E82" s="0" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="F82" s="0" t="s">
         <v>40</v>
@@ -3298,15 +3301,15 @@
         <v>111</v>
       </c>
       <c r="J82" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="19">
-        <v>46316</v>
+        <v>46318</v>
       </c>
       <c r="B83" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C83" s="0" t="s">
         <v>110</v>
@@ -3315,7 +3318,7 @@
         <v>23</v>
       </c>
       <c r="E83" s="0" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F83" s="0" t="s">
         <v>40</v>
@@ -3330,7 +3333,7 @@
         <v>111</v>
       </c>
       <c r="J83" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="84">
@@ -3347,13 +3350,13 @@
         <v>23</v>
       </c>
       <c r="E84" s="0" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="F84" s="0" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="G84" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H84" s="0">
         <v>1008</v>
@@ -3362,7 +3365,7 @@
         <v>111</v>
       </c>
       <c r="J84" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="85">
@@ -3379,13 +3382,13 @@
         <v>23</v>
       </c>
       <c r="E85" s="0" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="F85" s="0" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G85" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H85" s="0">
         <v>1008</v>
@@ -3394,7 +3397,7 @@
         <v>111</v>
       </c>
       <c r="J85" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="86">
@@ -3411,13 +3414,13 @@
         <v>23</v>
       </c>
       <c r="E86" s="0" t="s">
-        <v>129</v>
+        <v>59</v>
       </c>
       <c r="F86" s="0" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G86" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H86" s="0">
         <v>1008</v>
@@ -3431,28 +3434,28 @@
     </row>
     <row r="87">
       <c r="A87" s="19">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="B87" s="0" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="C87" s="0" t="s">
         <v>110</v>
       </c>
       <c r="D87" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E87" s="0" t="s">
-        <v>19</v>
+        <v>97</v>
       </c>
       <c r="F87" s="0" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G87" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H87" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I87" s="0" t="s">
         <v>111</v>
@@ -3463,34 +3466,34 @@
     </row>
     <row r="88">
       <c r="A88" s="19">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C88" s="0" t="s">
         <v>110</v>
       </c>
       <c r="D88" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>21</v>
+        <v>132</v>
       </c>
       <c r="F88" s="0" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G88" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H88" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I88" s="0" t="s">
         <v>111</v>
       </c>
       <c r="J88" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="89">
@@ -3507,7 +3510,7 @@
         <v>12</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F89" s="0" t="s">
         <v>14</v>
@@ -3522,7 +3525,7 @@
         <v>111</v>
       </c>
       <c r="J89" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="90">
@@ -3539,7 +3542,7 @@
         <v>12</v>
       </c>
       <c r="E90" s="0" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F90" s="0" t="s">
         <v>14</v>
@@ -3554,7 +3557,7 @@
         <v>111</v>
       </c>
       <c r="J90" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="91">
@@ -3586,7 +3589,7 @@
         <v>111</v>
       </c>
       <c r="J91" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -3609,7 +3612,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>23</v>
@@ -3641,10 +3644,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3">
@@ -3661,10 +3664,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4">
@@ -3681,10 +3684,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5">
@@ -3701,10 +3704,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6">
@@ -3721,10 +3724,10 @@
         <v>1050</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7">
@@ -3741,10 +3744,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -3762,57 +3765,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -3860,10 +3863,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3">
@@ -3877,10 +3880,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4">
@@ -3894,10 +3897,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5">
@@ -3905,16 +3908,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6">
@@ -3928,10 +3931,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7">
@@ -3945,10 +3948,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8">
@@ -3962,10 +3965,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="9">
@@ -3973,16 +3976,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="10">
@@ -3996,10 +3999,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11">
@@ -4013,10 +4016,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="12">
@@ -4030,10 +4033,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13">
@@ -4041,16 +4044,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -4086,10 +4089,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>8</v>
@@ -4115,7 +4118,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3">
@@ -4138,7 +4141,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4">
@@ -4161,7 +4164,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5">
@@ -4172,7 +4175,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -4184,7 +4187,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="6">
@@ -4207,7 +4210,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7">
@@ -4230,7 +4233,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8">
@@ -4253,7 +4256,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9">
@@ -4264,7 +4267,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -4276,7 +4279,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10">
@@ -4299,7 +4302,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="11">
@@ -4322,7 +4325,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="12">
@@ -4345,7 +4348,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="13">
@@ -4356,7 +4359,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -4368,7 +4371,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="14">
@@ -4391,7 +4394,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="15">
@@ -4402,7 +4405,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -4414,7 +4417,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16">
@@ -4437,7 +4440,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17">
@@ -4460,7 +4463,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -4480,10 +4483,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -4491,35 +4494,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -4539,10 +4542,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>23</v>
@@ -4554,10 +4557,10 @@
         <v>105</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>8</v>
@@ -4586,7 +4589,7 @@
         <f>C2+D2+E2</f>
       </c>
       <c r="H2" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3">
@@ -4612,7 +4615,7 @@
         <f>C3+D3+E3</f>
       </c>
       <c r="H3" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="4">
@@ -4638,7 +4641,7 @@
         <f>C4+D4+E4</f>
       </c>
       <c r="H4" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5">
@@ -4664,7 +4667,7 @@
         <f>C5+D5+E5</f>
       </c>
       <c r="H5" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6">
@@ -4690,7 +4693,7 @@
         <f>C6+D6+E6</f>
       </c>
       <c r="H6" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7">
@@ -4716,7 +4719,7 @@
         <f>C7+D7+E7</f>
       </c>
       <c r="H7" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="8">
@@ -4742,7 +4745,7 @@
         <f>C8+D8+E8</f>
       </c>
       <c r="H8" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="9">
@@ -4768,7 +4771,7 @@
         <f>C9+D9+E9</f>
       </c>
       <c r="H9" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="10">
@@ -4794,7 +4797,7 @@
         <f>C10+D10+E10</f>
       </c>
       <c r="H10" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="11">
@@ -4820,7 +4823,7 @@
         <f>C11+D11+E11</f>
       </c>
       <c r="H11" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12">
@@ -4846,7 +4849,7 @@
         <f>C12+D12+E12</f>
       </c>
       <c r="H12" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13">
@@ -4872,12 +4875,12 @@
         <f>C13+D13+E13</f>
       </c>
       <c r="H13" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: carga extra de Jhony Viera sab 17/10; sab 24 cierra 27.040
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="189">
   <si>
     <t>fecha</t>
   </si>
@@ -419,6 +419,15 @@
   </si>
   <si>
     <t>planificacion 15/10: Guido 1 (7,5 USD): lunes</t>
+  </si>
+  <si>
+    <t>Jhony Viera</t>
+  </si>
+  <si>
+    <t>Gonzalo 15/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 15/10: carga extra sabado 17 (Gonzalo 15/10: "hay una carga extra sabado 17 de jony viera")</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -624,11 +633,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -944,7 +954,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J90"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -3837,6 +3847,38 @@
       </c>
       <c r="J90" s="0" t="s">
         <v>130</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5">
+        <v>46312</v>
+      </c>
+      <c r="B91" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C91" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="D91" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E91" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="F91" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G91" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H91" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I91" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="J91" s="0" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -3858,7 +3900,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>23</v>
@@ -3890,10 +3932,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3">
@@ -3910,10 +3952,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4">
@@ -3930,10 +3972,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5">
@@ -3950,10 +3992,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6">
@@ -3970,10 +4012,10 @@
         <v>1050</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7">
@@ -3990,10 +4032,10 @@
         <v>1278</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -4012,57 +4054,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -4110,10 +4152,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3">
@@ -4127,10 +4169,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4">
@@ -4144,10 +4186,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5">
@@ -4155,16 +4197,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6">
@@ -4178,10 +4220,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7">
@@ -4195,10 +4237,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8">
@@ -4212,10 +4254,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9">
@@ -4223,16 +4265,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10">
@@ -4246,10 +4288,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11">
@@ -4263,10 +4305,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="12">
@@ -4280,10 +4322,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="13">
@@ -4291,16 +4333,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -4334,10 +4376,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -4363,7 +4405,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3">
@@ -4386,7 +4428,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4">
@@ -4409,7 +4451,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5">
@@ -4420,7 +4462,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -4432,7 +4474,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6">
@@ -4455,7 +4497,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7">
@@ -4478,7 +4520,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8">
@@ -4501,7 +4543,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9">
@@ -4512,7 +4554,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -4524,7 +4566,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="10">
@@ -4547,7 +4589,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11">
@@ -4570,7 +4612,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="12">
@@ -4593,7 +4635,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="13">
@@ -4604,7 +4646,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -4616,7 +4658,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="14">
@@ -4639,7 +4681,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="15">
@@ -4650,7 +4692,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -4662,7 +4704,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="16">
@@ -4685,7 +4727,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="17">
@@ -4708,7 +4750,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -4729,10 +4771,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -4740,35 +4782,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -4789,10 +4831,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>23</v>
@@ -4804,10 +4846,10 @@
         <v>84</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -4837,7 +4879,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3">
@@ -4864,7 +4906,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4">
@@ -4891,7 +4933,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5">
@@ -4918,7 +4960,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6">
@@ -4945,7 +4987,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7">
@@ -4972,7 +5014,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8">
@@ -4999,7 +5041,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9">
@@ -5026,7 +5068,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10">
@@ -5053,7 +5095,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11">
@@ -5080,7 +5122,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12">
@@ -5107,7 +5149,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13">
@@ -5134,12 +5176,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: venta prevista 20.500 para la semana del 19/10 (dictado); sab 24 23.740, faltan 4
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="196">
   <si>
     <t>fecha</t>
   </si>
@@ -473,6 +473,12 @@
   </si>
   <si>
     <t>Gonzalo 11/10/2026 "vamos por el 1": venta prevista = promedio real de las ultimas 10 semanas (Aloha); el generador pisa BR/PY/BO en cada corrida. Si Gonzalo dicta una semana, poner fuente "Gonzalo dd/MM..." y sus numeros.</t>
+  </si>
+  <si>
+    <t>Gonzalo 15/10: "la idea es semana que viene vender 20 o 21 mil cajas" = 20.500 (punto medio)</t>
+  </si>
+  <si>
+    <t>reparto BR/PY/BO con el mix real de las ultimas 10 semanas; desde el mie 21 la pisa la estimacion con los dias reales</t>
   </si>
   <si>
     <t>notas</t>
@@ -4104,19 +4110,19 @@
         <v>46314</v>
       </c>
       <c r="B7" s="0">
-        <v>11106</v>
+        <v>11111</v>
       </c>
       <c r="C7" s="0">
-        <v>5616</v>
+        <v>8036</v>
       </c>
       <c r="D7" s="0">
-        <v>1278</v>
+        <v>1353</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -4135,57 +4141,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -4233,10 +4239,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3">
@@ -4250,10 +4256,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4">
@@ -4267,10 +4273,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5">
@@ -4278,16 +4284,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6">
@@ -4301,10 +4307,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7">
@@ -4318,10 +4324,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8">
@@ -4335,10 +4341,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="9">
@@ -4346,16 +4352,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10">
@@ -4369,10 +4375,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11">
@@ -4386,10 +4392,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="12">
@@ -4403,10 +4409,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="13">
@@ -4414,16 +4420,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -4457,10 +4463,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -4486,7 +4492,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3">
@@ -4509,7 +4515,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4">
@@ -4532,7 +4538,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5">
@@ -4543,7 +4549,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -4555,7 +4561,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6">
@@ -4578,7 +4584,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="7">
@@ -4601,7 +4607,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8">
@@ -4624,7 +4630,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9">
@@ -4635,7 +4641,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -4647,7 +4653,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10">
@@ -4670,7 +4676,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="11">
@@ -4693,7 +4699,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12">
@@ -4716,7 +4722,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13">
@@ -4727,7 +4733,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -4739,7 +4745,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="14">
@@ -4762,7 +4768,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="15">
@@ -4773,7 +4779,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -4785,7 +4791,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="16">
@@ -4808,7 +4814,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17">
@@ -4831,7 +4837,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -4852,10 +4858,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -4863,35 +4869,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -4915,7 +4921,7 @@
         <v>139</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>23</v>
@@ -4927,10 +4933,10 @@
         <v>84</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -4960,7 +4966,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3">
@@ -4987,7 +4993,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4">
@@ -5014,7 +5020,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5">
@@ -5041,7 +5047,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6">
@@ -5068,7 +5074,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7">
@@ -5095,7 +5101,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8">
@@ -5122,7 +5128,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9">
@@ -5149,7 +5155,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="10">
@@ -5176,7 +5182,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11">
@@ -5203,7 +5209,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="12">
@@ -5230,7 +5236,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="13">
@@ -5257,12 +5263,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: venta dictada 18.000 esta semana; la venta dictada manda sobre la estimacion por dias; sab 24 23.540, faltan 4
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -469,10 +469,10 @@
     <t>total 16.000 = BO 1.050 (1 carga) + BR 9929 + PY 5021 (resto con el mix BR/PY del ERP ult. 4 sem)</t>
   </si>
   <si>
-    <t>AUTO</t>
-  </si>
-  <si>
-    <t>Gonzalo 11/10/2026 "vamos por el 1": venta prevista = promedio real de las ultimas 10 semanas (Aloha); el generador pisa BR/PY/BO en cada corrida. Si Gonzalo dicta una semana, poner fuente "Gonzalo dd/MM..." y sus numeros.</t>
+    <t>Gonzalo 15/10: "esta semana se va a vender 18 mil" = 18.000</t>
+  </si>
+  <si>
+    <t>reparto con el mix real de las ultimas 10 semanas</t>
   </si>
   <si>
     <t>Gonzalo 15/10: "la idea es semana que viene vender 20 o 21 mil cajas" = 20.500 (punto medio)</t>
@@ -4090,13 +4090,13 @@
         <v>46307</v>
       </c>
       <c r="B6" s="0">
-        <v>10593</v>
+        <v>9756</v>
       </c>
       <c r="C6" s="0">
-        <v>5357</v>
+        <v>7056</v>
       </c>
       <c r="D6" s="0">
-        <v>1050</v>
+        <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
         <v>147</v>

</xml_diff>

<commit_message>
plan de compras: confirmacion de las semanas 12-17 y 19-25 (Guido vuelve, Muller 3, Agro 1, PY solo Guido); sab 24 24.548, faltan 3
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="197">
   <si>
     <t>fecha</t>
   </si>
@@ -394,15 +394,12 @@
     <t>Jaime Zimerman</t>
   </si>
   <si>
-    <t>planificacion 15/10: Jaime Zimerman 1 (38): cuarta (nuevo)</t>
+    <t>planificacion 15/10: Jaime Zimerman 1 (38): cuarta (nuevo); transporte Nilton (confirmacion 15/10)</t>
   </si>
   <si>
     <t>planificacion 15/10: Agro 2 (precio pendiente): cuarta</t>
   </si>
   <si>
-    <t>planificacion 15/10: Agro 2 (precio pendiente): sexta (SUPUESTO: el dictado solo decia cuarta; se mantuvo la sexta del 14/10)</t>
-  </si>
-  <si>
     <t>planificacion 15/10: Gilson 1 (38): cuarta</t>
   </si>
   <si>
@@ -412,9 +409,6 @@
     <t>planificacion 15/10: Wagner 1 (38): sexta</t>
   </si>
   <si>
-    <t>planificacion 15/10: Milciades 1 (7 USD): lunes</t>
-  </si>
-  <si>
     <t>Paraguay GM</t>
   </si>
   <si>
@@ -443,6 +437,15 @@
   </si>
   <si>
     <t>dictado 15/10: Sergio Correia 1 (36): sabado (Gonzalo 15/10)</t>
+  </si>
+  <si>
+    <t>Gonzalo 15/10 confirmacion (chat)</t>
+  </si>
+  <si>
+    <t>confirmacion 15/10: Guido 1: martes (confirmacion 15/10: vuelve a esta semana)</t>
+  </si>
+  <si>
+    <t>confirmacion 15/10: Miuller Fabricio 3 (via Curuca): cuarta (confirmacion 15/10: pasa a 3)</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -654,11 +657,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -3601,10 +3605,10 @@
         <v>121</v>
       </c>
       <c r="F82" s="0" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G82" s="0" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H82" s="0">
         <v>1008</v>
@@ -3650,10 +3654,10 @@
     </row>
     <row r="84">
       <c r="A84" s="4">
-        <v>46318</v>
+        <v>46316</v>
       </c>
       <c r="B84" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C84" s="0" t="s">
         <v>110</v>
@@ -3662,7 +3666,7 @@
         <v>23</v>
       </c>
       <c r="E84" s="0" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F84" s="0" t="s">
         <v>40</v>
@@ -3694,7 +3698,7 @@
         <v>23</v>
       </c>
       <c r="E85" s="0" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="F85" s="0" t="s">
         <v>40</v>
@@ -3709,15 +3713,15 @@
         <v>89</v>
       </c>
       <c r="J85" s="0" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4">
-        <v>46316</v>
+        <v>46318</v>
       </c>
       <c r="B86" s="0" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C86" s="0" t="s">
         <v>110</v>
@@ -3726,7 +3730,7 @@
         <v>23</v>
       </c>
       <c r="E86" s="0" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
       <c r="F86" s="0" t="s">
         <v>40</v>
@@ -3741,7 +3745,7 @@
         <v>89</v>
       </c>
       <c r="J86" s="0" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="87">
@@ -3758,7 +3762,7 @@
         <v>23</v>
       </c>
       <c r="E87" s="0" t="s">
-        <v>103</v>
+        <v>125</v>
       </c>
       <c r="F87" s="0" t="s">
         <v>40</v>
@@ -3773,56 +3777,56 @@
         <v>89</v>
       </c>
       <c r="J87" s="0" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4">
-        <v>46318</v>
+        <v>46314</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C88" s="0" t="s">
         <v>110</v>
       </c>
       <c r="D88" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F88" s="0" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G88" s="0" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H88" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I88" s="0" t="s">
         <v>89</v>
       </c>
       <c r="J88" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="4">
-        <v>46314</v>
+      <c r="A89" s="5">
+        <v>46312</v>
       </c>
       <c r="B89" s="0" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="C89" s="0" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="D89" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>19</v>
+        <v>129</v>
       </c>
       <c r="F89" s="0" t="s">
         <v>14</v>
@@ -3831,117 +3835,117 @@
         <v>14</v>
       </c>
       <c r="H89" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I89" s="0" t="s">
-        <v>89</v>
+        <v>130</v>
       </c>
       <c r="J89" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="4">
-        <v>46314</v>
+      <c r="A90" s="6">
+        <v>46318</v>
       </c>
       <c r="B90" s="0" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C90" s="0" t="s">
         <v>110</v>
       </c>
       <c r="D90" s="0" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E90" s="0" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="F90" s="0" t="s">
-        <v>14</v>
+        <v>133</v>
       </c>
       <c r="G90" s="0" t="s">
         <v>14</v>
       </c>
       <c r="H90" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I90" s="0" t="s">
-        <v>89</v>
+        <v>130</v>
       </c>
       <c r="J90" s="0" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="5">
-        <v>46312</v>
+      <c r="A91" s="7">
+        <v>46319</v>
       </c>
       <c r="B91" s="0" t="s">
         <v>29</v>
       </c>
       <c r="C91" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D91" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E91" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="F91" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G91" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H91" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I91" s="0" t="s">
+        <v>130</v>
+      </c>
+      <c r="J91" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="8">
+        <v>46308</v>
+      </c>
+      <c r="B92" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C92" s="0" t="s">
         <v>88</v>
       </c>
-      <c r="D91" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E91" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F91" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G91" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H91" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I91" s="0" t="s">
-        <v>132</v>
-      </c>
-      <c r="J91" s="0" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="6">
-        <v>46318</v>
-      </c>
-      <c r="B92" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="C92" s="0" t="s">
-        <v>110</v>
-      </c>
       <c r="D92" s="0" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E92" s="0" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="F92" s="0" t="s">
-        <v>135</v>
+        <v>14</v>
       </c>
       <c r="G92" s="0" t="s">
         <v>14</v>
       </c>
       <c r="H92" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I92" s="0" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="J92" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="7">
-        <v>46319</v>
+      <c r="A93" s="8">
+        <v>46316</v>
       </c>
       <c r="B93" s="0" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="C93" s="0" t="s">
         <v>110</v>
@@ -3950,22 +3954,22 @@
         <v>23</v>
       </c>
       <c r="E93" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="F93" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="G93" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H93" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I93" s="0" t="s">
         <v>137</v>
       </c>
-      <c r="F93" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G93" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H93" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I93" s="0" t="s">
-        <v>132</v>
-      </c>
       <c r="J93" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -3987,7 +3991,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>23</v>
@@ -4019,10 +4023,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3">
@@ -4039,10 +4043,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4">
@@ -4059,10 +4063,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5">
@@ -4079,10 +4083,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6">
@@ -4099,10 +4103,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7">
@@ -4119,10 +4123,10 @@
         <v>1353</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -4141,57 +4145,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -4239,10 +4243,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3">
@@ -4256,10 +4260,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4">
@@ -4273,10 +4277,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5">
@@ -4284,16 +4288,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="6">
@@ -4307,10 +4311,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7">
@@ -4324,10 +4328,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8">
@@ -4341,10 +4345,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9">
@@ -4352,16 +4356,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="10">
@@ -4375,10 +4379,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11">
@@ -4392,10 +4396,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="12">
@@ -4409,10 +4413,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="13">
@@ -4420,16 +4424,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -4463,10 +4467,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -4492,7 +4496,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3">
@@ -4515,7 +4519,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4">
@@ -4538,7 +4542,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5">
@@ -4549,7 +4553,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -4561,7 +4565,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6">
@@ -4584,7 +4588,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7">
@@ -4607,7 +4611,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="8">
@@ -4630,7 +4634,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="9">
@@ -4641,7 +4645,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -4653,7 +4657,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="10">
@@ -4676,7 +4680,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11">
@@ -4699,7 +4703,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="12">
@@ -4722,7 +4726,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="13">
@@ -4733,7 +4737,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -4745,7 +4749,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="14">
@@ -4768,7 +4772,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="15">
@@ -4779,7 +4783,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -4791,7 +4795,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="16">
@@ -4814,7 +4818,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="17">
@@ -4837,7 +4841,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -4858,10 +4862,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -4869,35 +4873,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -4918,10 +4922,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>23</v>
@@ -4933,10 +4937,10 @@
         <v>84</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -4966,7 +4970,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3">
@@ -4993,7 +4997,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4">
@@ -5020,7 +5024,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5">
@@ -5047,7 +5051,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6">
@@ -5074,7 +5078,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7">
@@ -5101,7 +5105,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8">
@@ -5128,7 +5132,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9">
@@ -5155,7 +5159,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="10">
@@ -5182,7 +5186,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11">
@@ -5209,7 +5213,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="12">
@@ -5236,7 +5240,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="13">
@@ -5263,12 +5267,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: semana 19-25 con Jhony tersa, segunda de Gilson y dos medias cargas (Furlani, Josemar); sab 24 cierra 27.428
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="202">
   <si>
     <t>fecha</t>
   </si>
@@ -446,6 +446,21 @@
   </si>
   <si>
     <t>confirmacion 15/10: Miuller Fabricio 3 (via Curuca): cuarta (confirmacion 15/10: pasa a 3)</t>
+  </si>
+  <si>
+    <t>Gonzalo 15/10 noche (chat)</t>
+  </si>
+  <si>
+    <t>dictado 15/10 noche: 1/2 carga: 12 pallets en el camion de exoticos, tersa</t>
+  </si>
+  <si>
+    <t>dictado 15/10 noche: 1/2 carga: 12 pallets en el camion de exoticos, cuarta</t>
+  </si>
+  <si>
+    <t>dictado 15/10 noche: Jony 1: tersa</t>
+  </si>
+  <si>
+    <t>dictado 15/10 noche: Gilson 2: la segunda, tambien cuarta</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -657,11 +672,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -981,7 +997,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J93"/>
+  <dimension ref="A1:J97"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -3970,6 +3986,134 @@
       </c>
       <c r="J93" s="0" t="s">
         <v>139</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="9">
+        <v>46315</v>
+      </c>
+      <c r="B94" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C94" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D94" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E94" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="F94" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G94" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H94" s="0">
+        <v>432</v>
+      </c>
+      <c r="I94" s="0" t="s">
+        <v>140</v>
+      </c>
+      <c r="J94" s="0" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="9">
+        <v>46316</v>
+      </c>
+      <c r="B95" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C95" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D95" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E95" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="F95" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G95" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H95" s="0">
+        <v>432</v>
+      </c>
+      <c r="I95" s="0" t="s">
+        <v>140</v>
+      </c>
+      <c r="J95" s="0" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="9">
+        <v>46315</v>
+      </c>
+      <c r="B96" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C96" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D96" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E96" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="F96" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G96" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H96" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I96" s="0" t="s">
+        <v>140</v>
+      </c>
+      <c r="J96" s="0" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="9">
+        <v>46316</v>
+      </c>
+      <c r="B97" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C97" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D97" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E97" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="F97" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="G97" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="H97" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I97" s="0" t="s">
+        <v>140</v>
+      </c>
+      <c r="J97" s="0" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -3991,7 +4135,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>23</v>
@@ -4023,10 +4167,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3">
@@ -4043,10 +4187,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4">
@@ -4063,10 +4207,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5">
@@ -4083,10 +4227,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6">
@@ -4103,10 +4247,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7">
@@ -4123,10 +4267,10 @@
         <v>1353</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -4145,57 +4289,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -4243,10 +4387,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3">
@@ -4260,10 +4404,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4">
@@ -4277,10 +4421,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5">
@@ -4288,16 +4432,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6">
@@ -4311,10 +4455,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7">
@@ -4328,10 +4472,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="8">
@@ -4345,10 +4489,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9">
@@ -4356,16 +4500,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10">
@@ -4379,10 +4523,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11">
@@ -4396,10 +4540,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12">
@@ -4413,10 +4557,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13">
@@ -4424,16 +4568,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -4467,10 +4611,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -4496,7 +4640,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3">
@@ -4519,7 +4663,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4">
@@ -4542,7 +4686,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5">
@@ -4553,7 +4697,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -4565,7 +4709,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6">
@@ -4588,7 +4732,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7">
@@ -4611,7 +4755,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8">
@@ -4634,7 +4778,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9">
@@ -4645,7 +4789,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -4657,7 +4801,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10">
@@ -4680,7 +4824,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="11">
@@ -4703,7 +4847,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="12">
@@ -4726,7 +4870,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="13">
@@ -4737,7 +4881,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -4749,7 +4893,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="14">
@@ -4772,7 +4916,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="15">
@@ -4783,7 +4927,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -4795,7 +4939,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="16">
@@ -4818,7 +4962,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="17">
@@ -4841,7 +4985,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -4862,10 +5006,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -4873,35 +5017,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>
@@ -4922,10 +5066,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>23</v>
@@ -4937,10 +5081,10 @@
         <v>84</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -4970,7 +5114,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3">
@@ -4997,7 +5141,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4">
@@ -5024,7 +5168,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5">
@@ -5051,7 +5195,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6">
@@ -5078,7 +5222,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="7">
@@ -5105,7 +5249,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8">
@@ -5132,7 +5276,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9">
@@ -5159,7 +5303,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10">
@@ -5186,7 +5330,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11">
@@ -5213,7 +5357,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="12">
@@ -5240,7 +5384,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13">
@@ -5267,12 +5411,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: descarga real de los dictados (columna descarga); 5 ya descargados el 16/10 y Guido 13/10 cancelado
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -58,6 +58,9 @@
     <t>nota</t>
   </si>
   <si>
+    <t>descarga</t>
+  </si>
+  <si>
     <t>dom</t>
   </si>
   <si>
@@ -319,6 +322,9 @@
     <t>planificacion 15/10: Stein 2 (38): cuarta</t>
   </si>
   <si>
+    <t>2026-10-16</t>
+  </si>
+  <si>
     <t>planificacion 15/10: Stein 2 (38): sexta</t>
   </si>
   <si>
@@ -367,112 +373,106 @@
     <t>dictado 15/10: carga extra sabado 17 (Gonzalo 15/10: "hay una carga extra sabado 17 de jony viera")</t>
   </si>
   <si>
+    <t>2026-10-18</t>
+  </si>
+  <si>
+    <t>Gonzalo 16/10 definitivo (chat)</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: 1/2 carga exoticos: tersa</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: 1/2 carga exoticos: cuarta</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Fisher 2: tersa</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Fisher 2: cuarta</t>
+  </si>
+  <si>
+    <t>Muller Fabricio</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Muller 3 (Curuca): tersa</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Muller 3 (Curuca): cuarta</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Muller 3 (Curuca): sexta</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Stein 3: segunda</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Stein 3: tersa</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Stein 3: sexta</t>
+  </si>
+  <si>
+    <t>BAHIA</t>
+  </si>
+  <si>
+    <t>Silvio</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Sergio 2: Bahia sexta (Silvio)</t>
+  </si>
+  <si>
+    <t>Sergio</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Sergio 2: SC sabado</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Cassio 3: tersa</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Cassio 3: cuarta</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Cassio 3: sexta</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Jony 1: tersa</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Celso 1: cuarta</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Ivo 1: tersa</t>
+  </si>
+  <si>
+    <t>Jaime Zimerman</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Jaime Zimerman 1: cuarta</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Agro 2: cuarta</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Agro 2: sexta</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Gilson 1: tersa</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Marconi 1: cuarta</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Shapo 1: tersa</t>
+  </si>
+  <si>
+    <t>Wagner</t>
+  </si>
+  <si>
+    <t>definitivo 16/10: Wagner 1: sexta</t>
+  </si>
+  <si>
     <t>Paraguay GM</t>
-  </si>
-  <si>
-    <t>Gonzalo 15/10 confirmacion (chat)</t>
-  </si>
-  <si>
-    <t>confirmacion 15/10: Guido 1: martes (confirmacion 15/10: vuelve a esta semana)</t>
-  </si>
-  <si>
-    <t>2026-10-18</t>
-  </si>
-  <si>
-    <t>Gonzalo 16/10 definitivo (chat)</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: 1/2 carga exoticos: tersa</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: 1/2 carga exoticos: cuarta</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Fisher 2: tersa</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Fisher 2: cuarta</t>
-  </si>
-  <si>
-    <t>Muller Fabricio</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Muller 3 (Curuca): tersa</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Muller 3 (Curuca): cuarta</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Muller 3 (Curuca): sexta</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Stein 3: segunda</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Stein 3: tersa</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Stein 3: sexta</t>
-  </si>
-  <si>
-    <t>BAHIA</t>
-  </si>
-  <si>
-    <t>Silvio</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Sergio 2: Bahia sexta (Silvio)</t>
-  </si>
-  <si>
-    <t>Sergio</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Sergio 2: SC sabado</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Cassio 3: tersa</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Cassio 3: cuarta</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Cassio 3: sexta</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Jony 1: tersa</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Celso 1: cuarta</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Ivo 1: tersa</t>
-  </si>
-  <si>
-    <t>Jaime Zimerman</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Jaime Zimerman 1: cuarta</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Agro 2: cuarta</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Agro 2: sexta</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Gilson 1: tersa</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Marconi 1: cuarta</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Shapo 1: tersa</t>
-  </si>
-  <si>
-    <t>Wagner</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Wagner 1: sexta</t>
   </si>
   <si>
     <t>definitivo 16/10: Guido 1: lunes</t>
@@ -687,12 +687,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -1010,7 +1009,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J98"/>
+  <dimension ref="A1:K97"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -1056,37 +1055,40 @@
       <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="0" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
         <v>46278</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" s="0">
         <v>980</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -1094,31 +1096,31 @@
         <v>46278</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H3" s="0">
         <v>980</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -1126,31 +1128,31 @@
         <v>46278</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H4" s="0">
         <v>980</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -1158,31 +1160,31 @@
         <v>46279</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H5" s="0">
         <v>980</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -1190,31 +1192,31 @@
         <v>46279</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H6" s="0">
         <v>980</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J6" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -1222,31 +1224,31 @@
         <v>46279</v>
       </c>
       <c r="B7" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="0" t="s">
-        <v>17</v>
-      </c>
       <c r="F7" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H7" s="0">
         <v>980</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J7" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -1254,31 +1256,31 @@
         <v>46280</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H8" s="0">
         <v>980</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J8" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -1286,31 +1288,31 @@
         <v>46280</v>
       </c>
       <c r="B9" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="0" t="s">
-        <v>19</v>
-      </c>
       <c r="F9" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H9" s="0">
         <v>980</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J9" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
@@ -1318,31 +1320,31 @@
         <v>46283</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H10" s="0">
         <v>936</v>
       </c>
       <c r="I10" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J10" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
@@ -1350,31 +1352,31 @@
         <v>46283</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H11" s="0">
         <v>936</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J11" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -1382,31 +1384,31 @@
         <v>46284</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H12" s="0">
         <v>1008</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J12" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13">
@@ -1414,31 +1416,31 @@
         <v>46287</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H13" s="0">
         <v>1008</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J13" s="0" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14">
@@ -1446,31 +1448,31 @@
         <v>46290</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H14" s="0">
         <v>936</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15">
@@ -1478,31 +1480,31 @@
         <v>46290</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H15" s="0">
         <v>1008</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J15" s="0" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16">
@@ -1510,31 +1512,31 @@
         <v>46290</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H16" s="0">
         <v>1008</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J16" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17">
@@ -1542,31 +1544,31 @@
         <v>46285</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H17" s="0">
         <v>980</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J17" s="0" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18">
@@ -1574,31 +1576,31 @@
         <v>46286</v>
       </c>
       <c r="B18" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="D18" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" s="0" t="s">
-        <v>17</v>
-      </c>
       <c r="F18" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H18" s="0">
         <v>980</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J18" s="0" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="19">
@@ -1606,31 +1608,31 @@
         <v>46287</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H19" s="0">
         <v>980</v>
       </c>
       <c r="I19" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J19" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20">
@@ -1638,31 +1640,31 @@
         <v>46286</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G20" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H20" s="0">
         <v>980</v>
       </c>
       <c r="I20" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J20" s="0" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21">
@@ -1670,31 +1672,31 @@
         <v>46287</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G21" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H21" s="0">
         <v>980</v>
       </c>
       <c r="I21" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J21" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22">
@@ -1702,31 +1704,31 @@
         <v>46286</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G22" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H22" s="0">
         <v>980</v>
       </c>
       <c r="I22" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J22" s="0" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23">
@@ -1734,31 +1736,31 @@
         <v>46287</v>
       </c>
       <c r="B23" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="D23" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E23" s="0" t="s">
-        <v>19</v>
-      </c>
       <c r="F23" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H23" s="0">
         <v>980</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J23" s="0" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24">
@@ -1766,31 +1768,31 @@
         <v>46295</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H24" s="0">
         <v>1008</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J24" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25">
@@ -1798,31 +1800,31 @@
         <v>46297</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H25" s="0">
         <v>1008</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J25" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26">
@@ -1830,31 +1832,31 @@
         <v>46295</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G26" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H26" s="0">
         <v>1008</v>
       </c>
       <c r="I26" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J26" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27">
@@ -1862,31 +1864,31 @@
         <v>46294</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H27" s="0">
         <v>1008</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J27" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28">
@@ -1894,31 +1896,31 @@
         <v>46297</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F28" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G28" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H28" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I28" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="J28" s="0" t="s">
         <v>55</v>
-      </c>
-      <c r="G28" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H28" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I28" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="J28" s="0" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="29">
@@ -1926,31 +1928,31 @@
         <v>46297</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G29" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H29" s="0">
         <v>1008</v>
       </c>
       <c r="I29" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J29" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="30">
@@ -1958,31 +1960,31 @@
         <v>46297</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H30" s="0">
         <v>1008</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J30" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31">
@@ -1990,31 +1992,31 @@
         <v>46297</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D31" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H31" s="0">
         <v>1008</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J31" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32">
@@ -2022,31 +2024,31 @@
         <v>46297</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F32" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G32" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I32" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="J32" s="0" t="s">
         <v>55</v>
-      </c>
-      <c r="G32" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H32" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I32" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="J32" s="0" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="33">
@@ -2054,31 +2056,31 @@
         <v>46293</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D33" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G33" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H33" s="0">
         <v>980</v>
       </c>
       <c r="I33" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J33" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34">
@@ -2086,31 +2088,31 @@
         <v>46293</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G34" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H34" s="0">
         <v>980</v>
       </c>
       <c r="I34" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J34" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35">
@@ -2118,31 +2120,31 @@
         <v>46294</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H35" s="0">
         <v>980</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J35" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="36">
@@ -2150,31 +2152,31 @@
         <v>46293</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D36" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H36" s="0">
         <v>980</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37">
@@ -2182,31 +2184,31 @@
         <v>46295</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H37" s="0">
         <v>1008</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J37" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="38">
@@ -2214,31 +2216,31 @@
         <v>46295</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D38" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G38" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H38" s="0">
         <v>936</v>
       </c>
       <c r="I38" s="0" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J38" s="0" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="39">
@@ -2246,31 +2248,31 @@
         <v>46301</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D39" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F39" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G39" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H39" s="0">
         <v>1008</v>
       </c>
       <c r="I39" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J39" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="40">
@@ -2278,31 +2280,31 @@
         <v>46304</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H40" s="0">
         <v>1008</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="41">
@@ -2310,31 +2312,31 @@
         <v>46302</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H41" s="0">
         <v>1008</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J41" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="42">
@@ -2342,31 +2344,31 @@
         <v>46302</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G42" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H42" s="0">
         <v>936</v>
       </c>
       <c r="I42" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J42" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="43">
@@ -2374,31 +2376,31 @@
         <v>46302</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H43" s="0">
         <v>1008</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="44">
@@ -2406,31 +2408,31 @@
         <v>46301</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H44" s="0">
         <v>1008</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="45">
@@ -2438,31 +2440,31 @@
         <v>46302</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H45" s="0">
         <v>1008</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="46">
@@ -2470,31 +2472,31 @@
         <v>46301</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G46" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H46" s="0">
         <v>1008</v>
       </c>
       <c r="I46" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J46" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="47">
@@ -2502,31 +2504,31 @@
         <v>46300</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H47" s="0">
         <v>980</v>
       </c>
       <c r="I47" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J47" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48">
@@ -2534,31 +2536,31 @@
         <v>46301</v>
       </c>
       <c r="B48" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C48" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="D48" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E48" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="C48" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="D48" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E48" s="0" t="s">
-        <v>19</v>
-      </c>
       <c r="F48" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H48" s="0">
         <v>980</v>
       </c>
       <c r="I48" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J48" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="49">
@@ -2566,31 +2568,31 @@
         <v>46300</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C49" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D49" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F49" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G49" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H49" s="0">
         <v>980</v>
       </c>
       <c r="I49" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J49" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="50">
@@ -2598,31 +2600,31 @@
         <v>46301</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C50" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D50" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G50" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H50" s="0">
         <v>980</v>
       </c>
       <c r="I50" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J50" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="51">
@@ -2630,31 +2632,31 @@
         <v>46300</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D51" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G51" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H51" s="0">
         <v>980</v>
       </c>
       <c r="I51" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J51" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="52">
@@ -2662,31 +2664,31 @@
         <v>46304</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G52" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H52" s="0">
         <v>1050</v>
       </c>
       <c r="I52" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J52" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="53">
@@ -2694,31 +2696,31 @@
         <v>46309</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D53" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H53" s="0">
         <v>1008</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J53" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="54">
@@ -2726,31 +2728,31 @@
         <v>46312</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H54" s="0">
         <v>1008</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J54" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="55">
@@ -2758,31 +2760,31 @@
         <v>46309</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C55" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D55" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H55" s="0">
         <v>1008</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J55" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="56">
@@ -2790,31 +2792,31 @@
         <v>46311</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H56" s="0">
         <v>1008</v>
       </c>
       <c r="I56" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J56" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="57">
@@ -2822,31 +2824,31 @@
         <v>46309</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C57" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H57" s="0">
         <v>1008</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J57" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="58">
@@ -2854,31 +2856,31 @@
         <v>46311</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C58" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G58" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H58" s="0">
         <v>1008</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="59">
@@ -2886,31 +2888,34 @@
         <v>46309</v>
       </c>
       <c r="B59" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G59" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H59" s="0">
         <v>1008</v>
       </c>
       <c r="I59" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J59" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
+      </c>
+      <c r="K59" s="0" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="60">
@@ -2918,31 +2923,31 @@
         <v>46311</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G60" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H60" s="0">
         <v>1008</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J60" s="0" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="61">
@@ -2950,30 +2955,33 @@
         <v>46309</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H61" s="0">
         <v>1008</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J61" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="K61" s="0" t="s">
         <v>98</v>
       </c>
     </row>
@@ -2982,31 +2990,34 @@
         <v>46309</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C62" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G62" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H62" s="0">
         <v>1008</v>
       </c>
       <c r="I62" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J62" s="0" t="s">
-        <v>99</v>
+        <v>101</v>
+      </c>
+      <c r="K62" s="0" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="63">
@@ -3014,31 +3025,31 @@
         <v>46309</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D63" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G63" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H63" s="0">
         <v>1008</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="64">
@@ -3046,31 +3057,34 @@
         <v>46309</v>
       </c>
       <c r="B64" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G64" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H64" s="0">
         <v>1008</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J64" s="0" t="s">
-        <v>101</v>
+        <v>103</v>
+      </c>
+      <c r="K64" s="0" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="65">
@@ -3078,31 +3092,31 @@
         <v>46311</v>
       </c>
       <c r="B65" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C65" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F65" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G65" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H65" s="0">
         <v>1008</v>
       </c>
       <c r="I65" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J65" s="0" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="66">
@@ -3110,31 +3124,31 @@
         <v>46311</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C66" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F66" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G66" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H66" s="0">
         <v>1008</v>
       </c>
       <c r="I66" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J66" s="0" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="67">
@@ -3142,31 +3156,31 @@
         <v>46308</v>
       </c>
       <c r="B67" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C67" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E67" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F67" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G67" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H67" s="0">
         <v>432</v>
       </c>
       <c r="I67" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J67" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="68">
@@ -3174,31 +3188,34 @@
         <v>46308</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C68" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D68" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E68" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F68" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G68" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H68" s="0">
         <v>980</v>
       </c>
       <c r="I68" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J68" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
+      </c>
+      <c r="K68" s="0" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="69">
@@ -3206,31 +3223,31 @@
         <v>46309</v>
       </c>
       <c r="B69" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C69" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D69" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E69" s="0" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G69" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H69" s="0">
         <v>980</v>
       </c>
       <c r="I69" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J69" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="70">
@@ -3238,31 +3255,31 @@
         <v>46311</v>
       </c>
       <c r="B70" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C70" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D70" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E70" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F70" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G70" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H70" s="0">
         <v>1050</v>
       </c>
       <c r="I70" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J70" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="71">
@@ -3270,894 +3287,862 @@
         <v>46312</v>
       </c>
       <c r="B71" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C71" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D71" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E71" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F71" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G71" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H71" s="0">
         <v>1008</v>
       </c>
       <c r="I71" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="J71" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="6">
-        <v>46308</v>
+        <v>46315</v>
       </c>
       <c r="B72" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C72" s="0" t="s">
-        <v>88</v>
+        <v>115</v>
       </c>
       <c r="D72" s="0" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E72" s="0" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="F72" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G72" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H72" s="0">
-        <v>980</v>
+        <v>432</v>
       </c>
       <c r="I72" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="J72" s="0" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6">
+        <v>46316</v>
+      </c>
+      <c r="B73" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C73" s="0" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="7">
-        <v>46315</v>
-      </c>
-      <c r="B73" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="C73" s="0" t="s">
-        <v>116</v>
-      </c>
       <c r="D73" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E73" s="0" t="s">
-        <v>105</v>
+        <v>58</v>
       </c>
       <c r="F73" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G73" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H73" s="0">
         <v>432</v>
       </c>
       <c r="I73" s="0" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J73" s="0" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="7">
-        <v>46316</v>
+      <c r="A74" s="6">
+        <v>46315</v>
       </c>
       <c r="B74" s="0" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="C74" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D74" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E74" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="F74" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="G74" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H74" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I74" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D74" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E74" s="0" t="s">
-        <v>57</v>
-      </c>
-      <c r="F74" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G74" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H74" s="0">
-        <v>432</v>
-      </c>
-      <c r="I74" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J74" s="0" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="7">
-        <v>46315</v>
+      <c r="A75" s="6">
+        <v>46316</v>
       </c>
       <c r="B75" s="0" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="C75" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D75" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E75" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="F75" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="G75" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H75" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I75" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D75" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E75" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="F75" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="G75" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H75" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I75" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J75" s="0" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="7">
+      <c r="A76" s="6">
+        <v>46315</v>
+      </c>
+      <c r="B76" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C76" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D76" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E76" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="F76" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G76" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H76" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I76" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="J76" s="0" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6">
         <v>46316</v>
       </c>
-      <c r="B76" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="C76" s="0" t="s">
+      <c r="B77" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C77" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D77" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E77" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="F77" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G77" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H77" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I77" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D76" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E76" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="F76" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="G76" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H76" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I76" s="0" t="s">
-        <v>117</v>
-      </c>
-      <c r="J76" s="0" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="7">
-        <v>46315</v>
-      </c>
-      <c r="B77" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="C77" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="D77" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E77" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="F77" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="G77" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H77" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I77" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J77" s="0" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="7">
-        <v>46316</v>
+      <c r="A78" s="6">
+        <v>46318</v>
       </c>
       <c r="B78" s="0" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="C78" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D78" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E78" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="F78" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G78" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H78" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I78" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D78" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E78" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="F78" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="G78" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H78" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I78" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J78" s="0" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="7">
-        <v>46318</v>
+      <c r="A79" s="6">
+        <v>46314</v>
       </c>
       <c r="B79" s="0" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C79" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D79" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E79" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F79" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G79" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H79" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I79" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D79" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E79" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="F79" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="G79" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H79" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I79" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J79" s="0" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="7">
-        <v>46314</v>
+      <c r="A80" s="6">
+        <v>46315</v>
       </c>
       <c r="B80" s="0" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C80" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D80" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E80" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F80" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G80" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H80" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I80" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D80" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E80" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="F80" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="G80" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H80" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I80" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J80" s="0" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="7">
-        <v>46315</v>
+      <c r="A81" s="6">
+        <v>46318</v>
       </c>
       <c r="B81" s="0" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C81" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D81" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E81" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F81" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G81" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H81" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I81" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D81" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E81" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="F81" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="G81" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H81" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I81" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J81" s="0" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="7">
+      <c r="A82" s="6">
         <v>46318</v>
       </c>
       <c r="B82" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C82" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D82" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E82" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="F82" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="G82" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H82" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I82" s="0" t="s">
         <v>116</v>
       </c>
-      <c r="D82" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E82" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="F82" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="G82" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H82" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I82" s="0" t="s">
-        <v>117</v>
-      </c>
       <c r="J82" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="7">
-        <v>46318</v>
+      <c r="A83" s="6">
+        <v>46319</v>
       </c>
       <c r="B83" s="0" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="C83" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D83" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E83" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="F83" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G83" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H83" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I83" s="0" t="s">
         <v>116</v>
       </c>
-      <c r="D83" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E83" s="0" t="s">
-        <v>129</v>
-      </c>
-      <c r="F83" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="G83" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H83" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I83" s="0" t="s">
-        <v>117</v>
-      </c>
       <c r="J83" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="7">
-        <v>46319</v>
+      <c r="A84" s="6">
+        <v>46315</v>
       </c>
       <c r="B84" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C84" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D84" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E84" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F84" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="G84" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="C84" s="0" t="s">
+      <c r="H84" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I84" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D84" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E84" s="0" t="s">
-        <v>132</v>
-      </c>
-      <c r="F84" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G84" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H84" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I84" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J84" s="0" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="7">
-        <v>46315</v>
+      <c r="A85" s="6">
+        <v>46316</v>
       </c>
       <c r="B85" s="0" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="C85" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D85" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E85" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F85" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G85" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H85" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I85" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D85" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E85" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="F85" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="G85" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="H85" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I85" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J85" s="0" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="7">
-        <v>46316</v>
+      <c r="A86" s="6">
+        <v>46318</v>
       </c>
       <c r="B86" s="0" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="C86" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D86" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E86" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F86" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G86" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H86" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I86" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D86" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E86" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="F86" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G86" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H86" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I86" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J86" s="0" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="7">
-        <v>46318</v>
+      <c r="A87" s="6">
+        <v>46315</v>
       </c>
       <c r="B87" s="0" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C87" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D87" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E87" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="F87" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G87" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H87" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I87" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D87" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E87" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="F87" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G87" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H87" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I87" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J87" s="0" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="7">
-        <v>46315</v>
+      <c r="A88" s="6">
+        <v>46316</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="C88" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D88" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E88" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="F88" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G88" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H88" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I88" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D88" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E88" s="0" t="s">
-        <v>110</v>
-      </c>
-      <c r="F88" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G88" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H88" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I88" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J88" s="0" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="7">
-        <v>46316</v>
+      <c r="A89" s="6">
+        <v>46315</v>
       </c>
       <c r="B89" s="0" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="C89" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D89" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E89" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F89" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G89" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H89" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I89" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D89" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E89" s="0" t="s">
-        <v>74</v>
-      </c>
-      <c r="F89" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G89" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H89" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I89" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J89" s="0" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="7">
-        <v>46315</v>
+      <c r="A90" s="6">
+        <v>46316</v>
       </c>
       <c r="B90" s="0" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="C90" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D90" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E90" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="F90" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G90" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H90" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I90" s="0" t="s">
         <v>116</v>
       </c>
-      <c r="D90" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E90" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="F90" s="0" t="s">
+      <c r="J90" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="6">
+        <v>46316</v>
+      </c>
+      <c r="B91" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C91" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D91" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E91" s="0" t="s">
         <v>40</v>
       </c>
-      <c r="G90" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H90" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I90" s="0" t="s">
-        <v>117</v>
-      </c>
-      <c r="J90" s="0" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="7">
-        <v>46316</v>
-      </c>
-      <c r="B91" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="C91" s="0" t="s">
+      <c r="F91" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G91" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H91" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I91" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D91" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E91" s="0" t="s">
-        <v>140</v>
-      </c>
-      <c r="F91" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G91" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H91" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I91" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J91" s="0" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="7">
-        <v>46316</v>
+      <c r="A92" s="6">
+        <v>46318</v>
       </c>
       <c r="B92" s="0" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="C92" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D92" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E92" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="F92" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G92" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H92" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I92" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D92" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E92" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="F92" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G92" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H92" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I92" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J92" s="0" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="7">
-        <v>46318</v>
+      <c r="A93" s="6">
+        <v>46315</v>
       </c>
       <c r="B93" s="0" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C93" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D93" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E93" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="F93" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G93" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H93" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I93" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D93" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E93" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="F93" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G93" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H93" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I93" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J93" s="0" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="7">
-        <v>46315</v>
+      <c r="A94" s="6">
+        <v>46316</v>
       </c>
       <c r="B94" s="0" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="C94" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D94" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E94" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="F94" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G94" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H94" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I94" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D94" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E94" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="F94" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G94" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H94" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I94" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J94" s="0" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="7">
-        <v>46316</v>
+      <c r="A95" s="6">
+        <v>46315</v>
       </c>
       <c r="B95" s="0" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="C95" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D95" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E95" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="F95" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G95" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H95" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I95" s="0" t="s">
         <v>116</v>
-      </c>
-      <c r="D95" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E95" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="F95" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G95" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H95" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I95" s="0" t="s">
-        <v>117</v>
       </c>
       <c r="J95" s="0" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="7">
-        <v>46315</v>
+      <c r="A96" s="6">
+        <v>46318</v>
       </c>
       <c r="B96" s="0" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C96" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D96" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E96" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="F96" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G96" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H96" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I96" s="0" t="s">
         <v>116</v>
       </c>
-      <c r="D96" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E96" s="0" t="s">
-        <v>103</v>
-      </c>
-      <c r="F96" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G96" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H96" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I96" s="0" t="s">
-        <v>117</v>
-      </c>
       <c r="J96" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="7">
-        <v>46318</v>
+      <c r="A97" s="6">
+        <v>46314</v>
       </c>
       <c r="B97" s="0" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C97" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D97" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E97" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="F97" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G97" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H97" s="0">
+        <v>980</v>
+      </c>
+      <c r="I97" s="0" t="s">
         <v>116</v>
       </c>
-      <c r="D97" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E97" s="0" t="s">
-        <v>147</v>
-      </c>
-      <c r="F97" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G97" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="H97" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I97" s="0" t="s">
-        <v>117</v>
-      </c>
       <c r="J97" s="0" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="7">
-        <v>46314</v>
-      </c>
-      <c r="B98" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="C98" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="D98" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E98" s="0" t="s">
-        <v>113</v>
-      </c>
-      <c r="F98" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G98" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H98" s="0">
-        <v>980</v>
-      </c>
-      <c r="I98" s="0" t="s">
-        <v>117</v>
-      </c>
-      <c r="J98" s="0" t="s">
         <v>149</v>
       </c>
     </row>
@@ -4183,13 +4168,13 @@
         <v>150</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>8</v>
@@ -4426,7 +4411,7 @@
         <v>46282</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C2" s="0">
         <v>14475</v>
@@ -4443,7 +4428,7 @@
         <v>46282</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3" s="0">
         <v>12345</v>
@@ -4460,7 +4445,7 @@
         <v>46282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C4" s="0">
         <v>2604</v>
@@ -4494,7 +4479,7 @@
         <v>46291</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C6" s="0">
         <v>11653</v>
@@ -4511,7 +4496,7 @@
         <v>46291</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" s="0">
         <v>13673</v>
@@ -4528,7 +4513,7 @@
         <v>46291</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C8" s="0">
         <v>1646</v>
@@ -4562,7 +4547,7 @@
         <v>46298</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C10" s="0">
         <v>12269</v>
@@ -4579,7 +4564,7 @@
         <v>46298</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C11" s="0">
         <v>9676</v>
@@ -4596,7 +4581,7 @@
         <v>46298</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C12" s="0">
         <v>1500</v>
@@ -4670,10 +4655,10 @@
         <v>46280</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D2" s="0">
         <v>964</v>
@@ -4693,10 +4678,10 @@
         <v>46280</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D3" s="0">
         <v>725</v>
@@ -4716,10 +4701,10 @@
         <v>46280</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D4" s="0">
         <v>98</v>
@@ -4739,7 +4724,7 @@
         <v>46280</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
         <v>177</v>
@@ -4762,10 +4747,10 @@
         <v>46281</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D6" s="0">
         <v>1301</v>
@@ -4785,10 +4770,10 @@
         <v>46281</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D7" s="0">
         <v>710</v>
@@ -4808,10 +4793,10 @@
         <v>46281</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D8" s="0">
         <v>114</v>
@@ -4831,7 +4816,7 @@
         <v>46281</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
         <v>177</v>
@@ -4854,10 +4839,10 @@
         <v>46284</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D10" s="0">
         <v>749</v>
@@ -4877,10 +4862,10 @@
         <v>46284</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D11" s="0">
         <v>686</v>
@@ -4900,10 +4885,10 @@
         <v>46284</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D12" s="0">
         <v>139</v>
@@ -4923,7 +4908,7 @@
         <v>46284</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
         <v>177</v>
@@ -4946,10 +4931,10 @@
         <v>46291</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D14" s="0">
         <v>901</v>
@@ -4969,7 +4954,7 @@
         <v>46291</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
         <v>177</v>
@@ -4992,10 +4977,10 @@
         <v>46291</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D16" s="0">
         <v>233</v>
@@ -5015,10 +5000,10 @@
         <v>46291</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D17" s="0">
         <v>134</v>
@@ -5117,13 +5102,13 @@
         <v>203</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>177</v>

</xml_diff>

<commit_message>
plan de compras: venta de las semanas 26/10 (17900) y 2/11 (14000) por la UAM cerrada el lunes 2/11
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="211">
   <si>
     <t>fecha</t>
   </si>
@@ -512,6 +512,18 @@
   </si>
   <si>
     <t>reparto BR/PY/BO con el mix real de las ultimas 10 semanas; desde el mie 21 la pisa la estimacion con los dias reales</t>
+  </si>
+  <si>
+    <t>Gonzalo 16/10: lun 2/11 UAM cerrada, el sabado 31 vende 800 mas = estacional 17100 + 800</t>
+  </si>
+  <si>
+    <t>el resto de la semana como la venta estacional</t>
+  </si>
+  <si>
+    <t>Gonzalo 16/10: lun 2/11 UAM cerrada (sin venta), el martes 3 vende 700 mas = estacional 17500 sin el lunes (23,9 %) + 700</t>
+  </si>
+  <si>
+    <t>feriado Finados en Brasil el mismo lunes: frontera cerrada</t>
   </si>
   <si>
     <t>notas</t>
@@ -687,7 +699,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -695,6 +707,7 @@
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4154,7 +4167,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.28515625" customWidth="1"/>
@@ -4301,6 +4314,46 @@
       </c>
       <c r="F7" s="0" t="s">
         <v>161</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7">
+        <v>46321</v>
+      </c>
+      <c r="B8" s="0">
+        <v>9702</v>
+      </c>
+      <c r="C8" s="0">
+        <v>7017</v>
+      </c>
+      <c r="D8" s="0">
+        <v>1181</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="F8" s="0" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7">
+        <v>46328</v>
+      </c>
+      <c r="B9" s="0">
+        <v>7588</v>
+      </c>
+      <c r="C9" s="0">
+        <v>5488</v>
+      </c>
+      <c r="D9" s="0">
+        <v>924</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="F9" s="0" t="s">
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -4319,57 +4372,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -4417,10 +4470,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3">
@@ -4434,10 +4487,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4">
@@ -4451,10 +4504,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5">
@@ -4462,16 +4515,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6">
@@ -4485,10 +4538,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7">
@@ -4502,10 +4555,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8">
@@ -4519,10 +4572,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9">
@@ -4530,16 +4583,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10">
@@ -4553,10 +4606,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11">
@@ -4570,10 +4623,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12">
@@ -4587,10 +4640,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
     </row>
     <row r="13">
@@ -4598,16 +4651,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -4641,10 +4694,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -4670,7 +4723,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3">
@@ -4693,7 +4746,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4">
@@ -4716,7 +4769,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5">
@@ -4727,7 +4780,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -4739,7 +4792,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6">
@@ -4762,7 +4815,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="7">
@@ -4785,7 +4838,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="8">
@@ -4808,7 +4861,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9">
@@ -4819,7 +4872,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -4831,7 +4884,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="10">
@@ -4854,7 +4907,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="11">
@@ -4877,7 +4930,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="12">
@@ -4900,7 +4953,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="13">
@@ -4911,7 +4964,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -4923,7 +4976,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="14">
@@ -4946,7 +4999,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="15">
@@ -4957,7 +5010,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -4969,7 +5022,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="16">
@@ -4992,7 +5045,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="17">
@@ -5015,7 +5068,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -5036,10 +5089,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -5047,35 +5100,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -5099,7 +5152,7 @@
         <v>150</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -5111,10 +5164,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -5144,7 +5197,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3">
@@ -5171,7 +5224,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4">
@@ -5198,7 +5251,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5">
@@ -5225,7 +5278,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6">
@@ -5252,7 +5305,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7">
@@ -5279,7 +5332,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8">
@@ -5306,7 +5359,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9">
@@ -5333,7 +5386,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10">
@@ -5360,7 +5413,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="11">
@@ -5387,7 +5440,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12">
@@ -5414,7 +5467,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13">
@@ -5441,12 +5494,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: venta 16.000 en la semana del 2/11 (dictado)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -520,7 +520,7 @@
     <t>el resto de la semana como la venta estacional</t>
   </si>
   <si>
-    <t>Gonzalo 16/10: lun 2/11 UAM cerrada (sin venta), el martes 3 vende 700 mas = estacional 17500 sin el lunes (23,9 %) + 700</t>
+    <t>Gonzalo 16/10: "la venta de la semana del feriado va a ser de 16 mil la semana toda" (lun 2/11 UAM cerrada)</t>
   </si>
   <si>
     <t>feriado Finados en Brasil el mismo lunes: frontera cerrada</t>
@@ -4341,13 +4341,13 @@
         <v>46328</v>
       </c>
       <c r="B9" s="0">
-        <v>7588</v>
+        <v>8672</v>
       </c>
       <c r="C9" s="0">
-        <v>5488</v>
+        <v>6272</v>
       </c>
       <c r="D9" s="0">
-        <v>924</v>
+        <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
         <v>164</v>

</xml_diff>

<commit_message>
plan de compras: venta dictada 20.000 / 21.000 / 16.000 para las semanas 19/10, 26/10 y 2/11
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="210">
   <si>
     <t>fecha</t>
   </si>
@@ -508,19 +508,16 @@
     <t>reparto con el mix real de las ultimas 10 semanas</t>
   </si>
   <si>
-    <t>Gonzalo 15/10: "la idea es semana que viene vender 20 o 21 mil cajas" = 20.500 (punto medio)</t>
+    <t>Gonzalo 16/10: "semana que viene se venden 20, la siguiente 21 mil, la del feriado 16 mil" = 20000</t>
   </si>
   <si>
     <t>reparto BR/PY/BO con el mix real de las ultimas 10 semanas; desde el mie 21 la pisa la estimacion con los dias reales</t>
   </si>
   <si>
-    <t>Gonzalo 16/10: lun 2/11 UAM cerrada, el sabado 31 vende 800 mas = estacional 17100 + 800</t>
+    <t xml:space="preserve">Gonzalo 16/10: "semana que viene se venden 20, la siguiente 21 mil, la del feriado 16 mil" = </t>
   </si>
   <si>
     <t>el resto de la semana como la venta estacional</t>
-  </si>
-  <si>
-    <t>Gonzalo 16/10: "la venta de la semana del feriado va a ser de 16 mil la semana toda" (lun 2/11 UAM cerrada)</t>
   </si>
   <si>
     <t>feriado Finados en Brasil el mismo lunes: frontera cerrada</t>
@@ -4301,13 +4298,13 @@
         <v>46314</v>
       </c>
       <c r="B7" s="0">
-        <v>11111</v>
+        <v>10840</v>
       </c>
       <c r="C7" s="0">
-        <v>8036</v>
+        <v>7840</v>
       </c>
       <c r="D7" s="0">
-        <v>1353</v>
+        <v>1320</v>
       </c>
       <c r="E7" s="0" t="s">
         <v>160</v>
@@ -4321,13 +4318,13 @@
         <v>46321</v>
       </c>
       <c r="B8" s="0">
-        <v>9702</v>
+        <v>0</v>
       </c>
       <c r="C8" s="0">
-        <v>7017</v>
+        <v>0</v>
       </c>
       <c r="D8" s="0">
-        <v>1181</v>
+        <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
         <v>162</v>
@@ -4341,19 +4338,19 @@
         <v>46328</v>
       </c>
       <c r="B9" s="0">
-        <v>8672</v>
+        <v>0</v>
       </c>
       <c r="C9" s="0">
-        <v>6272</v>
+        <v>0</v>
       </c>
       <c r="D9" s="0">
-        <v>1056</v>
+        <v>0</v>
       </c>
       <c r="E9" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="F9" s="0" t="s">
         <v>164</v>
-      </c>
-      <c r="F9" s="0" t="s">
-        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -4372,57 +4369,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -4470,10 +4467,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="E2" s="0" t="s">
         <v>177</v>
-      </c>
-      <c r="E2" s="0" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="3">
@@ -4487,10 +4484,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4">
@@ -4504,10 +4501,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5">
@@ -4515,16 +4512,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6">
@@ -4538,10 +4535,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
+        <v>182</v>
+      </c>
+      <c r="E6" s="0" t="s">
         <v>183</v>
-      </c>
-      <c r="E6" s="0" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="7">
@@ -4555,10 +4552,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8">
@@ -4572,10 +4569,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="9">
@@ -4583,16 +4580,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="10">
@@ -4606,10 +4603,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
+        <v>187</v>
+      </c>
+      <c r="E10" s="0" t="s">
         <v>188</v>
-      </c>
-      <c r="E10" s="0" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="11">
@@ -4623,10 +4620,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12">
@@ -4640,10 +4637,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13">
@@ -4651,16 +4648,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -4694,10 +4691,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>194</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -4723,7 +4720,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3">
@@ -4746,7 +4743,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4">
@@ -4769,7 +4766,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5">
@@ -4780,7 +4777,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -4792,7 +4789,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6">
@@ -4815,7 +4812,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7">
@@ -4838,7 +4835,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8">
@@ -4861,7 +4858,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9">
@@ -4872,7 +4869,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -4884,7 +4881,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="10">
@@ -4907,7 +4904,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="11">
@@ -4930,7 +4927,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12">
@@ -4953,7 +4950,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="13">
@@ -4964,7 +4961,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -4976,7 +4973,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="14">
@@ -4999,7 +4996,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="15">
@@ -5010,7 +5007,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -5022,7 +5019,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="16">
@@ -5045,7 +5042,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="17">
@@ -5068,7 +5065,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>
@@ -5089,10 +5086,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="B1" s="0" t="s">
         <v>199</v>
-      </c>
-      <c r="B1" s="0" t="s">
-        <v>200</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -5100,35 +5097,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -5152,7 +5149,7 @@
         <v>150</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -5164,10 +5161,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -5197,7 +5194,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3">
@@ -5224,7 +5221,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4">
@@ -5251,7 +5248,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5">
@@ -5278,7 +5275,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6">
@@ -5305,7 +5302,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7">
@@ -5332,7 +5329,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8">
@@ -5359,7 +5356,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9">
@@ -5386,7 +5383,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="10">
@@ -5413,7 +5410,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="11">
@@ -5440,7 +5437,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="12">
@@ -5467,7 +5464,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="13">
@@ -5494,12 +5491,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: venta 21.000 y 16.000 de las semanas 26/10 y 2/11 (habian quedado en 0)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="211">
   <si>
     <t>fecha</t>
   </si>
@@ -514,10 +514,13 @@
     <t>reparto BR/PY/BO con el mix real de las ultimas 10 semanas; desde el mie 21 la pisa la estimacion con los dias reales</t>
   </si>
   <si>
-    <t xml:space="preserve">Gonzalo 16/10: "semana que viene se venden 20, la siguiente 21 mil, la del feriado 16 mil" = </t>
+    <t>Gonzalo 16/10: "semana que viene se venden 20, la siguiente 21 mil, la del feriado 16 mil" = 21000</t>
   </si>
   <si>
     <t>el resto de la semana como la venta estacional</t>
+  </si>
+  <si>
+    <t>Gonzalo 16/10: "semana que viene se venden 20, la siguiente 21 mil, la del feriado 16 mil" = 16000</t>
   </si>
   <si>
     <t>feriado Finados en Brasil el mismo lunes: frontera cerrada</t>
@@ -4318,13 +4321,13 @@
         <v>46321</v>
       </c>
       <c r="B8" s="0">
-        <v>0</v>
+        <v>11382</v>
       </c>
       <c r="C8" s="0">
-        <v>0</v>
+        <v>8232</v>
       </c>
       <c r="D8" s="0">
-        <v>0</v>
+        <v>1386</v>
       </c>
       <c r="E8" s="0" t="s">
         <v>162</v>
@@ -4338,19 +4341,19 @@
         <v>46328</v>
       </c>
       <c r="B9" s="0">
-        <v>0</v>
+        <v>8672</v>
       </c>
       <c r="C9" s="0">
-        <v>0</v>
+        <v>6272</v>
       </c>
       <c r="D9" s="0">
-        <v>0</v>
+        <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -4369,57 +4372,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -4467,10 +4470,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3">
@@ -4484,10 +4487,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4">
@@ -4501,10 +4504,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5">
@@ -4512,16 +4515,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6">
@@ -4535,10 +4538,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7">
@@ -4552,10 +4555,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8">
@@ -4569,10 +4572,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9">
@@ -4580,16 +4583,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10">
@@ -4603,10 +4606,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11">
@@ -4620,10 +4623,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12">
@@ -4637,10 +4640,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="13">
@@ -4648,16 +4651,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -4691,10 +4694,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -4720,7 +4723,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3">
@@ -4743,7 +4746,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4">
@@ -4766,7 +4769,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5">
@@ -4777,7 +4780,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -4789,7 +4792,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6">
@@ -4812,7 +4815,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="7">
@@ -4835,7 +4838,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="8">
@@ -4858,7 +4861,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9">
@@ -4869,7 +4872,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -4881,7 +4884,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="10">
@@ -4904,7 +4907,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="11">
@@ -4927,7 +4930,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="12">
@@ -4950,7 +4953,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="13">
@@ -4961,7 +4964,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -4973,7 +4976,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="14">
@@ -4996,7 +4999,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="15">
@@ -5007,7 +5010,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -5019,7 +5022,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="16">
@@ -5042,7 +5045,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="17">
@@ -5065,7 +5068,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -5086,10 +5089,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -5097,35 +5100,35 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -5149,7 +5152,7 @@
         <v>150</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -5161,10 +5164,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -5194,7 +5197,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3">
@@ -5221,7 +5224,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4">
@@ -5248,7 +5251,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5">
@@ -5275,7 +5278,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6">
@@ -5302,7 +5305,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7">
@@ -5329,7 +5332,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8">
@@ -5356,7 +5359,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9">
@@ -5383,7 +5386,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10">
@@ -5410,7 +5413,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="11">
@@ -5437,7 +5440,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12">
@@ -5464,7 +5467,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13">
@@ -5491,12 +5494,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: piso de venta 18.000 por semana y semana 26/10 en 20.500
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="213">
   <si>
     <t>fecha</t>
   </si>
@@ -514,7 +514,7 @@
     <t>reparto BR/PY/BO con el mix real de las ultimas 10 semanas; desde el mie 21 la pisa la estimacion con los dias reales</t>
   </si>
   <si>
-    <t>Gonzalo 16/10: "semana que viene se venden 20, la siguiente 21 mil, la del feriado 16 mil" = 21000</t>
+    <t>Gonzalo 18/10: "las dos semanas de 20 y 20.5" = 20.500</t>
   </si>
   <si>
     <t>el resto de la semana como la venta estacional</t>
@@ -647,6 +647,12 @@
   </si>
   <si>
     <t>Gonzalo 14/10/2026: "Uruguay quiere cierre de los sabados a 27 mil" (antes 25.000 desde el 01/10; 22.500 antes)</t>
+  </si>
+  <si>
+    <t>venta_minima_semana</t>
+  </si>
+  <si>
+    <t>Gonzalo 18/10/2026: "18 mil es el promedio semanal minimo" (piso de la venta automatica; las semanas dictadas mandan)</t>
   </si>
   <si>
     <t>sabado</t>
@@ -4321,13 +4327,13 @@
         <v>46321</v>
       </c>
       <c r="B8" s="0">
-        <v>11382</v>
+        <v>11111</v>
       </c>
       <c r="C8" s="0">
-        <v>8232</v>
+        <v>8036</v>
       </c>
       <c r="D8" s="0">
-        <v>1386</v>
+        <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
         <v>162</v>
@@ -5079,7 +5085,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.85546875" customWidth="1"/>
@@ -5129,6 +5135,17 @@
       </c>
       <c r="C4" s="0" t="s">
         <v>206</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="B5" s="0">
+        <v>18000</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -5152,7 +5169,7 @@
         <v>150</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -5167,7 +5184,7 @@
         <v>181</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -5197,7 +5214,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="3">
@@ -5224,7 +5241,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4">
@@ -5251,7 +5268,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5">
@@ -5278,7 +5295,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6">
@@ -5305,7 +5322,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7">
@@ -5332,7 +5349,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8">
@@ -5359,7 +5376,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="9">
@@ -5386,7 +5403,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="10">
@@ -5413,7 +5430,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="11">
@@ -5440,7 +5457,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="12">
@@ -5467,7 +5484,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="13">
@@ -5494,12 +5511,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Celso mie 21 cancelado, lo cubre Ivo vie 23
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="214">
   <si>
     <t>fecha</t>
   </si>
@@ -439,9 +439,6 @@
     <t>definitivo 16/10: Jony 1: tersa</t>
   </si>
   <si>
-    <t>definitivo 16/10: Celso 1: cuarta</t>
-  </si>
-  <si>
     <t>definitivo 16/10: Ivo 1: tersa</t>
   </si>
   <si>
@@ -476,6 +473,12 @@
   </si>
   <si>
     <t>definitivo 16/10: Guido 1: lunes</t>
+  </si>
+  <si>
+    <t>Gonzalo 19/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 19/10: reemplaza la carga cancelada de Celso (Gonzalo 19/10)</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -705,7 +708,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -714,6 +717,7 @@
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3847,10 +3851,10 @@
     </row>
     <row r="88">
       <c r="A88" s="6">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C88" s="0" t="s">
         <v>115</v>
@@ -3859,7 +3863,7 @@
         <v>24</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="F88" s="0" t="s">
         <v>41</v>
@@ -3879,10 +3883,10 @@
     </row>
     <row r="89">
       <c r="A89" s="6">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B89" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C89" s="0" t="s">
         <v>115</v>
@@ -3891,7 +3895,7 @@
         <v>24</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>25</v>
+        <v>138</v>
       </c>
       <c r="F89" s="0" t="s">
         <v>41</v>
@@ -3906,7 +3910,7 @@
         <v>116</v>
       </c>
       <c r="J89" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="90">
@@ -3923,7 +3927,7 @@
         <v>24</v>
       </c>
       <c r="E90" s="0" t="s">
-        <v>139</v>
+        <v>40</v>
       </c>
       <c r="F90" s="0" t="s">
         <v>41</v>
@@ -3943,10 +3947,10 @@
     </row>
     <row r="91">
       <c r="A91" s="6">
-        <v>46316</v>
+        <v>46318</v>
       </c>
       <c r="B91" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C91" s="0" t="s">
         <v>115</v>
@@ -3975,10 +3979,10 @@
     </row>
     <row r="92">
       <c r="A92" s="6">
-        <v>46318</v>
+        <v>46315</v>
       </c>
       <c r="B92" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C92" s="0" t="s">
         <v>115</v>
@@ -3987,7 +3991,7 @@
         <v>24</v>
       </c>
       <c r="E92" s="0" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F92" s="0" t="s">
         <v>41</v>
@@ -4007,10 +4011,10 @@
     </row>
     <row r="93">
       <c r="A93" s="6">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B93" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C93" s="0" t="s">
         <v>115</v>
@@ -4019,7 +4023,7 @@
         <v>24</v>
       </c>
       <c r="E93" s="0" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F93" s="0" t="s">
         <v>41</v>
@@ -4039,10 +4043,10 @@
     </row>
     <row r="94">
       <c r="A94" s="6">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="B94" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C94" s="0" t="s">
         <v>115</v>
@@ -4051,7 +4055,7 @@
         <v>24</v>
       </c>
       <c r="E94" s="0" t="s">
-        <v>60</v>
+        <v>105</v>
       </c>
       <c r="F94" s="0" t="s">
         <v>41</v>
@@ -4071,10 +4075,10 @@
     </row>
     <row r="95">
       <c r="A95" s="6">
-        <v>46315</v>
+        <v>46318</v>
       </c>
       <c r="B95" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C95" s="0" t="s">
         <v>115</v>
@@ -4083,7 +4087,7 @@
         <v>24</v>
       </c>
       <c r="E95" s="0" t="s">
-        <v>105</v>
+        <v>145</v>
       </c>
       <c r="F95" s="0" t="s">
         <v>41</v>
@@ -4098,71 +4102,71 @@
         <v>116</v>
       </c>
       <c r="J95" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="6">
-        <v>46318</v>
+        <v>46314</v>
       </c>
       <c r="B96" s="0" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C96" s="0" t="s">
         <v>115</v>
       </c>
       <c r="D96" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E96" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F96" s="0" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G96" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H96" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I96" s="0" t="s">
         <v>116</v>
       </c>
       <c r="J96" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="6">
-        <v>46314</v>
+      <c r="A97" s="8">
+        <v>46318</v>
       </c>
       <c r="B97" s="0" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C97" s="0" t="s">
         <v>115</v>
       </c>
       <c r="D97" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E97" s="0" t="s">
-        <v>148</v>
+        <v>25</v>
       </c>
       <c r="F97" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G97" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H97" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I97" s="0" t="s">
-        <v>116</v>
+        <v>149</v>
       </c>
       <c r="J97" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -4184,7 +4188,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -4216,10 +4220,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3">
@@ -4236,10 +4240,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4">
@@ -4256,10 +4260,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5">
@@ -4276,10 +4280,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6">
@@ -4296,10 +4300,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7">
@@ -4316,10 +4320,10 @@
         <v>1320</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8">
@@ -4336,10 +4340,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9">
@@ -4356,10 +4360,10 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -4378,57 +4382,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -4476,10 +4480,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3">
@@ -4493,10 +4497,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4">
@@ -4510,10 +4514,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5">
@@ -4521,16 +4525,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6">
@@ -4544,10 +4548,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7">
@@ -4561,10 +4565,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8">
@@ -4578,10 +4582,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9">
@@ -4589,16 +4593,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="10">
@@ -4612,10 +4616,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="11">
@@ -4629,10 +4633,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="12">
@@ -4646,10 +4650,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="13">
@@ -4657,16 +4661,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -4700,10 +4704,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -4729,7 +4733,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3">
@@ -4752,7 +4756,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="4">
@@ -4775,7 +4779,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5">
@@ -4786,7 +4790,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -4798,7 +4802,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6">
@@ -4821,7 +4825,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7">
@@ -4844,7 +4848,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8">
@@ -4867,7 +4871,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9">
@@ -4878,7 +4882,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -4890,7 +4894,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10">
@@ -4913,7 +4917,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="11">
@@ -4936,7 +4940,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="12">
@@ -4959,7 +4963,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="13">
@@ -4970,7 +4974,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -4982,7 +4986,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="14">
@@ -5005,7 +5009,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="15">
@@ -5016,7 +5020,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -5028,7 +5032,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="16">
@@ -5051,7 +5055,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="17">
@@ -5074,7 +5078,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>
@@ -5095,10 +5099,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -5106,46 +5110,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -5166,10 +5170,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -5181,10 +5185,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -5214,7 +5218,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3">
@@ -5241,7 +5245,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4">
@@ -5268,7 +5272,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5">
@@ -5295,7 +5299,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6">
@@ -5322,7 +5326,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="7">
@@ -5349,7 +5353,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="8">
@@ -5376,7 +5380,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9">
@@ -5403,7 +5407,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="10">
@@ -5430,7 +5434,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="11">
@@ -5457,7 +5461,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="12">
@@ -5484,7 +5488,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="13">
@@ -5511,12 +5515,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: dictado de la semana de carga 26-31/10 (18 BR + 3 PY)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="237">
   <si>
     <t>fecha</t>
   </si>
@@ -479,6 +479,75 @@
   </si>
   <si>
     <t>dictado 19/10: reemplaza la carga cancelada de Celso (Gonzalo 19/10)</t>
+  </si>
+  <si>
+    <t>2026-10-25</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Fisher 2: tersa</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Fisher 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Casio 2: tersa</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Casio 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Stein 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Stein 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Miuller 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Miuller 2: sexta</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Agro 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Gilson 1: sexta</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Wagner 1: sexta</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Bahia 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Sergio 1: sabado</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Jony 1: tersa</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Ivo 1: sexta</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Josemar 1: sexta</t>
+  </si>
+  <si>
+    <t>Aryste Mittelman</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Aryste Mittelman 1: sexta (nuevo)</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Shapo 1: sexta</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Alvarito 1: lunes</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Milciades 1: martes</t>
+  </si>
+  <si>
+    <t>dictado 19/10: Guido 1: martes</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -708,7 +777,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -717,6 +786,7 @@
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1032,7 +1102,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K97"/>
+  <dimension ref="A1:K118"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -4167,6 +4237,678 @@
       </c>
       <c r="J97" s="0" t="s">
         <v>150</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="9">
+        <v>46322</v>
+      </c>
+      <c r="B98" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C98" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D98" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E98" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="F98" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="G98" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H98" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I98" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J98" s="0" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="9">
+        <v>46325</v>
+      </c>
+      <c r="B99" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C99" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D99" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E99" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="F99" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="G99" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H99" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I99" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J99" s="0" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="9">
+        <v>46322</v>
+      </c>
+      <c r="B100" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C100" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D100" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E100" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F100" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="G100" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="H100" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I100" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J100" s="0" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="9">
+        <v>46325</v>
+      </c>
+      <c r="B101" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C101" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D101" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E101" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F101" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G101" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H101" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I101" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J101" s="0" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="9">
+        <v>46323</v>
+      </c>
+      <c r="B102" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C102" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D102" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E102" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F102" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G102" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H102" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I102" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J102" s="0" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="9">
+        <v>46325</v>
+      </c>
+      <c r="B103" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C103" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D103" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E103" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F103" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G103" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H103" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I103" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J103" s="0" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="9">
+        <v>46323</v>
+      </c>
+      <c r="B104" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C104" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D104" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E104" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="F104" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G104" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H104" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I104" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J104" s="0" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="9">
+        <v>46325</v>
+      </c>
+      <c r="B105" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C105" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D105" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E105" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="F105" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G105" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H105" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I105" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J105" s="0" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="9">
+        <v>46323</v>
+      </c>
+      <c r="B106" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C106" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D106" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E106" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="F106" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G106" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H106" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I106" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J106" s="0" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="9">
+        <v>46325</v>
+      </c>
+      <c r="B107" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C107" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D107" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E107" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="F107" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G107" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H107" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I107" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J107" s="0" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="9">
+        <v>46325</v>
+      </c>
+      <c r="B108" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C108" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D108" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E108" s="0" t="s">
+        <v>145</v>
+      </c>
+      <c r="F108" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G108" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H108" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I108" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J108" s="0" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="9">
+        <v>46323</v>
+      </c>
+      <c r="B109" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C109" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D109" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E109" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="F109" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="G109" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H109" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I109" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J109" s="0" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="9">
+        <v>46326</v>
+      </c>
+      <c r="B110" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="C110" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D110" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E110" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="F110" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G110" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H110" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I110" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J110" s="0" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="9">
+        <v>46322</v>
+      </c>
+      <c r="B111" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C111" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D111" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E111" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="F111" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G111" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H111" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I111" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J111" s="0" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="9">
+        <v>46325</v>
+      </c>
+      <c r="B112" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C112" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D112" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E112" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F112" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G112" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H112" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I112" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J112" s="0" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="9">
+        <v>46325</v>
+      </c>
+      <c r="B113" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C113" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D113" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E113" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="F113" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G113" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H113" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I113" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J113" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="9">
+        <v>46325</v>
+      </c>
+      <c r="B114" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C114" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D114" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E114" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="F114" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G114" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H114" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I114" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J114" s="0" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="9">
+        <v>46325</v>
+      </c>
+      <c r="B115" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C115" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D115" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E115" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="F115" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G115" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H115" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I115" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J115" s="0" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="9">
+        <v>46321</v>
+      </c>
+      <c r="B116" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C116" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D116" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E116" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="F116" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G116" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H116" s="0">
+        <v>980</v>
+      </c>
+      <c r="I116" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J116" s="0" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="9">
+        <v>46322</v>
+      </c>
+      <c r="B117" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C117" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D117" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E117" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="F117" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G117" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H117" s="0">
+        <v>980</v>
+      </c>
+      <c r="I117" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J117" s="0" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="9">
+        <v>46322</v>
+      </c>
+      <c r="B118" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C118" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D118" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E118" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="F118" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G118" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H118" s="0">
+        <v>980</v>
+      </c>
+      <c r="I118" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="J118" s="0" t="s">
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -4188,7 +4930,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>151</v>
+        <v>174</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -4220,10 +4962,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>153</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3">
@@ -4240,10 +4982,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>154</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4">
@@ -4260,10 +5002,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>156</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5">
@@ -4280,10 +5022,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>157</v>
+        <v>180</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6">
@@ -4300,10 +5042,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>160</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7">
@@ -4320,10 +5062,10 @@
         <v>1320</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>161</v>
+        <v>184</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>162</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8">
@@ -4340,10 +5082,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9">
@@ -4360,10 +5102,10 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>165</v>
+        <v>188</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -4382,57 +5124,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>167</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>168</v>
+        <v>191</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>169</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>171</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>172</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>173</v>
+        <v>196</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>174</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>175</v>
+        <v>198</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>176</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>177</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -4480,10 +5222,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>178</v>
+        <v>201</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>179</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3">
@@ -4497,10 +5239,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>178</v>
+        <v>201</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>180</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4">
@@ -4514,10 +5256,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>178</v>
+        <v>201</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
     </row>
     <row r="5">
@@ -4525,16 +5267,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>182</v>
+        <v>205</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>178</v>
+        <v>201</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>183</v>
+        <v>206</v>
       </c>
     </row>
     <row r="6">
@@ -4548,10 +5290,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>184</v>
+        <v>207</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>185</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7">
@@ -4565,10 +5307,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>184</v>
+        <v>207</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>186</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8">
@@ -4582,10 +5324,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>184</v>
+        <v>207</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>187</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9">
@@ -4593,16 +5335,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>182</v>
+        <v>205</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>184</v>
+        <v>207</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>188</v>
+        <v>211</v>
       </c>
     </row>
     <row r="10">
@@ -4616,10 +5358,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>189</v>
+        <v>212</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>190</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11">
@@ -4633,10 +5375,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>189</v>
+        <v>212</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>191</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12">
@@ -4650,10 +5392,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>189</v>
+        <v>212</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>192</v>
+        <v>215</v>
       </c>
     </row>
     <row r="13">
@@ -4661,16 +5403,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>182</v>
+        <v>205</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>189</v>
+        <v>212</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>193</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -4704,10 +5446,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>194</v>
+        <v>217</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -4733,7 +5475,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>196</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3">
@@ -4756,7 +5498,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>196</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4">
@@ -4779,7 +5521,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>196</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5">
@@ -4790,7 +5532,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>182</v>
+        <v>205</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -4802,7 +5544,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>196</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6">
@@ -4825,7 +5567,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>197</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7">
@@ -4848,7 +5590,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>197</v>
+        <v>220</v>
       </c>
     </row>
     <row r="8">
@@ -4871,7 +5613,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>197</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9">
@@ -4882,7 +5624,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>182</v>
+        <v>205</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -4894,7 +5636,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>197</v>
+        <v>220</v>
       </c>
     </row>
     <row r="10">
@@ -4917,7 +5659,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>198</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11">
@@ -4940,7 +5682,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>198</v>
+        <v>221</v>
       </c>
     </row>
     <row r="12">
@@ -4963,7 +5705,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>198</v>
+        <v>221</v>
       </c>
     </row>
     <row r="13">
@@ -4974,7 +5716,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>182</v>
+        <v>205</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -4986,7 +5728,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>198</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14">
@@ -5009,7 +5751,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>199</v>
+        <v>222</v>
       </c>
     </row>
     <row r="15">
@@ -5020,7 +5762,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>182</v>
+        <v>205</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -5032,7 +5774,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>199</v>
+        <v>222</v>
       </c>
     </row>
     <row r="16">
@@ -5055,7 +5797,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>199</v>
+        <v>222</v>
       </c>
     </row>
     <row r="17">
@@ -5078,7 +5820,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>199</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -5099,10 +5841,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>200</v>
+        <v>223</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>201</v>
+        <v>224</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -5110,46 +5852,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>202</v>
+        <v>225</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>203</v>
+        <v>226</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>204</v>
+        <v>227</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>205</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>206</v>
+        <v>229</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>207</v>
+        <v>230</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>208</v>
+        <v>231</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>209</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -5170,10 +5912,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>151</v>
+        <v>174</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>210</v>
+        <v>233</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -5185,10 +5927,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>182</v>
+        <v>205</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>211</v>
+        <v>234</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -5218,7 +5960,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3">
@@ -5245,7 +5987,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4">
@@ -5272,7 +6014,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5">
@@ -5299,7 +6041,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6">
@@ -5326,7 +6068,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7">
@@ -5353,7 +6095,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
     </row>
     <row r="8">
@@ -5380,7 +6122,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9">
@@ -5407,7 +6149,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
     </row>
     <row r="10">
@@ -5434,7 +6176,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
     </row>
     <row r="11">
@@ -5461,7 +6203,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
     </row>
     <row r="12">
@@ -5488,7 +6230,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
     </row>
     <row r="13">
@@ -5515,12 +6257,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>213</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: semana 26-31/10 re-dictada con cargas adelantadas; venta 19.500 esta semana
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -484,70 +484,70 @@
     <t>2026-10-25</t>
   </si>
   <si>
-    <t>dictado 19/10: Fisher 2: tersa</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Fisher 2: sexta</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Casio 2: tersa</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Casio 2: sexta</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Stein 2: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Stein 2: sexta</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Miuller 2: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Miuller 2: sexta</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Agro 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Gilson 1: sexta</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Wagner 1: sexta</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Bahia 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Sergio 1: sabado</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Jony 1: tersa</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Ivo 1: sexta</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Josemar 1: sexta</t>
+    <t>Gonzalo 20/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Fisher 2: tersa</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Fisher 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Casio 2: tersa</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Casio 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Stein 2: tersa</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Stein 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Miuller 2: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Miuller 2: sabado</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Agro 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Gilson 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Wagner 1: sabado</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Bahia 1: cuarta</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Sergio 1: sabado</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Jony 1: tersa</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Ivo 1: sabado</t>
   </si>
   <si>
     <t>Aryste Mittelman</t>
   </si>
   <si>
-    <t>dictado 19/10: Aryste Mittelman 1: sexta (nuevo)</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Shapo 1: sexta</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Alvarito 1: lunes</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Milciades 1: martes</t>
-  </si>
-  <si>
-    <t>dictado 19/10: Guido 1: martes</t>
+    <t>dictado 20/10: Aryste Mittelman 1: sabado</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Shapo 1: sabado</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Alvarito 1: lunes</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Milciades 1: martes</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Guido 1: martes</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -580,7 +580,7 @@
     <t>reparto con el mix real de las ultimas 10 semanas</t>
   </si>
   <si>
-    <t>Gonzalo 16/10: "semana que viene se venden 20, la siguiente 21 mil, la del feriado 16 mil" = 20000</t>
+    <t>Gonzalo 20/10: "contando con una venta de 19500 esta semana"</t>
   </si>
   <si>
     <t>reparto BR/PY/BO con el mix real de las ultimas 10 semanas; desde el mie 21 la pisa la estimacion con los dias reales</t>
@@ -1102,7 +1102,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K118"/>
+  <dimension ref="A1:K117"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -4265,18 +4265,18 @@
         <v>1008</v>
       </c>
       <c r="I98" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J98" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="9">
-        <v>46325</v>
+        <v>46323</v>
       </c>
       <c r="B99" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C99" s="0" t="s">
         <v>151</v>
@@ -4297,10 +4297,10 @@
         <v>1008</v>
       </c>
       <c r="I99" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J99" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="100">
@@ -4329,18 +4329,18 @@
         <v>1008</v>
       </c>
       <c r="I100" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J100" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="9">
-        <v>46325</v>
+        <v>46323</v>
       </c>
       <c r="B101" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C101" s="0" t="s">
         <v>151</v>
@@ -4361,18 +4361,18 @@
         <v>1008</v>
       </c>
       <c r="I101" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J101" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="9">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="B102" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C102" s="0" t="s">
         <v>151</v>
@@ -4393,18 +4393,18 @@
         <v>1008</v>
       </c>
       <c r="I102" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J102" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="9">
-        <v>46325</v>
+        <v>46323</v>
       </c>
       <c r="B103" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C103" s="0" t="s">
         <v>151</v>
@@ -4425,10 +4425,10 @@
         <v>1008</v>
       </c>
       <c r="I103" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J103" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="104">
@@ -4457,18 +4457,18 @@
         <v>1008</v>
       </c>
       <c r="I104" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J104" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="9">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B105" s="0" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C105" s="0" t="s">
         <v>151</v>
@@ -4489,10 +4489,10 @@
         <v>1008</v>
       </c>
       <c r="I105" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J105" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="106">
@@ -4521,18 +4521,18 @@
         <v>1008</v>
       </c>
       <c r="I106" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J106" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="9">
-        <v>46325</v>
+        <v>46323</v>
       </c>
       <c r="B107" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C107" s="0" t="s">
         <v>151</v>
@@ -4553,18 +4553,18 @@
         <v>1008</v>
       </c>
       <c r="I107" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J107" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="9">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B108" s="0" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C108" s="0" t="s">
         <v>151</v>
@@ -4585,10 +4585,10 @@
         <v>1008</v>
       </c>
       <c r="I108" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J108" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="109">
@@ -4617,10 +4617,10 @@
         <v>1008</v>
       </c>
       <c r="I109" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J109" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="110">
@@ -4649,10 +4649,10 @@
         <v>1008</v>
       </c>
       <c r="I110" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J110" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="111">
@@ -4681,18 +4681,18 @@
         <v>1008</v>
       </c>
       <c r="I111" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J111" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="9">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B112" s="0" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C112" s="0" t="s">
         <v>151</v>
@@ -4713,18 +4713,18 @@
         <v>1008</v>
       </c>
       <c r="I112" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J112" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="9">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B113" s="0" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C113" s="0" t="s">
         <v>151</v>
@@ -4733,30 +4733,30 @@
         <v>24</v>
       </c>
       <c r="E113" s="0" t="s">
-        <v>58</v>
+        <v>168</v>
       </c>
       <c r="F113" s="0" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G113" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H113" s="0">
         <v>1008</v>
       </c>
       <c r="I113" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J113" s="0" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="9">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B114" s="0" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C114" s="0" t="s">
         <v>151</v>
@@ -4765,62 +4765,62 @@
         <v>24</v>
       </c>
       <c r="E114" s="0" t="s">
-        <v>168</v>
+        <v>105</v>
       </c>
       <c r="F114" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G114" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H114" s="0">
         <v>1008</v>
       </c>
       <c r="I114" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J114" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9">
-        <v>46325</v>
+        <v>46321</v>
       </c>
       <c r="B115" s="0" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C115" s="0" t="s">
         <v>151</v>
       </c>
       <c r="D115" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E115" s="0" t="s">
-        <v>105</v>
+        <v>22</v>
       </c>
       <c r="F115" s="0" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G115" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H115" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I115" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J115" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="9">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="B116" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C116" s="0" t="s">
         <v>151</v>
@@ -4829,7 +4829,7 @@
         <v>13</v>
       </c>
       <c r="E116" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F116" s="0" t="s">
         <v>15</v>
@@ -4841,10 +4841,10 @@
         <v>980</v>
       </c>
       <c r="I116" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J116" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="117">
@@ -4861,7 +4861,7 @@
         <v>13</v>
       </c>
       <c r="E117" s="0" t="s">
-        <v>20</v>
+        <v>147</v>
       </c>
       <c r="F117" s="0" t="s">
         <v>15</v>
@@ -4873,41 +4873,9 @@
         <v>980</v>
       </c>
       <c r="I117" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J117" s="0" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="9">
-        <v>46322</v>
-      </c>
-      <c r="B118" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="C118" s="0" t="s">
-        <v>151</v>
-      </c>
-      <c r="D118" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="E118" s="0" t="s">
-        <v>147</v>
-      </c>
-      <c r="F118" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G118" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H118" s="0">
-        <v>980</v>
-      </c>
-      <c r="I118" s="0" t="s">
-        <v>149</v>
-      </c>
-      <c r="J118" s="0" t="s">
         <v>173</v>
       </c>
     </row>
@@ -5053,13 +5021,13 @@
         <v>46314</v>
       </c>
       <c r="B7" s="0">
-        <v>10840</v>
+        <v>10569</v>
       </c>
       <c r="C7" s="0">
-        <v>7840</v>
+        <v>7644</v>
       </c>
       <c r="D7" s="0">
-        <v>1320</v>
+        <v>1287</v>
       </c>
       <c r="E7" s="0" t="s">
         <v>184</v>

</xml_diff>

<commit_message>
plan de compras: dictado de las semanas 26-31/10 y 2-7/11
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="252">
   <si>
     <t>fecha</t>
   </si>
@@ -487,67 +487,112 @@
     <t>Gonzalo 20/10 (chat)</t>
   </si>
   <si>
-    <t>dictado 20/10: Fisher 2: tersa</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Fisher 2: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Casio 2: tersa</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Casio 2: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Stein 2: tersa</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Stein 2: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Miuller 2: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Miuller 2: sabado</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Agro 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Gilson 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Wagner 1: sabado</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Bahia 1: cuarta</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Sergio 1: sabado</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Jony 1: tersa</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Ivo 1: sabado</t>
+    <t>dictado 20/10: Fisher 2026-10-27</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Cassio 2026-10-27</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Stein 2026-10-27</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Muller Fabricio 2026-10-28</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Agrocurupa 2026-10-28</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Gilson 2026-10-28</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Wagner 2026-10-31</t>
+  </si>
+  <si>
+    <t>dictado 20/10: BAHIA 2026-10-28</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Jhony Viera 2026-10-27</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Ivo zimer 2026-10-28</t>
   </si>
   <si>
     <t>Aryste Mittelman</t>
   </si>
   <si>
-    <t>dictado 20/10: Aryste Mittelman 1: sabado</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Shapo 1: sabado</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Alvarito 1: lunes</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Milciades 1: martes</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Guido 1: martes</t>
+    <t>dictado 20/10: Aryste Mittelman 2026-10-28</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Shapo 2026-10-27</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Paraguay AS 2026-10-26</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Paraguay MS 2026-10-27</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Paraguay GM 2026-10-27</t>
+  </si>
+  <si>
+    <t>2026-11-01</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Fisher 2026-11-03</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Fisher 2026-11-04</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Fisher 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Cassio 2026-11-03</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Cassio 2026-11-04</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Cassio 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Gilson 2026-11-03</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Gilson 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Stein 2026-11-03</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Stein 2026-11-04</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Stein 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Agrocurupa 2026-11-04</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Agrocurupa 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Muller Fabricio 2026-11-03</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Muller Fabricio 2026-11-04</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Muller Fabricio 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Paraguay GM 2026-11-02</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Paraguay AS 2026-11-03</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Paraguay MS 2026-11-02</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -1102,7 +1147,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K117"/>
+  <dimension ref="A1:K131"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -4273,10 +4318,10 @@
     </row>
     <row r="99">
       <c r="A99" s="9">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="B99" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C99" s="0" t="s">
         <v>151</v>
@@ -4285,13 +4330,13 @@
         <v>24</v>
       </c>
       <c r="E99" s="0" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F99" s="0" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="G99" s="0" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H99" s="0">
         <v>1008</v>
@@ -4317,13 +4362,13 @@
         <v>24</v>
       </c>
       <c r="E100" s="0" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="F100" s="0" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="G100" s="0" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="H100" s="0">
         <v>1008</v>
@@ -4349,13 +4394,13 @@
         <v>24</v>
       </c>
       <c r="E101" s="0" t="s">
-        <v>27</v>
+        <v>121</v>
       </c>
       <c r="F101" s="0" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G101" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H101" s="0">
         <v>1008</v>
@@ -4369,10 +4414,10 @@
     </row>
     <row r="102">
       <c r="A102" s="9">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B102" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C102" s="0" t="s">
         <v>151</v>
@@ -4381,13 +4426,13 @@
         <v>24</v>
       </c>
       <c r="E102" s="0" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="F102" s="0" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="G102" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H102" s="0">
         <v>1008</v>
@@ -4413,13 +4458,13 @@
         <v>24</v>
       </c>
       <c r="E103" s="0" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="F103" s="0" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="G103" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H103" s="0">
         <v>1008</v>
@@ -4433,10 +4478,10 @@
     </row>
     <row r="104">
       <c r="A104" s="9">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="B104" s="0" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C104" s="0" t="s">
         <v>151</v>
@@ -4445,13 +4490,13 @@
         <v>24</v>
       </c>
       <c r="E104" s="0" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="F104" s="0" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="G104" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H104" s="0">
         <v>1008</v>
@@ -4465,10 +4510,10 @@
     </row>
     <row r="105">
       <c r="A105" s="9">
-        <v>46326</v>
+        <v>46323</v>
       </c>
       <c r="B105" s="0" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="C105" s="0" t="s">
         <v>151</v>
@@ -4477,10 +4522,10 @@
         <v>24</v>
       </c>
       <c r="E105" s="0" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="F105" s="0" t="s">
-        <v>56</v>
+        <v>129</v>
       </c>
       <c r="G105" s="0" t="s">
         <v>15</v>
@@ -4497,10 +4542,10 @@
     </row>
     <row r="106">
       <c r="A106" s="9">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="B106" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C106" s="0" t="s">
         <v>151</v>
@@ -4509,7 +4554,7 @@
         <v>24</v>
       </c>
       <c r="E106" s="0" t="s">
-        <v>40</v>
+        <v>112</v>
       </c>
       <c r="F106" s="0" t="s">
         <v>41</v>
@@ -4541,7 +4586,7 @@
         <v>24</v>
       </c>
       <c r="E107" s="0" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="F107" s="0" t="s">
         <v>41</v>
@@ -4561,10 +4606,10 @@
     </row>
     <row r="108">
       <c r="A108" s="9">
-        <v>46326</v>
+        <v>46323</v>
       </c>
       <c r="B108" s="0" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="C108" s="0" t="s">
         <v>151</v>
@@ -4573,13 +4618,13 @@
         <v>24</v>
       </c>
       <c r="E108" s="0" t="s">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="F108" s="0" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G108" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H108" s="0">
         <v>1008</v>
@@ -4588,15 +4633,15 @@
         <v>152</v>
       </c>
       <c r="J108" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="9">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="B109" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C109" s="0" t="s">
         <v>151</v>
@@ -4605,13 +4650,13 @@
         <v>24</v>
       </c>
       <c r="E109" s="0" t="s">
-        <v>128</v>
+        <v>105</v>
       </c>
       <c r="F109" s="0" t="s">
-        <v>129</v>
+        <v>41</v>
       </c>
       <c r="G109" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H109" s="0">
         <v>1008</v>
@@ -4620,39 +4665,39 @@
         <v>152</v>
       </c>
       <c r="J109" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="9">
-        <v>46326</v>
+        <v>46321</v>
       </c>
       <c r="B110" s="0" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="C110" s="0" t="s">
         <v>151</v>
       </c>
       <c r="D110" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E110" s="0" t="s">
-        <v>131</v>
+        <v>22</v>
       </c>
       <c r="F110" s="0" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G110" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H110" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I110" s="0" t="s">
         <v>152</v>
       </c>
       <c r="J110" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="111">
@@ -4666,80 +4711,80 @@
         <v>151</v>
       </c>
       <c r="D111" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E111" s="0" t="s">
-        <v>112</v>
+        <v>20</v>
       </c>
       <c r="F111" s="0" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G111" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H111" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I111" s="0" t="s">
         <v>152</v>
       </c>
       <c r="J111" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="9">
-        <v>46326</v>
+        <v>46322</v>
       </c>
       <c r="B112" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C112" s="0" t="s">
         <v>151</v>
       </c>
       <c r="D112" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E112" s="0" t="s">
-        <v>25</v>
+        <v>147</v>
       </c>
       <c r="F112" s="0" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G112" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H112" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I112" s="0" t="s">
         <v>152</v>
       </c>
       <c r="J112" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="9">
-        <v>46326</v>
+        <v>46329</v>
       </c>
       <c r="B113" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C113" s="0" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="D113" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E113" s="0" t="s">
-        <v>168</v>
+        <v>31</v>
       </c>
       <c r="F113" s="0" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="G113" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H113" s="0">
         <v>1008</v>
@@ -4748,27 +4793,27 @@
         <v>152</v>
       </c>
       <c r="J113" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="9">
-        <v>46326</v>
+        <v>46330</v>
       </c>
       <c r="B114" s="0" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="C114" s="0" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="D114" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E114" s="0" t="s">
-        <v>105</v>
+        <v>31</v>
       </c>
       <c r="F114" s="0" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="G114" s="0" t="s">
         <v>35</v>
@@ -4780,103 +4825,551 @@
         <v>152</v>
       </c>
       <c r="J114" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9">
-        <v>46321</v>
+        <v>46332</v>
       </c>
       <c r="B115" s="0" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C115" s="0" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="D115" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E115" s="0" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F115" s="0" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="G115" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H115" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I115" s="0" t="s">
         <v>152</v>
       </c>
       <c r="J115" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="9">
-        <v>46322</v>
+        <v>46329</v>
       </c>
       <c r="B116" s="0" t="s">
         <v>21</v>
       </c>
       <c r="C116" s="0" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="D116" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E116" s="0" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F116" s="0" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G116" s="0" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="H116" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I116" s="0" t="s">
         <v>152</v>
       </c>
       <c r="J116" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="9">
-        <v>46322</v>
+        <v>46330</v>
       </c>
       <c r="B117" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C117" s="0" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="D117" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E117" s="0" t="s">
-        <v>147</v>
+        <v>27</v>
       </c>
       <c r="F117" s="0" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G117" s="0" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="H117" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I117" s="0" t="s">
         <v>152</v>
       </c>
       <c r="J117" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="9">
+        <v>46332</v>
+      </c>
+      <c r="B118" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C118" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D118" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E118" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F118" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="G118" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="H118" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I118" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J118" s="0" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="9">
+        <v>46329</v>
+      </c>
+      <c r="B119" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C119" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D119" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E119" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="F119" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G119" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H119" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I119" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J119" s="0" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="9">
+        <v>46332</v>
+      </c>
+      <c r="B120" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C120" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D120" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E120" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="F120" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G120" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H120" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I120" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J120" s="0" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="9">
+        <v>46329</v>
+      </c>
+      <c r="B121" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C121" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D121" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E121" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F121" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G121" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H121" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I121" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J121" s="0" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="9">
+        <v>46330</v>
+      </c>
+      <c r="B122" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C122" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D122" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E122" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F122" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G122" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H122" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I122" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J122" s="0" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="9">
+        <v>46332</v>
+      </c>
+      <c r="B123" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C123" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D123" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E123" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F123" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G123" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H123" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I123" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J123" s="0" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="9">
+        <v>46330</v>
+      </c>
+      <c r="B124" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C124" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D124" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E124" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="F124" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G124" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H124" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I124" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J124" s="0" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="9">
+        <v>46332</v>
+      </c>
+      <c r="B125" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C125" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D125" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E125" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="F125" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G125" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H125" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I125" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J125" s="0" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="9">
+        <v>46329</v>
+      </c>
+      <c r="B126" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C126" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D126" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E126" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="F126" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G126" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H126" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I126" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J126" s="0" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="9">
+        <v>46330</v>
+      </c>
+      <c r="B127" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C127" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D127" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E127" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="F127" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G127" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H127" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I127" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J127" s="0" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="9">
+        <v>46332</v>
+      </c>
+      <c r="B128" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C128" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D128" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E128" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="F128" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G128" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H128" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I128" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J128" s="0" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="9">
+        <v>46328</v>
+      </c>
+      <c r="B129" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C129" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D129" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E129" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="F129" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G129" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H129" s="0">
+        <v>980</v>
+      </c>
+      <c r="I129" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J129" s="0" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="9">
+        <v>46329</v>
+      </c>
+      <c r="B130" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C130" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D130" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E130" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="F130" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G130" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H130" s="0">
+        <v>980</v>
+      </c>
+      <c r="I130" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J130" s="0" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="9">
+        <v>46328</v>
+      </c>
+      <c r="B131" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C131" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D131" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E131" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="F131" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G131" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H131" s="0">
+        <v>980</v>
+      </c>
+      <c r="I131" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J131" s="0" t="s">
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -4898,7 +5391,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -4930,10 +5423,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
     </row>
     <row r="3">
@@ -4950,10 +5443,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4">
@@ -4970,10 +5463,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5">
@@ -4990,10 +5483,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6">
@@ -5010,10 +5503,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7">
@@ -5030,10 +5523,10 @@
         <v>1287</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>185</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8">
@@ -5050,10 +5543,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
     </row>
     <row r="9">
@@ -5070,10 +5563,10 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -5092,57 +5585,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>197</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -5190,10 +5683,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>202</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3">
@@ -5207,10 +5700,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4">
@@ -5224,10 +5717,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>204</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5">
@@ -5235,16 +5728,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6">
@@ -5258,10 +5751,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>208</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7">
@@ -5275,10 +5768,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>209</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8">
@@ -5292,10 +5785,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>210</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9">
@@ -5303,16 +5796,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>211</v>
+        <v>226</v>
       </c>
     </row>
     <row r="10">
@@ -5326,10 +5819,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>213</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11">
@@ -5343,10 +5836,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>214</v>
+        <v>229</v>
       </c>
     </row>
     <row r="12">
@@ -5360,10 +5853,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>215</v>
+        <v>230</v>
       </c>
     </row>
     <row r="13">
@@ -5371,16 +5864,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>216</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -5414,10 +5907,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>217</v>
+        <v>232</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>218</v>
+        <v>233</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -5443,7 +5936,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>219</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3">
@@ -5466,7 +5959,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>219</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4">
@@ -5489,7 +5982,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>219</v>
+        <v>234</v>
       </c>
     </row>
     <row r="5">
@@ -5500,7 +5993,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -5512,7 +6005,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>219</v>
+        <v>234</v>
       </c>
     </row>
     <row r="6">
@@ -5535,7 +6028,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>220</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7">
@@ -5558,7 +6051,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>220</v>
+        <v>235</v>
       </c>
     </row>
     <row r="8">
@@ -5581,7 +6074,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>220</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9">
@@ -5592,7 +6085,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -5604,7 +6097,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>220</v>
+        <v>235</v>
       </c>
     </row>
     <row r="10">
@@ -5627,7 +6120,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>221</v>
+        <v>236</v>
       </c>
     </row>
     <row r="11">
@@ -5650,7 +6143,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>221</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12">
@@ -5673,7 +6166,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>221</v>
+        <v>236</v>
       </c>
     </row>
     <row r="13">
@@ -5684,7 +6177,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -5696,7 +6189,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>221</v>
+        <v>236</v>
       </c>
     </row>
     <row r="14">
@@ -5719,7 +6212,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
     </row>
     <row r="15">
@@ -5730,7 +6223,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -5742,7 +6235,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
     </row>
     <row r="16">
@@ -5765,7 +6258,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
     </row>
     <row r="17">
@@ -5788,7 +6281,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -5809,10 +6302,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>223</v>
+        <v>238</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -5820,46 +6313,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>226</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>227</v>
+        <v>242</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>228</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>229</v>
+        <v>244</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>230</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>231</v>
+        <v>246</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>232</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -5880,10 +6373,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -5895,10 +6388,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -5928,7 +6421,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3">
@@ -5955,7 +6448,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4">
@@ -5982,7 +6475,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5">
@@ -6009,7 +6502,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6">
@@ -6036,7 +6529,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7">
@@ -6063,7 +6556,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8">
@@ -6090,7 +6583,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9">
@@ -6117,7 +6610,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10">
@@ -6144,7 +6637,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11">
@@ -6171,7 +6664,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12">
@@ -6198,7 +6691,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13">
@@ -6225,12 +6718,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: semana 26-31/10 con Wagner martes, Jaime Zimerman y Andre Pauli
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="255">
   <si>
     <t>fecha</t>
   </si>
@@ -505,7 +505,16 @@
     <t>dictado 20/10: Gilson 2026-10-28</t>
   </si>
   <si>
-    <t>dictado 20/10: Wagner 2026-10-31</t>
+    <t>dictado 20/10: Wagner 2026-10-27</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Jaime Zimerman 2026-10-28</t>
+  </si>
+  <si>
+    <t>Andre Pauli</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Andre Pauli 2026-10-27</t>
   </si>
   <si>
     <t>dictado 20/10: BAHIA 2026-10-28</t>
@@ -1147,7 +1156,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K131"/>
+  <dimension ref="A1:K133"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -4478,10 +4487,10 @@
     </row>
     <row r="104">
       <c r="A104" s="9">
-        <v>46326</v>
+        <v>46322</v>
       </c>
       <c r="B104" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C104" s="0" t="s">
         <v>151</v>
@@ -4522,13 +4531,13 @@
         <v>24</v>
       </c>
       <c r="E105" s="0" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="F105" s="0" t="s">
-        <v>129</v>
+        <v>41</v>
       </c>
       <c r="G105" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H105" s="0">
         <v>1008</v>
@@ -4554,13 +4563,13 @@
         <v>24</v>
       </c>
       <c r="E106" s="0" t="s">
-        <v>112</v>
+        <v>161</v>
       </c>
       <c r="F106" s="0" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G106" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H106" s="0">
         <v>1008</v>
@@ -4569,7 +4578,7 @@
         <v>152</v>
       </c>
       <c r="J106" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="107">
@@ -4586,13 +4595,13 @@
         <v>24</v>
       </c>
       <c r="E107" s="0" t="s">
-        <v>25</v>
+        <v>128</v>
       </c>
       <c r="F107" s="0" t="s">
-        <v>41</v>
+        <v>129</v>
       </c>
       <c r="G107" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H107" s="0">
         <v>1008</v>
@@ -4601,15 +4610,15 @@
         <v>152</v>
       </c>
       <c r="J107" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="9">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="B108" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C108" s="0" t="s">
         <v>151</v>
@@ -4618,13 +4627,13 @@
         <v>24</v>
       </c>
       <c r="E108" s="0" t="s">
-        <v>163</v>
+        <v>112</v>
       </c>
       <c r="F108" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G108" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H108" s="0">
         <v>1008</v>
@@ -4638,10 +4647,10 @@
     </row>
     <row r="109">
       <c r="A109" s="9">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B109" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C109" s="0" t="s">
         <v>151</v>
@@ -4650,7 +4659,7 @@
         <v>24</v>
       </c>
       <c r="E109" s="0" t="s">
-        <v>105</v>
+        <v>25</v>
       </c>
       <c r="F109" s="0" t="s">
         <v>41</v>
@@ -4670,19 +4679,19 @@
     </row>
     <row r="110">
       <c r="A110" s="9">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="B110" s="0" t="s">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="C110" s="0" t="s">
         <v>151</v>
       </c>
       <c r="D110" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E110" s="0" t="s">
-        <v>22</v>
+        <v>166</v>
       </c>
       <c r="F110" s="0" t="s">
         <v>15</v>
@@ -4691,13 +4700,13 @@
         <v>15</v>
       </c>
       <c r="H110" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I110" s="0" t="s">
         <v>152</v>
       </c>
       <c r="J110" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="111">
@@ -4711,33 +4720,33 @@
         <v>151</v>
       </c>
       <c r="D111" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E111" s="0" t="s">
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="F111" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G111" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H111" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I111" s="0" t="s">
         <v>152</v>
       </c>
       <c r="J111" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="9">
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="B112" s="0" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C112" s="0" t="s">
         <v>151</v>
@@ -4746,7 +4755,7 @@
         <v>13</v>
       </c>
       <c r="E112" s="0" t="s">
-        <v>147</v>
+        <v>22</v>
       </c>
       <c r="F112" s="0" t="s">
         <v>15</v>
@@ -4761,33 +4770,33 @@
         <v>152</v>
       </c>
       <c r="J112" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="9">
-        <v>46329</v>
+        <v>46322</v>
       </c>
       <c r="B113" s="0" t="s">
         <v>21</v>
       </c>
       <c r="C113" s="0" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="D113" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E113" s="0" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="F113" s="0" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="G113" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H113" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I113" s="0" t="s">
         <v>152</v>
@@ -4798,28 +4807,28 @@
     </row>
     <row r="114">
       <c r="A114" s="9">
-        <v>46330</v>
+        <v>46322</v>
       </c>
       <c r="B114" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C114" s="0" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="D114" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E114" s="0" t="s">
-        <v>31</v>
+        <v>147</v>
       </c>
       <c r="F114" s="0" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="G114" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H114" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I114" s="0" t="s">
         <v>152</v>
@@ -4830,13 +4839,13 @@
     </row>
     <row r="115">
       <c r="A115" s="9">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B115" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C115" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D115" s="0" t="s">
         <v>24</v>
@@ -4857,30 +4866,30 @@
         <v>152</v>
       </c>
       <c r="J115" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="9">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="B116" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C116" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D116" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E116" s="0" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F116" s="0" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="G116" s="0" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H116" s="0">
         <v>1008</v>
@@ -4889,30 +4898,30 @@
         <v>152</v>
       </c>
       <c r="J116" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="9">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B117" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C117" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D117" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E117" s="0" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F117" s="0" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="G117" s="0" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H117" s="0">
         <v>1008</v>
@@ -4921,18 +4930,18 @@
         <v>152</v>
       </c>
       <c r="J117" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="9">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B118" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C118" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D118" s="0" t="s">
         <v>24</v>
@@ -4953,30 +4962,30 @@
         <v>152</v>
       </c>
       <c r="J118" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="9">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="B119" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C119" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D119" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E119" s="0" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="F119" s="0" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G119" s="0" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H119" s="0">
         <v>1008</v>
@@ -4985,7 +4994,7 @@
         <v>152</v>
       </c>
       <c r="J119" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="120">
@@ -4996,19 +5005,19 @@
         <v>23</v>
       </c>
       <c r="C120" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D120" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E120" s="0" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="F120" s="0" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G120" s="0" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H120" s="0">
         <v>1008</v>
@@ -5017,7 +5026,7 @@
         <v>152</v>
       </c>
       <c r="J120" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="121">
@@ -5028,19 +5037,19 @@
         <v>21</v>
       </c>
       <c r="C121" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D121" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E121" s="0" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="F121" s="0" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="G121" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H121" s="0">
         <v>1008</v>
@@ -5049,30 +5058,30 @@
         <v>152</v>
       </c>
       <c r="J121" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="9">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B122" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C122" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D122" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E122" s="0" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="F122" s="0" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="G122" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H122" s="0">
         <v>1008</v>
@@ -5081,18 +5090,18 @@
         <v>152</v>
       </c>
       <c r="J122" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="9">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B123" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C123" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D123" s="0" t="s">
         <v>24</v>
@@ -5113,7 +5122,7 @@
         <v>152</v>
       </c>
       <c r="J123" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="124">
@@ -5124,19 +5133,19 @@
         <v>52</v>
       </c>
       <c r="C124" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D124" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E124" s="0" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="F124" s="0" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G124" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H124" s="0">
         <v>1008</v>
@@ -5145,7 +5154,7 @@
         <v>152</v>
       </c>
       <c r="J124" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="125">
@@ -5156,19 +5165,19 @@
         <v>23</v>
       </c>
       <c r="C125" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D125" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E125" s="0" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="F125" s="0" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G125" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H125" s="0">
         <v>1008</v>
@@ -5177,30 +5186,30 @@
         <v>152</v>
       </c>
       <c r="J125" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="9">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="B126" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C126" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D126" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E126" s="0" t="s">
-        <v>121</v>
+        <v>40</v>
       </c>
       <c r="F126" s="0" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="G126" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H126" s="0">
         <v>1008</v>
@@ -5209,30 +5218,30 @@
         <v>152</v>
       </c>
       <c r="J126" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="9">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B127" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C127" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D127" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E127" s="0" t="s">
-        <v>121</v>
+        <v>40</v>
       </c>
       <c r="F127" s="0" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="G127" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H127" s="0">
         <v>1008</v>
@@ -5241,18 +5250,18 @@
         <v>152</v>
       </c>
       <c r="J127" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="9">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B128" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C128" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D128" s="0" t="s">
         <v>24</v>
@@ -5273,71 +5282,71 @@
         <v>152</v>
       </c>
       <c r="J128" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="9">
-        <v>46328</v>
+        <v>46330</v>
       </c>
       <c r="B129" s="0" t="s">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="C129" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D129" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E129" s="0" t="s">
-        <v>147</v>
+        <v>121</v>
       </c>
       <c r="F129" s="0" t="s">
-        <v>15</v>
+        <v>56</v>
       </c>
       <c r="G129" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H129" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I129" s="0" t="s">
         <v>152</v>
       </c>
       <c r="J129" s="0" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="9">
-        <v>46329</v>
+        <v>46332</v>
       </c>
       <c r="B130" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C130" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D130" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E130" s="0" t="s">
-        <v>22</v>
+        <v>121</v>
       </c>
       <c r="F130" s="0" t="s">
-        <v>15</v>
+        <v>56</v>
       </c>
       <c r="G130" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H130" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I130" s="0" t="s">
         <v>152</v>
       </c>
       <c r="J130" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="131">
@@ -5348,13 +5357,13 @@
         <v>19</v>
       </c>
       <c r="C131" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D131" s="0" t="s">
         <v>13</v>
       </c>
       <c r="E131" s="0" t="s">
-        <v>20</v>
+        <v>147</v>
       </c>
       <c r="F131" s="0" t="s">
         <v>15</v>
@@ -5369,7 +5378,71 @@
         <v>152</v>
       </c>
       <c r="J131" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="9">
+        <v>46329</v>
+      </c>
+      <c r="B132" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C132" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="D132" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E132" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="F132" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G132" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H132" s="0">
+        <v>980</v>
+      </c>
+      <c r="I132" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J132" s="0" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="9">
+        <v>46328</v>
+      </c>
+      <c r="B133" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C133" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="D133" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E133" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="F133" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G133" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H133" s="0">
+        <v>980</v>
+      </c>
+      <c r="I133" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J133" s="0" t="s">
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -5391,7 +5464,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5423,10 +5496,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3">
@@ -5443,10 +5516,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4">
@@ -5463,10 +5536,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5">
@@ -5483,10 +5556,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6">
@@ -5503,10 +5576,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7">
@@ -5523,10 +5596,10 @@
         <v>1287</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="8">
@@ -5543,10 +5616,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9">
@@ -5563,10 +5636,10 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -5585,57 +5658,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -5683,10 +5756,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3">
@@ -5700,10 +5773,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4">
@@ -5717,10 +5790,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5">
@@ -5728,16 +5801,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6">
@@ -5751,10 +5824,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7">
@@ -5768,10 +5841,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="8">
@@ -5785,10 +5858,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9">
@@ -5796,16 +5869,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="10">
@@ -5819,10 +5892,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11">
@@ -5836,10 +5909,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="12">
@@ -5853,10 +5926,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="13">
@@ -5864,16 +5937,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -5907,10 +5980,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -5936,7 +6009,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="3">
@@ -5959,7 +6032,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4">
@@ -5982,7 +6055,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5">
@@ -5993,7 +6066,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6005,7 +6078,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6">
@@ -6028,7 +6101,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7">
@@ -6051,7 +6124,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8">
@@ -6074,7 +6147,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9">
@@ -6085,7 +6158,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6097,7 +6170,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="10">
@@ -6120,7 +6193,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="11">
@@ -6143,7 +6216,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="12">
@@ -6166,7 +6239,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="13">
@@ -6177,7 +6250,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6189,7 +6262,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="14">
@@ -6212,7 +6285,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="15">
@@ -6223,7 +6296,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6235,7 +6308,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="16">
@@ -6258,7 +6331,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="17">
@@ -6281,7 +6354,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -6302,10 +6375,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6313,46 +6386,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -6373,10 +6446,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6388,10 +6461,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6421,7 +6494,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="3">
@@ -6448,7 +6521,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4">
@@ -6475,7 +6548,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5">
@@ -6502,7 +6575,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6">
@@ -6529,7 +6602,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="7">
@@ -6556,7 +6629,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8">
@@ -6583,7 +6656,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="9">
@@ -6610,7 +6683,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="10">
@@ -6637,7 +6710,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="11">
@@ -6664,7 +6737,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12">
@@ -6691,7 +6764,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="13">
@@ -6718,12 +6791,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: venta 21.000 en las semanas 9/11 y 16/11
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="256">
   <si>
     <t>fecha</t>
   </si>
@@ -650,6 +650,9 @@
   </si>
   <si>
     <t>feriado Finados en Brasil el mismo lunes: frontera cerrada</t>
+  </si>
+  <si>
+    <t>Gonzalo 20/10: "9 al 14 21 mil, 16 al 21 21 mil"</t>
   </si>
   <si>
     <t>notas</t>
@@ -831,7 +834,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -842,6 +845,7 @@
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5453,7 +5457,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.28515625" customWidth="1"/>
@@ -5640,6 +5644,40 @@
       </c>
       <c r="F9" s="0" t="s">
         <v>207</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10">
+        <v>46335</v>
+      </c>
+      <c r="B10" s="0">
+        <v>11382</v>
+      </c>
+      <c r="C10" s="0">
+        <v>8232</v>
+      </c>
+      <c r="D10" s="0">
+        <v>1386</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10">
+        <v>46342</v>
+      </c>
+      <c r="B11" s="0">
+        <v>11382</v>
+      </c>
+      <c r="C11" s="0">
+        <v>8232</v>
+      </c>
+      <c r="D11" s="0">
+        <v>1386</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -5658,57 +5696,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -5756,10 +5794,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="3">
@@ -5773,10 +5811,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4">
@@ -5790,10 +5828,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5">
@@ -5801,16 +5839,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6">
@@ -5824,10 +5862,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="7">
@@ -5841,10 +5879,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8">
@@ -5858,10 +5896,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9">
@@ -5869,16 +5907,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="10">
@@ -5892,10 +5930,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="11">
@@ -5909,10 +5947,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="12">
@@ -5926,10 +5964,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="13">
@@ -5937,16 +5975,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -5980,10 +6018,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6009,7 +6047,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3">
@@ -6032,7 +6070,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4">
@@ -6055,7 +6093,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5">
@@ -6066,7 +6104,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6078,7 +6116,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6">
@@ -6101,7 +6139,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="7">
@@ -6124,7 +6162,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="8">
@@ -6147,7 +6185,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9">
@@ -6158,7 +6196,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6170,7 +6208,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10">
@@ -6193,7 +6231,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11">
@@ -6216,7 +6254,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="12">
@@ -6239,7 +6277,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="13">
@@ -6250,7 +6288,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6262,7 +6300,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14">
@@ -6285,7 +6323,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="15">
@@ -6296,7 +6334,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6308,7 +6346,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="16">
@@ -6331,7 +6369,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="17">
@@ -6354,7 +6392,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>
@@ -6375,10 +6413,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6386,46 +6424,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -6449,7 +6487,7 @@
         <v>192</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6461,10 +6499,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6494,7 +6532,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3">
@@ -6521,7 +6559,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4">
@@ -6548,7 +6586,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5">
@@ -6575,7 +6613,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6">
@@ -6602,7 +6640,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7">
@@ -6629,7 +6667,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8">
@@ -6656,7 +6694,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9">
@@ -6683,7 +6721,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10">
@@ -6710,7 +6748,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="11">
@@ -6737,7 +6775,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="12">
@@ -6764,7 +6802,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13">
@@ -6791,12 +6829,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: re-dictado de las semanas 26-31/10 y 2-7/11
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="259">
   <si>
     <t>fecha</t>
   </si>
@@ -490,13 +490,16 @@
     <t>dictado 20/10: Fisher 2026-10-27</t>
   </si>
   <si>
+    <t>dictado 20/10: Fisher 2026-10-31</t>
+  </si>
+  <si>
     <t>dictado 20/10: Cassio 2026-10-27</t>
   </si>
   <si>
     <t>dictado 20/10: Stein 2026-10-27</t>
   </si>
   <si>
-    <t>dictado 20/10: Muller Fabricio 2026-10-28</t>
+    <t>dictado 20/10: Muller Fabricio 2026-10-31</t>
   </si>
   <si>
     <t>dictado 20/10: Agrocurupa 2026-10-28</t>
@@ -505,16 +508,16 @@
     <t>dictado 20/10: Gilson 2026-10-28</t>
   </si>
   <si>
-    <t>dictado 20/10: Wagner 2026-10-27</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Jaime Zimerman 2026-10-28</t>
+    <t>dictado 20/10: Wagner 2026-10-31</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Jaime Zimerman 2026-10-31</t>
   </si>
   <si>
     <t>Andre Pauli</t>
   </si>
   <si>
-    <t>dictado 20/10: Andre Pauli 2026-10-27</t>
+    <t>dictado 20/10: Andre Pauli 2026-10-31</t>
   </si>
   <si>
     <t>dictado 20/10: BAHIA 2026-10-28</t>
@@ -523,16 +526,16 @@
     <t>dictado 20/10: Jhony Viera 2026-10-27</t>
   </si>
   <si>
-    <t>dictado 20/10: Ivo zimer 2026-10-28</t>
+    <t>dictado 20/10: Ivo zimer 2026-10-31</t>
   </si>
   <si>
     <t>Aryste Mittelman</t>
   </si>
   <si>
-    <t>dictado 20/10: Aryste Mittelman 2026-10-28</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Shapo 2026-10-27</t>
+    <t>dictado 20/10: Aryste Mittelman 2026-10-31</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Shapo 2026-10-31</t>
   </si>
   <si>
     <t>dictado 20/10: Paraguay AS 2026-10-26</t>
@@ -547,9 +550,6 @@
     <t>2026-11-01</t>
   </si>
   <si>
-    <t>dictado 20/10: Fisher 2026-11-03</t>
-  </si>
-  <si>
     <t>dictado 20/10: Fisher 2026-11-04</t>
   </si>
   <si>
@@ -559,12 +559,12 @@
     <t>dictado 20/10: Cassio 2026-11-03</t>
   </si>
   <si>
-    <t>dictado 20/10: Cassio 2026-11-04</t>
-  </si>
-  <si>
     <t>dictado 20/10: Cassio 2026-11-06</t>
   </si>
   <si>
+    <t>dictado 20/10: Cassio 2026-11-07</t>
+  </si>
+  <si>
     <t>dictado 20/10: Gilson 2026-11-03</t>
   </si>
   <si>
@@ -586,22 +586,31 @@
     <t>dictado 20/10: Agrocurupa 2026-11-06</t>
   </si>
   <si>
-    <t>dictado 20/10: Muller Fabricio 2026-11-03</t>
-  </si>
-  <si>
     <t>dictado 20/10: Muller Fabricio 2026-11-04</t>
   </si>
   <si>
     <t>dictado 20/10: Muller Fabricio 2026-11-06</t>
   </si>
   <si>
-    <t>dictado 20/10: Paraguay GM 2026-11-02</t>
+    <t>dictado 20/10: Ivo zimer 2026-11-04</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Ivo zimer 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Jaime Zimerman 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Aryste Mittelman 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Andre Pauli 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Paraguay MS 2026-11-02</t>
   </si>
   <si>
     <t>dictado 20/10: Paraguay AS 2026-11-03</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Paraguay MS 2026-11-02</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -844,8 +853,8 @@
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1160,7 +1169,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K133"/>
+  <dimension ref="A1:K136"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -4298,7 +4307,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="9">
+      <c r="A98" s="10">
         <v>46322</v>
       </c>
       <c r="B98" s="0" t="s">
@@ -4330,11 +4339,11 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="9">
-        <v>46322</v>
+      <c r="A99" s="10">
+        <v>46326</v>
       </c>
       <c r="B99" s="0" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C99" s="0" t="s">
         <v>151</v>
@@ -4343,13 +4352,13 @@
         <v>24</v>
       </c>
       <c r="E99" s="0" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F99" s="0" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="G99" s="0" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H99" s="0">
         <v>1008</v>
@@ -4362,7 +4371,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="9">
+      <c r="A100" s="10">
         <v>46322</v>
       </c>
       <c r="B100" s="0" t="s">
@@ -4375,13 +4384,13 @@
         <v>24</v>
       </c>
       <c r="E100" s="0" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="F100" s="0" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="G100" s="0" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="H100" s="0">
         <v>1008</v>
@@ -4394,11 +4403,11 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="9">
-        <v>46323</v>
+      <c r="A101" s="10">
+        <v>46322</v>
       </c>
       <c r="B101" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C101" s="0" t="s">
         <v>151</v>
@@ -4407,7 +4416,7 @@
         <v>24</v>
       </c>
       <c r="E101" s="0" t="s">
-        <v>121</v>
+        <v>59</v>
       </c>
       <c r="F101" s="0" t="s">
         <v>56</v>
@@ -4426,11 +4435,11 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="9">
-        <v>46323</v>
+      <c r="A102" s="10">
+        <v>46326</v>
       </c>
       <c r="B102" s="0" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C102" s="0" t="s">
         <v>151</v>
@@ -4439,13 +4448,13 @@
         <v>24</v>
       </c>
       <c r="E102" s="0" t="s">
-        <v>40</v>
+        <v>121</v>
       </c>
       <c r="F102" s="0" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G102" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H102" s="0">
         <v>1008</v>
@@ -4458,7 +4467,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="9">
+      <c r="A103" s="10">
         <v>46323</v>
       </c>
       <c r="B103" s="0" t="s">
@@ -4471,7 +4480,7 @@
         <v>24</v>
       </c>
       <c r="E103" s="0" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F103" s="0" t="s">
         <v>41</v>
@@ -4490,11 +4499,11 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="9">
-        <v>46322</v>
+      <c r="A104" s="10">
+        <v>46323</v>
       </c>
       <c r="B104" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C104" s="0" t="s">
         <v>151</v>
@@ -4503,7 +4512,7 @@
         <v>24</v>
       </c>
       <c r="E104" s="0" t="s">
-        <v>145</v>
+        <v>43</v>
       </c>
       <c r="F104" s="0" t="s">
         <v>41</v>
@@ -4522,11 +4531,11 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="9">
-        <v>46323</v>
+      <c r="A105" s="10">
+        <v>46326</v>
       </c>
       <c r="B105" s="0" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C105" s="0" t="s">
         <v>151</v>
@@ -4535,7 +4544,7 @@
         <v>24</v>
       </c>
       <c r="E105" s="0" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="F105" s="0" t="s">
         <v>41</v>
@@ -4554,11 +4563,11 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="9">
-        <v>46322</v>
+      <c r="A106" s="10">
+        <v>46326</v>
       </c>
       <c r="B106" s="0" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C106" s="0" t="s">
         <v>151</v>
@@ -4567,13 +4576,13 @@
         <v>24</v>
       </c>
       <c r="E106" s="0" t="s">
-        <v>161</v>
+        <v>138</v>
       </c>
       <c r="F106" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G106" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H106" s="0">
         <v>1008</v>
@@ -4582,15 +4591,15 @@
         <v>152</v>
       </c>
       <c r="J106" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="9">
-        <v>46323</v>
+      <c r="A107" s="10">
+        <v>46326</v>
       </c>
       <c r="B107" s="0" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C107" s="0" t="s">
         <v>151</v>
@@ -4599,10 +4608,10 @@
         <v>24</v>
       </c>
       <c r="E107" s="0" t="s">
-        <v>128</v>
+        <v>162</v>
       </c>
       <c r="F107" s="0" t="s">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="G107" s="0" t="s">
         <v>15</v>
@@ -4618,11 +4627,11 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="9">
-        <v>46322</v>
+      <c r="A108" s="10">
+        <v>46323</v>
       </c>
       <c r="B108" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C108" s="0" t="s">
         <v>151</v>
@@ -4631,13 +4640,13 @@
         <v>24</v>
       </c>
       <c r="E108" s="0" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="F108" s="0" t="s">
-        <v>41</v>
+        <v>129</v>
       </c>
       <c r="G108" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H108" s="0">
         <v>1008</v>
@@ -4650,11 +4659,11 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="9">
-        <v>46323</v>
+      <c r="A109" s="10">
+        <v>46322</v>
       </c>
       <c r="B109" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C109" s="0" t="s">
         <v>151</v>
@@ -4663,7 +4672,7 @@
         <v>24</v>
       </c>
       <c r="E109" s="0" t="s">
-        <v>25</v>
+        <v>112</v>
       </c>
       <c r="F109" s="0" t="s">
         <v>41</v>
@@ -4682,11 +4691,11 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="9">
-        <v>46323</v>
+      <c r="A110" s="10">
+        <v>46326</v>
       </c>
       <c r="B110" s="0" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C110" s="0" t="s">
         <v>151</v>
@@ -4695,13 +4704,13 @@
         <v>24</v>
       </c>
       <c r="E110" s="0" t="s">
-        <v>166</v>
+        <v>25</v>
       </c>
       <c r="F110" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G110" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H110" s="0">
         <v>1008</v>
@@ -4710,15 +4719,15 @@
         <v>152</v>
       </c>
       <c r="J110" s="0" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="9">
-        <v>46322</v>
+      <c r="A111" s="10">
+        <v>46326</v>
       </c>
       <c r="B111" s="0" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C111" s="0" t="s">
         <v>151</v>
@@ -4727,13 +4736,13 @@
         <v>24</v>
       </c>
       <c r="E111" s="0" t="s">
-        <v>105</v>
+        <v>167</v>
       </c>
       <c r="F111" s="0" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G111" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H111" s="0">
         <v>1008</v>
@@ -4746,29 +4755,29 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="9">
-        <v>46321</v>
+      <c r="A112" s="10">
+        <v>46326</v>
       </c>
       <c r="B112" s="0" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="C112" s="0" t="s">
         <v>151</v>
       </c>
       <c r="D112" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E112" s="0" t="s">
-        <v>22</v>
+        <v>105</v>
       </c>
       <c r="F112" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G112" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H112" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I112" s="0" t="s">
         <v>152</v>
@@ -4778,11 +4787,11 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="9">
-        <v>46322</v>
+      <c r="A113" s="10">
+        <v>46321</v>
       </c>
       <c r="B113" s="0" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C113" s="0" t="s">
         <v>151</v>
@@ -4791,7 +4800,7 @@
         <v>13</v>
       </c>
       <c r="E113" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F113" s="0" t="s">
         <v>15</v>
@@ -4810,7 +4819,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="9">
+      <c r="A114" s="10">
         <v>46322</v>
       </c>
       <c r="B114" s="0" t="s">
@@ -4823,7 +4832,7 @@
         <v>13</v>
       </c>
       <c r="E114" s="0" t="s">
-        <v>147</v>
+        <v>20</v>
       </c>
       <c r="F114" s="0" t="s">
         <v>15</v>
@@ -4842,46 +4851,46 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="9">
-        <v>46329</v>
+      <c r="A115" s="10">
+        <v>46322</v>
       </c>
       <c r="B115" s="0" t="s">
         <v>21</v>
       </c>
       <c r="C115" s="0" t="s">
-        <v>172</v>
+        <v>151</v>
       </c>
       <c r="D115" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E115" s="0" t="s">
-        <v>31</v>
+        <v>147</v>
       </c>
       <c r="F115" s="0" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="G115" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H115" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I115" s="0" t="s">
         <v>152</v>
       </c>
       <c r="J115" s="0" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="9">
+      <c r="A116" s="10">
         <v>46330</v>
       </c>
       <c r="B116" s="0" t="s">
         <v>52</v>
       </c>
       <c r="C116" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D116" s="0" t="s">
         <v>24</v>
@@ -4906,14 +4915,14 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="9">
+      <c r="A117" s="10">
         <v>46332</v>
       </c>
       <c r="B117" s="0" t="s">
         <v>23</v>
       </c>
       <c r="C117" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D117" s="0" t="s">
         <v>24</v>
@@ -4938,14 +4947,14 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="9">
+      <c r="A118" s="10">
         <v>46329</v>
       </c>
       <c r="B118" s="0" t="s">
         <v>21</v>
       </c>
       <c r="C118" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D118" s="0" t="s">
         <v>24</v>
@@ -4970,14 +4979,14 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="9">
-        <v>46330</v>
+      <c r="A119" s="10">
+        <v>46332</v>
       </c>
       <c r="B119" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C119" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D119" s="0" t="s">
         <v>24</v>
@@ -5002,14 +5011,14 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="9">
-        <v>46332</v>
+      <c r="A120" s="10">
+        <v>46333</v>
       </c>
       <c r="B120" s="0" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C120" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D120" s="0" t="s">
         <v>24</v>
@@ -5034,14 +5043,14 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="9">
+      <c r="A121" s="10">
         <v>46329</v>
       </c>
       <c r="B121" s="0" t="s">
         <v>21</v>
       </c>
       <c r="C121" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D121" s="0" t="s">
         <v>24</v>
@@ -5066,14 +5075,14 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="9">
+      <c r="A122" s="10">
         <v>46332</v>
       </c>
       <c r="B122" s="0" t="s">
         <v>23</v>
       </c>
       <c r="C122" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D122" s="0" t="s">
         <v>24</v>
@@ -5098,14 +5107,14 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="9">
+      <c r="A123" s="10">
         <v>46329</v>
       </c>
       <c r="B123" s="0" t="s">
         <v>21</v>
       </c>
       <c r="C123" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D123" s="0" t="s">
         <v>24</v>
@@ -5130,14 +5139,14 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="9">
+      <c r="A124" s="10">
         <v>46330</v>
       </c>
       <c r="B124" s="0" t="s">
         <v>52</v>
       </c>
       <c r="C124" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D124" s="0" t="s">
         <v>24</v>
@@ -5162,14 +5171,14 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="9">
+      <c r="A125" s="10">
         <v>46332</v>
       </c>
       <c r="B125" s="0" t="s">
         <v>23</v>
       </c>
       <c r="C125" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D125" s="0" t="s">
         <v>24</v>
@@ -5194,14 +5203,14 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="9">
+      <c r="A126" s="10">
         <v>46330</v>
       </c>
       <c r="B126" s="0" t="s">
         <v>52</v>
       </c>
       <c r="C126" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D126" s="0" t="s">
         <v>24</v>
@@ -5226,14 +5235,14 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="9">
+      <c r="A127" s="10">
         <v>46332</v>
       </c>
       <c r="B127" s="0" t="s">
         <v>23</v>
       </c>
       <c r="C127" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D127" s="0" t="s">
         <v>24</v>
@@ -5258,14 +5267,14 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="9">
-        <v>46329</v>
+      <c r="A128" s="10">
+        <v>46330</v>
       </c>
       <c r="B128" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C128" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D128" s="0" t="s">
         <v>24</v>
@@ -5290,14 +5299,14 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="9">
-        <v>46330</v>
+      <c r="A129" s="10">
+        <v>46332</v>
       </c>
       <c r="B129" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C129" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D129" s="0" t="s">
         <v>24</v>
@@ -5322,26 +5331,26 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="9">
-        <v>46332</v>
+      <c r="A130" s="10">
+        <v>46330</v>
       </c>
       <c r="B130" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C130" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D130" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E130" s="0" t="s">
-        <v>121</v>
+        <v>25</v>
       </c>
       <c r="F130" s="0" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="G130" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H130" s="0">
         <v>1008</v>
@@ -5354,29 +5363,29 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="9">
-        <v>46328</v>
+      <c r="A131" s="10">
+        <v>46332</v>
       </c>
       <c r="B131" s="0" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C131" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D131" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E131" s="0" t="s">
-        <v>147</v>
+        <v>25</v>
       </c>
       <c r="F131" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G131" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H131" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I131" s="0" t="s">
         <v>152</v>
@@ -5386,29 +5395,29 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="9">
-        <v>46329</v>
+      <c r="A132" s="10">
+        <v>46332</v>
       </c>
       <c r="B132" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C132" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D132" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E132" s="0" t="s">
-        <v>22</v>
+        <v>138</v>
       </c>
       <c r="F132" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G132" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H132" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I132" s="0" t="s">
         <v>152</v>
@@ -5418,20 +5427,20 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="9">
-        <v>46328</v>
+      <c r="A133" s="10">
+        <v>46332</v>
       </c>
       <c r="B133" s="0" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C133" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D133" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E133" s="0" t="s">
-        <v>20</v>
+        <v>167</v>
       </c>
       <c r="F133" s="0" t="s">
         <v>15</v>
@@ -5440,13 +5449,109 @@
         <v>15</v>
       </c>
       <c r="H133" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I133" s="0" t="s">
         <v>152</v>
       </c>
       <c r="J133" s="0" t="s">
         <v>191</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="10">
+        <v>46332</v>
+      </c>
+      <c r="B134" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C134" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="D134" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E134" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="F134" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G134" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H134" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I134" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J134" s="0" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="10">
+        <v>46328</v>
+      </c>
+      <c r="B135" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C135" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="D135" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E135" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="F135" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G135" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H135" s="0">
+        <v>980</v>
+      </c>
+      <c r="I135" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J135" s="0" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="10">
+        <v>46329</v>
+      </c>
+      <c r="B136" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C136" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="D136" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E136" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="F136" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G136" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H136" s="0">
+        <v>980</v>
+      </c>
+      <c r="I136" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="J136" s="0" t="s">
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -5468,7 +5573,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5500,10 +5605,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3">
@@ -5520,10 +5625,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4">
@@ -5540,10 +5645,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5">
@@ -5560,10 +5665,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="6">
@@ -5580,10 +5685,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="7">
@@ -5600,10 +5705,10 @@
         <v>1287</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="8">
@@ -5620,10 +5725,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9">
@@ -5640,14 +5745,14 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10">
+      <c r="A10" s="9">
         <v>46335</v>
       </c>
       <c r="B10" s="0">
@@ -5660,11 +5765,11 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10">
+      <c r="A11" s="9">
         <v>46342</v>
       </c>
       <c r="B11" s="0">
@@ -5677,7 +5782,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -5696,57 +5801,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -5794,10 +5899,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3">
@@ -5811,10 +5916,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="4">
@@ -5828,10 +5933,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5">
@@ -5839,16 +5944,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6">
@@ -5862,10 +5967,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="7">
@@ -5879,10 +5984,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8">
@@ -5896,10 +6001,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="9">
@@ -5907,16 +6012,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="10">
@@ -5930,10 +6035,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="11">
@@ -5947,10 +6052,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12">
@@ -5964,10 +6069,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="13">
@@ -5975,16 +6080,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -6018,10 +6123,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6047,7 +6152,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3">
@@ -6070,7 +6175,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4">
@@ -6093,7 +6198,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="5">
@@ -6104,7 +6209,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6116,7 +6221,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6">
@@ -6139,7 +6244,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="7">
@@ -6162,7 +6267,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="8">
@@ -6185,7 +6290,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9">
@@ -6196,7 +6301,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6208,7 +6313,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="10">
@@ -6231,7 +6336,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="11">
@@ -6254,7 +6359,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="12">
@@ -6277,7 +6382,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="13">
@@ -6288,7 +6393,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6300,7 +6405,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="14">
@@ -6323,7 +6428,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="15">
@@ -6334,7 +6439,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6346,7 +6451,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="16">
@@ -6369,7 +6474,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="17">
@@ -6392,7 +6497,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -6413,10 +6518,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6424,46 +6529,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -6484,10 +6589,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6499,10 +6604,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6532,7 +6637,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3">
@@ -6559,7 +6664,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="4">
@@ -6586,7 +6691,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="5">
@@ -6613,7 +6718,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6">
@@ -6640,7 +6745,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="7">
@@ -6667,7 +6772,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="8">
@@ -6694,7 +6799,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="9">
@@ -6721,7 +6826,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10">
@@ -6748,7 +6853,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="11">
@@ -6775,7 +6880,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="12">
@@ -6802,7 +6907,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="13">
@@ -6829,12 +6934,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Ivo y Aryste Mittelman al miercoles 28
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -526,13 +526,13 @@
     <t>dictado 20/10: Jhony Viera 2026-10-27</t>
   </si>
   <si>
-    <t>dictado 20/10: Ivo zimer 2026-10-31</t>
+    <t>dictado 20/10: Ivo zimer 2026-10-28</t>
   </si>
   <si>
     <t>Aryste Mittelman</t>
   </si>
   <si>
-    <t>dictado 20/10: Aryste Mittelman 2026-10-31</t>
+    <t>dictado 20/10: Aryste Mittelman 2026-10-28</t>
   </si>
   <si>
     <t>dictado 20/10: Shapo 2026-10-31</t>
@@ -4692,10 +4692,10 @@
     </row>
     <row r="110">
       <c r="A110" s="10">
-        <v>46326</v>
+        <v>46323</v>
       </c>
       <c r="B110" s="0" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="C110" s="0" t="s">
         <v>151</v>
@@ -4724,10 +4724,10 @@
     </row>
     <row r="111">
       <c r="A111" s="10">
-        <v>46326</v>
+        <v>46323</v>
       </c>
       <c r="B111" s="0" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="C111" s="0" t="s">
         <v>151</v>

</xml_diff>

<commit_message>
plan de compras: Stein de la segunda 19 descarga el miercoles 21 (Gonzalo)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="260">
   <si>
     <t>fecha</t>
   </si>
@@ -404,6 +404,9 @@
   </si>
   <si>
     <t>definitivo 16/10: Stein 3: segunda</t>
+  </si>
+  <si>
+    <t>2026-10-21</t>
   </si>
   <si>
     <t>definitivo 16/10: Stein 3: tersa</t>
@@ -3729,6 +3732,9 @@
       <c r="J79" s="0" t="s">
         <v>125</v>
       </c>
+      <c r="K79" s="0" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="6">
@@ -3759,7 +3765,7 @@
         <v>116</v>
       </c>
       <c r="J80" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="81">
@@ -3791,7 +3797,7 @@
         <v>116</v>
       </c>
       <c r="J81" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="82">
@@ -3808,10 +3814,10 @@
         <v>24</v>
       </c>
       <c r="E82" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F82" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G82" s="0" t="s">
         <v>15</v>
@@ -3823,7 +3829,7 @@
         <v>116</v>
       </c>
       <c r="J82" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="83">
@@ -3840,7 +3846,7 @@
         <v>24</v>
       </c>
       <c r="E83" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F83" s="0" t="s">
         <v>41</v>
@@ -3855,7 +3861,7 @@
         <v>116</v>
       </c>
       <c r="J83" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="84">
@@ -3887,7 +3893,7 @@
         <v>116</v>
       </c>
       <c r="J84" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="85">
@@ -3919,7 +3925,7 @@
         <v>116</v>
       </c>
       <c r="J85" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="86">
@@ -3951,7 +3957,7 @@
         <v>116</v>
       </c>
       <c r="J86" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="87">
@@ -3983,7 +3989,7 @@
         <v>116</v>
       </c>
       <c r="J87" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="88">
@@ -4015,7 +4021,7 @@
         <v>116</v>
       </c>
       <c r="J88" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="89">
@@ -4032,7 +4038,7 @@
         <v>24</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F89" s="0" t="s">
         <v>41</v>
@@ -4047,7 +4053,7 @@
         <v>116</v>
       </c>
       <c r="J89" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="90">
@@ -4079,7 +4085,7 @@
         <v>116</v>
       </c>
       <c r="J90" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="91">
@@ -4111,7 +4117,7 @@
         <v>116</v>
       </c>
       <c r="J91" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="92">
@@ -4143,7 +4149,7 @@
         <v>116</v>
       </c>
       <c r="J92" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="93">
@@ -4175,7 +4181,7 @@
         <v>116</v>
       </c>
       <c r="J93" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="94">
@@ -4207,7 +4213,7 @@
         <v>116</v>
       </c>
       <c r="J94" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="95">
@@ -4224,7 +4230,7 @@
         <v>24</v>
       </c>
       <c r="E95" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F95" s="0" t="s">
         <v>41</v>
@@ -4239,7 +4245,7 @@
         <v>116</v>
       </c>
       <c r="J95" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="96">
@@ -4256,7 +4262,7 @@
         <v>13</v>
       </c>
       <c r="E96" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F96" s="0" t="s">
         <v>15</v>
@@ -4271,7 +4277,7 @@
         <v>116</v>
       </c>
       <c r="J96" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="97">
@@ -4300,10 +4306,10 @@
         <v>1008</v>
       </c>
       <c r="I97" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J97" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="98">
@@ -4314,7 +4320,7 @@
         <v>21</v>
       </c>
       <c r="C98" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D98" s="0" t="s">
         <v>24</v>
@@ -4332,10 +4338,10 @@
         <v>1008</v>
       </c>
       <c r="I98" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J98" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="99">
@@ -4346,7 +4352,7 @@
         <v>30</v>
       </c>
       <c r="C99" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D99" s="0" t="s">
         <v>24</v>
@@ -4364,10 +4370,10 @@
         <v>1008</v>
       </c>
       <c r="I99" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J99" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="100">
@@ -4378,7 +4384,7 @@
         <v>21</v>
       </c>
       <c r="C100" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D100" s="0" t="s">
         <v>24</v>
@@ -4396,10 +4402,10 @@
         <v>1008</v>
       </c>
       <c r="I100" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J100" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="101">
@@ -4410,7 +4416,7 @@
         <v>21</v>
       </c>
       <c r="C101" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D101" s="0" t="s">
         <v>24</v>
@@ -4428,10 +4434,10 @@
         <v>1008</v>
       </c>
       <c r="I101" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J101" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="102">
@@ -4442,7 +4448,7 @@
         <v>30</v>
       </c>
       <c r="C102" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D102" s="0" t="s">
         <v>24</v>
@@ -4460,10 +4466,10 @@
         <v>1008</v>
       </c>
       <c r="I102" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J102" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="103">
@@ -4474,7 +4480,7 @@
         <v>52</v>
       </c>
       <c r="C103" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D103" s="0" t="s">
         <v>24</v>
@@ -4492,10 +4498,10 @@
         <v>1008</v>
       </c>
       <c r="I103" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J103" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="104">
@@ -4506,7 +4512,7 @@
         <v>52</v>
       </c>
       <c r="C104" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D104" s="0" t="s">
         <v>24</v>
@@ -4524,10 +4530,10 @@
         <v>1008</v>
       </c>
       <c r="I104" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J104" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="105">
@@ -4538,13 +4544,13 @@
         <v>30</v>
       </c>
       <c r="C105" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D105" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E105" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F105" s="0" t="s">
         <v>41</v>
@@ -4556,10 +4562,10 @@
         <v>1008</v>
       </c>
       <c r="I105" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J105" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="106">
@@ -4570,13 +4576,13 @@
         <v>30</v>
       </c>
       <c r="C106" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D106" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E106" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F106" s="0" t="s">
         <v>41</v>
@@ -4588,10 +4594,10 @@
         <v>1008</v>
       </c>
       <c r="I106" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J106" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="107">
@@ -4602,13 +4608,13 @@
         <v>30</v>
       </c>
       <c r="C107" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D107" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E107" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F107" s="0" t="s">
         <v>15</v>
@@ -4620,10 +4626,10 @@
         <v>1008</v>
       </c>
       <c r="I107" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J107" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="108">
@@ -4634,16 +4640,16 @@
         <v>52</v>
       </c>
       <c r="C108" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D108" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E108" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F108" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G108" s="0" t="s">
         <v>15</v>
@@ -4652,10 +4658,10 @@
         <v>1008</v>
       </c>
       <c r="I108" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J108" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="109">
@@ -4666,7 +4672,7 @@
         <v>21</v>
       </c>
       <c r="C109" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D109" s="0" t="s">
         <v>24</v>
@@ -4684,10 +4690,10 @@
         <v>1008</v>
       </c>
       <c r="I109" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J109" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="110">
@@ -4698,7 +4704,7 @@
         <v>52</v>
       </c>
       <c r="C110" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D110" s="0" t="s">
         <v>24</v>
@@ -4716,10 +4722,10 @@
         <v>1008</v>
       </c>
       <c r="I110" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J110" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="111">
@@ -4730,13 +4736,13 @@
         <v>52</v>
       </c>
       <c r="C111" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D111" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E111" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F111" s="0" t="s">
         <v>15</v>
@@ -4748,10 +4754,10 @@
         <v>1008</v>
       </c>
       <c r="I111" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J111" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="112">
@@ -4762,7 +4768,7 @@
         <v>30</v>
       </c>
       <c r="C112" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D112" s="0" t="s">
         <v>24</v>
@@ -4780,10 +4786,10 @@
         <v>1008</v>
       </c>
       <c r="I112" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J112" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="113">
@@ -4794,7 +4800,7 @@
         <v>19</v>
       </c>
       <c r="C113" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D113" s="0" t="s">
         <v>13</v>
@@ -4812,10 +4818,10 @@
         <v>980</v>
       </c>
       <c r="I113" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J113" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="114">
@@ -4826,7 +4832,7 @@
         <v>21</v>
       </c>
       <c r="C114" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D114" s="0" t="s">
         <v>13</v>
@@ -4844,10 +4850,10 @@
         <v>980</v>
       </c>
       <c r="I114" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J114" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="115">
@@ -4858,13 +4864,13 @@
         <v>21</v>
       </c>
       <c r="C115" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D115" s="0" t="s">
         <v>13</v>
       </c>
       <c r="E115" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F115" s="0" t="s">
         <v>15</v>
@@ -4876,10 +4882,10 @@
         <v>980</v>
       </c>
       <c r="I115" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J115" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="116">
@@ -4890,7 +4896,7 @@
         <v>52</v>
       </c>
       <c r="C116" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D116" s="0" t="s">
         <v>24</v>
@@ -4908,10 +4914,10 @@
         <v>1008</v>
       </c>
       <c r="I116" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J116" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="117">
@@ -4922,7 +4928,7 @@
         <v>23</v>
       </c>
       <c r="C117" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D117" s="0" t="s">
         <v>24</v>
@@ -4940,10 +4946,10 @@
         <v>1008</v>
       </c>
       <c r="I117" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J117" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="118">
@@ -4954,7 +4960,7 @@
         <v>21</v>
       </c>
       <c r="C118" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D118" s="0" t="s">
         <v>24</v>
@@ -4972,10 +4978,10 @@
         <v>1008</v>
       </c>
       <c r="I118" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J118" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="119">
@@ -4986,7 +4992,7 @@
         <v>23</v>
       </c>
       <c r="C119" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D119" s="0" t="s">
         <v>24</v>
@@ -5004,10 +5010,10 @@
         <v>1008</v>
       </c>
       <c r="I119" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J119" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="120">
@@ -5018,7 +5024,7 @@
         <v>30</v>
       </c>
       <c r="C120" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D120" s="0" t="s">
         <v>24</v>
@@ -5036,10 +5042,10 @@
         <v>1008</v>
       </c>
       <c r="I120" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J120" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="121">
@@ -5050,7 +5056,7 @@
         <v>21</v>
       </c>
       <c r="C121" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D121" s="0" t="s">
         <v>24</v>
@@ -5068,10 +5074,10 @@
         <v>1008</v>
       </c>
       <c r="I121" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J121" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="122">
@@ -5082,7 +5088,7 @@
         <v>23</v>
       </c>
       <c r="C122" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D122" s="0" t="s">
         <v>24</v>
@@ -5100,10 +5106,10 @@
         <v>1008</v>
       </c>
       <c r="I122" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J122" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="123">
@@ -5114,7 +5120,7 @@
         <v>21</v>
       </c>
       <c r="C123" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D123" s="0" t="s">
         <v>24</v>
@@ -5132,10 +5138,10 @@
         <v>1008</v>
       </c>
       <c r="I123" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J123" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="124">
@@ -5146,7 +5152,7 @@
         <v>52</v>
       </c>
       <c r="C124" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D124" s="0" t="s">
         <v>24</v>
@@ -5164,10 +5170,10 @@
         <v>1008</v>
       </c>
       <c r="I124" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J124" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="125">
@@ -5178,7 +5184,7 @@
         <v>23</v>
       </c>
       <c r="C125" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D125" s="0" t="s">
         <v>24</v>
@@ -5196,10 +5202,10 @@
         <v>1008</v>
       </c>
       <c r="I125" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J125" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="126">
@@ -5210,7 +5216,7 @@
         <v>52</v>
       </c>
       <c r="C126" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D126" s="0" t="s">
         <v>24</v>
@@ -5228,10 +5234,10 @@
         <v>1008</v>
       </c>
       <c r="I126" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J126" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="127">
@@ -5242,7 +5248,7 @@
         <v>23</v>
       </c>
       <c r="C127" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D127" s="0" t="s">
         <v>24</v>
@@ -5260,10 +5266,10 @@
         <v>1008</v>
       </c>
       <c r="I127" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J127" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="128">
@@ -5274,7 +5280,7 @@
         <v>52</v>
       </c>
       <c r="C128" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D128" s="0" t="s">
         <v>24</v>
@@ -5292,10 +5298,10 @@
         <v>1008</v>
       </c>
       <c r="I128" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J128" s="0" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="129">
@@ -5306,7 +5312,7 @@
         <v>23</v>
       </c>
       <c r="C129" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D129" s="0" t="s">
         <v>24</v>
@@ -5324,10 +5330,10 @@
         <v>1008</v>
       </c>
       <c r="I129" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J129" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="130">
@@ -5338,7 +5344,7 @@
         <v>52</v>
       </c>
       <c r="C130" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D130" s="0" t="s">
         <v>24</v>
@@ -5356,10 +5362,10 @@
         <v>1008</v>
       </c>
       <c r="I130" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J130" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="131">
@@ -5370,7 +5376,7 @@
         <v>23</v>
       </c>
       <c r="C131" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D131" s="0" t="s">
         <v>24</v>
@@ -5388,10 +5394,10 @@
         <v>1008</v>
       </c>
       <c r="I131" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J131" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="132">
@@ -5402,13 +5408,13 @@
         <v>23</v>
       </c>
       <c r="C132" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D132" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E132" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F132" s="0" t="s">
         <v>41</v>
@@ -5420,10 +5426,10 @@
         <v>1008</v>
       </c>
       <c r="I132" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J132" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="133">
@@ -5434,13 +5440,13 @@
         <v>23</v>
       </c>
       <c r="C133" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D133" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E133" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F133" s="0" t="s">
         <v>15</v>
@@ -5452,10 +5458,10 @@
         <v>1008</v>
       </c>
       <c r="I133" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J133" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="134">
@@ -5466,13 +5472,13 @@
         <v>23</v>
       </c>
       <c r="C134" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D134" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E134" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F134" s="0" t="s">
         <v>15</v>
@@ -5484,10 +5490,10 @@
         <v>1008</v>
       </c>
       <c r="I134" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J134" s="0" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="135">
@@ -5498,7 +5504,7 @@
         <v>19</v>
       </c>
       <c r="C135" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D135" s="0" t="s">
         <v>13</v>
@@ -5516,10 +5522,10 @@
         <v>980</v>
       </c>
       <c r="I135" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J135" s="0" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="136">
@@ -5530,7 +5536,7 @@
         <v>21</v>
       </c>
       <c r="C136" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D136" s="0" t="s">
         <v>13</v>
@@ -5548,10 +5554,10 @@
         <v>980</v>
       </c>
       <c r="I136" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J136" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -5573,7 +5579,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5605,10 +5611,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3">
@@ -5625,10 +5631,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4">
@@ -5645,10 +5651,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5">
@@ -5665,10 +5671,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6">
@@ -5685,10 +5691,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="7">
@@ -5705,10 +5711,10 @@
         <v>1287</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8">
@@ -5725,10 +5731,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9">
@@ -5745,10 +5751,10 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="10">
@@ -5765,7 +5771,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="11">
@@ -5782,7 +5788,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -5801,57 +5807,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>
@@ -5899,10 +5905,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3">
@@ -5916,10 +5922,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4">
@@ -5933,10 +5939,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5">
@@ -5944,16 +5950,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6">
@@ -5967,10 +5973,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7">
@@ -5984,10 +5990,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8">
@@ -6001,10 +6007,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="9">
@@ -6012,16 +6018,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="10">
@@ -6035,10 +6041,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="11">
@@ -6052,10 +6058,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="12">
@@ -6069,10 +6075,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="13">
@@ -6080,16 +6086,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -6123,10 +6129,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6152,7 +6158,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="3">
@@ -6175,7 +6181,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="4">
@@ -6198,7 +6204,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5">
@@ -6209,7 +6215,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6221,7 +6227,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6">
@@ -6244,7 +6250,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="7">
@@ -6267,7 +6273,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="8">
@@ -6290,7 +6296,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="9">
@@ -6301,7 +6307,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6313,7 +6319,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="10">
@@ -6336,7 +6342,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="11">
@@ -6359,7 +6365,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12">
@@ -6382,7 +6388,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13">
@@ -6393,7 +6399,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6405,7 +6411,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="14">
@@ -6428,7 +6434,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="15">
@@ -6439,7 +6445,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6451,7 +6457,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="16">
@@ -6474,7 +6480,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="17">
@@ -6497,7 +6503,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -6518,10 +6524,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6529,46 +6535,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -6589,10 +6595,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6604,10 +6610,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6637,7 +6643,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3">
@@ -6664,7 +6670,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4">
@@ -6691,7 +6697,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5">
@@ -6718,7 +6724,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6">
@@ -6745,7 +6751,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="7">
@@ -6772,7 +6778,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="8">
@@ -6799,7 +6805,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="9">
@@ -6826,7 +6832,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="10">
@@ -6853,7 +6859,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11">
@@ -6880,7 +6886,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="12">
@@ -6907,7 +6913,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13">
@@ -6934,12 +6940,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Milciades (camion roto) descarga hoy 21/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -358,7 +358,10 @@
     <t>planificacion 15/10: Alvarito 1 (7 USD): martes</t>
   </si>
   <si>
-    <t>planificacion 15/10: Milciades 1 (7 USD): miercoles</t>
+    <t>planificacion 15/10: Milciades 1 (7 USD): miercoles; camion roto, arribado 20/10, descarga 21/10 (Gonzalo)</t>
+  </si>
+  <si>
+    <t>2026-10-21</t>
   </si>
   <si>
     <t>planificacion 15/10: Bolivia 1 por semana (dictado 11/10, se mantiene)</t>
@@ -404,9 +407,6 @@
   </si>
   <si>
     <t>definitivo 16/10: Stein 3: segunda</t>
-  </si>
-  <si>
-    <t>2026-10-21</t>
   </si>
   <si>
     <t>definitivo 16/10: Stein 3: tersa</t>
@@ -3412,6 +3412,9 @@
       <c r="J69" s="0" t="s">
         <v>110</v>
       </c>
+      <c r="K69" s="0" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4">
@@ -3442,7 +3445,7 @@
         <v>90</v>
       </c>
       <c r="J70" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="71">
@@ -3459,7 +3462,7 @@
         <v>24</v>
       </c>
       <c r="E71" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F71" s="0" t="s">
         <v>15</v>
@@ -3471,10 +3474,10 @@
         <v>1008</v>
       </c>
       <c r="I71" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J71" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="72">
@@ -3485,7 +3488,7 @@
         <v>21</v>
       </c>
       <c r="C72" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D72" s="0" t="s">
         <v>24</v>
@@ -3503,10 +3506,10 @@
         <v>432</v>
       </c>
       <c r="I72" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J72" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="73">
@@ -3517,7 +3520,7 @@
         <v>52</v>
       </c>
       <c r="C73" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D73" s="0" t="s">
         <v>24</v>
@@ -3535,10 +3538,10 @@
         <v>432</v>
       </c>
       <c r="I73" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J73" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="74">
@@ -3549,7 +3552,7 @@
         <v>21</v>
       </c>
       <c r="C74" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D74" s="0" t="s">
         <v>24</v>
@@ -3567,10 +3570,10 @@
         <v>1008</v>
       </c>
       <c r="I74" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J74" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="75">
@@ -3581,7 +3584,7 @@
         <v>52</v>
       </c>
       <c r="C75" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D75" s="0" t="s">
         <v>24</v>
@@ -3599,10 +3602,10 @@
         <v>1008</v>
       </c>
       <c r="I75" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J75" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="76">
@@ -3613,13 +3616,13 @@
         <v>21</v>
       </c>
       <c r="C76" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D76" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E76" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F76" s="0" t="s">
         <v>56</v>
@@ -3631,10 +3634,10 @@
         <v>1008</v>
       </c>
       <c r="I76" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J76" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="77">
@@ -3645,13 +3648,13 @@
         <v>52</v>
       </c>
       <c r="C77" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D77" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E77" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F77" s="0" t="s">
         <v>56</v>
@@ -3663,10 +3666,10 @@
         <v>1008</v>
       </c>
       <c r="I77" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J77" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="78">
@@ -3677,13 +3680,13 @@
         <v>23</v>
       </c>
       <c r="C78" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D78" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E78" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F78" s="0" t="s">
         <v>56</v>
@@ -3695,10 +3698,10 @@
         <v>1008</v>
       </c>
       <c r="I78" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J78" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="79">
@@ -3709,7 +3712,7 @@
         <v>19</v>
       </c>
       <c r="C79" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D79" s="0" t="s">
         <v>24</v>
@@ -3727,13 +3730,13 @@
         <v>1008</v>
       </c>
       <c r="I79" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J79" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K79" s="0" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
     </row>
     <row r="80">
@@ -3744,7 +3747,7 @@
         <v>21</v>
       </c>
       <c r="C80" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D80" s="0" t="s">
         <v>24</v>
@@ -3762,7 +3765,7 @@
         <v>1008</v>
       </c>
       <c r="I80" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J80" s="0" t="s">
         <v>127</v>
@@ -3776,7 +3779,7 @@
         <v>23</v>
       </c>
       <c r="C81" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D81" s="0" t="s">
         <v>24</v>
@@ -3794,7 +3797,7 @@
         <v>1008</v>
       </c>
       <c r="I81" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J81" s="0" t="s">
         <v>128</v>
@@ -3808,7 +3811,7 @@
         <v>23</v>
       </c>
       <c r="C82" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D82" s="0" t="s">
         <v>24</v>
@@ -3826,7 +3829,7 @@
         <v>1008</v>
       </c>
       <c r="I82" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J82" s="0" t="s">
         <v>131</v>
@@ -3840,7 +3843,7 @@
         <v>30</v>
       </c>
       <c r="C83" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D83" s="0" t="s">
         <v>24</v>
@@ -3858,7 +3861,7 @@
         <v>1008</v>
       </c>
       <c r="I83" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J83" s="0" t="s">
         <v>133</v>
@@ -3872,7 +3875,7 @@
         <v>21</v>
       </c>
       <c r="C84" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D84" s="0" t="s">
         <v>24</v>
@@ -3890,7 +3893,7 @@
         <v>1008</v>
       </c>
       <c r="I84" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J84" s="0" t="s">
         <v>134</v>
@@ -3904,7 +3907,7 @@
         <v>52</v>
       </c>
       <c r="C85" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D85" s="0" t="s">
         <v>24</v>
@@ -3922,7 +3925,7 @@
         <v>1008</v>
       </c>
       <c r="I85" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J85" s="0" t="s">
         <v>135</v>
@@ -3936,7 +3939,7 @@
         <v>23</v>
       </c>
       <c r="C86" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D86" s="0" t="s">
         <v>24</v>
@@ -3954,7 +3957,7 @@
         <v>1008</v>
       </c>
       <c r="I86" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J86" s="0" t="s">
         <v>136</v>
@@ -3968,13 +3971,13 @@
         <v>21</v>
       </c>
       <c r="C87" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D87" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E87" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F87" s="0" t="s">
         <v>41</v>
@@ -3986,7 +3989,7 @@
         <v>1008</v>
       </c>
       <c r="I87" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J87" s="0" t="s">
         <v>137</v>
@@ -4000,7 +4003,7 @@
         <v>21</v>
       </c>
       <c r="C88" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D88" s="0" t="s">
         <v>24</v>
@@ -4018,7 +4021,7 @@
         <v>1008</v>
       </c>
       <c r="I88" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J88" s="0" t="s">
         <v>138</v>
@@ -4032,7 +4035,7 @@
         <v>52</v>
       </c>
       <c r="C89" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D89" s="0" t="s">
         <v>24</v>
@@ -4050,7 +4053,7 @@
         <v>1008</v>
       </c>
       <c r="I89" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J89" s="0" t="s">
         <v>140</v>
@@ -4064,7 +4067,7 @@
         <v>52</v>
       </c>
       <c r="C90" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D90" s="0" t="s">
         <v>24</v>
@@ -4082,7 +4085,7 @@
         <v>1008</v>
       </c>
       <c r="I90" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J90" s="0" t="s">
         <v>141</v>
@@ -4096,7 +4099,7 @@
         <v>23</v>
       </c>
       <c r="C91" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D91" s="0" t="s">
         <v>24</v>
@@ -4114,7 +4117,7 @@
         <v>1008</v>
       </c>
       <c r="I91" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J91" s="0" t="s">
         <v>142</v>
@@ -4128,7 +4131,7 @@
         <v>21</v>
       </c>
       <c r="C92" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D92" s="0" t="s">
         <v>24</v>
@@ -4146,7 +4149,7 @@
         <v>1008</v>
       </c>
       <c r="I92" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J92" s="0" t="s">
         <v>143</v>
@@ -4160,7 +4163,7 @@
         <v>52</v>
       </c>
       <c r="C93" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D93" s="0" t="s">
         <v>24</v>
@@ -4178,7 +4181,7 @@
         <v>1008</v>
       </c>
       <c r="I93" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J93" s="0" t="s">
         <v>144</v>
@@ -4192,7 +4195,7 @@
         <v>21</v>
       </c>
       <c r="C94" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D94" s="0" t="s">
         <v>24</v>
@@ -4210,7 +4213,7 @@
         <v>1008</v>
       </c>
       <c r="I94" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J94" s="0" t="s">
         <v>145</v>
@@ -4224,7 +4227,7 @@
         <v>23</v>
       </c>
       <c r="C95" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D95" s="0" t="s">
         <v>24</v>
@@ -4242,7 +4245,7 @@
         <v>1008</v>
       </c>
       <c r="I95" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J95" s="0" t="s">
         <v>147</v>
@@ -4256,7 +4259,7 @@
         <v>19</v>
       </c>
       <c r="C96" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D96" s="0" t="s">
         <v>13</v>
@@ -4274,7 +4277,7 @@
         <v>980</v>
       </c>
       <c r="I96" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J96" s="0" t="s">
         <v>149</v>
@@ -4288,7 +4291,7 @@
         <v>23</v>
       </c>
       <c r="C97" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D97" s="0" t="s">
         <v>24</v>
@@ -4454,7 +4457,7 @@
         <v>24</v>
       </c>
       <c r="E102" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F102" s="0" t="s">
         <v>56</v>
@@ -4678,7 +4681,7 @@
         <v>24</v>
       </c>
       <c r="E109" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F109" s="0" t="s">
         <v>41</v>
@@ -5286,7 +5289,7 @@
         <v>24</v>
       </c>
       <c r="E128" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F128" s="0" t="s">
         <v>56</v>
@@ -5318,7 +5321,7 @@
         <v>24</v>
       </c>
       <c r="E129" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F129" s="0" t="s">
         <v>56</v>

</xml_diff>

<commit_message>
plan de compras: Guido descarga el jueves 22
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="261">
   <si>
     <t>fecha</t>
   </si>
@@ -476,6 +476,9 @@
   </si>
   <si>
     <t>definitivo 16/10: Guido 1: lunes</t>
+  </si>
+  <si>
+    <t>2026-10-22</t>
   </si>
   <si>
     <t>Gonzalo 19/10 (chat)</t>
@@ -4282,6 +4285,9 @@
       <c r="J96" s="0" t="s">
         <v>149</v>
       </c>
+      <c r="K96" s="0" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="8">
@@ -4309,10 +4315,10 @@
         <v>1008</v>
       </c>
       <c r="I97" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J97" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="98">
@@ -4323,7 +4329,7 @@
         <v>21</v>
       </c>
       <c r="C98" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D98" s="0" t="s">
         <v>24</v>
@@ -4341,10 +4347,10 @@
         <v>1008</v>
       </c>
       <c r="I98" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J98" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="99">
@@ -4355,7 +4361,7 @@
         <v>30</v>
       </c>
       <c r="C99" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D99" s="0" t="s">
         <v>24</v>
@@ -4373,10 +4379,10 @@
         <v>1008</v>
       </c>
       <c r="I99" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J99" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="100">
@@ -4387,7 +4393,7 @@
         <v>21</v>
       </c>
       <c r="C100" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D100" s="0" t="s">
         <v>24</v>
@@ -4405,10 +4411,10 @@
         <v>1008</v>
       </c>
       <c r="I100" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J100" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="101">
@@ -4419,7 +4425,7 @@
         <v>21</v>
       </c>
       <c r="C101" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D101" s="0" t="s">
         <v>24</v>
@@ -4437,10 +4443,10 @@
         <v>1008</v>
       </c>
       <c r="I101" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J101" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="102">
@@ -4451,7 +4457,7 @@
         <v>30</v>
       </c>
       <c r="C102" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D102" s="0" t="s">
         <v>24</v>
@@ -4469,10 +4475,10 @@
         <v>1008</v>
       </c>
       <c r="I102" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J102" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="103">
@@ -4483,7 +4489,7 @@
         <v>52</v>
       </c>
       <c r="C103" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D103" s="0" t="s">
         <v>24</v>
@@ -4501,10 +4507,10 @@
         <v>1008</v>
       </c>
       <c r="I103" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J103" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="104">
@@ -4515,7 +4521,7 @@
         <v>52</v>
       </c>
       <c r="C104" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D104" s="0" t="s">
         <v>24</v>
@@ -4533,10 +4539,10 @@
         <v>1008</v>
       </c>
       <c r="I104" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J104" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="105">
@@ -4547,7 +4553,7 @@
         <v>30</v>
       </c>
       <c r="C105" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D105" s="0" t="s">
         <v>24</v>
@@ -4565,10 +4571,10 @@
         <v>1008</v>
       </c>
       <c r="I105" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J105" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="106">
@@ -4579,7 +4585,7 @@
         <v>30</v>
       </c>
       <c r="C106" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D106" s="0" t="s">
         <v>24</v>
@@ -4597,10 +4603,10 @@
         <v>1008</v>
       </c>
       <c r="I106" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J106" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="107">
@@ -4611,13 +4617,13 @@
         <v>30</v>
       </c>
       <c r="C107" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D107" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E107" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F107" s="0" t="s">
         <v>15</v>
@@ -4629,10 +4635,10 @@
         <v>1008</v>
       </c>
       <c r="I107" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J107" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="108">
@@ -4643,7 +4649,7 @@
         <v>52</v>
       </c>
       <c r="C108" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D108" s="0" t="s">
         <v>24</v>
@@ -4661,10 +4667,10 @@
         <v>1008</v>
       </c>
       <c r="I108" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J108" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="109">
@@ -4675,7 +4681,7 @@
         <v>21</v>
       </c>
       <c r="C109" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D109" s="0" t="s">
         <v>24</v>
@@ -4693,10 +4699,10 @@
         <v>1008</v>
       </c>
       <c r="I109" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J109" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="110">
@@ -4707,7 +4713,7 @@
         <v>52</v>
       </c>
       <c r="C110" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D110" s="0" t="s">
         <v>24</v>
@@ -4725,10 +4731,10 @@
         <v>1008</v>
       </c>
       <c r="I110" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J110" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="111">
@@ -4739,13 +4745,13 @@
         <v>52</v>
       </c>
       <c r="C111" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D111" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E111" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F111" s="0" t="s">
         <v>15</v>
@@ -4757,10 +4763,10 @@
         <v>1008</v>
       </c>
       <c r="I111" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J111" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="112">
@@ -4771,7 +4777,7 @@
         <v>30</v>
       </c>
       <c r="C112" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D112" s="0" t="s">
         <v>24</v>
@@ -4789,10 +4795,10 @@
         <v>1008</v>
       </c>
       <c r="I112" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J112" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="113">
@@ -4803,7 +4809,7 @@
         <v>19</v>
       </c>
       <c r="C113" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D113" s="0" t="s">
         <v>13</v>
@@ -4821,10 +4827,10 @@
         <v>980</v>
       </c>
       <c r="I113" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J113" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="114">
@@ -4835,7 +4841,7 @@
         <v>21</v>
       </c>
       <c r="C114" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D114" s="0" t="s">
         <v>13</v>
@@ -4853,10 +4859,10 @@
         <v>980</v>
       </c>
       <c r="I114" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J114" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="115">
@@ -4867,7 +4873,7 @@
         <v>21</v>
       </c>
       <c r="C115" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D115" s="0" t="s">
         <v>13</v>
@@ -4885,10 +4891,10 @@
         <v>980</v>
       </c>
       <c r="I115" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J115" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="116">
@@ -4899,7 +4905,7 @@
         <v>52</v>
       </c>
       <c r="C116" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D116" s="0" t="s">
         <v>24</v>
@@ -4917,10 +4923,10 @@
         <v>1008</v>
       </c>
       <c r="I116" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J116" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="117">
@@ -4931,7 +4937,7 @@
         <v>23</v>
       </c>
       <c r="C117" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D117" s="0" t="s">
         <v>24</v>
@@ -4949,10 +4955,10 @@
         <v>1008</v>
       </c>
       <c r="I117" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J117" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="118">
@@ -4963,7 +4969,7 @@
         <v>21</v>
       </c>
       <c r="C118" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D118" s="0" t="s">
         <v>24</v>
@@ -4981,10 +4987,10 @@
         <v>1008</v>
       </c>
       <c r="I118" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J118" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="119">
@@ -4995,7 +5001,7 @@
         <v>23</v>
       </c>
       <c r="C119" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D119" s="0" t="s">
         <v>24</v>
@@ -5013,10 +5019,10 @@
         <v>1008</v>
       </c>
       <c r="I119" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J119" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="120">
@@ -5027,7 +5033,7 @@
         <v>30</v>
       </c>
       <c r="C120" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D120" s="0" t="s">
         <v>24</v>
@@ -5045,10 +5051,10 @@
         <v>1008</v>
       </c>
       <c r="I120" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J120" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="121">
@@ -5059,7 +5065,7 @@
         <v>21</v>
       </c>
       <c r="C121" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D121" s="0" t="s">
         <v>24</v>
@@ -5077,10 +5083,10 @@
         <v>1008</v>
       </c>
       <c r="I121" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J121" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="122">
@@ -5091,7 +5097,7 @@
         <v>23</v>
       </c>
       <c r="C122" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D122" s="0" t="s">
         <v>24</v>
@@ -5109,10 +5115,10 @@
         <v>1008</v>
       </c>
       <c r="I122" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J122" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="123">
@@ -5123,7 +5129,7 @@
         <v>21</v>
       </c>
       <c r="C123" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D123" s="0" t="s">
         <v>24</v>
@@ -5141,10 +5147,10 @@
         <v>1008</v>
       </c>
       <c r="I123" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J123" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="124">
@@ -5155,7 +5161,7 @@
         <v>52</v>
       </c>
       <c r="C124" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D124" s="0" t="s">
         <v>24</v>
@@ -5173,10 +5179,10 @@
         <v>1008</v>
       </c>
       <c r="I124" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J124" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="125">
@@ -5187,7 +5193,7 @@
         <v>23</v>
       </c>
       <c r="C125" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D125" s="0" t="s">
         <v>24</v>
@@ -5205,10 +5211,10 @@
         <v>1008</v>
       </c>
       <c r="I125" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J125" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="126">
@@ -5219,7 +5225,7 @@
         <v>52</v>
       </c>
       <c r="C126" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D126" s="0" t="s">
         <v>24</v>
@@ -5237,10 +5243,10 @@
         <v>1008</v>
       </c>
       <c r="I126" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J126" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="127">
@@ -5251,7 +5257,7 @@
         <v>23</v>
       </c>
       <c r="C127" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D127" s="0" t="s">
         <v>24</v>
@@ -5269,10 +5275,10 @@
         <v>1008</v>
       </c>
       <c r="I127" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J127" s="0" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="128">
@@ -5283,7 +5289,7 @@
         <v>52</v>
       </c>
       <c r="C128" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D128" s="0" t="s">
         <v>24</v>
@@ -5301,10 +5307,10 @@
         <v>1008</v>
       </c>
       <c r="I128" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J128" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="129">
@@ -5315,7 +5321,7 @@
         <v>23</v>
       </c>
       <c r="C129" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D129" s="0" t="s">
         <v>24</v>
@@ -5333,10 +5339,10 @@
         <v>1008</v>
       </c>
       <c r="I129" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J129" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="130">
@@ -5347,7 +5353,7 @@
         <v>52</v>
       </c>
       <c r="C130" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D130" s="0" t="s">
         <v>24</v>
@@ -5365,10 +5371,10 @@
         <v>1008</v>
       </c>
       <c r="I130" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J130" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="131">
@@ -5379,7 +5385,7 @@
         <v>23</v>
       </c>
       <c r="C131" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D131" s="0" t="s">
         <v>24</v>
@@ -5397,10 +5403,10 @@
         <v>1008</v>
       </c>
       <c r="I131" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J131" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="132">
@@ -5411,7 +5417,7 @@
         <v>23</v>
       </c>
       <c r="C132" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D132" s="0" t="s">
         <v>24</v>
@@ -5429,10 +5435,10 @@
         <v>1008</v>
       </c>
       <c r="I132" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J132" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="133">
@@ -5443,13 +5449,13 @@
         <v>23</v>
       </c>
       <c r="C133" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D133" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E133" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F133" s="0" t="s">
         <v>15</v>
@@ -5461,10 +5467,10 @@
         <v>1008</v>
       </c>
       <c r="I133" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J133" s="0" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="134">
@@ -5475,13 +5481,13 @@
         <v>23</v>
       </c>
       <c r="C134" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D134" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E134" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F134" s="0" t="s">
         <v>15</v>
@@ -5493,10 +5499,10 @@
         <v>1008</v>
       </c>
       <c r="I134" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J134" s="0" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="135">
@@ -5507,7 +5513,7 @@
         <v>19</v>
       </c>
       <c r="C135" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D135" s="0" t="s">
         <v>13</v>
@@ -5525,10 +5531,10 @@
         <v>980</v>
       </c>
       <c r="I135" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J135" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="136">
@@ -5539,7 +5545,7 @@
         <v>21</v>
       </c>
       <c r="C136" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D136" s="0" t="s">
         <v>13</v>
@@ -5557,10 +5563,10 @@
         <v>980</v>
       </c>
       <c r="I136" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J136" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -5582,7 +5588,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5614,10 +5620,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3">
@@ -5634,10 +5640,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4">
@@ -5654,10 +5660,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5">
@@ -5674,10 +5680,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6">
@@ -5694,10 +5700,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7">
@@ -5714,10 +5720,10 @@
         <v>1287</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8">
@@ -5734,10 +5740,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9">
@@ -5754,10 +5760,10 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="10">
@@ -5774,7 +5780,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11">
@@ -5791,7 +5797,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -5810,57 +5816,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -5908,10 +5914,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="3">
@@ -5925,10 +5931,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4">
@@ -5942,10 +5948,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5">
@@ -5953,16 +5959,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6">
@@ -5976,10 +5982,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7">
@@ -5993,10 +5999,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="8">
@@ -6010,10 +6016,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9">
@@ -6021,16 +6027,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="10">
@@ -6044,10 +6050,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="11">
@@ -6061,10 +6067,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="12">
@@ -6078,10 +6084,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="13">
@@ -6089,16 +6095,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -6132,10 +6138,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6161,7 +6167,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3">
@@ -6184,7 +6190,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4">
@@ -6207,7 +6213,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="5">
@@ -6218,7 +6224,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6230,7 +6236,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="6">
@@ -6253,7 +6259,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7">
@@ -6276,7 +6282,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="8">
@@ -6299,7 +6305,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9">
@@ -6310,7 +6316,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6322,7 +6328,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10">
@@ -6345,7 +6351,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11">
@@ -6368,7 +6374,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="12">
@@ -6391,7 +6397,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="13">
@@ -6402,7 +6408,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6414,7 +6420,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14">
@@ -6437,7 +6443,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15">
@@ -6448,7 +6454,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6460,7 +6466,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="16">
@@ -6483,7 +6489,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="17">
@@ -6506,7 +6512,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -6527,10 +6533,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6538,46 +6544,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -6598,10 +6604,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6613,10 +6619,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6646,7 +6652,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3">
@@ -6673,7 +6679,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="4">
@@ -6700,7 +6706,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5">
@@ -6727,7 +6733,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="6">
@@ -6754,7 +6760,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="7">
@@ -6781,7 +6787,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="8">
@@ -6808,7 +6814,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="9">
@@ -6835,7 +6841,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="10">
@@ -6862,7 +6868,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11">
@@ -6889,7 +6895,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12">
@@ -6916,7 +6922,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="13">
@@ -6943,12 +6949,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Muller y Stein de la tersa 20 descargan el jueves 22
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -400,6 +400,9 @@
     <t>definitivo 16/10: Muller 3 (Curuca): tersa</t>
   </si>
   <si>
+    <t>2026-10-22</t>
+  </si>
+  <si>
     <t>definitivo 16/10: Muller 3 (Curuca): cuarta</t>
   </si>
   <si>
@@ -476,9 +479,6 @@
   </si>
   <si>
     <t>definitivo 16/10: Guido 1: lunes</t>
-  </si>
-  <si>
-    <t>2026-10-22</t>
   </si>
   <si>
     <t>Gonzalo 19/10 (chat)</t>
@@ -3642,6 +3642,9 @@
       <c r="J76" s="0" t="s">
         <v>123</v>
       </c>
+      <c r="K76" s="0" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="6">
@@ -3672,7 +3675,7 @@
         <v>117</v>
       </c>
       <c r="J77" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="78">
@@ -3704,7 +3707,7 @@
         <v>117</v>
       </c>
       <c r="J78" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="79">
@@ -3736,7 +3739,7 @@
         <v>117</v>
       </c>
       <c r="J79" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="K79" s="0" t="s">
         <v>111</v>
@@ -3771,7 +3774,10 @@
         <v>117</v>
       </c>
       <c r="J80" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
+      </c>
+      <c r="K80" s="0" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="81">
@@ -3803,7 +3809,7 @@
         <v>117</v>
       </c>
       <c r="J81" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="82">
@@ -3820,10 +3826,10 @@
         <v>24</v>
       </c>
       <c r="E82" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F82" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G82" s="0" t="s">
         <v>15</v>
@@ -3835,7 +3841,7 @@
         <v>117</v>
       </c>
       <c r="J82" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="83">
@@ -3852,7 +3858,7 @@
         <v>24</v>
       </c>
       <c r="E83" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F83" s="0" t="s">
         <v>41</v>
@@ -3867,7 +3873,7 @@
         <v>117</v>
       </c>
       <c r="J83" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="84">
@@ -3899,7 +3905,7 @@
         <v>117</v>
       </c>
       <c r="J84" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="85">
@@ -3931,7 +3937,7 @@
         <v>117</v>
       </c>
       <c r="J85" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="86">
@@ -3963,7 +3969,7 @@
         <v>117</v>
       </c>
       <c r="J86" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="87">
@@ -3995,7 +4001,7 @@
         <v>117</v>
       </c>
       <c r="J87" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="88">
@@ -4027,7 +4033,7 @@
         <v>117</v>
       </c>
       <c r="J88" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="89">
@@ -4044,7 +4050,7 @@
         <v>24</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F89" s="0" t="s">
         <v>41</v>
@@ -4059,7 +4065,7 @@
         <v>117</v>
       </c>
       <c r="J89" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="90">
@@ -4091,7 +4097,7 @@
         <v>117</v>
       </c>
       <c r="J90" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="91">
@@ -4123,7 +4129,7 @@
         <v>117</v>
       </c>
       <c r="J91" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="92">
@@ -4155,7 +4161,7 @@
         <v>117</v>
       </c>
       <c r="J92" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="93">
@@ -4187,7 +4193,7 @@
         <v>117</v>
       </c>
       <c r="J93" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="94">
@@ -4219,7 +4225,7 @@
         <v>117</v>
       </c>
       <c r="J94" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="95">
@@ -4236,7 +4242,7 @@
         <v>24</v>
       </c>
       <c r="E95" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F95" s="0" t="s">
         <v>41</v>
@@ -4251,7 +4257,7 @@
         <v>117</v>
       </c>
       <c r="J95" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="96">
@@ -4268,7 +4274,7 @@
         <v>13</v>
       </c>
       <c r="E96" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F96" s="0" t="s">
         <v>15</v>
@@ -4283,10 +4289,10 @@
         <v>117</v>
       </c>
       <c r="J96" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="K96" s="0" t="s">
-        <v>150</v>
+        <v>124</v>
       </c>
     </row>
     <row r="97">
@@ -4559,7 +4565,7 @@
         <v>24</v>
       </c>
       <c r="E105" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F105" s="0" t="s">
         <v>41</v>
@@ -4591,7 +4597,7 @@
         <v>24</v>
       </c>
       <c r="E106" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F106" s="0" t="s">
         <v>41</v>
@@ -4655,10 +4661,10 @@
         <v>24</v>
       </c>
       <c r="E108" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F108" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G108" s="0" t="s">
         <v>15</v>
@@ -4879,7 +4885,7 @@
         <v>13</v>
       </c>
       <c r="E115" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F115" s="0" t="s">
         <v>15</v>
@@ -5423,7 +5429,7 @@
         <v>24</v>
       </c>
       <c r="E132" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F132" s="0" t="s">
         <v>41</v>

</xml_diff>

<commit_message>
plan de compras: Shapo de la tersa 20 no cargo (no esta en Aloha; carga el viernes 23)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="260">
   <si>
     <t>fecha</t>
   </si>
@@ -464,9 +464,6 @@
   </si>
   <si>
     <t>definitivo 16/10: Marconi 1: cuarta</t>
-  </si>
-  <si>
-    <t>definitivo 16/10: Shapo 1: tersa</t>
   </si>
   <si>
     <t>Wagner</t>
@@ -1175,7 +1172,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K136"/>
+  <dimension ref="A1:K135"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -4201,10 +4198,10 @@
     </row>
     <row r="94">
       <c r="A94" s="6">
-        <v>46315</v>
+        <v>46318</v>
       </c>
       <c r="B94" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C94" s="0" t="s">
         <v>116</v>
@@ -4213,7 +4210,7 @@
         <v>24</v>
       </c>
       <c r="E94" s="0" t="s">
-        <v>105</v>
+        <v>146</v>
       </c>
       <c r="F94" s="0" t="s">
         <v>41</v>
@@ -4228,94 +4225,94 @@
         <v>117</v>
       </c>
       <c r="J94" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="6">
-        <v>46318</v>
+        <v>46314</v>
       </c>
       <c r="B95" s="0" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C95" s="0" t="s">
         <v>116</v>
       </c>
       <c r="D95" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E95" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F95" s="0" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G95" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H95" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I95" s="0" t="s">
         <v>117</v>
       </c>
       <c r="J95" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
+      </c>
+      <c r="K95" s="0" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="6">
-        <v>46314</v>
+      <c r="A96" s="8">
+        <v>46318</v>
       </c>
       <c r="B96" s="0" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C96" s="0" t="s">
         <v>116</v>
       </c>
       <c r="D96" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E96" s="0" t="s">
-        <v>149</v>
+        <v>25</v>
       </c>
       <c r="F96" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G96" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H96" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I96" s="0" t="s">
-        <v>117</v>
+        <v>150</v>
       </c>
       <c r="J96" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="K96" s="0" t="s">
-        <v>124</v>
+        <v>151</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="8">
-        <v>46318</v>
+      <c r="A97" s="10">
+        <v>46322</v>
       </c>
       <c r="B97" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C97" s="0" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="D97" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E97" s="0" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F97" s="0" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="G97" s="0" t="s">
         <v>35</v>
@@ -4324,21 +4321,21 @@
         <v>1008</v>
       </c>
       <c r="I97" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="J97" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="10">
-        <v>46322</v>
+        <v>46326</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C98" s="0" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D98" s="0" t="s">
         <v>24</v>
@@ -4356,7 +4353,7 @@
         <v>1008</v>
       </c>
       <c r="I98" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J98" s="0" t="s">
         <v>155</v>
@@ -4364,31 +4361,31 @@
     </row>
     <row r="99">
       <c r="A99" s="10">
-        <v>46326</v>
+        <v>46322</v>
       </c>
       <c r="B99" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C99" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D99" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E99" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F99" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="G99" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="H99" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I99" s="0" t="s">
         <v>153</v>
-      </c>
-      <c r="D99" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E99" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="F99" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="G99" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="H99" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I99" s="0" t="s">
-        <v>154</v>
       </c>
       <c r="J99" s="0" t="s">
         <v>156</v>
@@ -4402,25 +4399,25 @@
         <v>21</v>
       </c>
       <c r="C100" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D100" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E100" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F100" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="G100" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H100" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I100" s="0" t="s">
         <v>153</v>
-      </c>
-      <c r="D100" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E100" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="F100" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="G100" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="H100" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I100" s="0" t="s">
-        <v>154</v>
       </c>
       <c r="J100" s="0" t="s">
         <v>157</v>
@@ -4428,19 +4425,19 @@
     </row>
     <row r="101">
       <c r="A101" s="10">
-        <v>46322</v>
+        <v>46326</v>
       </c>
       <c r="B101" s="0" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C101" s="0" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D101" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E101" s="0" t="s">
-        <v>59</v>
+        <v>122</v>
       </c>
       <c r="F101" s="0" t="s">
         <v>56</v>
@@ -4452,7 +4449,7 @@
         <v>1008</v>
       </c>
       <c r="I101" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J101" s="0" t="s">
         <v>158</v>
@@ -4460,31 +4457,31 @@
     </row>
     <row r="102">
       <c r="A102" s="10">
-        <v>46326</v>
+        <v>46323</v>
       </c>
       <c r="B102" s="0" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="C102" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D102" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E102" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="F102" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G102" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H102" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I102" s="0" t="s">
         <v>153</v>
-      </c>
-      <c r="D102" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E102" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="F102" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="G102" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H102" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I102" s="0" t="s">
-        <v>154</v>
       </c>
       <c r="J102" s="0" t="s">
         <v>159</v>
@@ -4498,13 +4495,13 @@
         <v>52</v>
       </c>
       <c r="C103" s="0" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D103" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E103" s="0" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F103" s="0" t="s">
         <v>41</v>
@@ -4516,7 +4513,7 @@
         <v>1008</v>
       </c>
       <c r="I103" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J103" s="0" t="s">
         <v>160</v>
@@ -4524,19 +4521,19 @@
     </row>
     <row r="104">
       <c r="A104" s="10">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="B104" s="0" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C104" s="0" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D104" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E104" s="0" t="s">
-        <v>43</v>
+        <v>146</v>
       </c>
       <c r="F104" s="0" t="s">
         <v>41</v>
@@ -4548,7 +4545,7 @@
         <v>1008</v>
       </c>
       <c r="I104" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J104" s="0" t="s">
         <v>161</v>
@@ -4562,13 +4559,13 @@
         <v>30</v>
       </c>
       <c r="C105" s="0" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D105" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E105" s="0" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="F105" s="0" t="s">
         <v>41</v>
@@ -4580,7 +4577,7 @@
         <v>1008</v>
       </c>
       <c r="I105" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J105" s="0" t="s">
         <v>162</v>
@@ -4594,57 +4591,57 @@
         <v>30</v>
       </c>
       <c r="C106" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D106" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E106" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="F106" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G106" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H106" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I106" s="0" t="s">
         <v>153</v>
       </c>
-      <c r="D106" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E106" s="0" t="s">
-        <v>140</v>
-      </c>
-      <c r="F106" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G106" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="H106" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I106" s="0" t="s">
-        <v>154</v>
-      </c>
       <c r="J106" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="10">
-        <v>46326</v>
+        <v>46323</v>
       </c>
       <c r="B107" s="0" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="C107" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D107" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E107" s="0" t="s">
+        <v>130</v>
+      </c>
+      <c r="F107" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="G107" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H107" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I107" s="0" t="s">
         <v>153</v>
-      </c>
-      <c r="D107" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E107" s="0" t="s">
-        <v>164</v>
-      </c>
-      <c r="F107" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G107" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H107" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I107" s="0" t="s">
-        <v>154</v>
       </c>
       <c r="J107" s="0" t="s">
         <v>165</v>
@@ -4652,31 +4649,31 @@
     </row>
     <row r="108">
       <c r="A108" s="10">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="B108" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C108" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D108" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E108" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="F108" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G108" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H108" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I108" s="0" t="s">
         <v>153</v>
-      </c>
-      <c r="D108" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E108" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="F108" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="G108" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H108" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I108" s="0" t="s">
-        <v>154</v>
       </c>
       <c r="J108" s="0" t="s">
         <v>166</v>
@@ -4684,19 +4681,19 @@
     </row>
     <row r="109">
       <c r="A109" s="10">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B109" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C109" s="0" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D109" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E109" s="0" t="s">
-        <v>113</v>
+        <v>25</v>
       </c>
       <c r="F109" s="0" t="s">
         <v>41</v>
@@ -4708,7 +4705,7 @@
         <v>1008</v>
       </c>
       <c r="I109" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J109" s="0" t="s">
         <v>167</v>
@@ -4722,57 +4719,57 @@
         <v>52</v>
       </c>
       <c r="C110" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D110" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E110" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="F110" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G110" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H110" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I110" s="0" t="s">
         <v>153</v>
       </c>
-      <c r="D110" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E110" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="F110" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G110" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="H110" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I110" s="0" t="s">
-        <v>154</v>
-      </c>
       <c r="J110" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="10">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="B111" s="0" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C111" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D111" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E111" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="F111" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G111" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H111" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I111" s="0" t="s">
         <v>153</v>
-      </c>
-      <c r="D111" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E111" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="F111" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G111" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H111" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I111" s="0" t="s">
-        <v>154</v>
       </c>
       <c r="J111" s="0" t="s">
         <v>170</v>
@@ -4780,31 +4777,31 @@
     </row>
     <row r="112">
       <c r="A112" s="10">
-        <v>46326</v>
+        <v>46321</v>
       </c>
       <c r="B112" s="0" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="C112" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D112" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E112" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="F112" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G112" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H112" s="0">
+        <v>980</v>
+      </c>
+      <c r="I112" s="0" t="s">
         <v>153</v>
-      </c>
-      <c r="D112" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E112" s="0" t="s">
-        <v>105</v>
-      </c>
-      <c r="F112" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G112" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="H112" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I112" s="0" t="s">
-        <v>154</v>
       </c>
       <c r="J112" s="0" t="s">
         <v>171</v>
@@ -4812,19 +4809,19 @@
     </row>
     <row r="113">
       <c r="A113" s="10">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="B113" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C113" s="0" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D113" s="0" t="s">
         <v>13</v>
       </c>
       <c r="E113" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F113" s="0" t="s">
         <v>15</v>
@@ -4836,7 +4833,7 @@
         <v>980</v>
       </c>
       <c r="I113" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J113" s="0" t="s">
         <v>172</v>
@@ -4850,13 +4847,13 @@
         <v>21</v>
       </c>
       <c r="C114" s="0" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D114" s="0" t="s">
         <v>13</v>
       </c>
       <c r="E114" s="0" t="s">
-        <v>20</v>
+        <v>148</v>
       </c>
       <c r="F114" s="0" t="s">
         <v>15</v>
@@ -4868,7 +4865,7 @@
         <v>980</v>
       </c>
       <c r="I114" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J114" s="0" t="s">
         <v>173</v>
@@ -4876,45 +4873,45 @@
     </row>
     <row r="115">
       <c r="A115" s="10">
-        <v>46322</v>
+        <v>46330</v>
       </c>
       <c r="B115" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C115" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="D115" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E115" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="F115" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="G115" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H115" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I115" s="0" t="s">
         <v>153</v>
       </c>
-      <c r="D115" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="E115" s="0" t="s">
-        <v>149</v>
-      </c>
-      <c r="F115" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G115" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H115" s="0">
-        <v>980</v>
-      </c>
-      <c r="I115" s="0" t="s">
-        <v>154</v>
-      </c>
       <c r="J115" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B116" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C116" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D116" s="0" t="s">
         <v>24</v>
@@ -4932,7 +4929,7 @@
         <v>1008</v>
       </c>
       <c r="I116" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J116" s="0" t="s">
         <v>176</v>
@@ -4940,31 +4937,31 @@
     </row>
     <row r="117">
       <c r="A117" s="10">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B117" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C117" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D117" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E117" s="0" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F117" s="0" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="G117" s="0" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H117" s="0">
         <v>1008</v>
       </c>
       <c r="I117" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J117" s="0" t="s">
         <v>177</v>
@@ -4972,13 +4969,13 @@
     </row>
     <row r="118">
       <c r="A118" s="10">
-        <v>46329</v>
+        <v>46332</v>
       </c>
       <c r="B118" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C118" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D118" s="0" t="s">
         <v>24</v>
@@ -4996,7 +4993,7 @@
         <v>1008</v>
       </c>
       <c r="I118" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J118" s="0" t="s">
         <v>178</v>
@@ -5004,13 +5001,13 @@
     </row>
     <row r="119">
       <c r="A119" s="10">
-        <v>46332</v>
+        <v>46333</v>
       </c>
       <c r="B119" s="0" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C119" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D119" s="0" t="s">
         <v>24</v>
@@ -5028,7 +5025,7 @@
         <v>1008</v>
       </c>
       <c r="I119" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J119" s="0" t="s">
         <v>179</v>
@@ -5036,31 +5033,31 @@
     </row>
     <row r="120">
       <c r="A120" s="10">
-        <v>46333</v>
+        <v>46329</v>
       </c>
       <c r="B120" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C120" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D120" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E120" s="0" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="F120" s="0" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G120" s="0" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H120" s="0">
         <v>1008</v>
       </c>
       <c r="I120" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J120" s="0" t="s">
         <v>180</v>
@@ -5068,13 +5065,13 @@
     </row>
     <row r="121">
       <c r="A121" s="10">
-        <v>46329</v>
+        <v>46332</v>
       </c>
       <c r="B121" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C121" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D121" s="0" t="s">
         <v>24</v>
@@ -5092,7 +5089,7 @@
         <v>1008</v>
       </c>
       <c r="I121" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J121" s="0" t="s">
         <v>181</v>
@@ -5100,31 +5097,31 @@
     </row>
     <row r="122">
       <c r="A122" s="10">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B122" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C122" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D122" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E122" s="0" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="F122" s="0" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G122" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H122" s="0">
         <v>1008</v>
       </c>
       <c r="I122" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J122" s="0" t="s">
         <v>182</v>
@@ -5132,13 +5129,13 @@
     </row>
     <row r="123">
       <c r="A123" s="10">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="B123" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C123" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D123" s="0" t="s">
         <v>24</v>
@@ -5156,7 +5153,7 @@
         <v>1008</v>
       </c>
       <c r="I123" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J123" s="0" t="s">
         <v>183</v>
@@ -5164,13 +5161,13 @@
     </row>
     <row r="124">
       <c r="A124" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B124" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C124" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D124" s="0" t="s">
         <v>24</v>
@@ -5188,7 +5185,7 @@
         <v>1008</v>
       </c>
       <c r="I124" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J124" s="0" t="s">
         <v>184</v>
@@ -5196,31 +5193,31 @@
     </row>
     <row r="125">
       <c r="A125" s="10">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B125" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C125" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D125" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E125" s="0" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="F125" s="0" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="G125" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H125" s="0">
         <v>1008</v>
       </c>
       <c r="I125" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J125" s="0" t="s">
         <v>185</v>
@@ -5228,13 +5225,13 @@
     </row>
     <row r="126">
       <c r="A126" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B126" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C126" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D126" s="0" t="s">
         <v>24</v>
@@ -5252,7 +5249,7 @@
         <v>1008</v>
       </c>
       <c r="I126" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J126" s="0" t="s">
         <v>186</v>
@@ -5260,31 +5257,31 @@
     </row>
     <row r="127">
       <c r="A127" s="10">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B127" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C127" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D127" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E127" s="0" t="s">
-        <v>40</v>
+        <v>122</v>
       </c>
       <c r="F127" s="0" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G127" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H127" s="0">
         <v>1008</v>
       </c>
       <c r="I127" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J127" s="0" t="s">
         <v>187</v>
@@ -5292,13 +5289,13 @@
     </row>
     <row r="128">
       <c r="A128" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B128" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C128" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D128" s="0" t="s">
         <v>24</v>
@@ -5316,7 +5313,7 @@
         <v>1008</v>
       </c>
       <c r="I128" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J128" s="0" t="s">
         <v>188</v>
@@ -5324,31 +5321,31 @@
     </row>
     <row r="129">
       <c r="A129" s="10">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B129" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C129" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D129" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E129" s="0" t="s">
-        <v>122</v>
+        <v>25</v>
       </c>
       <c r="F129" s="0" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="G129" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H129" s="0">
         <v>1008</v>
       </c>
       <c r="I129" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J129" s="0" t="s">
         <v>189</v>
@@ -5356,13 +5353,13 @@
     </row>
     <row r="130">
       <c r="A130" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B130" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C130" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D130" s="0" t="s">
         <v>24</v>
@@ -5380,7 +5377,7 @@
         <v>1008</v>
       </c>
       <c r="I130" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J130" s="0" t="s">
         <v>190</v>
@@ -5394,13 +5391,13 @@
         <v>23</v>
       </c>
       <c r="C131" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D131" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E131" s="0" t="s">
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="F131" s="0" t="s">
         <v>41</v>
@@ -5412,7 +5409,7 @@
         <v>1008</v>
       </c>
       <c r="I131" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J131" s="0" t="s">
         <v>191</v>
@@ -5426,25 +5423,25 @@
         <v>23</v>
       </c>
       <c r="C132" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D132" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E132" s="0" t="s">
-        <v>140</v>
+        <v>168</v>
       </c>
       <c r="F132" s="0" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G132" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H132" s="0">
         <v>1008</v>
       </c>
       <c r="I132" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J132" s="0" t="s">
         <v>192</v>
@@ -5458,13 +5455,13 @@
         <v>23</v>
       </c>
       <c r="C133" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D133" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E133" s="0" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="F133" s="0" t="s">
         <v>15</v>
@@ -5476,7 +5473,7 @@
         <v>1008</v>
       </c>
       <c r="I133" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J133" s="0" t="s">
         <v>193</v>
@@ -5484,19 +5481,19 @@
     </row>
     <row r="134">
       <c r="A134" s="10">
-        <v>46332</v>
+        <v>46328</v>
       </c>
       <c r="B134" s="0" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C134" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D134" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E134" s="0" t="s">
-        <v>164</v>
+        <v>20</v>
       </c>
       <c r="F134" s="0" t="s">
         <v>15</v>
@@ -5505,10 +5502,10 @@
         <v>15</v>
       </c>
       <c r="H134" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I134" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J134" s="0" t="s">
         <v>194</v>
@@ -5516,19 +5513,19 @@
     </row>
     <row r="135">
       <c r="A135" s="10">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="B135" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C135" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D135" s="0" t="s">
         <v>13</v>
       </c>
       <c r="E135" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F135" s="0" t="s">
         <v>15</v>
@@ -5540,42 +5537,10 @@
         <v>980</v>
       </c>
       <c r="I135" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J135" s="0" t="s">
         <v>195</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="10">
-        <v>46329</v>
-      </c>
-      <c r="B136" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="C136" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="D136" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="E136" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="F136" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G136" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H136" s="0">
-        <v>980</v>
-      </c>
-      <c r="I136" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="J136" s="0" t="s">
-        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -5597,7 +5562,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5629,10 +5594,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
+        <v>197</v>
+      </c>
+      <c r="F2" s="0" t="s">
         <v>198</v>
-      </c>
-      <c r="F2" s="0" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="3">
@@ -5649,10 +5614,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4">
@@ -5669,10 +5634,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
+        <v>200</v>
+      </c>
+      <c r="F4" s="0" t="s">
         <v>201</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="5">
@@ -5689,10 +5654,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
+        <v>202</v>
+      </c>
+      <c r="F5" s="0" t="s">
         <v>203</v>
-      </c>
-      <c r="F5" s="0" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="6">
@@ -5709,10 +5674,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
+        <v>204</v>
+      </c>
+      <c r="F6" s="0" t="s">
         <v>205</v>
-      </c>
-      <c r="F6" s="0" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="7">
@@ -5729,10 +5694,10 @@
         <v>1287</v>
       </c>
       <c r="E7" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="F7" s="0" t="s">
         <v>207</v>
-      </c>
-      <c r="F7" s="0" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="8">
@@ -5749,10 +5714,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="F8" s="0" t="s">
         <v>209</v>
-      </c>
-      <c r="F8" s="0" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="9">
@@ -5769,10 +5734,10 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
+        <v>210</v>
+      </c>
+      <c r="F9" s="0" t="s">
         <v>211</v>
-      </c>
-      <c r="F9" s="0" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="10">
@@ -5789,7 +5754,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="11">
@@ -5806,7 +5771,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -5825,57 +5790,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>
@@ -5923,10 +5888,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
+        <v>224</v>
+      </c>
+      <c r="E2" s="0" t="s">
         <v>225</v>
-      </c>
-      <c r="E2" s="0" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="3">
@@ -5940,10 +5905,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4">
@@ -5957,10 +5922,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5">
@@ -5968,16 +5933,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6">
@@ -5991,10 +5956,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="E6" s="0" t="s">
         <v>231</v>
-      </c>
-      <c r="E6" s="0" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="7">
@@ -6008,10 +5973,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8">
@@ -6025,10 +5990,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="9">
@@ -6036,16 +6001,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="10">
@@ -6059,10 +6024,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
+        <v>235</v>
+      </c>
+      <c r="E10" s="0" t="s">
         <v>236</v>
-      </c>
-      <c r="E10" s="0" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="11">
@@ -6076,10 +6041,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="12">
@@ -6093,10 +6058,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="13">
@@ -6104,16 +6069,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -6147,10 +6112,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>241</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>242</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6176,7 +6141,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="3">
@@ -6199,7 +6164,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="4">
@@ -6222,7 +6187,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5">
@@ -6233,7 +6198,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6245,7 +6210,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6">
@@ -6268,7 +6233,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="7">
@@ -6291,7 +6256,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="8">
@@ -6314,7 +6279,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="9">
@@ -6325,7 +6290,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6337,7 +6302,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="10">
@@ -6360,7 +6325,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="11">
@@ -6383,7 +6348,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12">
@@ -6406,7 +6371,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13">
@@ -6417,7 +6382,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6429,7 +6394,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="14">
@@ -6452,7 +6417,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="15">
@@ -6463,7 +6428,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6475,7 +6440,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="16">
@@ -6498,7 +6463,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="17">
@@ -6521,7 +6486,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -6542,10 +6507,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
+        <v>246</v>
+      </c>
+      <c r="B1" s="0" t="s">
         <v>247</v>
-      </c>
-      <c r="B1" s="0" t="s">
-        <v>248</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6553,46 +6518,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -6613,10 +6578,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6628,10 +6593,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6661,7 +6626,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3">
@@ -6688,7 +6653,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4">
@@ -6715,7 +6680,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5">
@@ -6742,7 +6707,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6">
@@ -6769,7 +6734,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="7">
@@ -6796,7 +6761,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="8">
@@ -6823,7 +6788,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="9">
@@ -6850,7 +6815,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="10">
@@ -6877,7 +6842,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11">
@@ -6904,7 +6869,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="12">
@@ -6931,7 +6896,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13">
@@ -6958,12 +6923,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: semana de carga 26-31/10 re-dictada
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="261">
   <si>
     <t>fecha</t>
   </si>
@@ -493,24 +493,45 @@
     <t>dictado 20/10: Fisher 2026-10-27</t>
   </si>
   <si>
-    <t>dictado 20/10: Fisher 2026-10-31</t>
+    <t>dictado 20/10: Fisher 2026-10-28</t>
   </si>
   <si>
     <t>dictado 20/10: Cassio 2026-10-27</t>
   </si>
   <si>
+    <t>dictado 20/10: Cassio 2026-10-28</t>
+  </si>
+  <si>
     <t>dictado 20/10: Stein 2026-10-27</t>
   </si>
   <si>
+    <t>dictado 20/10: Agrocurupa 2026-10-28</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Gilson 2026-10-28</t>
+  </si>
+  <si>
+    <t>dictado 20/10: BAHIA 2026-10-28</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Jhony Viera 2026-10-27</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Ivo zimer 2026-10-28</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Marconi 2026-10-28</t>
+  </si>
+  <si>
+    <t>Aryste Mittelman</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Aryste Mittelman 2026-10-28</t>
+  </si>
+  <si>
     <t>dictado 20/10: Muller Fabricio 2026-10-31</t>
   </si>
   <si>
-    <t>dictado 20/10: Agrocurupa 2026-10-28</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Gilson 2026-10-28</t>
-  </si>
-  <si>
     <t>dictado 20/10: Wagner 2026-10-31</t>
   </si>
   <si>
@@ -523,28 +544,10 @@
     <t>dictado 20/10: Andre Pauli 2026-10-31</t>
   </si>
   <si>
-    <t>dictado 20/10: BAHIA 2026-10-28</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Jhony Viera 2026-10-27</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Ivo zimer 2026-10-28</t>
-  </si>
-  <si>
-    <t>Aryste Mittelman</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Aryste Mittelman 2026-10-28</t>
-  </si>
-  <si>
     <t>dictado 20/10: Shapo 2026-10-31</t>
   </si>
   <si>
     <t>dictado 20/10: Paraguay AS 2026-10-26</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Paraguay MS 2026-10-27</t>
   </si>
   <si>
     <t>dictado 20/10: Paraguay GM 2026-10-27</t>
@@ -1172,7 +1175,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K135"/>
+  <dimension ref="A1:K136"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -4329,10 +4332,10 @@
     </row>
     <row r="98">
       <c r="A98" s="10">
-        <v>46326</v>
+        <v>46323</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="C98" s="0" t="s">
         <v>152</v>
@@ -4393,10 +4396,10 @@
     </row>
     <row r="100">
       <c r="A100" s="10">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B100" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C100" s="0" t="s">
         <v>152</v>
@@ -4405,13 +4408,13 @@
         <v>24</v>
       </c>
       <c r="E100" s="0" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="F100" s="0" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="G100" s="0" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="H100" s="0">
         <v>1008</v>
@@ -4425,10 +4428,10 @@
     </row>
     <row r="101">
       <c r="A101" s="10">
-        <v>46326</v>
+        <v>46322</v>
       </c>
       <c r="B101" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C101" s="0" t="s">
         <v>152</v>
@@ -4437,7 +4440,7 @@
         <v>24</v>
       </c>
       <c r="E101" s="0" t="s">
-        <v>122</v>
+        <v>59</v>
       </c>
       <c r="F101" s="0" t="s">
         <v>56</v>
@@ -4521,10 +4524,10 @@
     </row>
     <row r="104">
       <c r="A104" s="10">
-        <v>46326</v>
+        <v>46323</v>
       </c>
       <c r="B104" s="0" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="C104" s="0" t="s">
         <v>152</v>
@@ -4533,13 +4536,13 @@
         <v>24</v>
       </c>
       <c r="E104" s="0" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="F104" s="0" t="s">
-        <v>41</v>
+        <v>131</v>
       </c>
       <c r="G104" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H104" s="0">
         <v>1008</v>
@@ -4553,10 +4556,10 @@
     </row>
     <row r="105">
       <c r="A105" s="10">
-        <v>46326</v>
+        <v>46322</v>
       </c>
       <c r="B105" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C105" s="0" t="s">
         <v>152</v>
@@ -4565,7 +4568,7 @@
         <v>24</v>
       </c>
       <c r="E105" s="0" t="s">
-        <v>140</v>
+        <v>113</v>
       </c>
       <c r="F105" s="0" t="s">
         <v>41</v>
@@ -4585,10 +4588,10 @@
     </row>
     <row r="106">
       <c r="A106" s="10">
-        <v>46326</v>
+        <v>46323</v>
       </c>
       <c r="B106" s="0" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="C106" s="0" t="s">
         <v>152</v>
@@ -4597,13 +4600,13 @@
         <v>24</v>
       </c>
       <c r="E106" s="0" t="s">
-        <v>163</v>
+        <v>25</v>
       </c>
       <c r="F106" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G106" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H106" s="0">
         <v>1008</v>
@@ -4612,7 +4615,7 @@
         <v>153</v>
       </c>
       <c r="J106" s="0" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="107">
@@ -4629,13 +4632,13 @@
         <v>24</v>
       </c>
       <c r="E107" s="0" t="s">
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="F107" s="0" t="s">
-        <v>131</v>
+        <v>41</v>
       </c>
       <c r="G107" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H107" s="0">
         <v>1008</v>
@@ -4644,15 +4647,15 @@
         <v>153</v>
       </c>
       <c r="J107" s="0" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="10">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B108" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C108" s="0" t="s">
         <v>152</v>
@@ -4661,13 +4664,13 @@
         <v>24</v>
       </c>
       <c r="E108" s="0" t="s">
-        <v>113</v>
+        <v>165</v>
       </c>
       <c r="F108" s="0" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G108" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H108" s="0">
         <v>1008</v>
@@ -4681,10 +4684,10 @@
     </row>
     <row r="109">
       <c r="A109" s="10">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="B109" s="0" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C109" s="0" t="s">
         <v>152</v>
@@ -4693,13 +4696,13 @@
         <v>24</v>
       </c>
       <c r="E109" s="0" t="s">
-        <v>25</v>
+        <v>122</v>
       </c>
       <c r="F109" s="0" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G109" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H109" s="0">
         <v>1008</v>
@@ -4713,10 +4716,10 @@
     </row>
     <row r="110">
       <c r="A110" s="10">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="B110" s="0" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C110" s="0" t="s">
         <v>152</v>
@@ -4725,13 +4728,13 @@
         <v>24</v>
       </c>
       <c r="E110" s="0" t="s">
-        <v>168</v>
+        <v>146</v>
       </c>
       <c r="F110" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G110" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H110" s="0">
         <v>1008</v>
@@ -4740,7 +4743,7 @@
         <v>153</v>
       </c>
       <c r="J110" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="111">
@@ -4757,7 +4760,7 @@
         <v>24</v>
       </c>
       <c r="E111" s="0" t="s">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="F111" s="0" t="s">
         <v>41</v>
@@ -4772,24 +4775,24 @@
         <v>153</v>
       </c>
       <c r="J111" s="0" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="10">
-        <v>46321</v>
+        <v>46326</v>
       </c>
       <c r="B112" s="0" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="C112" s="0" t="s">
         <v>152</v>
       </c>
       <c r="D112" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E112" s="0" t="s">
-        <v>22</v>
+        <v>170</v>
       </c>
       <c r="F112" s="0" t="s">
         <v>15</v>
@@ -4798,7 +4801,7 @@
         <v>15</v>
       </c>
       <c r="H112" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I112" s="0" t="s">
         <v>153</v>
@@ -4809,28 +4812,28 @@
     </row>
     <row r="113">
       <c r="A113" s="10">
-        <v>46322</v>
+        <v>46326</v>
       </c>
       <c r="B113" s="0" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C113" s="0" t="s">
         <v>152</v>
       </c>
       <c r="D113" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E113" s="0" t="s">
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="F113" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G113" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H113" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I113" s="0" t="s">
         <v>153</v>
@@ -4841,10 +4844,10 @@
     </row>
     <row r="114">
       <c r="A114" s="10">
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="B114" s="0" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C114" s="0" t="s">
         <v>152</v>
@@ -4853,7 +4856,7 @@
         <v>13</v>
       </c>
       <c r="E114" s="0" t="s">
-        <v>148</v>
+        <v>22</v>
       </c>
       <c r="F114" s="0" t="s">
         <v>15</v>
@@ -4873,45 +4876,45 @@
     </row>
     <row r="115">
       <c r="A115" s="10">
-        <v>46330</v>
+        <v>46322</v>
       </c>
       <c r="B115" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C115" s="0" t="s">
-        <v>174</v>
+        <v>152</v>
       </c>
       <c r="D115" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E115" s="0" t="s">
-        <v>31</v>
+        <v>148</v>
       </c>
       <c r="F115" s="0" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="G115" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H115" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I115" s="0" t="s">
         <v>153</v>
       </c>
       <c r="J115" s="0" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="10">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B116" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C116" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D116" s="0" t="s">
         <v>24</v>
@@ -4937,25 +4940,25 @@
     </row>
     <row r="117">
       <c r="A117" s="10">
-        <v>46329</v>
+        <v>46332</v>
       </c>
       <c r="B117" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C117" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D117" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E117" s="0" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F117" s="0" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="G117" s="0" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H117" s="0">
         <v>1008</v>
@@ -4969,13 +4972,13 @@
     </row>
     <row r="118">
       <c r="A118" s="10">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B118" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C118" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D118" s="0" t="s">
         <v>24</v>
@@ -5001,13 +5004,13 @@
     </row>
     <row r="119">
       <c r="A119" s="10">
-        <v>46333</v>
+        <v>46332</v>
       </c>
       <c r="B119" s="0" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C119" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D119" s="0" t="s">
         <v>24</v>
@@ -5033,25 +5036,25 @@
     </row>
     <row r="120">
       <c r="A120" s="10">
-        <v>46329</v>
+        <v>46333</v>
       </c>
       <c r="B120" s="0" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C120" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D120" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E120" s="0" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="F120" s="0" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G120" s="0" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H120" s="0">
         <v>1008</v>
@@ -5065,13 +5068,13 @@
     </row>
     <row r="121">
       <c r="A121" s="10">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B121" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C121" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D121" s="0" t="s">
         <v>24</v>
@@ -5097,25 +5100,25 @@
     </row>
     <row r="122">
       <c r="A122" s="10">
-        <v>46329</v>
+        <v>46332</v>
       </c>
       <c r="B122" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C122" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D122" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E122" s="0" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="F122" s="0" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="G122" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H122" s="0">
         <v>1008</v>
@@ -5129,13 +5132,13 @@
     </row>
     <row r="123">
       <c r="A123" s="10">
-        <v>46330</v>
+        <v>46329</v>
       </c>
       <c r="B123" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C123" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D123" s="0" t="s">
         <v>24</v>
@@ -5161,13 +5164,13 @@
     </row>
     <row r="124">
       <c r="A124" s="10">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B124" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C124" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D124" s="0" t="s">
         <v>24</v>
@@ -5193,25 +5196,25 @@
     </row>
     <row r="125">
       <c r="A125" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B125" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C125" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D125" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E125" s="0" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="F125" s="0" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G125" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H125" s="0">
         <v>1008</v>
@@ -5225,13 +5228,13 @@
     </row>
     <row r="126">
       <c r="A126" s="10">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B126" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C126" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D126" s="0" t="s">
         <v>24</v>
@@ -5257,25 +5260,25 @@
     </row>
     <row r="127">
       <c r="A127" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B127" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C127" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D127" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E127" s="0" t="s">
-        <v>122</v>
+        <v>40</v>
       </c>
       <c r="F127" s="0" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="G127" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H127" s="0">
         <v>1008</v>
@@ -5289,13 +5292,13 @@
     </row>
     <row r="128">
       <c r="A128" s="10">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B128" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C128" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D128" s="0" t="s">
         <v>24</v>
@@ -5321,25 +5324,25 @@
     </row>
     <row r="129">
       <c r="A129" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B129" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C129" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D129" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E129" s="0" t="s">
-        <v>25</v>
+        <v>122</v>
       </c>
       <c r="F129" s="0" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G129" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H129" s="0">
         <v>1008</v>
@@ -5353,13 +5356,13 @@
     </row>
     <row r="130">
       <c r="A130" s="10">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B130" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C130" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D130" s="0" t="s">
         <v>24</v>
@@ -5391,13 +5394,13 @@
         <v>23</v>
       </c>
       <c r="C131" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D131" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E131" s="0" t="s">
-        <v>140</v>
+        <v>25</v>
       </c>
       <c r="F131" s="0" t="s">
         <v>41</v>
@@ -5423,19 +5426,19 @@
         <v>23</v>
       </c>
       <c r="C132" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D132" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E132" s="0" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="F132" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G132" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H132" s="0">
         <v>1008</v>
@@ -5455,13 +5458,13 @@
         <v>23</v>
       </c>
       <c r="C133" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D133" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E133" s="0" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F133" s="0" t="s">
         <v>15</v>
@@ -5481,19 +5484,19 @@
     </row>
     <row r="134">
       <c r="A134" s="10">
-        <v>46328</v>
+        <v>46332</v>
       </c>
       <c r="B134" s="0" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C134" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D134" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E134" s="0" t="s">
-        <v>20</v>
+        <v>170</v>
       </c>
       <c r="F134" s="0" t="s">
         <v>15</v>
@@ -5502,7 +5505,7 @@
         <v>15</v>
       </c>
       <c r="H134" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I134" s="0" t="s">
         <v>153</v>
@@ -5513,19 +5516,19 @@
     </row>
     <row r="135">
       <c r="A135" s="10">
-        <v>46329</v>
+        <v>46328</v>
       </c>
       <c r="B135" s="0" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C135" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D135" s="0" t="s">
         <v>13</v>
       </c>
       <c r="E135" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F135" s="0" t="s">
         <v>15</v>
@@ -5541,6 +5544,38 @@
       </c>
       <c r="J135" s="0" t="s">
         <v>195</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="10">
+        <v>46329</v>
+      </c>
+      <c r="B136" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C136" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="D136" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E136" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="F136" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G136" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H136" s="0">
+        <v>980</v>
+      </c>
+      <c r="I136" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="J136" s="0" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -5562,7 +5597,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5594,10 +5629,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3">
@@ -5614,10 +5649,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4">
@@ -5634,10 +5669,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5">
@@ -5654,10 +5689,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6">
@@ -5674,10 +5709,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7">
@@ -5694,10 +5729,10 @@
         <v>1287</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8">
@@ -5714,10 +5749,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9">
@@ -5734,10 +5769,10 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="10">
@@ -5754,7 +5789,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11">
@@ -5771,7 +5806,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -5790,57 +5825,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -5888,10 +5923,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="3">
@@ -5905,10 +5940,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4">
@@ -5922,10 +5957,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5">
@@ -5933,16 +5968,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6">
@@ -5956,10 +5991,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7">
@@ -5973,10 +6008,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="8">
@@ -5990,10 +6025,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9">
@@ -6001,16 +6036,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="10">
@@ -6024,10 +6059,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="11">
@@ -6041,10 +6076,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="12">
@@ -6058,10 +6093,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="13">
@@ -6069,16 +6104,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -6112,10 +6147,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6141,7 +6176,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3">
@@ -6164,7 +6199,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4">
@@ -6187,7 +6222,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="5">
@@ -6198,7 +6233,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6210,7 +6245,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="6">
@@ -6233,7 +6268,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7">
@@ -6256,7 +6291,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="8">
@@ -6279,7 +6314,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9">
@@ -6290,7 +6325,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6302,7 +6337,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10">
@@ -6325,7 +6360,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11">
@@ -6348,7 +6383,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="12">
@@ -6371,7 +6406,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="13">
@@ -6382,7 +6417,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6394,7 +6429,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14">
@@ -6417,7 +6452,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15">
@@ -6428,7 +6463,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6440,7 +6475,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="16">
@@ -6463,7 +6498,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="17">
@@ -6486,7 +6521,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -6507,10 +6542,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6518,46 +6553,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -6578,10 +6613,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6593,10 +6628,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6626,7 +6661,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3">
@@ -6653,7 +6688,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="4">
@@ -6680,7 +6715,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5">
@@ -6707,7 +6742,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="6">
@@ -6734,7 +6769,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="7">
@@ -6761,7 +6796,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="8">
@@ -6788,7 +6823,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="9">
@@ -6815,7 +6850,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="10">
@@ -6842,7 +6877,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11">
@@ -6869,7 +6904,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12">
@@ -6896,7 +6931,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="13">
@@ -6923,12 +6958,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: venta de la semana 19/10 = 19.900 (faltan 9.800 jue-sab) y Cassio 20/10 con 936 cajas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -649,7 +649,7 @@
     <t>reparto con el mix real de las ultimas 10 semanas</t>
   </si>
   <si>
-    <t>Gonzalo 20/10: "contando con una venta de 19500 esta semana"</t>
+    <t>Gonzalo 21/10: faltan vender 9.800 jue-sab (vendido lun-mie 9.944) = 19.900</t>
   </si>
   <si>
     <t>reparto BR/PY/BO con el mix real de las ultimas 10 semanas; desde el mie 21 la pisa la estimacion con los dias reales</t>
@@ -3899,7 +3899,7 @@
         <v>29</v>
       </c>
       <c r="H84" s="0">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I84" s="0" t="s">
         <v>117</v>
@@ -5720,13 +5720,13 @@
         <v>46314</v>
       </c>
       <c r="B7" s="0">
-        <v>10569</v>
+        <v>10786</v>
       </c>
       <c r="C7" s="0">
-        <v>7644</v>
+        <v>7801</v>
       </c>
       <c r="D7" s="0">
-        <v>1287</v>
+        <v>1313</v>
       </c>
       <c r="E7" s="0" t="s">
         <v>207</v>

</xml_diff>

<commit_message>
plan de compras: Gilson extra y Shapo el viernes 23 (descargan el martes 27)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="264">
   <si>
     <t>fecha</t>
   </si>
@@ -617,6 +617,15 @@
   </si>
   <si>
     <t>dictado 20/10: Paraguay AS 2026-11-03</t>
+  </si>
+  <si>
+    <t>Gonzalo 21/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 21/10: carga extra viernes 23 (Gonzalo 21/10)</t>
+  </si>
+  <si>
+    <t>dictado 21/10: la de la tersa 20 que no cargo pasa al viernes 23 (Gonzalo 21/10)</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -849,7 +858,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -860,6 +869,8 @@
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1175,7 +1186,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K136"/>
+  <dimension ref="A1:K138"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -5576,6 +5587,70 @@
       </c>
       <c r="J136" s="0" t="s">
         <v>196</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="11">
+        <v>46318</v>
+      </c>
+      <c r="B137" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C137" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="D137" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E137" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="F137" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G137" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H137" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I137" s="0" t="s">
+        <v>197</v>
+      </c>
+      <c r="J137" s="0" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="12">
+        <v>46318</v>
+      </c>
+      <c r="B138" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C138" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="D138" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E138" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="F138" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G138" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H138" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I138" s="0" t="s">
+        <v>197</v>
+      </c>
+      <c r="J138" s="0" t="s">
+        <v>199</v>
       </c>
     </row>
   </sheetData>
@@ -5597,7 +5672,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5629,10 +5704,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3">
@@ -5649,10 +5724,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4">
@@ -5669,10 +5744,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="5">
@@ -5689,10 +5764,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="6">
@@ -5709,10 +5784,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7">
@@ -5729,10 +5804,10 @@
         <v>1313</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8">
@@ -5749,10 +5824,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9">
@@ -5769,10 +5844,10 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="10">
@@ -5789,7 +5864,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="11">
@@ -5806,7 +5881,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -5825,57 +5900,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -5923,10 +5998,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3">
@@ -5940,10 +6015,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4">
@@ -5957,10 +6032,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="5">
@@ -5968,16 +6043,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="6">
@@ -5991,10 +6066,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7">
@@ -6008,10 +6083,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="8">
@@ -6025,10 +6100,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="9">
@@ -6036,16 +6111,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="10">
@@ -6059,10 +6134,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11">
@@ -6076,10 +6151,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="12">
@@ -6093,10 +6168,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="13">
@@ -6104,16 +6179,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -6147,10 +6222,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6176,7 +6251,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3">
@@ -6199,7 +6274,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4">
@@ -6222,7 +6297,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5">
@@ -6233,7 +6308,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6245,7 +6320,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6">
@@ -6268,7 +6343,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="7">
@@ -6291,7 +6366,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="8">
@@ -6314,7 +6389,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9">
@@ -6325,7 +6400,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6337,7 +6412,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="10">
@@ -6360,7 +6435,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="11">
@@ -6383,7 +6458,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="12">
@@ -6406,7 +6481,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="13">
@@ -6417,7 +6492,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6429,7 +6504,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="14">
@@ -6452,7 +6527,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="15">
@@ -6463,7 +6538,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6475,7 +6550,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="16">
@@ -6498,7 +6573,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="17">
@@ -6521,7 +6596,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -6542,10 +6617,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6553,46 +6628,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
   </sheetData>
@@ -6613,10 +6688,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6628,10 +6703,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6661,7 +6736,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3">
@@ -6688,7 +6763,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4">
@@ -6715,7 +6790,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="5">
@@ -6742,7 +6817,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="6">
@@ -6769,7 +6844,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="7">
@@ -6796,7 +6871,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8">
@@ -6823,7 +6898,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="9">
@@ -6850,7 +6925,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="10">
@@ -6877,7 +6952,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="11">
@@ -6904,7 +6979,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="12">
@@ -6931,7 +7006,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="13">
@@ -6958,12 +7033,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Milciades carga lunes 26/10 (Paraguay 3)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="265">
   <si>
     <t>fecha</t>
   </si>
@@ -626,6 +626,9 @@
   </si>
   <si>
     <t>dictado 21/10: la de la tersa 20 que no cargo pasa al viernes 23 (Gonzalo 21/10)</t>
+  </si>
+  <si>
+    <t>dictado 21/10: Milciades lunes (Paraguay 3: Guido, Alvarito, Milciades)</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -858,7 +861,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -869,6 +872,7 @@
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -1186,7 +1190,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K138"/>
+  <dimension ref="A1:K139"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -5651,6 +5655,38 @@
       </c>
       <c r="J138" s="0" t="s">
         <v>199</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B139" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C139" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D139" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E139" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="F139" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G139" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H139" s="0">
+        <v>980</v>
+      </c>
+      <c r="I139" s="0" t="s">
+        <v>197</v>
+      </c>
+      <c r="J139" s="0" t="s">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -5672,7 +5708,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5704,10 +5740,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3">
@@ -5724,10 +5760,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4">
@@ -5744,10 +5780,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5">
@@ -5764,10 +5800,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6">
@@ -5784,10 +5820,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7">
@@ -5804,10 +5840,10 @@
         <v>1313</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="8">
@@ -5824,10 +5860,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9">
@@ -5844,10 +5880,10 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10">
@@ -5864,7 +5900,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11">
@@ -5881,7 +5917,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -5900,57 +5936,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -5998,10 +6034,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="3">
@@ -6015,10 +6051,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4">
@@ -6032,10 +6068,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5">
@@ -6043,16 +6079,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="6">
@@ -6066,10 +6102,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="7">
@@ -6083,10 +6119,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8">
@@ -6100,10 +6136,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9">
@@ -6111,16 +6147,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10">
@@ -6134,10 +6170,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="11">
@@ -6151,10 +6187,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12">
@@ -6168,10 +6204,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="13">
@@ -6179,16 +6215,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -6222,10 +6258,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6251,7 +6287,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3">
@@ -6274,7 +6310,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4">
@@ -6297,7 +6333,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5">
@@ -6308,7 +6344,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6320,7 +6356,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6">
@@ -6343,7 +6379,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7">
@@ -6366,7 +6402,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8">
@@ -6389,7 +6425,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9">
@@ -6400,7 +6436,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6412,7 +6448,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10">
@@ -6435,7 +6471,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="11">
@@ -6458,7 +6494,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="12">
@@ -6481,7 +6517,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="13">
@@ -6492,7 +6528,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6504,7 +6540,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="14">
@@ -6527,7 +6563,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15">
@@ -6538,7 +6574,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6550,7 +6586,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16">
@@ -6573,7 +6609,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="17">
@@ -6596,7 +6632,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -6617,10 +6653,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6628,46 +6664,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>
@@ -6688,10 +6724,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6703,10 +6739,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6736,7 +6772,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3">
@@ -6763,7 +6799,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4">
@@ -6790,7 +6826,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5">
@@ -6817,7 +6853,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6">
@@ -6844,7 +6880,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="7">
@@ -6871,7 +6907,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="8">
@@ -6898,7 +6934,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9">
@@ -6925,7 +6961,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10">
@@ -6952,7 +6988,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="11">
@@ -6979,7 +7015,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="12">
@@ -7006,7 +7042,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="13">
@@ -7033,12 +7069,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: cruce con Aloha por camion y base fija del ERP; Fischer 30/10 y Jhony 31/10
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -493,7 +493,7 @@
     <t>dictado 20/10: Fisher 2026-10-27</t>
   </si>
   <si>
-    <t>dictado 20/10: Fisher 2026-10-28</t>
+    <t>dictado 20/10: Fisher 2026-10-28; 22/10: pasa de 28/10 a 30/10 (dictado)</t>
   </si>
   <si>
     <t>dictado 20/10: Cassio 2026-10-27</t>
@@ -514,7 +514,7 @@
     <t>dictado 20/10: BAHIA 2026-10-28</t>
   </si>
   <si>
-    <t>dictado 20/10: Jhony Viera 2026-10-27</t>
+    <t>dictado 20/10: Jhony Viera 2026-10-27; 22/10: pasa de 27/10 a 31/10 (dictado)</t>
   </si>
   <si>
     <t>dictado 20/10: Ivo zimer 2026-10-28</t>
@@ -4347,10 +4347,10 @@
     </row>
     <row r="98">
       <c r="A98" s="10">
-        <v>46323</v>
+        <v>46325</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C98" s="0" t="s">
         <v>152</v>
@@ -4571,10 +4571,10 @@
     </row>
     <row r="105">
       <c r="A105" s="10">
-        <v>46322</v>
+        <v>46326</v>
       </c>
       <c r="B105" s="0" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C105" s="0" t="s">
         <v>152</v>

</xml_diff>

<commit_message>
plan de compras: Ivo carga el miercoles 21, descarga el sabado 24
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -445,7 +445,7 @@
     <t>definitivo 16/10: Jony 1: tersa</t>
   </si>
   <si>
-    <t>definitivo 16/10: Ivo 1: tersa</t>
+    <t>definitivo 16/10: Ivo 1: tersa; 22/10: cargo el miercoles 21, no el martes 20 (Gonzalo)</t>
   </si>
   <si>
     <t>Jaime Zimerman</t>
@@ -4021,10 +4021,10 @@
     </row>
     <row r="88">
       <c r="A88" s="6">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C88" s="0" t="s">
         <v>116</v>

</xml_diff>

<commit_message>
plan de compras: semana de carga 26-31/10 definitiva
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="266">
   <si>
     <t>fecha</t>
   </si>
@@ -493,13 +493,13 @@
     <t>dictado 20/10: Fisher 2026-10-27</t>
   </si>
   <si>
-    <t>dictado 20/10: Fisher 2026-10-28; 22/10: pasa de 28/10 a 30/10 (dictado)</t>
+    <t>dictado 20/10: Fisher 2026-10-28; 22/10: pasa de 28/10 a 30/10 (dictado); 22/10 definitivo (Gonzalo)</t>
   </si>
   <si>
     <t>dictado 20/10: Cassio 2026-10-27</t>
   </si>
   <si>
-    <t>dictado 20/10: Cassio 2026-10-28</t>
+    <t>dictado 20/10: Cassio 2026-10-28; 22/10 definitivo (Gonzalo)</t>
   </si>
   <si>
     <t>dictado 20/10: Stein 2026-10-27</t>
@@ -511,28 +511,31 @@
     <t>dictado 20/10: Gilson 2026-10-28</t>
   </si>
   <si>
-    <t>dictado 20/10: BAHIA 2026-10-28</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Jhony Viera 2026-10-27; 22/10: pasa de 27/10 a 31/10 (dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Ivo zimer 2026-10-28</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Marconi 2026-10-28</t>
+    <t>Gral</t>
+  </si>
+  <si>
+    <t>dictado 20/10: BAHIA 2026-10-28; 22/10 definitivo (Gonzalo)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Jhony Viera 2026-10-27; 22/10: pasa de 27/10 a 31/10 (dictado); 22/10 definitivo (Gonzalo)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Ivo zimer 2026-10-28; 22/10 definitivo (Gonzalo)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Marconi 2026-10-28; 22/10 definitivo (Gonzalo)</t>
   </si>
   <si>
     <t>Aryste Mittelman</t>
   </si>
   <si>
-    <t>dictado 20/10: Aryste Mittelman 2026-10-28</t>
+    <t>dictado 20/10: Aryste Mittelman 2026-10-28; 22/10 definitivo (Gonzalo)</t>
   </si>
   <si>
     <t>dictado 20/10: Muller Fabricio 2026-10-31</t>
   </si>
   <si>
-    <t>dictado 20/10: Wagner 2026-10-31</t>
+    <t>dictado 20/10: Wagner 2026-10-31; 22/10 definitivo (Gonzalo)</t>
   </si>
   <si>
     <t>dictado 20/10: Jaime Zimerman 2026-10-31</t>
@@ -541,7 +544,7 @@
     <t>Andre Pauli</t>
   </si>
   <si>
-    <t>dictado 20/10: Andre Pauli 2026-10-31</t>
+    <t>dictado 20/10: Andre Pauli 2026-10-31; 22/10 definitivo (Gonzalo)</t>
   </si>
   <si>
     <t>dictado 20/10: Shapo 2026-10-31</t>
@@ -4347,10 +4350,10 @@
     </row>
     <row r="98">
       <c r="A98" s="10">
-        <v>46325</v>
+        <v>46323</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C98" s="0" t="s">
         <v>152</v>
@@ -4426,10 +4429,10 @@
         <v>27</v>
       </c>
       <c r="F100" s="0" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G100" s="0" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="H100" s="0">
         <v>1008</v>
@@ -4554,7 +4557,7 @@
         <v>130</v>
       </c>
       <c r="F104" s="0" t="s">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="G104" s="0" t="s">
         <v>15</v>
@@ -4566,15 +4569,15 @@
         <v>153</v>
       </c>
       <c r="J104" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="10">
-        <v>46326</v>
+        <v>46322</v>
       </c>
       <c r="B105" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C105" s="0" t="s">
         <v>152</v>
@@ -4598,7 +4601,7 @@
         <v>153</v>
       </c>
       <c r="J105" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="106">
@@ -4618,10 +4621,10 @@
         <v>25</v>
       </c>
       <c r="F106" s="0" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G106" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H106" s="0">
         <v>1008</v>
@@ -4630,7 +4633,7 @@
         <v>153</v>
       </c>
       <c r="J106" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="107">
@@ -4650,10 +4653,10 @@
         <v>60</v>
       </c>
       <c r="F107" s="0" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G107" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H107" s="0">
         <v>1008</v>
@@ -4662,7 +4665,7 @@
         <v>153</v>
       </c>
       <c r="J107" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="108">
@@ -4679,10 +4682,10 @@
         <v>24</v>
       </c>
       <c r="E108" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F108" s="0" t="s">
-        <v>15</v>
+        <v>56</v>
       </c>
       <c r="G108" s="0" t="s">
         <v>15</v>
@@ -4694,7 +4697,7 @@
         <v>153</v>
       </c>
       <c r="J108" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="109">
@@ -4726,7 +4729,7 @@
         <v>153</v>
       </c>
       <c r="J109" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="110">
@@ -4746,10 +4749,10 @@
         <v>146</v>
       </c>
       <c r="F110" s="0" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G110" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H110" s="0">
         <v>1008</v>
@@ -4758,7 +4761,7 @@
         <v>153</v>
       </c>
       <c r="J110" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="111">
@@ -4790,7 +4793,7 @@
         <v>153</v>
       </c>
       <c r="J111" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="112">
@@ -4807,10 +4810,10 @@
         <v>24</v>
       </c>
       <c r="E112" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F112" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G112" s="0" t="s">
         <v>15</v>
@@ -4822,7 +4825,7 @@
         <v>153</v>
       </c>
       <c r="J112" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="113">
@@ -4854,7 +4857,7 @@
         <v>153</v>
       </c>
       <c r="J113" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="114">
@@ -4886,7 +4889,7 @@
         <v>153</v>
       </c>
       <c r="J114" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="115">
@@ -4918,7 +4921,7 @@
         <v>153</v>
       </c>
       <c r="J115" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="116">
@@ -4929,7 +4932,7 @@
         <v>52</v>
       </c>
       <c r="C116" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D116" s="0" t="s">
         <v>24</v>
@@ -4950,7 +4953,7 @@
         <v>153</v>
       </c>
       <c r="J116" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="117">
@@ -4961,7 +4964,7 @@
         <v>23</v>
       </c>
       <c r="C117" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D117" s="0" t="s">
         <v>24</v>
@@ -4982,7 +4985,7 @@
         <v>153</v>
       </c>
       <c r="J117" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="118">
@@ -4993,7 +4996,7 @@
         <v>21</v>
       </c>
       <c r="C118" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D118" s="0" t="s">
         <v>24</v>
@@ -5014,7 +5017,7 @@
         <v>153</v>
       </c>
       <c r="J118" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="119">
@@ -5025,7 +5028,7 @@
         <v>23</v>
       </c>
       <c r="C119" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D119" s="0" t="s">
         <v>24</v>
@@ -5046,7 +5049,7 @@
         <v>153</v>
       </c>
       <c r="J119" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="120">
@@ -5057,7 +5060,7 @@
         <v>30</v>
       </c>
       <c r="C120" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D120" s="0" t="s">
         <v>24</v>
@@ -5078,7 +5081,7 @@
         <v>153</v>
       </c>
       <c r="J120" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="121">
@@ -5089,7 +5092,7 @@
         <v>21</v>
       </c>
       <c r="C121" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D121" s="0" t="s">
         <v>24</v>
@@ -5110,7 +5113,7 @@
         <v>153</v>
       </c>
       <c r="J121" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="122">
@@ -5121,7 +5124,7 @@
         <v>23</v>
       </c>
       <c r="C122" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D122" s="0" t="s">
         <v>24</v>
@@ -5142,7 +5145,7 @@
         <v>153</v>
       </c>
       <c r="J122" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="123">
@@ -5153,7 +5156,7 @@
         <v>21</v>
       </c>
       <c r="C123" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D123" s="0" t="s">
         <v>24</v>
@@ -5174,7 +5177,7 @@
         <v>153</v>
       </c>
       <c r="J123" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="124">
@@ -5185,7 +5188,7 @@
         <v>52</v>
       </c>
       <c r="C124" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D124" s="0" t="s">
         <v>24</v>
@@ -5206,7 +5209,7 @@
         <v>153</v>
       </c>
       <c r="J124" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="125">
@@ -5217,7 +5220,7 @@
         <v>23</v>
       </c>
       <c r="C125" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D125" s="0" t="s">
         <v>24</v>
@@ -5238,7 +5241,7 @@
         <v>153</v>
       </c>
       <c r="J125" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="126">
@@ -5249,7 +5252,7 @@
         <v>52</v>
       </c>
       <c r="C126" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D126" s="0" t="s">
         <v>24</v>
@@ -5270,7 +5273,7 @@
         <v>153</v>
       </c>
       <c r="J126" s="0" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="127">
@@ -5281,7 +5284,7 @@
         <v>23</v>
       </c>
       <c r="C127" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D127" s="0" t="s">
         <v>24</v>
@@ -5302,7 +5305,7 @@
         <v>153</v>
       </c>
       <c r="J127" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="128">
@@ -5313,7 +5316,7 @@
         <v>52</v>
       </c>
       <c r="C128" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D128" s="0" t="s">
         <v>24</v>
@@ -5334,7 +5337,7 @@
         <v>153</v>
       </c>
       <c r="J128" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="129">
@@ -5345,7 +5348,7 @@
         <v>23</v>
       </c>
       <c r="C129" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D129" s="0" t="s">
         <v>24</v>
@@ -5366,7 +5369,7 @@
         <v>153</v>
       </c>
       <c r="J129" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="130">
@@ -5377,7 +5380,7 @@
         <v>52</v>
       </c>
       <c r="C130" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D130" s="0" t="s">
         <v>24</v>
@@ -5398,7 +5401,7 @@
         <v>153</v>
       </c>
       <c r="J130" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="131">
@@ -5409,7 +5412,7 @@
         <v>23</v>
       </c>
       <c r="C131" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D131" s="0" t="s">
         <v>24</v>
@@ -5430,7 +5433,7 @@
         <v>153</v>
       </c>
       <c r="J131" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="132">
@@ -5441,7 +5444,7 @@
         <v>23</v>
       </c>
       <c r="C132" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D132" s="0" t="s">
         <v>24</v>
@@ -5462,7 +5465,7 @@
         <v>153</v>
       </c>
       <c r="J132" s="0" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="133">
@@ -5473,13 +5476,13 @@
         <v>23</v>
       </c>
       <c r="C133" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D133" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E133" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F133" s="0" t="s">
         <v>15</v>
@@ -5494,7 +5497,7 @@
         <v>153</v>
       </c>
       <c r="J133" s="0" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="134">
@@ -5505,13 +5508,13 @@
         <v>23</v>
       </c>
       <c r="C134" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D134" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E134" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F134" s="0" t="s">
         <v>15</v>
@@ -5526,7 +5529,7 @@
         <v>153</v>
       </c>
       <c r="J134" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="135">
@@ -5537,7 +5540,7 @@
         <v>19</v>
       </c>
       <c r="C135" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D135" s="0" t="s">
         <v>13</v>
@@ -5558,7 +5561,7 @@
         <v>153</v>
       </c>
       <c r="J135" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="136">
@@ -5569,7 +5572,7 @@
         <v>21</v>
       </c>
       <c r="C136" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D136" s="0" t="s">
         <v>13</v>
@@ -5590,7 +5593,7 @@
         <v>153</v>
       </c>
       <c r="J136" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="137">
@@ -5619,10 +5622,10 @@
         <v>1008</v>
       </c>
       <c r="I137" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J137" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="138">
@@ -5651,10 +5654,10 @@
         <v>1008</v>
       </c>
       <c r="I138" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J138" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="139">
@@ -5683,10 +5686,10 @@
         <v>980</v>
       </c>
       <c r="I139" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J139" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -5708,7 +5711,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5740,10 +5743,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3">
@@ -5760,10 +5763,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4">
@@ -5780,10 +5783,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5">
@@ -5800,10 +5803,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6">
@@ -5820,10 +5823,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7">
@@ -5840,10 +5843,10 @@
         <v>1313</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8">
@@ -5860,10 +5863,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9">
@@ -5880,10 +5883,10 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10">
@@ -5900,7 +5903,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11">
@@ -5917,7 +5920,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -5936,57 +5939,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -6034,10 +6037,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="3">
@@ -6051,10 +6054,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4">
@@ -6068,10 +6071,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5">
@@ -6079,16 +6082,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6">
@@ -6102,10 +6105,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7">
@@ -6119,10 +6122,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8">
@@ -6136,10 +6139,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9">
@@ -6147,16 +6150,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="10">
@@ -6170,10 +6173,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11">
@@ -6187,10 +6190,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="12">
@@ -6204,10 +6207,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13">
@@ -6215,16 +6218,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -6258,10 +6261,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6287,7 +6290,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3">
@@ -6310,7 +6313,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4">
@@ -6333,7 +6336,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5">
@@ -6344,7 +6347,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6356,7 +6359,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6">
@@ -6379,7 +6382,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7">
@@ -6402,7 +6405,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="8">
@@ -6425,7 +6428,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="9">
@@ -6436,7 +6439,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6448,7 +6451,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="10">
@@ -6471,7 +6474,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11">
@@ -6494,7 +6497,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12">
@@ -6517,7 +6520,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13">
@@ -6528,7 +6531,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6540,7 +6543,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="14">
@@ -6563,7 +6566,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="15">
@@ -6574,7 +6577,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6586,7 +6589,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16">
@@ -6609,7 +6612,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="17">
@@ -6632,7 +6635,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -6653,10 +6656,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6664,46 +6667,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B4" s="0">
         <v>27000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -6724,10 +6727,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6739,10 +6742,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6772,7 +6775,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="3">
@@ -6799,7 +6802,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4">
@@ -6826,7 +6829,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5">
@@ -6853,7 +6856,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="6">
@@ -6880,7 +6883,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="7">
@@ -6907,7 +6910,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="8">
@@ -6934,7 +6937,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="9">
@@ -6961,7 +6964,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="10">
@@ -6988,7 +6991,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="11">
@@ -7015,7 +7018,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="12">
@@ -7042,7 +7045,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="13">
@@ -7069,12 +7072,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: sin transportistas supuestos en la semana 2-7/11
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -559,55 +559,55 @@
     <t>2026-11-01</t>
   </si>
   <si>
-    <t>dictado 20/10: Fisher 2026-11-04</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Fisher 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Cassio 2026-11-03</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Cassio 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Cassio 2026-11-07</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Gilson 2026-11-03</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Gilson 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Stein 2026-11-03</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Stein 2026-11-04</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Stein 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Agrocurupa 2026-11-04</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Agrocurupa 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Muller Fabricio 2026-11-04</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Muller Fabricio 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Ivo zimer 2026-11-04</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Ivo zimer 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Jaime Zimerman 2026-11-06</t>
+    <t>dictado 20/10: Fisher 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Fisher 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Cassio 2026-11-03; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Cassio 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Cassio 2026-11-07; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Gilson 2026-11-03; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Gilson 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Stein 2026-11-03; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Stein 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Stein 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Agrocurupa 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Agrocurupa 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Muller Fabricio 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Muller Fabricio 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Ivo zimer 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Ivo zimer 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Jaime Zimerman 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
   </si>
   <si>
     <t>dictado 20/10: Aryste Mittelman 2026-11-06</t>
@@ -4940,12 +4940,6 @@
       <c r="E116" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="F116" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="G116" s="0" t="s">
-        <v>35</v>
-      </c>
       <c r="H116" s="0">
         <v>1008</v>
       </c>
@@ -4972,12 +4966,6 @@
       <c r="E117" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="F117" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="G117" s="0" t="s">
-        <v>35</v>
-      </c>
       <c r="H117" s="0">
         <v>1008</v>
       </c>
@@ -5004,12 +4992,6 @@
       <c r="E118" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="F118" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="G118" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="H118" s="0">
         <v>1008</v>
       </c>
@@ -5036,12 +5018,6 @@
       <c r="E119" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="F119" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="G119" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="H119" s="0">
         <v>1008</v>
       </c>
@@ -5068,12 +5044,6 @@
       <c r="E120" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="F120" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="G120" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="H120" s="0">
         <v>1008</v>
       </c>
@@ -5100,12 +5070,6 @@
       <c r="E121" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="F121" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G121" s="0" t="s">
-        <v>35</v>
-      </c>
       <c r="H121" s="0">
         <v>1008</v>
       </c>
@@ -5132,12 +5096,6 @@
       <c r="E122" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="F122" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G122" s="0" t="s">
-        <v>35</v>
-      </c>
       <c r="H122" s="0">
         <v>1008</v>
       </c>
@@ -5164,12 +5122,6 @@
       <c r="E123" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="F123" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="G123" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="H123" s="0">
         <v>1008</v>
       </c>
@@ -5196,12 +5148,6 @@
       <c r="E124" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="F124" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="G124" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="H124" s="0">
         <v>1008</v>
       </c>
@@ -5228,12 +5174,6 @@
       <c r="E125" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="F125" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="G125" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="H125" s="0">
         <v>1008</v>
       </c>
@@ -5260,12 +5200,6 @@
       <c r="E126" s="0" t="s">
         <v>40</v>
       </c>
-      <c r="F126" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G126" s="0" t="s">
-        <v>35</v>
-      </c>
       <c r="H126" s="0">
         <v>1008</v>
       </c>
@@ -5292,12 +5226,6 @@
       <c r="E127" s="0" t="s">
         <v>40</v>
       </c>
-      <c r="F127" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G127" s="0" t="s">
-        <v>35</v>
-      </c>
       <c r="H127" s="0">
         <v>1008</v>
       </c>
@@ -5324,12 +5252,6 @@
       <c r="E128" s="0" t="s">
         <v>122</v>
       </c>
-      <c r="F128" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="G128" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="H128" s="0">
         <v>1008</v>
       </c>
@@ -5356,12 +5278,6 @@
       <c r="E129" s="0" t="s">
         <v>122</v>
       </c>
-      <c r="F129" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="G129" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="H129" s="0">
         <v>1008</v>
       </c>
@@ -5388,12 +5304,6 @@
       <c r="E130" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="F130" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G130" s="0" t="s">
-        <v>35</v>
-      </c>
       <c r="H130" s="0">
         <v>1008</v>
       </c>
@@ -5420,12 +5330,6 @@
       <c r="E131" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="F131" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G131" s="0" t="s">
-        <v>35</v>
-      </c>
       <c r="H131" s="0">
         <v>1008</v>
       </c>
@@ -5451,12 +5355,6 @@
       </c>
       <c r="E132" s="0" t="s">
         <v>140</v>
-      </c>
-      <c r="F132" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G132" s="0" t="s">
-        <v>35</v>
       </c>
       <c r="H132" s="0">
         <v>1008</v>

</xml_diff>

<commit_message>
plan de compras: objetivo del sabado 30.000 (maduracion lenta, protocolo invierno)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -805,7 +805,7 @@
     <t>minimo_cajas_sabado</t>
   </si>
   <si>
-    <t>Gonzalo 14/10/2026: "Uruguay quiere cierre de los sabados a 27 mil" (antes 25.000 desde el 01/10; 22.500 antes)</t>
+    <t>Gonzalo 22/10: Uruguay sube el stock a 30 mil (Charlie: la banana tarda mas en tomar color, protocolo invierno)</t>
   </si>
   <si>
     <t>venta_minima_semana</t>
@@ -6590,7 +6590,7 @@
         <v>258</v>
       </c>
       <c r="B4" s="0">
-        <v>27000</v>
+        <v>30000</v>
       </c>
       <c r="C4" s="0" t="s">
         <v>259</v>

</xml_diff>

<commit_message>
plan de compras: cancelada la carga de Guido del martes 27/10
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="265">
   <si>
     <t>fecha</t>
   </si>
@@ -551,9 +551,6 @@
   </si>
   <si>
     <t>dictado 20/10: Paraguay AS 2026-10-26</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Paraguay GM 2026-10-27</t>
   </si>
   <si>
     <t>2026-11-01</t>
@@ -1193,7 +1190,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K139"/>
+  <dimension ref="A1:K138"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -4894,45 +4891,39 @@
     </row>
     <row r="115">
       <c r="A115" s="10">
-        <v>46322</v>
+        <v>46330</v>
       </c>
       <c r="B115" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C115" s="0" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="D115" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E115" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="F115" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G115" s="0" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="H115" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I115" s="0" t="s">
         <v>153</v>
       </c>
       <c r="J115" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B116" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C116" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D116" s="0" t="s">
         <v>24</v>
@@ -4952,19 +4943,19 @@
     </row>
     <row r="117">
       <c r="A117" s="10">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B117" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C117" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D117" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E117" s="0" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="H117" s="0">
         <v>1008</v>
@@ -4978,13 +4969,13 @@
     </row>
     <row r="118">
       <c r="A118" s="10">
-        <v>46329</v>
+        <v>46332</v>
       </c>
       <c r="B118" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C118" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D118" s="0" t="s">
         <v>24</v>
@@ -5004,13 +4995,13 @@
     </row>
     <row r="119">
       <c r="A119" s="10">
-        <v>46332</v>
+        <v>46333</v>
       </c>
       <c r="B119" s="0" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C119" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D119" s="0" t="s">
         <v>24</v>
@@ -5030,19 +5021,19 @@
     </row>
     <row r="120">
       <c r="A120" s="10">
-        <v>46333</v>
+        <v>46329</v>
       </c>
       <c r="B120" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C120" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D120" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E120" s="0" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="H120" s="0">
         <v>1008</v>
@@ -5056,13 +5047,13 @@
     </row>
     <row r="121">
       <c r="A121" s="10">
-        <v>46329</v>
+        <v>46332</v>
       </c>
       <c r="B121" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C121" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D121" s="0" t="s">
         <v>24</v>
@@ -5082,19 +5073,19 @@
     </row>
     <row r="122">
       <c r="A122" s="10">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B122" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C122" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D122" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E122" s="0" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="H122" s="0">
         <v>1008</v>
@@ -5108,13 +5099,13 @@
     </row>
     <row r="123">
       <c r="A123" s="10">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="B123" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C123" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D123" s="0" t="s">
         <v>24</v>
@@ -5134,13 +5125,13 @@
     </row>
     <row r="124">
       <c r="A124" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B124" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C124" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D124" s="0" t="s">
         <v>24</v>
@@ -5160,19 +5151,19 @@
     </row>
     <row r="125">
       <c r="A125" s="10">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B125" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C125" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D125" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E125" s="0" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="H125" s="0">
         <v>1008</v>
@@ -5186,13 +5177,13 @@
     </row>
     <row r="126">
       <c r="A126" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B126" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C126" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D126" s="0" t="s">
         <v>24</v>
@@ -5212,19 +5203,19 @@
     </row>
     <row r="127">
       <c r="A127" s="10">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B127" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C127" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D127" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E127" s="0" t="s">
-        <v>40</v>
+        <v>122</v>
       </c>
       <c r="H127" s="0">
         <v>1008</v>
@@ -5238,13 +5229,13 @@
     </row>
     <row r="128">
       <c r="A128" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B128" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C128" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D128" s="0" t="s">
         <v>24</v>
@@ -5264,19 +5255,19 @@
     </row>
     <row r="129">
       <c r="A129" s="10">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B129" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C129" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D129" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E129" s="0" t="s">
-        <v>122</v>
+        <v>25</v>
       </c>
       <c r="H129" s="0">
         <v>1008</v>
@@ -5290,13 +5281,13 @@
     </row>
     <row r="130">
       <c r="A130" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B130" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C130" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D130" s="0" t="s">
         <v>24</v>
@@ -5322,13 +5313,13 @@
         <v>23</v>
       </c>
       <c r="C131" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D131" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E131" s="0" t="s">
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="H131" s="0">
         <v>1008</v>
@@ -5348,13 +5339,19 @@
         <v>23</v>
       </c>
       <c r="C132" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D132" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E132" s="0" t="s">
-        <v>140</v>
+        <v>166</v>
+      </c>
+      <c r="F132" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G132" s="0" t="s">
+        <v>15</v>
       </c>
       <c r="H132" s="0">
         <v>1008</v>
@@ -5374,13 +5371,13 @@
         <v>23</v>
       </c>
       <c r="C133" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D133" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E133" s="0" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="F133" s="0" t="s">
         <v>15</v>
@@ -5400,19 +5397,19 @@
     </row>
     <row r="134">
       <c r="A134" s="10">
-        <v>46332</v>
+        <v>46328</v>
       </c>
       <c r="B134" s="0" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C134" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D134" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E134" s="0" t="s">
-        <v>171</v>
+        <v>20</v>
       </c>
       <c r="F134" s="0" t="s">
         <v>15</v>
@@ -5421,7 +5418,7 @@
         <v>15</v>
       </c>
       <c r="H134" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I134" s="0" t="s">
         <v>153</v>
@@ -5432,19 +5429,19 @@
     </row>
     <row r="135">
       <c r="A135" s="10">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="B135" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C135" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D135" s="0" t="s">
         <v>13</v>
       </c>
       <c r="E135" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F135" s="0" t="s">
         <v>15</v>
@@ -5463,39 +5460,39 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="10">
-        <v>46329</v>
+      <c r="A136" s="11">
+        <v>46318</v>
       </c>
       <c r="B136" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C136" s="0" t="s">
-        <v>176</v>
+        <v>116</v>
       </c>
       <c r="D136" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E136" s="0" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="F136" s="0" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="G136" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H136" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I136" s="0" t="s">
-        <v>153</v>
+        <v>197</v>
       </c>
       <c r="J136" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="11">
+      <c r="A137" s="12">
         <v>46318</v>
       </c>
       <c r="B137" s="0" t="s">
@@ -5508,7 +5505,7 @@
         <v>24</v>
       </c>
       <c r="E137" s="0" t="s">
-        <v>43</v>
+        <v>105</v>
       </c>
       <c r="F137" s="0" t="s">
         <v>41</v>
@@ -5520,74 +5517,42 @@
         <v>1008</v>
       </c>
       <c r="I137" s="0" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J137" s="0" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="12">
-        <v>46318</v>
+      <c r="A138" s="13">
+        <v>46321</v>
       </c>
       <c r="B138" s="0" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C138" s="0" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="D138" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E138" s="0" t="s">
-        <v>105</v>
+        <v>20</v>
       </c>
       <c r="F138" s="0" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G138" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H138" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I138" s="0" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J138" s="0" t="s">
         <v>200</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="13">
-        <v>46321</v>
-      </c>
-      <c r="B139" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="C139" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="D139" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="E139" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="F139" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G139" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H139" s="0">
-        <v>980</v>
-      </c>
-      <c r="I139" s="0" t="s">
-        <v>198</v>
-      </c>
-      <c r="J139" s="0" t="s">
-        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -5609,7 +5574,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5641,10 +5606,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
+        <v>202</v>
+      </c>
+      <c r="F2" s="0" t="s">
         <v>203</v>
-      </c>
-      <c r="F2" s="0" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="3">
@@ -5661,10 +5626,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4">
@@ -5681,10 +5646,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="F4" s="0" t="s">
         <v>206</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="5">
@@ -5701,10 +5666,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="F5" s="0" t="s">
         <v>208</v>
-      </c>
-      <c r="F5" s="0" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="6">
@@ -5721,10 +5686,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="F6" s="0" t="s">
         <v>210</v>
-      </c>
-      <c r="F6" s="0" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="7">
@@ -5741,10 +5706,10 @@
         <v>1313</v>
       </c>
       <c r="E7" s="0" t="s">
+        <v>211</v>
+      </c>
+      <c r="F7" s="0" t="s">
         <v>212</v>
-      </c>
-      <c r="F7" s="0" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="8">
@@ -5761,10 +5726,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="F8" s="0" t="s">
         <v>214</v>
-      </c>
-      <c r="F8" s="0" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="9">
@@ -5781,10 +5746,10 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
+        <v>215</v>
+      </c>
+      <c r="F9" s="0" t="s">
         <v>216</v>
-      </c>
-      <c r="F9" s="0" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="10">
@@ -5801,7 +5766,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11">
@@ -5818,7 +5783,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -5837,57 +5802,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -5935,10 +5900,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="E2" s="0" t="s">
         <v>230</v>
-      </c>
-      <c r="E2" s="0" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="3">
@@ -5952,10 +5917,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4">
@@ -5969,10 +5934,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5">
@@ -5980,16 +5945,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="6">
@@ -6003,10 +5968,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
+        <v>235</v>
+      </c>
+      <c r="E6" s="0" t="s">
         <v>236</v>
-      </c>
-      <c r="E6" s="0" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="7">
@@ -6020,10 +5985,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8">
@@ -6037,10 +6002,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9">
@@ -6048,16 +6013,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10">
@@ -6071,10 +6036,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
+        <v>240</v>
+      </c>
+      <c r="E10" s="0" t="s">
         <v>241</v>
-      </c>
-      <c r="E10" s="0" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="11">
@@ -6088,10 +6053,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12">
@@ -6105,10 +6070,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="13">
@@ -6116,16 +6081,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -6159,10 +6124,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>246</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>247</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6188,7 +6153,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3">
@@ -6211,7 +6176,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4">
@@ -6234,7 +6199,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5">
@@ -6245,7 +6210,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6257,7 +6222,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6">
@@ -6280,7 +6245,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7">
@@ -6303,7 +6268,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8">
@@ -6326,7 +6291,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9">
@@ -6337,7 +6302,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6349,7 +6314,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10">
@@ -6372,7 +6337,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="11">
@@ -6395,7 +6360,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="12">
@@ -6418,7 +6383,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="13">
@@ -6429,7 +6394,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6441,7 +6406,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="14">
@@ -6464,7 +6429,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15">
@@ -6475,7 +6440,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6487,7 +6452,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16">
@@ -6510,7 +6475,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="17">
@@ -6533,7 +6498,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -6554,10 +6519,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
+        <v>251</v>
+      </c>
+      <c r="B1" s="0" t="s">
         <v>252</v>
-      </c>
-      <c r="B1" s="0" t="s">
-        <v>253</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6565,46 +6530,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B4" s="0">
         <v>30000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>
@@ -6625,10 +6590,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6640,10 +6605,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6673,7 +6638,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3">
@@ -6700,7 +6665,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4">
@@ -6727,7 +6692,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5">
@@ -6754,7 +6719,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6">
@@ -6781,7 +6746,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="7">
@@ -6808,7 +6773,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="8">
@@ -6835,7 +6800,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9">
@@ -6862,7 +6827,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10">
@@ -6889,7 +6854,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="11">
@@ -6916,7 +6881,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="12">
@@ -6943,7 +6908,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="13">
@@ -6970,12 +6935,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: canceladas las 8 cargas del miercoles 28/10 (feriado corrido al viernes 30)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="256">
   <si>
     <t>fecha</t>
   </si>
@@ -493,118 +493,91 @@
     <t>dictado 20/10: Fisher 2026-10-27</t>
   </si>
   <si>
-    <t>dictado 20/10: Fisher 2026-10-28; 22/10: pasa de 28/10 a 30/10 (dictado); 22/10 definitivo (Gonzalo)</t>
-  </si>
-  <si>
     <t>dictado 20/10: Cassio 2026-10-27</t>
   </si>
   <si>
-    <t>dictado 20/10: Cassio 2026-10-28; 22/10 definitivo (Gonzalo)</t>
-  </si>
-  <si>
     <t>dictado 20/10: Stein 2026-10-27</t>
   </si>
   <si>
-    <t>dictado 20/10: Agrocurupa 2026-10-28</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Gilson 2026-10-28</t>
-  </si>
-  <si>
-    <t>Gral</t>
-  </si>
-  <si>
-    <t>dictado 20/10: BAHIA 2026-10-28; 22/10 definitivo (Gonzalo)</t>
-  </si>
-  <si>
     <t>dictado 20/10: Jhony Viera 2026-10-27; 22/10: pasa de 27/10 a 31/10 (dictado); 22/10 definitivo (Gonzalo)</t>
   </si>
   <si>
-    <t>dictado 20/10: Ivo zimer 2026-10-28; 22/10 definitivo (Gonzalo)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Marconi 2026-10-28; 22/10 definitivo (Gonzalo)</t>
+    <t>dictado 20/10: Muller Fabricio 2026-10-31</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Wagner 2026-10-31; 22/10 definitivo (Gonzalo)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Jaime Zimerman 2026-10-31</t>
+  </si>
+  <si>
+    <t>Andre Pauli</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Andre Pauli 2026-10-31; 22/10 definitivo (Gonzalo)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Shapo 2026-10-31</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Paraguay AS 2026-10-26</t>
+  </si>
+  <si>
+    <t>2026-11-01</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Fisher 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Fisher 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Cassio 2026-11-03; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Cassio 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Cassio 2026-11-07; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Gilson 2026-11-03; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Gilson 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Stein 2026-11-03; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Stein 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Stein 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Agrocurupa 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Agrocurupa 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Muller Fabricio 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Muller Fabricio 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Ivo zimer 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Ivo zimer 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Jaime Zimerman 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
   </si>
   <si>
     <t>Aryste Mittelman</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Aryste Mittelman 2026-10-28; 22/10 definitivo (Gonzalo)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Muller Fabricio 2026-10-31</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Wagner 2026-10-31; 22/10 definitivo (Gonzalo)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Jaime Zimerman 2026-10-31</t>
-  </si>
-  <si>
-    <t>Andre Pauli</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Andre Pauli 2026-10-31; 22/10 definitivo (Gonzalo)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Shapo 2026-10-31</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Paraguay AS 2026-10-26</t>
-  </si>
-  <si>
-    <t>2026-11-01</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Fisher 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Fisher 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Cassio 2026-11-03; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Cassio 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Cassio 2026-11-07; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Gilson 2026-11-03; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Gilson 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Stein 2026-11-03; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Stein 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Stein 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Agrocurupa 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Agrocurupa 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Muller Fabricio 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Muller Fabricio 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Ivo zimer 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Ivo zimer 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Jaime Zimerman 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
   </si>
   <si>
     <t>dictado 20/10: Aryste Mittelman 2026-11-06</t>
@@ -1190,7 +1163,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K138"/>
+  <dimension ref="A1:K130"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -4347,10 +4320,10 @@
     </row>
     <row r="98">
       <c r="A98" s="10">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C98" s="0" t="s">
         <v>152</v>
@@ -4359,13 +4332,13 @@
         <v>24</v>
       </c>
       <c r="E98" s="0" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F98" s="0" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="G98" s="0" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H98" s="0">
         <v>1008</v>
@@ -4391,13 +4364,13 @@
         <v>24</v>
       </c>
       <c r="E99" s="0" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="F99" s="0" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="G99" s="0" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="H99" s="0">
         <v>1008</v>
@@ -4411,10 +4384,10 @@
     </row>
     <row r="100">
       <c r="A100" s="10">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="B100" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C100" s="0" t="s">
         <v>152</v>
@@ -4423,13 +4396,13 @@
         <v>24</v>
       </c>
       <c r="E100" s="0" t="s">
-        <v>27</v>
+        <v>113</v>
       </c>
       <c r="F100" s="0" t="s">
         <v>41</v>
       </c>
       <c r="G100" s="0" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H100" s="0">
         <v>1008</v>
@@ -4443,10 +4416,10 @@
     </row>
     <row r="101">
       <c r="A101" s="10">
-        <v>46322</v>
+        <v>46326</v>
       </c>
       <c r="B101" s="0" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C101" s="0" t="s">
         <v>152</v>
@@ -4455,7 +4428,7 @@
         <v>24</v>
       </c>
       <c r="E101" s="0" t="s">
-        <v>59</v>
+        <v>122</v>
       </c>
       <c r="F101" s="0" t="s">
         <v>56</v>
@@ -4475,10 +4448,10 @@
     </row>
     <row r="102">
       <c r="A102" s="10">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="B102" s="0" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C102" s="0" t="s">
         <v>152</v>
@@ -4487,13 +4460,13 @@
         <v>24</v>
       </c>
       <c r="E102" s="0" t="s">
-        <v>40</v>
+        <v>146</v>
       </c>
       <c r="F102" s="0" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G102" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H102" s="0">
         <v>1008</v>
@@ -4507,10 +4480,10 @@
     </row>
     <row r="103">
       <c r="A103" s="10">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="B103" s="0" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C103" s="0" t="s">
         <v>152</v>
@@ -4519,7 +4492,7 @@
         <v>24</v>
       </c>
       <c r="E103" s="0" t="s">
-        <v>43</v>
+        <v>140</v>
       </c>
       <c r="F103" s="0" t="s">
         <v>41</v>
@@ -4539,10 +4512,10 @@
     </row>
     <row r="104">
       <c r="A104" s="10">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="B104" s="0" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C104" s="0" t="s">
         <v>152</v>
@@ -4551,10 +4524,10 @@
         <v>24</v>
       </c>
       <c r="E104" s="0" t="s">
-        <v>130</v>
+        <v>161</v>
       </c>
       <c r="F104" s="0" t="s">
-        <v>161</v>
+        <v>41</v>
       </c>
       <c r="G104" s="0" t="s">
         <v>15</v>
@@ -4571,10 +4544,10 @@
     </row>
     <row r="105">
       <c r="A105" s="10">
-        <v>46322</v>
+        <v>46326</v>
       </c>
       <c r="B105" s="0" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C105" s="0" t="s">
         <v>152</v>
@@ -4583,7 +4556,7 @@
         <v>24</v>
       </c>
       <c r="E105" s="0" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="F105" s="0" t="s">
         <v>41</v>
@@ -4603,28 +4576,28 @@
     </row>
     <row r="106">
       <c r="A106" s="10">
-        <v>46323</v>
+        <v>46321</v>
       </c>
       <c r="B106" s="0" t="s">
-        <v>52</v>
+        <v>19</v>
       </c>
       <c r="C106" s="0" t="s">
         <v>152</v>
       </c>
       <c r="D106" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E106" s="0" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F106" s="0" t="s">
-        <v>56</v>
+        <v>15</v>
       </c>
       <c r="G106" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H106" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I106" s="0" t="s">
         <v>153</v>
@@ -4635,25 +4608,19 @@
     </row>
     <row r="107">
       <c r="A107" s="10">
-        <v>46323</v>
+        <v>46330</v>
       </c>
       <c r="B107" s="0" t="s">
         <v>52</v>
       </c>
       <c r="C107" s="0" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D107" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E107" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="F107" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="G107" s="0" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="H107" s="0">
         <v>1008</v>
@@ -4662,30 +4629,24 @@
         <v>153</v>
       </c>
       <c r="J107" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="10">
-        <v>46323</v>
+        <v>46332</v>
       </c>
       <c r="B108" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C108" s="0" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D108" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E108" s="0" t="s">
-        <v>166</v>
-      </c>
-      <c r="F108" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="G108" s="0" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="H108" s="0">
         <v>1008</v>
@@ -4699,25 +4660,19 @@
     </row>
     <row r="109">
       <c r="A109" s="10">
-        <v>46326</v>
+        <v>46329</v>
       </c>
       <c r="B109" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C109" s="0" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D109" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E109" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="F109" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="G109" s="0" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="H109" s="0">
         <v>1008</v>
@@ -4731,25 +4686,19 @@
     </row>
     <row r="110">
       <c r="A110" s="10">
-        <v>46326</v>
+        <v>46332</v>
       </c>
       <c r="B110" s="0" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C110" s="0" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D110" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E110" s="0" t="s">
-        <v>146</v>
-      </c>
-      <c r="F110" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="G110" s="0" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="H110" s="0">
         <v>1008</v>
@@ -4763,25 +4712,19 @@
     </row>
     <row r="111">
       <c r="A111" s="10">
-        <v>46326</v>
+        <v>46333</v>
       </c>
       <c r="B111" s="0" t="s">
         <v>30</v>
       </c>
       <c r="C111" s="0" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D111" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E111" s="0" t="s">
-        <v>140</v>
-      </c>
-      <c r="F111" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G111" s="0" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H111" s="0">
         <v>1008</v>
@@ -4795,25 +4738,19 @@
     </row>
     <row r="112">
       <c r="A112" s="10">
-        <v>46326</v>
+        <v>46329</v>
       </c>
       <c r="B112" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C112" s="0" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D112" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E112" s="0" t="s">
-        <v>171</v>
-      </c>
-      <c r="F112" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G112" s="0" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="H112" s="0">
         <v>1008</v>
@@ -4822,30 +4759,24 @@
         <v>153</v>
       </c>
       <c r="J112" s="0" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="10">
-        <v>46326</v>
+        <v>46332</v>
       </c>
       <c r="B113" s="0" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C113" s="0" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D113" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E113" s="0" t="s">
-        <v>105</v>
-      </c>
-      <c r="F113" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G113" s="0" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="H113" s="0">
         <v>1008</v>
@@ -4854,39 +4785,33 @@
         <v>153</v>
       </c>
       <c r="J113" s="0" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="10">
-        <v>46321</v>
+        <v>46329</v>
       </c>
       <c r="B114" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C114" s="0" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D114" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E114" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="F114" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G114" s="0" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="H114" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I114" s="0" t="s">
         <v>153</v>
       </c>
       <c r="J114" s="0" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="115">
@@ -4897,13 +4822,13 @@
         <v>52</v>
       </c>
       <c r="C115" s="0" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D115" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E115" s="0" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="H115" s="0">
         <v>1008</v>
@@ -4912,7 +4837,7 @@
         <v>153</v>
       </c>
       <c r="J115" s="0" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="116">
@@ -4923,13 +4848,13 @@
         <v>23</v>
       </c>
       <c r="C116" s="0" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D116" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E116" s="0" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="H116" s="0">
         <v>1008</v>
@@ -4938,24 +4863,24 @@
         <v>153</v>
       </c>
       <c r="J116" s="0" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="10">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="B117" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C117" s="0" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D117" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E117" s="0" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="H117" s="0">
         <v>1008</v>
@@ -4964,7 +4889,7 @@
         <v>153</v>
       </c>
       <c r="J117" s="0" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="118">
@@ -4975,13 +4900,13 @@
         <v>23</v>
       </c>
       <c r="C118" s="0" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D118" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E118" s="0" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="H118" s="0">
         <v>1008</v>
@@ -4990,24 +4915,24 @@
         <v>153</v>
       </c>
       <c r="J118" s="0" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="10">
-        <v>46333</v>
+        <v>46330</v>
       </c>
       <c r="B119" s="0" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="C119" s="0" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D119" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E119" s="0" t="s">
-        <v>27</v>
+        <v>122</v>
       </c>
       <c r="H119" s="0">
         <v>1008</v>
@@ -5016,24 +4941,24 @@
         <v>153</v>
       </c>
       <c r="J119" s="0" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="10">
-        <v>46329</v>
+        <v>46332</v>
       </c>
       <c r="B120" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C120" s="0" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D120" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E120" s="0" t="s">
-        <v>43</v>
+        <v>122</v>
       </c>
       <c r="H120" s="0">
         <v>1008</v>
@@ -5042,24 +4967,24 @@
         <v>153</v>
       </c>
       <c r="J120" s="0" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="10">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B121" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C121" s="0" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D121" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E121" s="0" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="H121" s="0">
         <v>1008</v>
@@ -5068,24 +4993,24 @@
         <v>153</v>
       </c>
       <c r="J121" s="0" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="10">
-        <v>46329</v>
+        <v>46332</v>
       </c>
       <c r="B122" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C122" s="0" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D122" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E122" s="0" t="s">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="H122" s="0">
         <v>1008</v>
@@ -5094,24 +5019,24 @@
         <v>153</v>
       </c>
       <c r="J122" s="0" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B123" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C123" s="0" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D123" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E123" s="0" t="s">
-        <v>59</v>
+        <v>140</v>
       </c>
       <c r="H123" s="0">
         <v>1008</v>
@@ -5120,7 +5045,7 @@
         <v>153</v>
       </c>
       <c r="J123" s="0" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="124">
@@ -5131,13 +5056,19 @@
         <v>23</v>
       </c>
       <c r="C124" s="0" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D124" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E124" s="0" t="s">
-        <v>59</v>
+        <v>183</v>
+      </c>
+      <c r="F124" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G124" s="0" t="s">
+        <v>15</v>
       </c>
       <c r="H124" s="0">
         <v>1008</v>
@@ -5146,24 +5077,30 @@
         <v>153</v>
       </c>
       <c r="J124" s="0" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="10">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B125" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C125" s="0" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D125" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E125" s="0" t="s">
-        <v>40</v>
+        <v>161</v>
+      </c>
+      <c r="F125" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G125" s="0" t="s">
+        <v>15</v>
       </c>
       <c r="H125" s="0">
         <v>1008</v>
@@ -5172,387 +5109,167 @@
         <v>153</v>
       </c>
       <c r="J125" s="0" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="10">
-        <v>46332</v>
+        <v>46328</v>
       </c>
       <c r="B126" s="0" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C126" s="0" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D126" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E126" s="0" t="s">
-        <v>40</v>
+        <v>20</v>
+      </c>
+      <c r="F126" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G126" s="0" t="s">
+        <v>15</v>
       </c>
       <c r="H126" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I126" s="0" t="s">
         <v>153</v>
       </c>
       <c r="J126" s="0" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="10">
-        <v>46330</v>
+        <v>46329</v>
       </c>
       <c r="B127" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C127" s="0" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D127" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E127" s="0" t="s">
-        <v>122</v>
+        <v>22</v>
+      </c>
+      <c r="F127" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G127" s="0" t="s">
+        <v>15</v>
       </c>
       <c r="H127" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I127" s="0" t="s">
         <v>153</v>
       </c>
       <c r="J127" s="0" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="10">
-        <v>46332</v>
+      <c r="A128" s="11">
+        <v>46318</v>
       </c>
       <c r="B128" s="0" t="s">
         <v>23</v>
       </c>
       <c r="C128" s="0" t="s">
-        <v>175</v>
+        <v>116</v>
       </c>
       <c r="D128" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E128" s="0" t="s">
-        <v>122</v>
+        <v>43</v>
+      </c>
+      <c r="F128" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G128" s="0" t="s">
+        <v>35</v>
       </c>
       <c r="H128" s="0">
         <v>1008</v>
       </c>
       <c r="I128" s="0" t="s">
-        <v>153</v>
+        <v>188</v>
       </c>
       <c r="J128" s="0" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="10">
-        <v>46330</v>
+      <c r="A129" s="12">
+        <v>46318</v>
       </c>
       <c r="B129" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C129" s="0" t="s">
-        <v>175</v>
+        <v>116</v>
       </c>
       <c r="D129" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E129" s="0" t="s">
-        <v>25</v>
+        <v>105</v>
+      </c>
+      <c r="F129" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G129" s="0" t="s">
+        <v>35</v>
       </c>
       <c r="H129" s="0">
         <v>1008</v>
       </c>
       <c r="I129" s="0" t="s">
-        <v>153</v>
+        <v>188</v>
       </c>
       <c r="J129" s="0" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="10">
-        <v>46332</v>
+      <c r="A130" s="13">
+        <v>46321</v>
       </c>
       <c r="B130" s="0" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C130" s="0" t="s">
-        <v>175</v>
+        <v>152</v>
       </c>
       <c r="D130" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E130" s="0" t="s">
-        <v>25</v>
+        <v>20</v>
+      </c>
+      <c r="F130" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G130" s="0" t="s">
+        <v>15</v>
       </c>
       <c r="H130" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I130" s="0" t="s">
-        <v>153</v>
+        <v>188</v>
       </c>
       <c r="J130" s="0" t="s">
         <v>191</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="10">
-        <v>46332</v>
-      </c>
-      <c r="B131" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C131" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="D131" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E131" s="0" t="s">
-        <v>140</v>
-      </c>
-      <c r="H131" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I131" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="J131" s="0" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="10">
-        <v>46332</v>
-      </c>
-      <c r="B132" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C132" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="D132" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E132" s="0" t="s">
-        <v>166</v>
-      </c>
-      <c r="F132" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G132" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H132" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I132" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="J132" s="0" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="10">
-        <v>46332</v>
-      </c>
-      <c r="B133" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C133" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="D133" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E133" s="0" t="s">
-        <v>171</v>
-      </c>
-      <c r="F133" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G133" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H133" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I133" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="J133" s="0" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="10">
-        <v>46328</v>
-      </c>
-      <c r="B134" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="C134" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="D134" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="E134" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="F134" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G134" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H134" s="0">
-        <v>980</v>
-      </c>
-      <c r="I134" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="J134" s="0" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="10">
-        <v>46329</v>
-      </c>
-      <c r="B135" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="C135" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="D135" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="E135" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="F135" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G135" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H135" s="0">
-        <v>980</v>
-      </c>
-      <c r="I135" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="J135" s="0" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="11">
-        <v>46318</v>
-      </c>
-      <c r="B136" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C136" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="D136" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E136" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="F136" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G136" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="H136" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I136" s="0" t="s">
-        <v>197</v>
-      </c>
-      <c r="J136" s="0" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="12">
-        <v>46318</v>
-      </c>
-      <c r="B137" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C137" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="D137" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E137" s="0" t="s">
-        <v>105</v>
-      </c>
-      <c r="F137" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G137" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="H137" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I137" s="0" t="s">
-        <v>197</v>
-      </c>
-      <c r="J137" s="0" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="13">
-        <v>46321</v>
-      </c>
-      <c r="B138" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="C138" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="D138" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="E138" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="F138" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G138" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H138" s="0">
-        <v>980</v>
-      </c>
-      <c r="I138" s="0" t="s">
-        <v>197</v>
-      </c>
-      <c r="J138" s="0" t="s">
-        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -5574,7 +5291,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5606,10 +5323,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3">
@@ -5626,10 +5343,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4">
@@ -5646,10 +5363,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5">
@@ -5666,10 +5383,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6">
@@ -5686,10 +5403,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7">
@@ -5706,10 +5423,10 @@
         <v>1313</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
     </row>
     <row r="8">
@@ -5726,10 +5443,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9">
@@ -5746,10 +5463,10 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
     </row>
     <row r="10">
@@ -5766,7 +5483,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
     </row>
     <row r="11">
@@ -5783,7 +5500,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -5802,57 +5519,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -5900,10 +5617,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
     </row>
     <row r="3">
@@ -5917,10 +5634,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4">
@@ -5934,10 +5651,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5">
@@ -5945,16 +5662,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6">
@@ -5968,10 +5685,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
     </row>
     <row r="7">
@@ -5985,10 +5702,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8">
@@ -6002,10 +5719,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9">
@@ -6013,16 +5730,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
     </row>
     <row r="10">
@@ -6036,10 +5753,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="11">
@@ -6053,10 +5770,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
     </row>
     <row r="12">
@@ -6070,10 +5787,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="13">
@@ -6081,16 +5798,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -6124,10 +5841,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6153,7 +5870,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3">
@@ -6176,7 +5893,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4">
@@ -6199,7 +5916,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5">
@@ -6210,7 +5927,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6222,7 +5939,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6">
@@ -6245,7 +5962,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
     </row>
     <row r="7">
@@ -6268,7 +5985,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
     </row>
     <row r="8">
@@ -6291,7 +6008,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9">
@@ -6302,7 +6019,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6314,7 +6031,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10">
@@ -6337,7 +6054,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11">
@@ -6360,7 +6077,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
     </row>
     <row r="12">
@@ -6383,7 +6100,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
     </row>
     <row r="13">
@@ -6394,7 +6111,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6406,7 +6123,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14">
@@ -6429,7 +6146,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
     </row>
     <row r="15">
@@ -6440,7 +6157,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6452,7 +6169,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
     </row>
     <row r="16">
@@ -6475,7 +6192,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
     </row>
     <row r="17">
@@ -6498,7 +6215,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>
@@ -6519,10 +6236,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6530,46 +6247,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="B4" s="0">
         <v>30000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>258</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -6590,10 +6307,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6605,10 +6322,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6638,7 +6355,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3">
@@ -6665,7 +6382,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4">
@@ -6692,7 +6409,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5">
@@ -6719,7 +6436,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6">
@@ -6746,7 +6463,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7">
@@ -6773,7 +6490,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8">
@@ -6800,7 +6517,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9">
@@ -6827,7 +6544,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10">
@@ -6854,7 +6571,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
     </row>
     <row r="11">
@@ -6881,7 +6598,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
     </row>
     <row r="12">
@@ -6908,7 +6625,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13">
@@ -6935,12 +6652,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: dictado 27/10 de la semana 26-31 (miercoles con descarga viernes, viernes y sabado al mie 4)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="265">
   <si>
     <t>fecha</t>
   </si>
@@ -602,6 +602,33 @@
   </si>
   <si>
     <t>dictado 21/10: Milciades lunes (Paraguay 3: Guido, Alvarito, Milciades)</t>
+  </si>
+  <si>
+    <t>Gonzalo 27/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 27/10: carga mie 28, descarga vie 30 confirmada (Gonzalo)</t>
+  </si>
+  <si>
+    <t>2026-10-30</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Fisher 2026-10-30</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Agrocurupa 2026-10-30</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Marconi 2026-10-31</t>
+  </si>
+  <si>
+    <t>Gral</t>
+  </si>
+  <si>
+    <t>dictado 27/10: carga mie 28, descarga sab 31 confirmada (Gonzalo)</t>
+  </si>
+  <si>
+    <t>2026-10-31</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -834,7 +861,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -845,6 +872,8 @@
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -1163,7 +1192,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K130"/>
+  <dimension ref="A1:K137"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -5270,6 +5299,221 @@
       </c>
       <c r="J130" s="0" t="s">
         <v>191</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="14">
+        <v>46323</v>
+      </c>
+      <c r="B131" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C131" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D131" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E131" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F131" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="H131" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I131" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="J131" s="0" t="s">
+        <v>193</v>
+      </c>
+      <c r="K131" s="0" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="14">
+        <v>46323</v>
+      </c>
+      <c r="B132" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C132" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D132" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E132" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F132" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="H132" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I132" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="J132" s="0" t="s">
+        <v>193</v>
+      </c>
+      <c r="K132" s="0" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="14">
+        <v>46323</v>
+      </c>
+      <c r="B133" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C133" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D133" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E133" s="0" t="s">
+        <v>183</v>
+      </c>
+      <c r="F133" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="H133" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I133" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="J133" s="0" t="s">
+        <v>193</v>
+      </c>
+      <c r="K133" s="0" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="14">
+        <v>46325</v>
+      </c>
+      <c r="B134" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C134" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D134" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E134" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="F134" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="H134" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I134" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="J134" s="0" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="14">
+        <v>46325</v>
+      </c>
+      <c r="B135" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C135" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D135" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E135" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="F135" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="H135" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I135" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="J135" s="0" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="14">
+        <v>46326</v>
+      </c>
+      <c r="B136" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="C136" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D136" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E136" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="F136" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="H136" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I136" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="J136" s="0" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="15">
+        <v>46323</v>
+      </c>
+      <c r="B137" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C137" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D137" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E137" s="0" t="s">
+        <v>130</v>
+      </c>
+      <c r="F137" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="H137" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I137" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="J137" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="K137" s="0" t="s">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -5291,7 +5535,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5323,10 +5567,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3">
@@ -5343,10 +5587,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4">
@@ -5363,10 +5607,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5">
@@ -5383,10 +5627,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6">
@@ -5403,10 +5647,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7">
@@ -5423,10 +5667,10 @@
         <v>1313</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
     </row>
     <row r="8">
@@ -5443,10 +5687,10 @@
         <v>1353</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9">
@@ -5463,10 +5707,10 @@
         <v>1056</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10">
@@ -5483,7 +5727,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11">
@@ -5500,7 +5744,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -5519,57 +5763,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -5617,10 +5861,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
     </row>
     <row r="3">
@@ -5634,10 +5878,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4">
@@ -5651,10 +5895,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5">
@@ -5662,16 +5906,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
     </row>
     <row r="6">
@@ -5685,10 +5929,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
     </row>
     <row r="7">
@@ -5702,10 +5946,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8">
@@ -5719,10 +5963,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9">
@@ -5730,16 +5974,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10">
@@ -5753,10 +5997,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
     </row>
     <row r="11">
@@ -5770,10 +6014,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12">
@@ -5787,10 +6031,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
     </row>
     <row r="13">
@@ -5798,16 +6042,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -5841,10 +6085,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -5870,7 +6114,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3">
@@ -5893,7 +6137,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4">
@@ -5916,7 +6160,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5">
@@ -5927,7 +6171,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -5939,7 +6183,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6">
@@ -5962,7 +6206,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7">
@@ -5985,7 +6229,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8">
@@ -6008,7 +6252,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9">
@@ -6019,7 +6263,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6031,7 +6275,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10">
@@ -6054,7 +6298,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="11">
@@ -6077,7 +6321,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="12">
@@ -6100,7 +6344,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="13">
@@ -6111,7 +6355,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6123,7 +6367,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="14">
@@ -6146,7 +6390,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15">
@@ -6157,7 +6401,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6169,7 +6413,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16">
@@ -6192,7 +6436,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
     </row>
     <row r="17">
@@ -6215,7 +6459,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -6236,10 +6480,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6247,46 +6491,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="B4" s="0">
         <v>30000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>
@@ -6307,10 +6551,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6322,10 +6566,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6355,7 +6599,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3">
@@ -6382,7 +6626,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4">
@@ -6409,7 +6653,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5">
@@ -6436,7 +6680,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6">
@@ -6463,7 +6707,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="7">
@@ -6490,7 +6734,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="8">
@@ -6517,7 +6761,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9">
@@ -6544,7 +6788,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10">
@@ -6571,7 +6815,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="11">
@@ -6598,7 +6842,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="12">
@@ -6625,7 +6869,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="13">
@@ -6652,12 +6896,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: dictado semana 2-7/11 y venta 22.000 / 18.000
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="266">
   <si>
     <t>fecha</t>
   </si>
@@ -526,93 +526,36 @@
     <t>2026-11-01</t>
   </si>
   <si>
-    <t>dictado 20/10: Fisher 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Fisher 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Cassio 2026-11-03; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Cassio 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Cassio 2026-11-07; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Gilson 2026-11-03; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Gilson 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Stein 2026-11-03; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Stein 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Stein 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Agrocurupa 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Agrocurupa 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Muller Fabricio 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Muller Fabricio 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Ivo zimer 2026-11-04; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Ivo zimer 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Jaime Zimerman 2026-11-06; 22/10: transportista borrado (lo habia puesto yo, no dictado)</t>
+    <t>dictado 20/10: Paraguay MS 2026-11-02</t>
+  </si>
+  <si>
+    <t>dictado 20/10: Paraguay AS 2026-11-03</t>
+  </si>
+  <si>
+    <t>Gonzalo 21/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 21/10: carga extra viernes 23 (Gonzalo 21/10)</t>
+  </si>
+  <si>
+    <t>dictado 21/10: la de la tersa 20 que no cargo pasa al viernes 23 (Gonzalo 21/10)</t>
+  </si>
+  <si>
+    <t>dictado 21/10: Milciades lunes (Paraguay 3: Guido, Alvarito, Milciades)</t>
+  </si>
+  <si>
+    <t>Gonzalo 27/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 27/10: carga mie 28, descarga vie 30 confirmada (Gonzalo)</t>
+  </si>
+  <si>
+    <t>2026-10-30</t>
   </si>
   <si>
     <t>Aryste Mittelman</t>
   </si>
   <si>
-    <t>dictado 20/10: Aryste Mittelman 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Andre Pauli 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Paraguay MS 2026-11-02</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Paraguay AS 2026-11-03</t>
-  </si>
-  <si>
-    <t>Gonzalo 21/10 (chat)</t>
-  </si>
-  <si>
-    <t>dictado 21/10: carga extra viernes 23 (Gonzalo 21/10)</t>
-  </si>
-  <si>
-    <t>dictado 21/10: la de la tersa 20 que no cargo pasa al viernes 23 (Gonzalo 21/10)</t>
-  </si>
-  <si>
-    <t>dictado 21/10: Milciades lunes (Paraguay 3: Guido, Alvarito, Milciades)</t>
-  </si>
-  <si>
-    <t>Gonzalo 27/10 (chat)</t>
-  </si>
-  <si>
-    <t>dictado 27/10: carga mie 28, descarga vie 30 confirmada (Gonzalo)</t>
-  </si>
-  <si>
-    <t>2026-10-30</t>
-  </si>
-  <si>
     <t>dictado 27/10: Fisher 2026-10-30</t>
   </si>
   <si>
@@ -631,6 +574,66 @@
     <t>2026-10-31</t>
   </si>
   <si>
+    <t>dictado 27/10: Cassio 2026-11-03</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Cassio 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Cassio 2026-11-07</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Gilson 2026-11-03</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Gilson 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Stein 2026-11-03</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Stein 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Agrocurupa 2026-11-04</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Agrocurupa 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Muller Fabricio 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Jaime Zimerman 2026-11-04</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Jaime Zimerman 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Aryste Mittelman 2026-11-04</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Aryste Mittelman 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Shapo 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Wagner 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Marconi 2026-11-04</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Josemar 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Jhony Viera 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 27/10: BAHIA 2026-11-04</t>
+  </si>
+  <si>
     <t>semana_lunes</t>
   </si>
   <si>
@@ -667,13 +670,13 @@
     <t>reparto BR/PY/BO con el mix real de las ultimas 10 semanas; desde el mie 21 la pisa la estimacion con los dias reales</t>
   </si>
   <si>
-    <t>Gonzalo 18/10: "las dos semanas de 20 y 20.5" = 20.500</t>
+    <t>Gonzalo 27/10: se preve una venta de 22 mil esta semana y 18 mil la que viene = 22000</t>
   </si>
   <si>
     <t>el resto de la semana como la venta estacional</t>
   </si>
   <si>
-    <t>Gonzalo 16/10: "semana que viene se venden 20, la siguiente 21 mil, la del feriado 16 mil" = 16000</t>
+    <t>Gonzalo 27/10: se preve una venta de 22 mil esta semana y 18 mil la que viene = 18000</t>
   </si>
   <si>
     <t>feriado Finados en Brasil el mismo lunes: frontera cerrada</t>
@@ -861,7 +864,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -872,6 +875,7 @@
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -1192,7 +1196,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K137"/>
+  <dimension ref="A1:K138"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -4637,22 +4641,28 @@
     </row>
     <row r="107">
       <c r="A107" s="10">
-        <v>46330</v>
+        <v>46328</v>
       </c>
       <c r="B107" s="0" t="s">
-        <v>52</v>
+        <v>19</v>
       </c>
       <c r="C107" s="0" t="s">
         <v>165</v>
       </c>
       <c r="D107" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E107" s="0" t="s">
-        <v>31</v>
+        <v>20</v>
+      </c>
+      <c r="F107" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G107" s="0" t="s">
+        <v>15</v>
       </c>
       <c r="H107" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I107" s="0" t="s">
         <v>153</v>
@@ -4663,22 +4673,28 @@
     </row>
     <row r="108">
       <c r="A108" s="10">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B108" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C108" s="0" t="s">
         <v>165</v>
       </c>
       <c r="D108" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E108" s="0" t="s">
-        <v>31</v>
+        <v>22</v>
+      </c>
+      <c r="F108" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G108" s="0" t="s">
+        <v>15</v>
       </c>
       <c r="H108" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I108" s="0" t="s">
         <v>153</v>
@@ -4688,271 +4704,322 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="10">
-        <v>46329</v>
+      <c r="A109" s="11">
+        <v>46318</v>
       </c>
       <c r="B109" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C109" s="0" t="s">
-        <v>165</v>
+        <v>116</v>
       </c>
       <c r="D109" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E109" s="0" t="s">
-        <v>27</v>
+        <v>43</v>
+      </c>
+      <c r="F109" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G109" s="0" t="s">
+        <v>35</v>
       </c>
       <c r="H109" s="0">
         <v>1008</v>
       </c>
       <c r="I109" s="0" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="J109" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="10">
-        <v>46332</v>
+      <c r="A110" s="12">
+        <v>46318</v>
       </c>
       <c r="B110" s="0" t="s">
         <v>23</v>
       </c>
       <c r="C110" s="0" t="s">
-        <v>165</v>
+        <v>116</v>
       </c>
       <c r="D110" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E110" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="F110" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G110" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H110" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I110" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="J110" s="0" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B111" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C111" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D111" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E111" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="F111" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="G111" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H111" s="0">
+        <v>980</v>
+      </c>
+      <c r="I111" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="J111" s="0" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="14">
+        <v>46323</v>
+      </c>
+      <c r="B112" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C112" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D112" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E112" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="H110" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I110" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="J110" s="0" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="10">
-        <v>46333</v>
-      </c>
-      <c r="B111" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="C111" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="D111" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E111" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="H111" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I111" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="J111" s="0" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="10">
-        <v>46329</v>
-      </c>
-      <c r="B112" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="C112" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="D112" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E112" s="0" t="s">
-        <v>43</v>
+      <c r="F112" s="0" t="s">
+        <v>41</v>
       </c>
       <c r="H112" s="0">
         <v>1008</v>
       </c>
       <c r="I112" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J112" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
+      </c>
+      <c r="K112" s="0" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="10">
-        <v>46332</v>
+      <c r="A113" s="14">
+        <v>46323</v>
       </c>
       <c r="B113" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C113" s="0" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="D113" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E113" s="0" t="s">
-        <v>43</v>
+        <v>25</v>
+      </c>
+      <c r="F113" s="0" t="s">
+        <v>56</v>
       </c>
       <c r="H113" s="0">
         <v>1008</v>
       </c>
       <c r="I113" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J113" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="K113" s="0" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="14">
+        <v>46323</v>
+      </c>
+      <c r="B114" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C114" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D114" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E114" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="F114" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="H114" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I114" s="0" t="s">
         <v>172</v>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="10">
-        <v>46329</v>
-      </c>
-      <c r="B114" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="C114" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="D114" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E114" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="H114" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I114" s="0" t="s">
-        <v>153</v>
       </c>
       <c r="J114" s="0" t="s">
         <v>173</v>
       </c>
+      <c r="K114" s="0" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="115">
-      <c r="A115" s="10">
-        <v>46330</v>
+      <c r="A115" s="14">
+        <v>46325</v>
       </c>
       <c r="B115" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C115" s="0" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="D115" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E115" s="0" t="s">
-        <v>59</v>
+        <v>31</v>
+      </c>
+      <c r="F115" s="0" t="s">
+        <v>26</v>
       </c>
       <c r="H115" s="0">
         <v>1008</v>
       </c>
       <c r="I115" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J115" s="0" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="10">
-        <v>46332</v>
+      <c r="A116" s="14">
+        <v>46325</v>
       </c>
       <c r="B116" s="0" t="s">
         <v>23</v>
       </c>
       <c r="C116" s="0" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="D116" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E116" s="0" t="s">
-        <v>59</v>
+        <v>40</v>
+      </c>
+      <c r="F116" s="0" t="s">
+        <v>41</v>
       </c>
       <c r="H116" s="0">
         <v>1008</v>
       </c>
       <c r="I116" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J116" s="0" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="10">
-        <v>46330</v>
+      <c r="A117" s="14">
+        <v>46326</v>
       </c>
       <c r="B117" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="C117" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D117" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E117" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="F117" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="H117" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I117" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="J117" s="0" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="15">
+        <v>46323</v>
+      </c>
+      <c r="B118" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="C117" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="D117" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E117" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="H117" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I117" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="J117" s="0" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="10">
-        <v>46332</v>
-      </c>
-      <c r="B118" s="0" t="s">
-        <v>23</v>
-      </c>
       <c r="C118" s="0" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="D118" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E118" s="0" t="s">
-        <v>40</v>
+        <v>130</v>
+      </c>
+      <c r="F118" s="0" t="s">
+        <v>179</v>
       </c>
       <c r="H118" s="0">
         <v>1008</v>
       </c>
       <c r="I118" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J118" s="0" t="s">
-        <v>177</v>
+        <v>180</v>
+      </c>
+      <c r="K118" s="0" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="10">
-        <v>46330</v>
+      <c r="A119" s="16">
+        <v>46329</v>
       </c>
       <c r="B119" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C119" s="0" t="s">
         <v>165</v>
@@ -4961,20 +5028,20 @@
         <v>24</v>
       </c>
       <c r="E119" s="0" t="s">
-        <v>122</v>
+        <v>27</v>
       </c>
       <c r="H119" s="0">
         <v>1008</v>
       </c>
       <c r="I119" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J119" s="0" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="10">
+      <c r="A120" s="16">
         <v>46332</v>
       </c>
       <c r="B120" s="0" t="s">
@@ -4987,24 +5054,24 @@
         <v>24</v>
       </c>
       <c r="E120" s="0" t="s">
-        <v>122</v>
+        <v>27</v>
       </c>
       <c r="H120" s="0">
         <v>1008</v>
       </c>
       <c r="I120" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J120" s="0" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="10">
-        <v>46330</v>
+      <c r="A121" s="16">
+        <v>46333</v>
       </c>
       <c r="B121" s="0" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C121" s="0" t="s">
         <v>165</v>
@@ -5013,24 +5080,24 @@
         <v>24</v>
       </c>
       <c r="E121" s="0" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H121" s="0">
         <v>1008</v>
       </c>
       <c r="I121" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J121" s="0" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="10">
-        <v>46332</v>
+      <c r="A122" s="16">
+        <v>46329</v>
       </c>
       <c r="B122" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C122" s="0" t="s">
         <v>165</v>
@@ -5039,20 +5106,20 @@
         <v>24</v>
       </c>
       <c r="E122" s="0" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="H122" s="0">
         <v>1008</v>
       </c>
       <c r="I122" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J122" s="0" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="10">
+      <c r="A123" s="16">
         <v>46332</v>
       </c>
       <c r="B123" s="0" t="s">
@@ -5065,24 +5132,24 @@
         <v>24</v>
       </c>
       <c r="E123" s="0" t="s">
-        <v>140</v>
+        <v>43</v>
       </c>
       <c r="H123" s="0">
         <v>1008</v>
       </c>
       <c r="I123" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J123" s="0" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="10">
-        <v>46332</v>
+      <c r="A124" s="16">
+        <v>46329</v>
       </c>
       <c r="B124" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C124" s="0" t="s">
         <v>165</v>
@@ -5091,26 +5158,20 @@
         <v>24</v>
       </c>
       <c r="E124" s="0" t="s">
-        <v>183</v>
-      </c>
-      <c r="F124" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G124" s="0" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="H124" s="0">
         <v>1008</v>
       </c>
       <c r="I124" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J124" s="0" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="10">
+      <c r="A125" s="16">
         <v>46332</v>
       </c>
       <c r="B125" s="0" t="s">
@@ -5123,397 +5184,354 @@
         <v>24</v>
       </c>
       <c r="E125" s="0" t="s">
-        <v>161</v>
-      </c>
-      <c r="F125" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G125" s="0" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="H125" s="0">
         <v>1008</v>
       </c>
       <c r="I125" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J125" s="0" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="10">
-        <v>46328</v>
+      <c r="A126" s="16">
+        <v>46330</v>
       </c>
       <c r="B126" s="0" t="s">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="C126" s="0" t="s">
         <v>165</v>
       </c>
       <c r="D126" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E126" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="F126" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G126" s="0" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="H126" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I126" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J126" s="0" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="10">
-        <v>46329</v>
+      <c r="A127" s="16">
+        <v>46332</v>
       </c>
       <c r="B127" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C127" s="0" t="s">
         <v>165</v>
       </c>
       <c r="D127" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E127" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="F127" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G127" s="0" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="H127" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I127" s="0" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J127" s="0" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="11">
-        <v>46318</v>
+      <c r="A128" s="16">
+        <v>46332</v>
       </c>
       <c r="B128" s="0" t="s">
         <v>23</v>
       </c>
       <c r="C128" s="0" t="s">
-        <v>116</v>
+        <v>165</v>
       </c>
       <c r="D128" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E128" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="F128" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G128" s="0" t="s">
-        <v>35</v>
+        <v>122</v>
       </c>
       <c r="H128" s="0">
         <v>1008</v>
       </c>
       <c r="I128" s="0" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="J128" s="0" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="12">
-        <v>46318</v>
+      <c r="A129" s="16">
+        <v>46330</v>
       </c>
       <c r="B129" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C129" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D129" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E129" s="0" t="s">
+        <v>140</v>
+      </c>
+      <c r="H129" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I129" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="J129" s="0" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="16">
+        <v>46332</v>
+      </c>
+      <c r="B130" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="C129" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="D129" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E129" s="0" t="s">
-        <v>105</v>
-      </c>
-      <c r="F129" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="G129" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="H129" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I129" s="0" t="s">
-        <v>188</v>
-      </c>
-      <c r="J129" s="0" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="13">
-        <v>46321</v>
-      </c>
-      <c r="B130" s="0" t="s">
-        <v>19</v>
-      </c>
       <c r="C130" s="0" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D130" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E130" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="F130" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G130" s="0" t="s">
-        <v>15</v>
+        <v>140</v>
       </c>
       <c r="H130" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I130" s="0" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="J130" s="0" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="14">
-        <v>46323</v>
+      <c r="A131" s="16">
+        <v>46330</v>
       </c>
       <c r="B131" s="0" t="s">
         <v>52</v>
       </c>
       <c r="C131" s="0" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D131" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E131" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="F131" s="0" t="s">
-        <v>41</v>
+        <v>175</v>
       </c>
       <c r="H131" s="0">
         <v>1008</v>
       </c>
       <c r="I131" s="0" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="J131" s="0" t="s">
-        <v>193</v>
-      </c>
-      <c r="K131" s="0" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="14">
-        <v>46323</v>
+      <c r="A132" s="16">
+        <v>46332</v>
       </c>
       <c r="B132" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C132" s="0" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D132" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E132" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="F132" s="0" t="s">
-        <v>56</v>
+        <v>175</v>
       </c>
       <c r="H132" s="0">
         <v>1008</v>
       </c>
       <c r="I132" s="0" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="J132" s="0" t="s">
-        <v>193</v>
-      </c>
-      <c r="K132" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="14">
-        <v>46323</v>
+      <c r="A133" s="16">
+        <v>46332</v>
       </c>
       <c r="B133" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C133" s="0" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D133" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E133" s="0" t="s">
-        <v>183</v>
-      </c>
-      <c r="F133" s="0" t="s">
-        <v>56</v>
+        <v>105</v>
       </c>
       <c r="H133" s="0">
         <v>1008</v>
       </c>
       <c r="I133" s="0" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="J133" s="0" t="s">
-        <v>193</v>
-      </c>
-      <c r="K133" s="0" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="14">
-        <v>46325</v>
+      <c r="A134" s="16">
+        <v>46332</v>
       </c>
       <c r="B134" s="0" t="s">
         <v>23</v>
       </c>
       <c r="C134" s="0" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D134" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E134" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="F134" s="0" t="s">
-        <v>26</v>
+        <v>146</v>
       </c>
       <c r="H134" s="0">
         <v>1008</v>
       </c>
       <c r="I134" s="0" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="J134" s="0" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="14">
-        <v>46325</v>
+      <c r="A135" s="16">
+        <v>46330</v>
       </c>
       <c r="B135" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C135" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D135" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E135" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="H135" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I135" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="J135" s="0" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="16">
+        <v>46332</v>
+      </c>
+      <c r="B136" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="C135" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="D135" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E135" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="F135" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="H135" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I135" s="0" t="s">
-        <v>192</v>
-      </c>
-      <c r="J135" s="0" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="14">
-        <v>46326</v>
-      </c>
-      <c r="B136" s="0" t="s">
-        <v>30</v>
-      </c>
       <c r="C136" s="0" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D136" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E136" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="F136" s="0" t="s">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="H136" s="0">
         <v>1008</v>
       </c>
       <c r="I136" s="0" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="J136" s="0" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="15">
-        <v>46323</v>
+      <c r="A137" s="16">
+        <v>46332</v>
       </c>
       <c r="B137" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C137" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D137" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E137" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="H137" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I137" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="J137" s="0" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="16">
+        <v>46330</v>
+      </c>
+      <c r="B138" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="C137" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="D137" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E137" s="0" t="s">
+      <c r="C138" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D138" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E138" s="0" t="s">
         <v>130</v>
       </c>
-      <c r="F137" s="0" t="s">
-        <v>198</v>
-      </c>
-      <c r="H137" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I137" s="0" t="s">
-        <v>192</v>
-      </c>
-      <c r="J137" s="0" t="s">
-        <v>199</v>
-      </c>
-      <c r="K137" s="0" t="s">
-        <v>200</v>
+      <c r="H138" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I138" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="J138" s="0" t="s">
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -5535,7 +5553,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5567,10 +5585,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3">
@@ -5587,10 +5605,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4">
@@ -5607,10 +5625,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5">
@@ -5627,10 +5645,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6">
@@ -5647,10 +5665,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7">
@@ -5667,10 +5685,10 @@
         <v>1313</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8">
@@ -5678,19 +5696,19 @@
         <v>46321</v>
       </c>
       <c r="B8" s="0">
-        <v>11111</v>
+        <v>12767</v>
       </c>
       <c r="C8" s="0">
-        <v>8036</v>
+        <v>9233</v>
       </c>
       <c r="D8" s="0">
-        <v>1353</v>
+        <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9">
@@ -5698,19 +5716,19 @@
         <v>46328</v>
       </c>
       <c r="B9" s="0">
-        <v>8672</v>
+        <v>10445</v>
       </c>
       <c r="C9" s="0">
-        <v>6272</v>
+        <v>7555</v>
       </c>
       <c r="D9" s="0">
-        <v>1056</v>
+        <v>0</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10">
@@ -5727,7 +5745,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11">
@@ -5744,7 +5762,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -5763,57 +5781,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -5861,10 +5879,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="3">
@@ -5878,10 +5896,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4">
@@ -5895,10 +5913,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5">
@@ -5906,16 +5924,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6">
@@ -5929,10 +5947,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7">
@@ -5946,10 +5964,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8">
@@ -5963,10 +5981,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9">
@@ -5974,16 +5992,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="10">
@@ -5997,10 +6015,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11">
@@ -6014,10 +6032,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="12">
@@ -6031,10 +6049,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13">
@@ -6042,16 +6060,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -6085,10 +6103,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6114,7 +6132,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3">
@@ -6137,7 +6155,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4">
@@ -6160,7 +6178,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5">
@@ -6171,7 +6189,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6183,7 +6201,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6">
@@ -6206,7 +6224,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7">
@@ -6229,7 +6247,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="8">
@@ -6252,7 +6270,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="9">
@@ -6263,7 +6281,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6275,7 +6293,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="10">
@@ -6298,7 +6316,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11">
@@ -6321,7 +6339,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12">
@@ -6344,7 +6362,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13">
@@ -6355,7 +6373,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6367,7 +6385,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="14">
@@ -6390,7 +6408,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="15">
@@ -6401,7 +6419,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6413,7 +6431,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16">
@@ -6436,7 +6454,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="17">
@@ -6459,7 +6477,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -6480,10 +6498,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6491,46 +6509,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B4" s="0">
         <v>30000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -6551,10 +6569,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6566,10 +6584,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6599,7 +6617,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="3">
@@ -6626,7 +6644,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4">
@@ -6653,7 +6671,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5">
@@ -6680,7 +6698,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="6">
@@ -6707,7 +6725,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="7">
@@ -6734,7 +6752,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="8">
@@ -6761,7 +6779,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="9">
@@ -6788,7 +6806,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="10">
@@ -6815,7 +6833,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="11">
@@ -6842,7 +6860,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="12">
@@ -6869,7 +6887,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="13">
@@ -6896,12 +6914,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Fischer 3 y Andre Pauli 2 en la semana 2-7/11
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="271">
   <si>
     <t>fecha</t>
   </si>
@@ -632,6 +632,21 @@
   </si>
   <si>
     <t>dictado 27/10: BAHIA 2026-11-04</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Fisher 2026-11-04</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Fisher 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Fisher 2026-11-07</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Andre Pauli 2026-11-04</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Andre Pauli 2026-11-06</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -864,7 +879,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -875,6 +890,7 @@
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -1196,7 +1212,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K138"/>
+  <dimension ref="A1:K143"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -5532,6 +5548,136 @@
       </c>
       <c r="J138" s="0" t="s">
         <v>201</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="17">
+        <v>46330</v>
+      </c>
+      <c r="B139" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C139" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D139" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E139" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="H139" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I139" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="J139" s="0" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="17">
+        <v>46332</v>
+      </c>
+      <c r="B140" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C140" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D140" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E140" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="H140" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I140" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="J140" s="0" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="17">
+        <v>46333</v>
+      </c>
+      <c r="B141" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="C141" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D141" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E141" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="H141" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I141" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="J141" s="0" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="17">
+        <v>46330</v>
+      </c>
+      <c r="B142" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C142" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D142" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E142" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="H142" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I142" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="J142" s="0" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="17">
+        <v>46332</v>
+      </c>
+      <c r="B143" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C143" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D143" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E143" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="H143" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I143" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="J143" s="0" t="s">
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -5553,7 +5699,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5585,10 +5731,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3">
@@ -5605,10 +5751,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4">
@@ -5625,10 +5771,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5">
@@ -5645,10 +5791,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6">
@@ -5665,10 +5811,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7">
@@ -5685,10 +5831,10 @@
         <v>1313</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8">
@@ -5705,10 +5851,10 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9">
@@ -5725,10 +5871,10 @@
         <v>0</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10">
@@ -5745,7 +5891,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
     </row>
     <row r="11">
@@ -5762,7 +5908,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>
@@ -5781,57 +5927,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -5879,10 +6025,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3">
@@ -5896,10 +6042,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4">
@@ -5913,10 +6059,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5">
@@ -5924,16 +6070,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6">
@@ -5947,10 +6093,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
     </row>
     <row r="7">
@@ -5964,10 +6110,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
     </row>
     <row r="8">
@@ -5981,10 +6127,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9">
@@ -5992,16 +6138,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="10">
@@ -6015,10 +6161,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
     </row>
     <row r="11">
@@ -6032,10 +6178,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
     </row>
     <row r="12">
@@ -6049,10 +6195,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
     </row>
     <row r="13">
@@ -6060,16 +6206,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -6103,10 +6249,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6132,7 +6278,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="3">
@@ -6155,7 +6301,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4">
@@ -6178,7 +6324,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5">
@@ -6189,7 +6335,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6201,7 +6347,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6">
@@ -6224,7 +6370,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7">
@@ -6247,7 +6393,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8">
@@ -6270,7 +6416,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9">
@@ -6281,7 +6427,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6293,7 +6439,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10">
@@ -6316,7 +6462,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="11">
@@ -6339,7 +6485,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="12">
@@ -6362,7 +6508,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13">
@@ -6373,7 +6519,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6385,7 +6531,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14">
@@ -6408,7 +6554,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
     </row>
     <row r="15">
@@ -6419,7 +6565,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6431,7 +6577,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
     </row>
     <row r="16">
@@ -6454,7 +6600,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
     </row>
     <row r="17">
@@ -6477,7 +6623,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -6498,10 +6644,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6509,46 +6655,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="B4" s="0">
         <v>30000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -6569,10 +6715,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6584,10 +6730,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6617,7 +6763,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3">
@@ -6644,7 +6790,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4">
@@ -6671,7 +6817,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5">
@@ -6698,7 +6844,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6">
@@ -6725,7 +6871,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7">
@@ -6752,7 +6898,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8">
@@ -6779,7 +6925,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9">
@@ -6806,7 +6952,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10">
@@ -6833,7 +6979,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11">
@@ -6860,7 +7006,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="12">
@@ -6887,7 +7033,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="13">
@@ -6914,12 +7060,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Muller, Josemar y Jhony al martes 3
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -601,7 +601,7 @@
     <t>dictado 27/10: Agrocurupa 2026-11-06</t>
   </si>
   <si>
-    <t>dictado 27/10: Muller Fabricio 2026-11-06</t>
+    <t>dictado 27/10: Muller Fabricio 2026-11-06; 27/10: pasa del vie 6 al mar 3 (dictado)</t>
   </si>
   <si>
     <t>dictado 27/10: Jaime Zimerman 2026-11-04</t>
@@ -625,10 +625,10 @@
     <t>dictado 27/10: Marconi 2026-11-04</t>
   </si>
   <si>
-    <t>dictado 27/10: Josemar 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Jhony Viera 2026-11-06</t>
+    <t>dictado 27/10: Josemar 2026-11-06; 27/10: pasa del vie 6 al mar 3 (dictado)</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Jhony Viera 2026-11-06; 27/10: pasa del vie 6 al mar 3 (dictado)</t>
   </si>
   <si>
     <t>dictado 27/10: BAHIA 2026-11-04</t>
@@ -5266,10 +5266,10 @@
     </row>
     <row r="128">
       <c r="A128" s="16">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B128" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C128" s="0" t="s">
         <v>165</v>
@@ -5474,10 +5474,10 @@
     </row>
     <row r="136">
       <c r="A136" s="16">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B136" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C136" s="0" t="s">
         <v>165</v>
@@ -5500,10 +5500,10 @@
     </row>
     <row r="137">
       <c r="A137" s="16">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B137" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C137" s="0" t="s">
         <v>165</v>

</xml_diff>

<commit_message>
plan de compras: sin cargas de Paraguay en la semana 2-7/11
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="269">
   <si>
     <t>fecha</t>
   </si>
@@ -523,55 +523,49 @@
     <t>dictado 20/10: Paraguay AS 2026-10-26</t>
   </si>
   <si>
+    <t>Gonzalo 21/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 21/10: carga extra viernes 23 (Gonzalo 21/10)</t>
+  </si>
+  <si>
+    <t>dictado 21/10: la de la tersa 20 que no cargo pasa al viernes 23 (Gonzalo 21/10)</t>
+  </si>
+  <si>
+    <t>dictado 21/10: Milciades lunes (Paraguay 3: Guido, Alvarito, Milciades)</t>
+  </si>
+  <si>
+    <t>Gonzalo 27/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 27/10: carga mie 28, descarga vie 30 confirmada (Gonzalo)</t>
+  </si>
+  <si>
+    <t>2026-10-30</t>
+  </si>
+  <si>
+    <t>Aryste Mittelman</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Fisher 2026-10-30</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Agrocurupa 2026-10-30</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Marconi 2026-10-31</t>
+  </si>
+  <si>
+    <t>Gral</t>
+  </si>
+  <si>
+    <t>dictado 27/10: carga mie 28, descarga sab 31 confirmada (Gonzalo)</t>
+  </si>
+  <si>
+    <t>2026-10-31</t>
+  </si>
+  <si>
     <t>2026-11-01</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Paraguay MS 2026-11-02</t>
-  </si>
-  <si>
-    <t>dictado 20/10: Paraguay AS 2026-11-03</t>
-  </si>
-  <si>
-    <t>Gonzalo 21/10 (chat)</t>
-  </si>
-  <si>
-    <t>dictado 21/10: carga extra viernes 23 (Gonzalo 21/10)</t>
-  </si>
-  <si>
-    <t>dictado 21/10: la de la tersa 20 que no cargo pasa al viernes 23 (Gonzalo 21/10)</t>
-  </si>
-  <si>
-    <t>dictado 21/10: Milciades lunes (Paraguay 3: Guido, Alvarito, Milciades)</t>
-  </si>
-  <si>
-    <t>Gonzalo 27/10 (chat)</t>
-  </si>
-  <si>
-    <t>dictado 27/10: carga mie 28, descarga vie 30 confirmada (Gonzalo)</t>
-  </si>
-  <si>
-    <t>2026-10-30</t>
-  </si>
-  <si>
-    <t>Aryste Mittelman</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Fisher 2026-10-30</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Agrocurupa 2026-10-30</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Marconi 2026-10-31</t>
-  </si>
-  <si>
-    <t>Gral</t>
-  </si>
-  <si>
-    <t>dictado 27/10: carga mie 28, descarga sab 31 confirmada (Gonzalo)</t>
-  </si>
-  <si>
-    <t>2026-10-31</t>
   </si>
   <si>
     <t>dictado 27/10: Cassio 2026-11-03</t>
@@ -1212,7 +1206,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K143"/>
+  <dimension ref="A1:K141"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -4656,162 +4650,162 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="10">
-        <v>46328</v>
+      <c r="A107" s="11">
+        <v>46318</v>
       </c>
       <c r="B107" s="0" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C107" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="D107" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E107" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="F107" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G107" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H107" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I107" s="0" t="s">
         <v>165</v>
-      </c>
-      <c r="D107" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="E107" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="F107" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G107" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H107" s="0">
-        <v>980</v>
-      </c>
-      <c r="I107" s="0" t="s">
-        <v>153</v>
       </c>
       <c r="J107" s="0" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="10">
-        <v>46329</v>
+      <c r="A108" s="12">
+        <v>46318</v>
       </c>
       <c r="B108" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C108" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="D108" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E108" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="F108" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="G108" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H108" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I108" s="0" t="s">
         <v>165</v>
-      </c>
-      <c r="D108" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="E108" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="F108" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G108" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H108" s="0">
-        <v>980</v>
-      </c>
-      <c r="I108" s="0" t="s">
-        <v>153</v>
       </c>
       <c r="J108" s="0" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="11">
-        <v>46318</v>
+      <c r="A109" s="13">
+        <v>46321</v>
       </c>
       <c r="B109" s="0" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C109" s="0" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="D109" s="0" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E109" s="0" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F109" s="0" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G109" s="0" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H109" s="0">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I109" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="J109" s="0" t="s">
         <v>168</v>
       </c>
-      <c r="J109" s="0" t="s">
-        <v>169</v>
-      </c>
     </row>
     <row r="110">
-      <c r="A110" s="12">
-        <v>46318</v>
+      <c r="A110" s="14">
+        <v>46323</v>
       </c>
       <c r="B110" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C110" s="0" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="D110" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E110" s="0" t="s">
-        <v>105</v>
+        <v>27</v>
       </c>
       <c r="F110" s="0" t="s">
         <v>41</v>
       </c>
-      <c r="G110" s="0" t="s">
-        <v>35</v>
-      </c>
       <c r="H110" s="0">
         <v>1008</v>
       </c>
       <c r="I110" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J110" s="0" t="s">
         <v>170</v>
       </c>
+      <c r="K110" s="0" t="s">
+        <v>171</v>
+      </c>
     </row>
     <row r="111">
-      <c r="A111" s="13">
-        <v>46321</v>
+      <c r="A111" s="14">
+        <v>46323</v>
       </c>
       <c r="B111" s="0" t="s">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="C111" s="0" t="s">
         <v>152</v>
       </c>
       <c r="D111" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E111" s="0" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F111" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G111" s="0" t="s">
-        <v>15</v>
+        <v>56</v>
       </c>
       <c r="H111" s="0">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I111" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J111" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="K111" s="0" t="s">
         <v>171</v>
       </c>
     </row>
@@ -4829,30 +4823,30 @@
         <v>24</v>
       </c>
       <c r="E112" s="0" t="s">
-        <v>27</v>
+        <v>172</v>
       </c>
       <c r="F112" s="0" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="H112" s="0">
         <v>1008</v>
       </c>
       <c r="I112" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J112" s="0" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="K112" s="0" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="14">
-        <v>46323</v>
+        <v>46325</v>
       </c>
       <c r="B113" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C113" s="0" t="s">
         <v>152</v>
@@ -4861,30 +4855,27 @@
         <v>24</v>
       </c>
       <c r="E113" s="0" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F113" s="0" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="H113" s="0">
         <v>1008</v>
       </c>
       <c r="I113" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J113" s="0" t="s">
         <v>173</v>
       </c>
-      <c r="K113" s="0" t="s">
-        <v>174</v>
-      </c>
     </row>
     <row r="114">
       <c r="A114" s="14">
-        <v>46323</v>
+        <v>46325</v>
       </c>
       <c r="B114" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C114" s="0" t="s">
         <v>152</v>
@@ -4893,30 +4884,27 @@
         <v>24</v>
       </c>
       <c r="E114" s="0" t="s">
-        <v>175</v>
+        <v>40</v>
       </c>
       <c r="F114" s="0" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="H114" s="0">
         <v>1008</v>
       </c>
       <c r="I114" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J114" s="0" t="s">
-        <v>173</v>
-      </c>
-      <c r="K114" s="0" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="14">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B115" s="0" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C115" s="0" t="s">
         <v>152</v>
@@ -4925,27 +4913,27 @@
         <v>24</v>
       </c>
       <c r="E115" s="0" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="F115" s="0" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="H115" s="0">
         <v>1008</v>
       </c>
       <c r="I115" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J115" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="14">
-        <v>46325</v>
+      <c r="A116" s="15">
+        <v>46323</v>
       </c>
       <c r="B116" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C116" s="0" t="s">
         <v>152</v>
@@ -4954,91 +4942,85 @@
         <v>24</v>
       </c>
       <c r="E116" s="0" t="s">
-        <v>40</v>
+        <v>130</v>
       </c>
       <c r="F116" s="0" t="s">
-        <v>41</v>
+        <v>176</v>
       </c>
       <c r="H116" s="0">
         <v>1008</v>
       </c>
       <c r="I116" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J116" s="0" t="s">
         <v>177</v>
       </c>
+      <c r="K116" s="0" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="117">
-      <c r="A117" s="14">
-        <v>46326</v>
+      <c r="A117" s="16">
+        <v>46329</v>
       </c>
       <c r="B117" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C117" s="0" t="s">
-        <v>152</v>
+        <v>179</v>
       </c>
       <c r="D117" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E117" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="F117" s="0" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="H117" s="0">
         <v>1008</v>
       </c>
       <c r="I117" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J117" s="0" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="15">
-        <v>46323</v>
+      <c r="A118" s="16">
+        <v>46332</v>
       </c>
       <c r="B118" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C118" s="0" t="s">
-        <v>152</v>
+        <v>179</v>
       </c>
       <c r="D118" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E118" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="F118" s="0" t="s">
-        <v>179</v>
+        <v>27</v>
       </c>
       <c r="H118" s="0">
         <v>1008</v>
       </c>
       <c r="I118" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J118" s="0" t="s">
-        <v>180</v>
-      </c>
-      <c r="K118" s="0" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="16">
-        <v>46329</v>
+        <v>46333</v>
       </c>
       <c r="B119" s="0" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C119" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D119" s="0" t="s">
         <v>24</v>
@@ -5050,7 +5032,7 @@
         <v>1008</v>
       </c>
       <c r="I119" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J119" s="0" t="s">
         <v>182</v>
@@ -5058,25 +5040,25 @@
     </row>
     <row r="120">
       <c r="A120" s="16">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B120" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C120" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D120" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E120" s="0" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="H120" s="0">
         <v>1008</v>
       </c>
       <c r="I120" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J120" s="0" t="s">
         <v>183</v>
@@ -5084,25 +5066,25 @@
     </row>
     <row r="121">
       <c r="A121" s="16">
-        <v>46333</v>
+        <v>46332</v>
       </c>
       <c r="B121" s="0" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C121" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D121" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E121" s="0" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="H121" s="0">
         <v>1008</v>
       </c>
       <c r="I121" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J121" s="0" t="s">
         <v>184</v>
@@ -5116,19 +5098,19 @@
         <v>21</v>
       </c>
       <c r="C122" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D122" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E122" s="0" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="H122" s="0">
         <v>1008</v>
       </c>
       <c r="I122" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J122" s="0" t="s">
         <v>185</v>
@@ -5142,19 +5124,19 @@
         <v>23</v>
       </c>
       <c r="C123" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D123" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E123" s="0" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="H123" s="0">
         <v>1008</v>
       </c>
       <c r="I123" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J123" s="0" t="s">
         <v>186</v>
@@ -5162,25 +5144,25 @@
     </row>
     <row r="124">
       <c r="A124" s="16">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="B124" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C124" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D124" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E124" s="0" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="H124" s="0">
         <v>1008</v>
       </c>
       <c r="I124" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J124" s="0" t="s">
         <v>187</v>
@@ -5194,19 +5176,19 @@
         <v>23</v>
       </c>
       <c r="C125" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D125" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E125" s="0" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="H125" s="0">
         <v>1008</v>
       </c>
       <c r="I125" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J125" s="0" t="s">
         <v>188</v>
@@ -5214,25 +5196,25 @@
     </row>
     <row r="126">
       <c r="A126" s="16">
-        <v>46330</v>
+        <v>46329</v>
       </c>
       <c r="B126" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C126" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D126" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E126" s="0" t="s">
-        <v>40</v>
+        <v>122</v>
       </c>
       <c r="H126" s="0">
         <v>1008</v>
       </c>
       <c r="I126" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J126" s="0" t="s">
         <v>189</v>
@@ -5240,25 +5222,25 @@
     </row>
     <row r="127">
       <c r="A127" s="16">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B127" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C127" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D127" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E127" s="0" t="s">
-        <v>40</v>
+        <v>140</v>
       </c>
       <c r="H127" s="0">
         <v>1008</v>
       </c>
       <c r="I127" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J127" s="0" t="s">
         <v>190</v>
@@ -5266,25 +5248,25 @@
     </row>
     <row r="128">
       <c r="A128" s="16">
-        <v>46329</v>
+        <v>46332</v>
       </c>
       <c r="B128" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C128" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D128" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E128" s="0" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="H128" s="0">
         <v>1008</v>
       </c>
       <c r="I128" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J128" s="0" t="s">
         <v>191</v>
@@ -5298,19 +5280,19 @@
         <v>52</v>
       </c>
       <c r="C129" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D129" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E129" s="0" t="s">
-        <v>140</v>
+        <v>172</v>
       </c>
       <c r="H129" s="0">
         <v>1008</v>
       </c>
       <c r="I129" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J129" s="0" t="s">
         <v>192</v>
@@ -5324,19 +5306,19 @@
         <v>23</v>
       </c>
       <c r="C130" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D130" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E130" s="0" t="s">
-        <v>140</v>
+        <v>172</v>
       </c>
       <c r="H130" s="0">
         <v>1008</v>
       </c>
       <c r="I130" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J130" s="0" t="s">
         <v>193</v>
@@ -5344,25 +5326,25 @@
     </row>
     <row r="131">
       <c r="A131" s="16">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B131" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C131" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D131" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E131" s="0" t="s">
-        <v>175</v>
+        <v>105</v>
       </c>
       <c r="H131" s="0">
         <v>1008</v>
       </c>
       <c r="I131" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J131" s="0" t="s">
         <v>194</v>
@@ -5376,19 +5358,19 @@
         <v>23</v>
       </c>
       <c r="C132" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D132" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E132" s="0" t="s">
-        <v>175</v>
+        <v>146</v>
       </c>
       <c r="H132" s="0">
         <v>1008</v>
       </c>
       <c r="I132" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J132" s="0" t="s">
         <v>195</v>
@@ -5396,25 +5378,25 @@
     </row>
     <row r="133">
       <c r="A133" s="16">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B133" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C133" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D133" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E133" s="0" t="s">
-        <v>105</v>
+        <v>60</v>
       </c>
       <c r="H133" s="0">
         <v>1008</v>
       </c>
       <c r="I133" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J133" s="0" t="s">
         <v>196</v>
@@ -5422,25 +5404,25 @@
     </row>
     <row r="134">
       <c r="A134" s="16">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B134" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C134" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D134" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E134" s="0" t="s">
-        <v>146</v>
+        <v>58</v>
       </c>
       <c r="H134" s="0">
         <v>1008</v>
       </c>
       <c r="I134" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J134" s="0" t="s">
         <v>197</v>
@@ -5448,25 +5430,25 @@
     </row>
     <row r="135">
       <c r="A135" s="16">
-        <v>46330</v>
+        <v>46329</v>
       </c>
       <c r="B135" s="0" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C135" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D135" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E135" s="0" t="s">
-        <v>60</v>
+        <v>113</v>
       </c>
       <c r="H135" s="0">
         <v>1008</v>
       </c>
       <c r="I135" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J135" s="0" t="s">
         <v>198</v>
@@ -5474,77 +5456,77 @@
     </row>
     <row r="136">
       <c r="A136" s="16">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="B136" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C136" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D136" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E136" s="0" t="s">
-        <v>58</v>
+        <v>130</v>
       </c>
       <c r="H136" s="0">
         <v>1008</v>
       </c>
       <c r="I136" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J136" s="0" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="16">
-        <v>46329</v>
+      <c r="A137" s="17">
+        <v>46330</v>
       </c>
       <c r="B137" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C137" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D137" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E137" s="0" t="s">
-        <v>113</v>
+        <v>31</v>
       </c>
       <c r="H137" s="0">
         <v>1008</v>
       </c>
       <c r="I137" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J137" s="0" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="16">
-        <v>46330</v>
+      <c r="A138" s="17">
+        <v>46332</v>
       </c>
       <c r="B138" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C138" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D138" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E138" s="0" t="s">
-        <v>130</v>
+        <v>31</v>
       </c>
       <c r="H138" s="0">
         <v>1008</v>
       </c>
       <c r="I138" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J138" s="0" t="s">
         <v>201</v>
@@ -5552,13 +5534,13 @@
     </row>
     <row r="139">
       <c r="A139" s="17">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="B139" s="0" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C139" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D139" s="0" t="s">
         <v>24</v>
@@ -5570,7 +5552,7 @@
         <v>1008</v>
       </c>
       <c r="I139" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J139" s="0" t="s">
         <v>202</v>
@@ -5578,25 +5560,25 @@
     </row>
     <row r="140">
       <c r="A140" s="17">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B140" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C140" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D140" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E140" s="0" t="s">
-        <v>31</v>
+        <v>161</v>
       </c>
       <c r="H140" s="0">
         <v>1008</v>
       </c>
       <c r="I140" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J140" s="0" t="s">
         <v>203</v>
@@ -5604,80 +5586,28 @@
     </row>
     <row r="141">
       <c r="A141" s="17">
-        <v>46333</v>
+        <v>46332</v>
       </c>
       <c r="B141" s="0" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C141" s="0" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D141" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E141" s="0" t="s">
-        <v>31</v>
+        <v>161</v>
       </c>
       <c r="H141" s="0">
         <v>1008</v>
       </c>
       <c r="I141" s="0" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J141" s="0" t="s">
         <v>204</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="17">
-        <v>46330</v>
-      </c>
-      <c r="B142" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="C142" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="D142" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E142" s="0" t="s">
-        <v>161</v>
-      </c>
-      <c r="H142" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I142" s="0" t="s">
-        <v>172</v>
-      </c>
-      <c r="J142" s="0" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="17">
-        <v>46332</v>
-      </c>
-      <c r="B143" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C143" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="D143" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E143" s="0" t="s">
-        <v>161</v>
-      </c>
-      <c r="H143" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I143" s="0" t="s">
-        <v>172</v>
-      </c>
-      <c r="J143" s="0" t="s">
-        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -5699,7 +5629,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5731,10 +5661,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="3">
@@ -5751,10 +5681,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="F3" s="0" t="s">
         <v>208</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="4">
@@ -5771,10 +5701,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5">
@@ -5791,10 +5721,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6">
@@ -5811,10 +5741,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7">
@@ -5831,10 +5761,10 @@
         <v>1313</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8">
@@ -5851,10 +5781,10 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="9">
@@ -5871,10 +5801,10 @@
         <v>0</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="10">
@@ -5891,7 +5821,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11">
@@ -5908,7 +5838,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -5927,57 +5857,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -6025,10 +5955,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3">
@@ -6042,10 +5972,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
+        <v>233</v>
+      </c>
+      <c r="E3" s="0" t="s">
         <v>235</v>
-      </c>
-      <c r="E3" s="0" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="4">
@@ -6059,10 +5989,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="5">
@@ -6070,16 +6000,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6">
@@ -6093,10 +6023,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="7">
@@ -6110,10 +6040,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
+        <v>239</v>
+      </c>
+      <c r="E7" s="0" t="s">
         <v>241</v>
-      </c>
-      <c r="E7" s="0" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="8">
@@ -6127,10 +6057,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9">
@@ -6138,16 +6068,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="10">
@@ -6161,10 +6091,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11">
@@ -6178,10 +6108,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
+        <v>244</v>
+      </c>
+      <c r="E11" s="0" t="s">
         <v>246</v>
-      </c>
-      <c r="E11" s="0" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="12">
@@ -6195,10 +6125,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="13">
@@ -6206,16 +6136,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>
@@ -6249,10 +6179,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6278,7 +6208,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3">
@@ -6301,7 +6231,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4">
@@ -6324,7 +6254,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5">
@@ -6335,7 +6265,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6347,7 +6277,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6">
@@ -6370,7 +6300,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="7">
@@ -6393,7 +6323,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8">
@@ -6416,7 +6346,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="9">
@@ -6427,7 +6357,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6439,7 +6369,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="10">
@@ -6462,7 +6392,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="11">
@@ -6485,7 +6415,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12">
@@ -6508,7 +6438,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="13">
@@ -6519,7 +6449,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6531,7 +6461,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="14">
@@ -6554,7 +6484,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="15">
@@ -6565,7 +6495,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6577,7 +6507,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="16">
@@ -6600,7 +6530,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="17">
@@ -6623,7 +6553,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -6644,10 +6574,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6655,46 +6585,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B4" s="0">
         <v>30000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -6715,10 +6645,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6730,10 +6660,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6763,7 +6693,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="3">
@@ -6790,7 +6720,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="4">
@@ -6817,7 +6747,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="5">
@@ -6844,7 +6774,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6">
@@ -6871,7 +6801,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="7">
@@ -6898,7 +6828,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="8">
@@ -6925,7 +6855,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="9">
@@ -6952,7 +6882,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="10">
@@ -6979,7 +6909,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="11">
@@ -7006,7 +6936,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="12">
@@ -7033,7 +6963,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="13">
@@ -7060,12 +6990,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Fischer al martes 3 y Muller 2 en la semana 2-7/11
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="270">
   <si>
     <t>fecha</t>
   </si>
@@ -631,7 +631,7 @@
     <t>dictado 27/10: Fisher 2026-11-04</t>
   </si>
   <si>
-    <t>dictado 27/10: Fisher 2026-11-06</t>
+    <t>dictado 27/10: Fisher 2026-11-06; 27/10: pasa del vie 6 al mar 3 (dictado)</t>
   </si>
   <si>
     <t>dictado 27/10: Fisher 2026-11-07</t>
@@ -641,6 +641,9 @@
   </si>
   <si>
     <t>dictado 27/10: Andre Pauli 2026-11-06</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Muller 2 (mar 3 y vie 6)</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -873,7 +876,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -884,6 +887,7 @@
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -1206,7 +1210,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K141"/>
+  <dimension ref="A1:K142"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -5508,10 +5512,10 @@
     </row>
     <row r="138">
       <c r="A138" s="17">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="B138" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C138" s="0" t="s">
         <v>179</v>
@@ -5608,6 +5612,32 @@
       </c>
       <c r="J141" s="0" t="s">
         <v>204</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="18">
+        <v>46332</v>
+      </c>
+      <c r="B142" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C142" s="0" t="s">
+        <v>179</v>
+      </c>
+      <c r="D142" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E142" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="H142" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I142" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="J142" s="0" t="s">
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -5629,7 +5659,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5661,10 +5691,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3">
@@ -5681,10 +5711,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4">
@@ -5701,10 +5731,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5">
@@ -5721,10 +5751,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6">
@@ -5741,10 +5771,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="7">
@@ -5761,10 +5791,10 @@
         <v>1313</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="8">
@@ -5781,10 +5811,10 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9">
@@ -5801,10 +5831,10 @@
         <v>0</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10">
@@ -5821,7 +5851,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11">
@@ -5838,7 +5868,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -5857,57 +5887,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -5955,10 +5985,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3">
@@ -5972,10 +6002,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4">
@@ -5989,10 +6019,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5">
@@ -6000,16 +6030,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="6">
@@ -6023,10 +6053,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="7">
@@ -6040,10 +6070,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="8">
@@ -6057,10 +6087,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="9">
@@ -6068,16 +6098,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10">
@@ -6091,10 +6121,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="11">
@@ -6108,10 +6138,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="12">
@@ -6125,10 +6155,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="13">
@@ -6136,16 +6166,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -6179,10 +6209,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6208,7 +6238,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3">
@@ -6231,7 +6261,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4">
@@ -6254,7 +6284,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5">
@@ -6265,7 +6295,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6277,7 +6307,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="6">
@@ -6300,7 +6330,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="7">
@@ -6323,7 +6353,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8">
@@ -6346,7 +6376,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="9">
@@ -6357,7 +6387,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6369,7 +6399,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="10">
@@ -6392,7 +6422,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="11">
@@ -6415,7 +6445,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="12">
@@ -6438,7 +6468,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13">
@@ -6449,7 +6479,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6461,7 +6491,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="14">
@@ -6484,7 +6514,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="15">
@@ -6495,7 +6525,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6507,7 +6537,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="16">
@@ -6530,7 +6560,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="17">
@@ -6553,7 +6583,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -6574,10 +6604,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6585,46 +6615,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B4" s="0">
         <v>30000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -6645,10 +6675,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6660,10 +6690,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6693,7 +6723,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="3">
@@ -6720,7 +6750,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="4">
@@ -6747,7 +6777,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5">
@@ -6774,7 +6804,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="6">
@@ -6801,7 +6831,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="7">
@@ -6828,7 +6858,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="8">
@@ -6855,7 +6885,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="9">
@@ -6882,7 +6912,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="10">
@@ -6909,7 +6939,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="11">
@@ -6936,7 +6966,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="12">
@@ -6963,7 +6993,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="13">
@@ -6990,12 +7020,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Cassio carga el sabado 31/10
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="271">
   <si>
     <t>fecha</t>
   </si>
@@ -644,6 +644,9 @@
   </si>
   <si>
     <t>dictado 27/10: Muller 2 (mar 3 y vie 6)</t>
+  </si>
+  <si>
+    <t>dictado 27/10: Cassio carga el sabado 31</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -876,7 +879,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -887,6 +890,7 @@
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -1210,7 +1214,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K142"/>
+  <dimension ref="A1:K143"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -5638,6 +5642,32 @@
       </c>
       <c r="J142" s="0" t="s">
         <v>205</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="19">
+        <v>46326</v>
+      </c>
+      <c r="B143" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="C143" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D143" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E143" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="H143" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I143" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="J143" s="0" t="s">
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -5659,7 +5689,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5691,10 +5721,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3">
@@ -5711,10 +5741,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4">
@@ -5731,10 +5761,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5">
@@ -5751,10 +5781,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6">
@@ -5771,10 +5801,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7">
@@ -5791,10 +5821,10 @@
         <v>1313</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8">
@@ -5811,10 +5841,10 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9">
@@ -5831,10 +5861,10 @@
         <v>0</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10">
@@ -5851,7 +5881,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="11">
@@ -5868,7 +5898,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>
@@ -5887,57 +5917,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -5985,10 +6015,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3">
@@ -6002,10 +6032,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4">
@@ -6019,10 +6049,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5">
@@ -6030,16 +6060,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6">
@@ -6053,10 +6083,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="7">
@@ -6070,10 +6100,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="8">
@@ -6087,10 +6117,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9">
@@ -6098,16 +6128,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="10">
@@ -6121,10 +6151,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="11">
@@ -6138,10 +6168,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="12">
@@ -6155,10 +6185,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="13">
@@ -6166,16 +6196,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -6209,10 +6239,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6238,7 +6268,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="3">
@@ -6261,7 +6291,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4">
@@ -6284,7 +6314,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5">
@@ -6295,7 +6325,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6307,7 +6337,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6">
@@ -6330,7 +6360,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7">
@@ -6353,7 +6383,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8">
@@ -6376,7 +6406,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9">
@@ -6387,7 +6417,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6399,7 +6429,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10">
@@ -6422,7 +6452,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="11">
@@ -6445,7 +6475,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="12">
@@ -6468,7 +6498,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13">
@@ -6479,7 +6509,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6491,7 +6521,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14">
@@ -6514,7 +6544,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="15">
@@ -6525,7 +6555,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6537,7 +6567,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="16">
@@ -6560,7 +6590,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="17">
@@ -6583,7 +6613,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -6604,10 +6634,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6615,46 +6645,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B4" s="0">
         <v>30000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -6675,10 +6705,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6690,10 +6720,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6723,7 +6753,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3">
@@ -6750,7 +6780,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4">
@@ -6777,7 +6807,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5">
@@ -6804,7 +6834,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6">
@@ -6831,7 +6861,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7">
@@ -6858,7 +6888,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8">
@@ -6885,7 +6915,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9">
@@ -6912,7 +6942,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10">
@@ -6939,7 +6969,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11">
@@ -6966,7 +6996,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="12">
@@ -6993,7 +7023,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="13">
@@ -7020,12 +7050,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Cassio del viernes 6 al miercoles 4
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -571,7 +571,7 @@
     <t>dictado 27/10: Cassio 2026-11-03</t>
   </si>
   <si>
-    <t>dictado 27/10: Cassio 2026-11-06</t>
+    <t>dictado 27/10: Cassio 2026-11-06; 28/10: pasa del vie 6 al mie 4 (dictado)</t>
   </si>
   <si>
     <t>dictado 27/10: Cassio 2026-11-07</t>
@@ -4996,10 +4996,10 @@
     </row>
     <row r="118">
       <c r="A118" s="16">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="B118" s="0" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C118" s="0" t="s">
         <v>179</v>

</xml_diff>

<commit_message>
plan de compras: semana 2-7/11 re-dictada con transportistas; sale BAHIA del mie 4
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="272">
   <si>
     <t>fecha</t>
   </si>
@@ -565,88 +565,91 @@
     <t>2026-10-31</t>
   </si>
   <si>
+    <t>dictado 27/10: Cassio carga el sabado 31</t>
+  </si>
+  <si>
     <t>2026-11-01</t>
   </si>
   <si>
-    <t>dictado 27/10: Cassio 2026-11-03</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Cassio 2026-11-06; 28/10: pasa del vie 6 al mie 4 (dictado)</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Cassio 2026-11-07</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Gilson 2026-11-03</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Gilson 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Stein 2026-11-03</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Stein 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Agrocurupa 2026-11-04</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Agrocurupa 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Muller Fabricio 2026-11-06; 27/10: pasa del vie 6 al mar 3 (dictado)</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Jaime Zimerman 2026-11-04</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Jaime Zimerman 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Aryste Mittelman 2026-11-04</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Aryste Mittelman 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Shapo 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Wagner 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Marconi 2026-11-04</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Josemar 2026-11-06; 27/10: pasa del vie 6 al mar 3 (dictado)</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Jhony Viera 2026-11-06; 27/10: pasa del vie 6 al mar 3 (dictado)</t>
-  </si>
-  <si>
-    <t>dictado 27/10: BAHIA 2026-11-04</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Fisher 2026-11-04</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Fisher 2026-11-06; 27/10: pasa del vie 6 al mar 3 (dictado)</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Fisher 2026-11-07</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Andre Pauli 2026-11-04</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Andre Pauli 2026-11-06</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Muller 2 (mar 3 y vie 6)</t>
-  </si>
-  <si>
-    <t>dictado 27/10: Cassio carga el sabado 31</t>
+    <t>Gonzalo 29/10 (chat)</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Fisher 2026-11-03 Amaro</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Fisher 2026-11-04 Amaro</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Fisher 2026-11-07 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Cassio 2026-11-03 Axt</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Cassio 2026-11-04 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Cassio 2026-11-07 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Gilson 2026-11-03 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Gilson 2026-11-06 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Stein 2026-11-03 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Stein 2026-11-06 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Agrocurupa 2026-11-04 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Agrocurupa 2026-11-06 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Muller Fabricio 2026-11-03 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Muller Fabricio 2026-11-06 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Jaime Zimerman 2026-11-04 Chabat</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Jaime Zimerman 2026-11-06 Chabat</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Aryste Mittelman 2026-11-03 Chabat</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Aryste Mittelman 2026-11-04 Chabat</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Aryste Mittelman 2026-11-06 Chabat</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Andre Pauli 2026-11-04 Chabat</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Andre Pauli 2026-11-06 Chabat</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Shapo 2026-11-06 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Wagner 2026-11-06 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Marconi 2026-11-06 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Josemar 2026-11-06 Nilton</t>
+  </si>
+  <si>
+    <t>dictado 29/10: Jhony Viera 2026-11-03 Nilton</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -879,7 +882,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -890,8 +893,6 @@
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -4970,13 +4971,13 @@
     </row>
     <row r="117">
       <c r="A117" s="16">
-        <v>46329</v>
+        <v>46326</v>
       </c>
       <c r="B117" s="0" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C117" s="0" t="s">
-        <v>179</v>
+        <v>152</v>
       </c>
       <c r="D117" s="0" t="s">
         <v>24</v>
@@ -4991,501 +4992,558 @@
         <v>169</v>
       </c>
       <c r="J117" s="0" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="17">
+        <v>46329</v>
+      </c>
+      <c r="B118" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C118" s="0" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="16">
+      <c r="D118" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E118" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="F118" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="H118" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I118" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="J118" s="0" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="17">
         <v>46330</v>
       </c>
-      <c r="B118" s="0" t="s">
+      <c r="B119" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="C118" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="D118" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E118" s="0" t="s">
+      <c r="C119" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="D119" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E119" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="F119" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="H119" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I119" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="J119" s="0" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="17">
+        <v>46333</v>
+      </c>
+      <c r="B120" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="C120" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="D120" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E120" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="F120" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="H120" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I120" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="J120" s="0" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="17">
+        <v>46329</v>
+      </c>
+      <c r="B121" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C121" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="D121" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E121" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="H118" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I118" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="J118" s="0" t="s">
+      <c r="F121" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H121" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I121" s="0" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="16">
+      <c r="J121" s="0" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="17">
+        <v>46330</v>
+      </c>
+      <c r="B122" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C122" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="D122" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E122" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F122" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="H122" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I122" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="J122" s="0" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="17">
         <v>46333</v>
       </c>
-      <c r="B119" s="0" t="s">
+      <c r="B123" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="C119" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="D119" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E119" s="0" t="s">
+      <c r="C123" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="D123" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E123" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="H119" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I119" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="J119" s="0" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="16">
+      <c r="F123" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="H123" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I123" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="J123" s="0" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="17">
         <v>46329</v>
       </c>
-      <c r="B120" s="0" t="s">
+      <c r="B124" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="C120" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="D120" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E120" s="0" t="s">
+      <c r="C124" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="D124" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E124" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="H120" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I120" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="J120" s="0" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="16">
-        <v>46332</v>
-      </c>
-      <c r="B121" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C121" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="D121" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E121" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="H121" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I121" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="J121" s="0" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="16">
-        <v>46329</v>
-      </c>
-      <c r="B122" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="C122" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="D122" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E122" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="H122" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I122" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="J122" s="0" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="16">
-        <v>46332</v>
-      </c>
-      <c r="B123" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C123" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="D123" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E123" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="H123" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I123" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="J123" s="0" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="16">
-        <v>46330</v>
-      </c>
-      <c r="B124" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="C124" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="D124" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E124" s="0" t="s">
-        <v>40</v>
+      <c r="F124" s="0" t="s">
+        <v>41</v>
       </c>
       <c r="H124" s="0">
         <v>1008</v>
       </c>
       <c r="I124" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J124" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="16">
+      <c r="A125" s="17">
         <v>46332</v>
       </c>
       <c r="B125" s="0" t="s">
         <v>23</v>
       </c>
       <c r="C125" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D125" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E125" s="0" t="s">
-        <v>40</v>
+        <v>43</v>
+      </c>
+      <c r="F125" s="0" t="s">
+        <v>41</v>
       </c>
       <c r="H125" s="0">
         <v>1008</v>
       </c>
       <c r="I125" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J125" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="16">
+      <c r="A126" s="17">
         <v>46329</v>
       </c>
       <c r="B126" s="0" t="s">
         <v>21</v>
       </c>
       <c r="C126" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D126" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E126" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F126" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="H126" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I126" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="J126" s="0" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="17">
+        <v>46332</v>
+      </c>
+      <c r="B127" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C127" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="D127" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E127" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="F127" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="H127" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I127" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="J127" s="0" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="17">
+        <v>46330</v>
+      </c>
+      <c r="B128" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C128" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="D128" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E128" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="F128" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="H128" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I128" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="J128" s="0" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="17">
+        <v>46332</v>
+      </c>
+      <c r="B129" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C129" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="D129" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E129" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="F129" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="H129" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I129" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="J129" s="0" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="17">
+        <v>46329</v>
+      </c>
+      <c r="B130" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C130" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="D130" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E130" s="0" t="s">
         <v>122</v>
       </c>
-      <c r="H126" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I126" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="J126" s="0" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="16">
-        <v>46330</v>
-      </c>
-      <c r="B127" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="C127" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="D127" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E127" s="0" t="s">
-        <v>140</v>
-      </c>
-      <c r="H127" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I127" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="J127" s="0" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="16">
-        <v>46332</v>
-      </c>
-      <c r="B128" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C128" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="D128" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E128" s="0" t="s">
-        <v>140</v>
-      </c>
-      <c r="H128" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I128" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="J128" s="0" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="16">
-        <v>46330</v>
-      </c>
-      <c r="B129" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="C129" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="D129" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E129" s="0" t="s">
-        <v>172</v>
-      </c>
-      <c r="H129" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I129" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="J129" s="0" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="16">
-        <v>46332</v>
-      </c>
-      <c r="B130" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C130" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="D130" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E130" s="0" t="s">
-        <v>172</v>
+      <c r="F130" s="0" t="s">
+        <v>41</v>
       </c>
       <c r="H130" s="0">
         <v>1008</v>
       </c>
       <c r="I130" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J130" s="0" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="16">
+      <c r="A131" s="17">
         <v>46332</v>
       </c>
       <c r="B131" s="0" t="s">
         <v>23</v>
       </c>
       <c r="C131" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D131" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E131" s="0" t="s">
-        <v>105</v>
+        <v>122</v>
+      </c>
+      <c r="F131" s="0" t="s">
+        <v>41</v>
       </c>
       <c r="H131" s="0">
         <v>1008</v>
       </c>
       <c r="I131" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J131" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="16">
+      <c r="A132" s="17">
+        <v>46330</v>
+      </c>
+      <c r="B132" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C132" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="D132" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E132" s="0" t="s">
+        <v>140</v>
+      </c>
+      <c r="F132" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="H132" s="0">
+        <v>1008</v>
+      </c>
+      <c r="I132" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="J132" s="0" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="17">
         <v>46332</v>
       </c>
-      <c r="B132" s="0" t="s">
+      <c r="B133" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="C132" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="D132" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E132" s="0" t="s">
-        <v>146</v>
-      </c>
-      <c r="H132" s="0">
-        <v>1008</v>
-      </c>
-      <c r="I132" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="J132" s="0" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="16">
-        <v>46330</v>
-      </c>
-      <c r="B133" s="0" t="s">
-        <v>52</v>
-      </c>
       <c r="C133" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D133" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E133" s="0" t="s">
-        <v>60</v>
+        <v>140</v>
+      </c>
+      <c r="F133" s="0" t="s">
+        <v>56</v>
       </c>
       <c r="H133" s="0">
         <v>1008</v>
       </c>
       <c r="I133" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J133" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="16">
+      <c r="A134" s="17">
         <v>46329</v>
       </c>
       <c r="B134" s="0" t="s">
         <v>21</v>
       </c>
       <c r="C134" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D134" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E134" s="0" t="s">
-        <v>58</v>
+        <v>172</v>
+      </c>
+      <c r="F134" s="0" t="s">
+        <v>56</v>
       </c>
       <c r="H134" s="0">
         <v>1008</v>
       </c>
       <c r="I134" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J134" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="16">
-        <v>46329</v>
+      <c r="A135" s="17">
+        <v>46330</v>
       </c>
       <c r="B135" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C135" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D135" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E135" s="0" t="s">
-        <v>113</v>
+        <v>172</v>
+      </c>
+      <c r="F135" s="0" t="s">
+        <v>56</v>
       </c>
       <c r="H135" s="0">
         <v>1008</v>
       </c>
       <c r="I135" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J135" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="16">
-        <v>46330</v>
+      <c r="A136" s="17">
+        <v>46332</v>
       </c>
       <c r="B136" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C136" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D136" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E136" s="0" t="s">
-        <v>130</v>
+        <v>172</v>
+      </c>
+      <c r="F136" s="0" t="s">
+        <v>56</v>
       </c>
       <c r="H136" s="0">
         <v>1008</v>
       </c>
       <c r="I136" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J136" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="137">
@@ -5496,100 +5554,112 @@
         <v>52</v>
       </c>
       <c r="C137" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D137" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E137" s="0" t="s">
-        <v>31</v>
+        <v>161</v>
+      </c>
+      <c r="F137" s="0" t="s">
+        <v>56</v>
       </c>
       <c r="H137" s="0">
         <v>1008</v>
       </c>
       <c r="I137" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J137" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="17">
-        <v>46329</v>
+        <v>46332</v>
       </c>
       <c r="B138" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C138" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D138" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E138" s="0" t="s">
-        <v>31</v>
+        <v>161</v>
+      </c>
+      <c r="F138" s="0" t="s">
+        <v>56</v>
       </c>
       <c r="H138" s="0">
         <v>1008</v>
       </c>
       <c r="I138" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J138" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="17">
-        <v>46333</v>
+        <v>46332</v>
       </c>
       <c r="B139" s="0" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C139" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D139" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E139" s="0" t="s">
-        <v>31</v>
+        <v>105</v>
+      </c>
+      <c r="F139" s="0" t="s">
+        <v>41</v>
       </c>
       <c r="H139" s="0">
         <v>1008</v>
       </c>
       <c r="I139" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J139" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="17">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B140" s="0" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C140" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D140" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E140" s="0" t="s">
-        <v>161</v>
+        <v>146</v>
+      </c>
+      <c r="F140" s="0" t="s">
+        <v>41</v>
       </c>
       <c r="H140" s="0">
         <v>1008</v>
       </c>
       <c r="I140" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J140" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="141">
@@ -5600,74 +5670,83 @@
         <v>23</v>
       </c>
       <c r="C141" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D141" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E141" s="0" t="s">
-        <v>161</v>
+        <v>60</v>
+      </c>
+      <c r="F141" s="0" t="s">
+        <v>41</v>
       </c>
       <c r="H141" s="0">
         <v>1008</v>
       </c>
       <c r="I141" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J141" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="18">
+      <c r="A142" s="17">
         <v>46332</v>
       </c>
       <c r="B142" s="0" t="s">
         <v>23</v>
       </c>
       <c r="C142" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D142" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E142" s="0" t="s">
-        <v>122</v>
+        <v>58</v>
+      </c>
+      <c r="F142" s="0" t="s">
+        <v>41</v>
       </c>
       <c r="H142" s="0">
         <v>1008</v>
       </c>
       <c r="I142" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J142" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="19">
-        <v>46326</v>
+      <c r="A143" s="17">
+        <v>46329</v>
       </c>
       <c r="B143" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C143" s="0" t="s">
-        <v>152</v>
+        <v>180</v>
       </c>
       <c r="D143" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E143" s="0" t="s">
-        <v>27</v>
+        <v>113</v>
+      </c>
+      <c r="F143" s="0" t="s">
+        <v>41</v>
       </c>
       <c r="H143" s="0">
         <v>1008</v>
       </c>
       <c r="I143" s="0" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J143" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -5689,7 +5768,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>24</v>
@@ -5721,10 +5800,10 @@
         <v>1492</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3">
@@ -5741,10 +5820,10 @@
         <v>705</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4">
@@ -5761,10 +5840,10 @@
         <v>1050</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5">
@@ -5781,10 +5860,10 @@
         <v>1050</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="6">
@@ -5801,10 +5880,10 @@
         <v>1188</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="7">
@@ -5821,10 +5900,10 @@
         <v>1313</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8">
@@ -5841,10 +5920,10 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9">
@@ -5861,10 +5940,10 @@
         <v>0</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10">
@@ -5881,7 +5960,7 @@
         <v>1386</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11">
@@ -5898,7 +5977,7 @@
         <v>1386</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -5917,57 +5996,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -6015,10 +6094,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="3">
@@ -6032,10 +6111,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4">
@@ -6049,10 +6128,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="5">
@@ -6060,16 +6139,16 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6">
@@ -6083,10 +6162,10 @@
         <v>11653</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="7">
@@ -6100,10 +6179,10 @@
         <v>13673</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="8">
@@ -6117,10 +6196,10 @@
         <v>1646</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="9">
@@ -6128,16 +6207,16 @@
         <v>46291</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C9" s="0">
         <v>21737</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="10">
@@ -6151,10 +6230,10 @@
         <v>12269</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="11">
@@ -6168,10 +6247,10 @@
         <v>9676</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="12">
@@ -6185,10 +6264,10 @@
         <v>1500</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13">
@@ -6196,16 +6275,16 @@
         <v>46298</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C13" s="0">
         <v>7993</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -6239,10 +6318,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -6268,7 +6347,7 @@
         <v>21026</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3">
@@ -6291,7 +6370,7 @@
         <v>10628</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4">
@@ -6314,7 +6393,7 @@
         <v>1958</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5">
@@ -6325,7 +6404,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D5" s="0">
         <v>996</v>
@@ -6337,7 +6416,7 @@
         <v>23023</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6">
@@ -6360,7 +6439,7 @@
         <v>19725</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="7">
@@ -6383,7 +6462,7 @@
         <v>11881</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="8">
@@ -6406,7 +6485,7 @@
         <v>1844</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="9">
@@ -6417,7 +6496,7 @@
         <v>52</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D9" s="0">
         <v>942</v>
@@ -6429,7 +6508,7 @@
         <v>22081</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10">
@@ -6452,7 +6531,7 @@
         <v>15893</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11">
@@ -6475,7 +6554,7 @@
         <v>14132</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12">
@@ -6498,7 +6577,7 @@
         <v>1972</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="13">
@@ -6509,7 +6588,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D13" s="0">
         <v>832</v>
@@ -6521,7 +6600,7 @@
         <v>20033</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="14">
@@ -6544,7 +6623,7 @@
         <v>12452</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="15">
@@ -6555,7 +6634,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D15" s="0">
         <v>855</v>
@@ -6567,7 +6646,7 @@
         <v>21955</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="16">
@@ -6590,7 +6669,7 @@
         <v>14786</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="17">
@@ -6613,7 +6692,7 @@
         <v>2017</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>
@@ -6634,10 +6713,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>9</v>
@@ -6645,46 +6724,46 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B2" s="0">
         <v>0</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B4" s="0">
         <v>30000</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B5" s="0">
         <v>18000</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -6705,10 +6784,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>24</v>
@@ -6720,10 +6799,10 @@
         <v>85</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>8</v>
@@ -6753,7 +6832,7 @@
         <v>14493</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3">
@@ -6780,7 +6859,7 @@
         <v>12498</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4">
@@ -6807,7 +6886,7 @@
         <v>14754</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5">
@@ -6834,7 +6913,7 @@
         <v>13944</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="6">
@@ -6861,7 +6940,7 @@
         <v>15938</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7">
@@ -6888,7 +6967,7 @@
         <v>14989</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="8">
@@ -6915,7 +6994,7 @@
         <v>13936</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="9">
@@ -6942,7 +7021,7 @@
         <v>14742</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="10">
@@ -6969,7 +7048,7 @@
         <v>17274</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="11">
@@ -6996,7 +7075,7 @@
         <v>16549</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="12">
@@ -7023,7 +7102,7 @@
         <v>15851</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="13">
@@ -7050,12 +7129,12 @@
         <v>14845</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
plan de compras: Jhony del martes 3 al viernes 6
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/plan_compras.xlsx
+++ b/plan_compras/plan_compras.xlsx
@@ -649,7 +649,7 @@
     <t>dictado 29/10: Josemar 2026-11-06 Nilton</t>
   </si>
   <si>
-    <t>dictado 29/10: Jhony Viera 2026-11-03 Nilton</t>
+    <t>dictado 29/10: Jhony Viera 2026-11-03 Nilton; 29/10: pasa del mar 3 al vie 6 (Gonzalo)</t>
   </si>
   <si>
     <t>semana_lunes</t>
@@ -5722,10 +5722,10 @@
     </row>
     <row r="143">
       <c r="A143" s="17">
-        <v>46329</v>
+        <v>46332</v>
       </c>
       <c r="B143" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C143" s="0" t="s">
         <v>180</v>

</xml_diff>